<commit_message>
feat: add refused colis and make it working, also fix a lot of bugs
</commit_message>
<xml_diff>
--- a/dummy-content/ECHEC-RETOUR_CLIENT-CASABLANCA.xlsx
+++ b/dummy-content/ECHEC-RETOUR_CLIENT-CASABLANCA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User1\Desktop\GoFleet-Enhancer\dummy-content\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3337EC3B-4410-4E6D-88D5-BB7A2B0EA9F5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65E33A46-2CCE-473D-A1E8-442A141F2726}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12110" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12110" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ECHEC CASA" sheetId="5" r:id="rId1"/>
@@ -100,7 +100,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="31">
+  <fonts count="29">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -112,21 +112,25 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="16"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -134,47 +138,55 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="13"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -182,29 +194,34 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="13"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <color rgb="FF212529"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
@@ -229,36 +246,6 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color rgb="FF212529"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -291,6 +278,22 @@
       <name val="IDAutomationHC39M Free Version"/>
       <family val="1"/>
       <charset val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="22">
@@ -1270,7 +1273,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="164">
+  <cellXfs count="160">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="15" fillId="13" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1322,64 +1325,18 @@
     <xf numFmtId="0" fontId="20" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="21" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="11" fontId="22" fillId="21" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="11" fontId="23" fillId="21" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="11" fontId="16" fillId="21" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -1412,10 +1369,141 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="71" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="15" fillId="21" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="21" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="15" fillId="21" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="65" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="15" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1444,95 +1532,18 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="19" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="65" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="26" fillId="14" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="17" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1547,26 +1558,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="20" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="19" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="28" fillId="3" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1890,121 +1881,121 @@
   <dimension ref="A1:K67"/>
   <sheetFormatPr defaultRowHeight="12.5"/>
   <cols>
-    <col min="1" max="1" width="23.54296875" style="40" customWidth="1"/>
-    <col min="2" max="2" width="13.26953125" style="40" customWidth="1"/>
-    <col min="3" max="3" width="4.90625" style="40" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="8.7265625" style="40"/>
-    <col min="5" max="5" width="29.81640625" style="40" customWidth="1"/>
-    <col min="6" max="9" width="14.54296875" style="40" customWidth="1"/>
-    <col min="10" max="10" width="8.7265625" style="40"/>
-    <col min="11" max="11" width="17.453125" style="40" customWidth="1"/>
+    <col min="1" max="1" width="23.54296875" style="28" customWidth="1"/>
+    <col min="2" max="2" width="13.26953125" style="28" customWidth="1"/>
+    <col min="3" max="3" width="4.90625" style="28" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="8.7265625" style="28"/>
+    <col min="5" max="5" width="29.81640625" style="28" customWidth="1"/>
+    <col min="6" max="9" width="14.54296875" style="28" customWidth="1"/>
+    <col min="10" max="10" width="8.7265625" style="28"/>
+    <col min="11" max="11" width="17.453125" style="28" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.5" customHeight="1">
-      <c r="A1" s="77"/>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="82" t="s">
+      <c r="A1" s="128"/>
+      <c r="B1" s="129"/>
+      <c r="C1" s="129"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="133" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="83"/>
-      <c r="G1" s="84"/>
-      <c r="H1" s="41"/>
-      <c r="I1" s="88" t="s">
+      <c r="F1" s="134"/>
+      <c r="G1" s="135"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="139" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="89"/>
-      <c r="K1" s="90"/>
+      <c r="J1" s="140"/>
+      <c r="K1" s="141"/>
     </row>
     <row r="2" spans="1:11" ht="15.5">
-      <c r="A2" s="79"/>
-      <c r="B2" s="80"/>
-      <c r="C2" s="81"/>
-      <c r="D2" s="69"/>
-      <c r="E2" s="85"/>
-      <c r="F2" s="86"/>
-      <c r="G2" s="87"/>
+      <c r="A2" s="130"/>
+      <c r="B2" s="131"/>
+      <c r="C2" s="132"/>
+      <c r="D2" s="53"/>
+      <c r="E2" s="136"/>
+      <c r="F2" s="137"/>
+      <c r="G2" s="138"/>
       <c r="H2" s="15"/>
-      <c r="I2" s="91">
+      <c r="I2" s="142">
         <f ca="1">TODAY()</f>
-        <v>45804</v>
-      </c>
-      <c r="J2" s="86"/>
-      <c r="K2" s="87"/>
+        <v>45811</v>
+      </c>
+      <c r="J2" s="137"/>
+      <c r="K2" s="138"/>
     </row>
     <row r="3" spans="1:11">
-      <c r="A3" s="46"/>
+      <c r="A3" s="32"/>
       <c r="B3" s="22"/>
       <c r="C3" s="13"/>
-      <c r="D3" s="52"/>
+      <c r="D3" s="36"/>
       <c r="E3" s="11"/>
       <c r="F3" s="22"/>
-      <c r="G3" s="47"/>
+      <c r="G3" s="33"/>
       <c r="H3" s="25"/>
       <c r="I3" s="22"/>
       <c r="J3" s="22"/>
-      <c r="K3" s="47"/>
+      <c r="K3" s="33"/>
     </row>
     <row r="4" spans="1:11" ht="17">
-      <c r="A4" s="92" t="s">
+      <c r="A4" s="143" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="93"/>
-      <c r="C4" s="94"/>
-      <c r="D4" s="68"/>
+      <c r="B4" s="113"/>
+      <c r="C4" s="72"/>
+      <c r="D4" s="52"/>
       <c r="E4" s="16" t="s">
         <v>21</v>
       </c>
       <c r="F4" s="1"/>
-      <c r="G4" s="71"/>
+      <c r="G4" s="55"/>
       <c r="H4" s="15"/>
       <c r="I4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="95"/>
-      <c r="K4" s="96"/>
+      <c r="J4" s="144"/>
+      <c r="K4" s="115"/>
     </row>
     <row r="5" spans="1:11" ht="18.5">
-      <c r="A5" s="97" t="s">
+      <c r="A5" s="121" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="98"/>
-      <c r="C5" s="99"/>
+      <c r="B5" s="80"/>
+      <c r="C5" s="96"/>
       <c r="D5" s="14"/>
-      <c r="E5" s="102" t="s">
+      <c r="E5" s="122" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="103"/>
-      <c r="G5" s="104"/>
+      <c r="F5" s="123"/>
+      <c r="G5" s="124"/>
       <c r="H5" s="22"/>
       <c r="I5" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="J5" s="105"/>
-      <c r="K5" s="96"/>
+      <c r="J5" s="125"/>
+      <c r="K5" s="115"/>
     </row>
     <row r="6" spans="1:11" ht="15.5">
-      <c r="A6" s="100"/>
-      <c r="B6" s="94"/>
-      <c r="C6" s="101"/>
+      <c r="A6" s="97"/>
+      <c r="B6" s="72"/>
+      <c r="C6" s="73"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="106" t="s">
+      <c r="E6" s="126" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="94"/>
-      <c r="G6" s="107"/>
-      <c r="H6" s="62"/>
+      <c r="F6" s="72"/>
+      <c r="G6" s="89"/>
+      <c r="H6" s="46"/>
       <c r="I6" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="J6" s="108">
+      <c r="J6" s="127">
         <v>1230</v>
       </c>
-      <c r="K6" s="96"/>
+      <c r="K6" s="115"/>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="46"/>
+      <c r="A7" s="32"/>
       <c r="B7" s="22"/>
       <c r="C7" s="22"/>
       <c r="D7" s="22"/>
@@ -2014,52 +2005,52 @@
       <c r="H7" s="22"/>
       <c r="I7" s="22"/>
       <c r="J7" s="22"/>
-      <c r="K7" s="47"/>
+      <c r="K7" s="33"/>
     </row>
     <row r="8" spans="1:11" ht="15.5">
-      <c r="A8" s="122" t="s">
+      <c r="A8" s="107" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="72" t="s">
+      <c r="B8" s="56" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="124" t="s">
+      <c r="C8" s="109" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="125"/>
-      <c r="E8" s="126"/>
+      <c r="D8" s="110"/>
+      <c r="E8" s="111"/>
       <c r="F8" s="14"/>
-      <c r="G8" s="127" t="s">
+      <c r="G8" s="112" t="s">
         <v>12</v>
       </c>
-      <c r="H8" s="93"/>
+      <c r="H8" s="113"/>
       <c r="I8" s="14"/>
-      <c r="J8" s="128" t="s">
+      <c r="J8" s="114" t="s">
         <v>13</v>
       </c>
-      <c r="K8" s="96"/>
+      <c r="K8" s="115"/>
     </row>
     <row r="9" spans="1:11" ht="17">
-      <c r="A9" s="123"/>
-      <c r="B9" s="73" t="s">
+      <c r="A9" s="108"/>
+      <c r="B9" s="57" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="129" t="s">
+      <c r="C9" s="116" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="94"/>
-      <c r="E9" s="114"/>
+      <c r="D9" s="72"/>
+      <c r="E9" s="81"/>
       <c r="F9" s="22"/>
-      <c r="G9" s="113">
+      <c r="G9" s="87">
         <v>1</v>
       </c>
-      <c r="H9" s="114"/>
+      <c r="H9" s="81"/>
       <c r="I9" s="22"/>
-      <c r="J9" s="115"/>
-      <c r="K9" s="107"/>
+      <c r="J9" s="88"/>
+      <c r="K9" s="89"/>
     </row>
     <row r="10" spans="1:11">
-      <c r="A10" s="46"/>
+      <c r="A10" s="32"/>
       <c r="B10" s="22"/>
       <c r="C10" s="22"/>
       <c r="D10" s="22"/>
@@ -2069,340 +2060,340 @@
       <c r="H10" s="19"/>
       <c r="I10" s="19"/>
       <c r="J10" s="22"/>
-      <c r="K10" s="48"/>
+      <c r="K10" s="34"/>
     </row>
     <row r="11" spans="1:11" ht="18.5">
-      <c r="A11" s="116" t="s">
+      <c r="A11" s="90" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="117"/>
-      <c r="C11" s="117"/>
-      <c r="D11" s="117"/>
-      <c r="E11" s="118"/>
-      <c r="F11" s="119"/>
-      <c r="G11" s="117"/>
-      <c r="H11" s="117"/>
-      <c r="I11" s="117"/>
-      <c r="J11" s="117"/>
-      <c r="K11" s="120"/>
-    </row>
-    <row r="12" spans="1:11" ht="13">
-      <c r="A12" s="121" t="s">
+      <c r="B11" s="91"/>
+      <c r="C11" s="91"/>
+      <c r="D11" s="91"/>
+      <c r="E11" s="92"/>
+      <c r="F11" s="93"/>
+      <c r="G11" s="91"/>
+      <c r="H11" s="91"/>
+      <c r="I11" s="91"/>
+      <c r="J11" s="91"/>
+      <c r="K11" s="94"/>
+    </row>
+    <row r="12" spans="1:11">
+      <c r="A12" s="95" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="99"/>
-      <c r="C12" s="99"/>
-      <c r="D12" s="99"/>
-      <c r="E12" s="114"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="44"/>
-      <c r="H12" s="49"/>
-      <c r="I12" s="45"/>
-      <c r="J12" s="130"/>
-      <c r="K12" s="131"/>
+      <c r="B12" s="96"/>
+      <c r="C12" s="96"/>
+      <c r="D12" s="96"/>
+      <c r="E12" s="81"/>
+      <c r="F12" s="59"/>
+      <c r="G12" s="31"/>
+      <c r="H12" s="60"/>
+      <c r="I12" s="31"/>
+      <c r="J12" s="117"/>
+      <c r="K12" s="118"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="100"/>
-      <c r="B13" s="94"/>
-      <c r="C13" s="94"/>
-      <c r="D13" s="94"/>
-      <c r="E13" s="101"/>
+      <c r="A13" s="97"/>
+      <c r="B13" s="72"/>
+      <c r="C13" s="72"/>
+      <c r="D13" s="72"/>
+      <c r="E13" s="73"/>
       <c r="F13" s="27"/>
-      <c r="G13" s="29"/>
-      <c r="H13" s="30"/>
+      <c r="G13" s="61"/>
+      <c r="H13" s="62"/>
       <c r="I13" s="2"/>
-      <c r="J13" s="75"/>
-      <c r="K13" s="76"/>
+      <c r="J13" s="119"/>
+      <c r="K13" s="120"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="155" t="str">
-        <f>""&amp;A12&amp;""</f>
-        <v>GOFEMM20052025001</v>
-      </c>
-      <c r="B14" s="156"/>
-      <c r="C14" s="156"/>
-      <c r="D14" s="156"/>
-      <c r="E14" s="157"/>
+      <c r="A14" s="98" t="str">
+        <f>"*"&amp;A12&amp;"*"</f>
+        <v>*GOFEMM20052025001*</v>
+      </c>
+      <c r="B14" s="99"/>
+      <c r="C14" s="99"/>
+      <c r="D14" s="99"/>
+      <c r="E14" s="100"/>
       <c r="F14" s="27"/>
-      <c r="G14" s="30"/>
-      <c r="H14" s="30"/>
+      <c r="G14" s="62"/>
+      <c r="H14" s="62"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="75"/>
-      <c r="K14" s="76"/>
+      <c r="J14" s="119"/>
+      <c r="K14" s="120"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="158"/>
-      <c r="B15" s="159"/>
-      <c r="C15" s="159"/>
-      <c r="D15" s="159"/>
-      <c r="E15" s="160"/>
+      <c r="A15" s="101"/>
+      <c r="B15" s="102"/>
+      <c r="C15" s="102"/>
+      <c r="D15" s="102"/>
+      <c r="E15" s="103"/>
       <c r="F15" s="27"/>
-      <c r="G15" s="30"/>
-      <c r="H15" s="30"/>
+      <c r="G15" s="62"/>
+      <c r="H15" s="62"/>
       <c r="I15" s="2"/>
-      <c r="J15" s="75"/>
-      <c r="K15" s="76"/>
+      <c r="J15" s="119"/>
+      <c r="K15" s="120"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="158"/>
-      <c r="B16" s="159"/>
-      <c r="C16" s="159"/>
-      <c r="D16" s="159"/>
-      <c r="E16" s="160"/>
-      <c r="F16" s="31"/>
-      <c r="G16" s="30"/>
-      <c r="H16" s="30"/>
+      <c r="A16" s="101"/>
+      <c r="B16" s="102"/>
+      <c r="C16" s="102"/>
+      <c r="D16" s="102"/>
+      <c r="E16" s="103"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="62"/>
+      <c r="H16" s="62"/>
       <c r="I16" s="2"/>
-      <c r="J16" s="75"/>
-      <c r="K16" s="76"/>
+      <c r="J16" s="119"/>
+      <c r="K16" s="120"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="158"/>
-      <c r="B17" s="159"/>
-      <c r="C17" s="159"/>
-      <c r="D17" s="159"/>
-      <c r="E17" s="160"/>
+      <c r="A17" s="101"/>
+      <c r="B17" s="102"/>
+      <c r="C17" s="102"/>
+      <c r="D17" s="102"/>
+      <c r="E17" s="103"/>
       <c r="F17" s="27"/>
-      <c r="G17" s="30"/>
-      <c r="H17" s="30"/>
+      <c r="G17" s="62"/>
+      <c r="H17" s="62"/>
       <c r="I17" s="2"/>
-      <c r="J17" s="75"/>
-      <c r="K17" s="76"/>
+      <c r="J17" s="119"/>
+      <c r="K17" s="120"/>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="158"/>
-      <c r="B18" s="159"/>
-      <c r="C18" s="159"/>
-      <c r="D18" s="159"/>
-      <c r="E18" s="160"/>
+      <c r="A18" s="101"/>
+      <c r="B18" s="102"/>
+      <c r="C18" s="102"/>
+      <c r="D18" s="102"/>
+      <c r="E18" s="103"/>
       <c r="F18" s="27"/>
-      <c r="G18" s="30"/>
-      <c r="H18" s="30"/>
+      <c r="G18" s="62"/>
+      <c r="H18" s="62"/>
       <c r="I18" s="8"/>
-      <c r="J18" s="75"/>
-      <c r="K18" s="76"/>
+      <c r="J18" s="119"/>
+      <c r="K18" s="120"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="161"/>
-      <c r="B19" s="162"/>
-      <c r="C19" s="162"/>
-      <c r="D19" s="162"/>
-      <c r="E19" s="163"/>
-      <c r="F19" s="32"/>
-      <c r="G19" s="30"/>
-      <c r="H19" s="30"/>
-      <c r="I19" s="28"/>
-      <c r="J19" s="75"/>
-      <c r="K19" s="76"/>
-    </row>
-    <row r="20" spans="1:11" ht="13">
-      <c r="A20" s="46"/>
+      <c r="A19" s="104"/>
+      <c r="B19" s="105"/>
+      <c r="C19" s="105"/>
+      <c r="D19" s="105"/>
+      <c r="E19" s="106"/>
+      <c r="F19" s="63"/>
+      <c r="G19" s="62"/>
+      <c r="H19" s="62"/>
+      <c r="I19" s="27"/>
+      <c r="J19" s="119"/>
+      <c r="K19" s="120"/>
+    </row>
+    <row r="20" spans="1:11">
+      <c r="A20" s="32"/>
       <c r="B20" s="22"/>
       <c r="C20" s="22"/>
       <c r="D20" s="22"/>
       <c r="E20" s="22"/>
-      <c r="F20" s="32"/>
-      <c r="G20" s="50"/>
-      <c r="H20" s="30"/>
-      <c r="I20" s="28"/>
-      <c r="J20" s="75"/>
-      <c r="K20" s="76"/>
+      <c r="F20" s="63"/>
+      <c r="G20" s="64"/>
+      <c r="H20" s="62"/>
+      <c r="I20" s="27"/>
+      <c r="J20" s="119"/>
+      <c r="K20" s="120"/>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="46"/>
+      <c r="A21" s="32"/>
       <c r="B21" s="22"/>
       <c r="C21" s="22"/>
       <c r="D21" s="22"/>
-      <c r="E21" s="51"/>
-      <c r="F21" s="32"/>
-      <c r="G21" s="30"/>
-      <c r="H21" s="30"/>
-      <c r="I21" s="28"/>
-      <c r="J21" s="75"/>
-      <c r="K21" s="76"/>
+      <c r="E21" s="35"/>
+      <c r="F21" s="63"/>
+      <c r="G21" s="62"/>
+      <c r="H21" s="62"/>
+      <c r="I21" s="27"/>
+      <c r="J21" s="119"/>
+      <c r="K21" s="120"/>
     </row>
     <row r="22" spans="1:11">
-      <c r="A22" s="46"/>
+      <c r="A22" s="32"/>
       <c r="B22" s="22"/>
       <c r="C22" s="22"/>
       <c r="D22" s="22"/>
-      <c r="E22" s="51"/>
-      <c r="F22" s="32"/>
-      <c r="G22" s="30"/>
-      <c r="H22" s="30"/>
-      <c r="I22" s="28"/>
-      <c r="J22" s="75"/>
-      <c r="K22" s="76"/>
+      <c r="E22" s="35"/>
+      <c r="F22" s="63"/>
+      <c r="G22" s="62"/>
+      <c r="H22" s="62"/>
+      <c r="I22" s="27"/>
+      <c r="J22" s="119"/>
+      <c r="K22" s="120"/>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="46"/>
+      <c r="A23" s="32"/>
       <c r="B23" s="22"/>
       <c r="C23" s="22"/>
       <c r="D23" s="22"/>
       <c r="E23" s="22"/>
-      <c r="F23" s="33"/>
+      <c r="F23" s="2"/>
       <c r="G23" s="27"/>
       <c r="H23" s="27"/>
-      <c r="I23" s="28"/>
-      <c r="J23" s="75"/>
-      <c r="K23" s="76"/>
+      <c r="I23" s="27"/>
+      <c r="J23" s="119"/>
+      <c r="K23" s="120"/>
     </row>
     <row r="24" spans="1:11">
-      <c r="A24" s="46"/>
+      <c r="A24" s="32"/>
       <c r="B24" s="22"/>
       <c r="C24" s="22"/>
       <c r="D24" s="22"/>
       <c r="E24" s="22"/>
-      <c r="F24" s="33"/>
-      <c r="G24" s="33"/>
-      <c r="H24" s="33"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
       <c r="I24" s="2"/>
-      <c r="J24" s="75"/>
-      <c r="K24" s="76"/>
+      <c r="J24" s="119"/>
+      <c r="K24" s="120"/>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="46"/>
+      <c r="A25" s="32"/>
       <c r="B25" s="22"/>
       <c r="C25" s="22"/>
       <c r="D25" s="22"/>
       <c r="E25" s="22"/>
-      <c r="F25" s="34"/>
-      <c r="G25" s="31"/>
-      <c r="H25" s="31"/>
+      <c r="F25" s="65"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="8"/>
       <c r="I25" s="9"/>
-      <c r="J25" s="75"/>
-      <c r="K25" s="76"/>
+      <c r="J25" s="119"/>
+      <c r="K25" s="120"/>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="109"/>
-      <c r="B26" s="98"/>
-      <c r="C26" s="98"/>
-      <c r="D26" s="98"/>
-      <c r="E26" s="110"/>
-      <c r="F26" s="35"/>
-      <c r="G26" s="36"/>
-      <c r="H26" s="31"/>
+      <c r="A26" s="83"/>
+      <c r="B26" s="80"/>
+      <c r="C26" s="80"/>
+      <c r="D26" s="80"/>
+      <c r="E26" s="84"/>
+      <c r="F26" s="66"/>
+      <c r="G26" s="67"/>
+      <c r="H26" s="8"/>
       <c r="I26" s="9"/>
-      <c r="J26" s="75"/>
-      <c r="K26" s="76"/>
+      <c r="J26" s="119"/>
+      <c r="K26" s="120"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="98"/>
-      <c r="B27" s="98"/>
-      <c r="C27" s="98"/>
-      <c r="D27" s="98"/>
-      <c r="E27" s="110"/>
-      <c r="F27" s="37"/>
-      <c r="G27" s="36"/>
-      <c r="H27" s="31"/>
+      <c r="A27" s="80"/>
+      <c r="B27" s="80"/>
+      <c r="C27" s="80"/>
+      <c r="D27" s="80"/>
+      <c r="E27" s="84"/>
+      <c r="F27" s="68"/>
+      <c r="G27" s="67"/>
+      <c r="H27" s="8"/>
       <c r="I27" s="9"/>
-      <c r="J27" s="75"/>
-      <c r="K27" s="76"/>
+      <c r="J27" s="119"/>
+      <c r="K27" s="120"/>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="98"/>
-      <c r="B28" s="98"/>
-      <c r="C28" s="98"/>
-      <c r="D28" s="98"/>
-      <c r="E28" s="110"/>
-      <c r="F28" s="37"/>
-      <c r="G28" s="36"/>
-      <c r="H28" s="31"/>
+      <c r="A28" s="80"/>
+      <c r="B28" s="80"/>
+      <c r="C28" s="80"/>
+      <c r="D28" s="80"/>
+      <c r="E28" s="84"/>
+      <c r="F28" s="68"/>
+      <c r="G28" s="67"/>
+      <c r="H28" s="8"/>
       <c r="I28" s="9"/>
-      <c r="J28" s="75"/>
-      <c r="K28" s="76"/>
+      <c r="J28" s="119"/>
+      <c r="K28" s="120"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="98"/>
-      <c r="B29" s="98"/>
-      <c r="C29" s="98"/>
-      <c r="D29" s="98"/>
-      <c r="E29" s="110"/>
-      <c r="F29" s="38"/>
-      <c r="G29" s="39"/>
-      <c r="H29" s="34"/>
+      <c r="A29" s="80"/>
+      <c r="B29" s="80"/>
+      <c r="C29" s="80"/>
+      <c r="D29" s="80"/>
+      <c r="E29" s="84"/>
+      <c r="F29" s="69"/>
+      <c r="G29" s="70"/>
+      <c r="H29" s="65"/>
       <c r="I29" s="23"/>
-      <c r="J29" s="75"/>
-      <c r="K29" s="76"/>
+      <c r="J29" s="119"/>
+      <c r="K29" s="120"/>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="111"/>
-      <c r="B30" s="111"/>
-      <c r="C30" s="111"/>
-      <c r="D30" s="111"/>
-      <c r="E30" s="112"/>
-      <c r="F30" s="65"/>
+      <c r="A30" s="85"/>
+      <c r="B30" s="85"/>
+      <c r="C30" s="85"/>
+      <c r="D30" s="85"/>
+      <c r="E30" s="86"/>
+      <c r="F30" s="49"/>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
-      <c r="J30" s="75"/>
-      <c r="K30" s="76"/>
+      <c r="J30" s="119"/>
+      <c r="K30" s="120"/>
     </row>
     <row r="31" spans="1:11" ht="15.5">
-      <c r="A31" s="132" t="s">
+      <c r="A31" s="71" t="s">
         <v>17</v>
       </c>
-      <c r="B31" s="94"/>
-      <c r="C31" s="101"/>
-      <c r="D31" s="66"/>
-      <c r="E31" s="133"/>
-      <c r="F31" s="134"/>
-      <c r="G31" s="134"/>
-      <c r="H31" s="134"/>
-      <c r="I31" s="135" t="s">
+      <c r="B31" s="72"/>
+      <c r="C31" s="73"/>
+      <c r="D31" s="50"/>
+      <c r="E31" s="74"/>
+      <c r="F31" s="75"/>
+      <c r="G31" s="75"/>
+      <c r="H31" s="75"/>
+      <c r="I31" s="76" t="s">
         <v>18</v>
       </c>
-      <c r="J31" s="136"/>
-      <c r="K31" s="137"/>
+      <c r="J31" s="77"/>
+      <c r="K31" s="78"/>
     </row>
     <row r="32" spans="1:11">
-      <c r="A32" s="53"/>
-      <c r="B32" s="70"/>
+      <c r="A32" s="37"/>
+      <c r="B32" s="54"/>
       <c r="C32" s="4"/>
-      <c r="D32" s="54"/>
+      <c r="D32" s="38"/>
       <c r="E32" s="3"/>
-      <c r="F32" s="138"/>
-      <c r="G32" s="98"/>
-      <c r="H32" s="114"/>
-      <c r="I32" s="138"/>
-      <c r="J32" s="98"/>
-      <c r="K32" s="139"/>
+      <c r="F32" s="79"/>
+      <c r="G32" s="80"/>
+      <c r="H32" s="81"/>
+      <c r="I32" s="79"/>
+      <c r="J32" s="80"/>
+      <c r="K32" s="82"/>
     </row>
     <row r="33" spans="1:11">
-      <c r="A33" s="55"/>
-      <c r="B33" s="61"/>
-      <c r="C33" s="57"/>
-      <c r="D33" s="58"/>
-      <c r="E33" s="59"/>
-      <c r="F33" s="56"/>
-      <c r="G33" s="56"/>
-      <c r="H33" s="60"/>
-      <c r="I33" s="56"/>
-      <c r="J33" s="56"/>
-      <c r="K33" s="61"/>
+      <c r="A33" s="39"/>
+      <c r="B33" s="45"/>
+      <c r="C33" s="41"/>
+      <c r="D33" s="42"/>
+      <c r="E33" s="43"/>
+      <c r="F33" s="40"/>
+      <c r="G33" s="40"/>
+      <c r="H33" s="44"/>
+      <c r="I33" s="40"/>
+      <c r="J33" s="40"/>
+      <c r="K33" s="45"/>
     </row>
     <row r="34" spans="1:11">
-      <c r="A34" s="42"/>
-      <c r="B34" s="42"/>
-      <c r="C34" s="42"/>
-      <c r="D34" s="42"/>
-      <c r="E34" s="42"/>
+      <c r="A34" s="30"/>
+      <c r="B34" s="30"/>
+      <c r="C34" s="30"/>
+      <c r="D34" s="30"/>
+      <c r="E34" s="30"/>
     </row>
     <row r="35" spans="1:11">
-      <c r="A35" s="42"/>
-      <c r="B35" s="42"/>
-      <c r="C35" s="42"/>
-      <c r="D35" s="42"/>
-      <c r="E35" s="42"/>
+      <c r="A35" s="30"/>
+      <c r="B35" s="30"/>
+      <c r="C35" s="30"/>
+      <c r="D35" s="30"/>
+      <c r="E35" s="30"/>
     </row>
     <row r="36" spans="1:11">
-      <c r="A36" s="42"/>
+      <c r="A36" s="30"/>
     </row>
     <row r="37" spans="1:11">
-      <c r="A37" s="42"/>
+      <c r="A37" s="30"/>
     </row>
     <row r="38" spans="1:11">
-      <c r="A38" s="42"/>
+      <c r="A38" s="30"/>
     </row>
     <row r="45" spans="1:11" ht="15.5">
       <c r="J45" s="5"/>
@@ -2445,11 +2436,32 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="E31:H31"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="E1:G2"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="A5:C6"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="J6:K6"/>
     <mergeCell ref="A26:E30"/>
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="J9:K9"/>
@@ -2466,32 +2478,11 @@
     <mergeCell ref="J13:K13"/>
     <mergeCell ref="J14:K14"/>
     <mergeCell ref="J15:K15"/>
-    <mergeCell ref="A5:C6"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="E6:G6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="E1:G2"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="E31:H31"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="I32:K32"/>
   </mergeCells>
   <conditionalFormatting sqref="F12:G15 I12 F17:F22 G17:G19 G21:G22">
     <cfRule type="expression" dxfId="7" priority="1">
@@ -2530,125 +2521,125 @@
   <dimension ref="A1:K67"/>
   <sheetFormatPr defaultRowHeight="12.5"/>
   <cols>
-    <col min="1" max="1" width="23.54296875" style="40" customWidth="1"/>
-    <col min="2" max="2" width="13.26953125" style="40" customWidth="1"/>
-    <col min="3" max="3" width="4.90625" style="40" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="8.7265625" style="40"/>
-    <col min="5" max="5" width="30.26953125" style="40" customWidth="1"/>
-    <col min="6" max="6" width="16.54296875" style="40" customWidth="1"/>
-    <col min="7" max="8" width="15.54296875" style="40" customWidth="1"/>
-    <col min="9" max="9" width="13.7265625" style="40" customWidth="1"/>
-    <col min="10" max="10" width="9.81640625" style="40" customWidth="1"/>
-    <col min="11" max="11" width="16.1796875" style="40" customWidth="1"/>
+    <col min="1" max="1" width="23.54296875" style="28" customWidth="1"/>
+    <col min="2" max="2" width="13.26953125" style="28" customWidth="1"/>
+    <col min="3" max="3" width="4.90625" style="28" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="8.7265625" style="28"/>
+    <col min="5" max="5" width="30.26953125" style="28" customWidth="1"/>
+    <col min="6" max="6" width="16.54296875" style="28" customWidth="1"/>
+    <col min="7" max="8" width="15.54296875" style="28" customWidth="1"/>
+    <col min="9" max="9" width="13.7265625" style="28" customWidth="1"/>
+    <col min="10" max="10" width="9.81640625" style="28" customWidth="1"/>
+    <col min="11" max="11" width="16.1796875" style="28" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.5" customHeight="1">
-      <c r="A1" s="77" t="s">
+      <c r="A1" s="128" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="140"/>
-      <c r="D1" s="74"/>
-      <c r="E1" s="142" t="s">
+      <c r="B1" s="129"/>
+      <c r="C1" s="150"/>
+      <c r="D1" s="58"/>
+      <c r="E1" s="152" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="143"/>
-      <c r="G1" s="144"/>
-      <c r="H1" s="41"/>
-      <c r="I1" s="88" t="s">
+      <c r="F1" s="153"/>
+      <c r="G1" s="154"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="139" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="89"/>
-      <c r="K1" s="90"/>
+      <c r="J1" s="140"/>
+      <c r="K1" s="141"/>
     </row>
     <row r="2" spans="1:11" ht="15.5">
-      <c r="A2" s="79"/>
-      <c r="B2" s="80"/>
-      <c r="C2" s="141"/>
-      <c r="D2" s="68"/>
-      <c r="E2" s="145"/>
-      <c r="F2" s="146"/>
-      <c r="G2" s="147"/>
+      <c r="A2" s="130"/>
+      <c r="B2" s="131"/>
+      <c r="C2" s="151"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="155"/>
+      <c r="F2" s="156"/>
+      <c r="G2" s="157"/>
       <c r="H2" s="15"/>
-      <c r="I2" s="91">
+      <c r="I2" s="142">
         <f ca="1">TODAY()</f>
-        <v>45804</v>
-      </c>
-      <c r="J2" s="86"/>
-      <c r="K2" s="87"/>
+        <v>45811</v>
+      </c>
+      <c r="J2" s="137"/>
+      <c r="K2" s="138"/>
     </row>
     <row r="3" spans="1:11">
-      <c r="A3" s="46"/>
+      <c r="A3" s="32"/>
       <c r="B3" s="22"/>
       <c r="C3" s="13"/>
-      <c r="D3" s="52"/>
+      <c r="D3" s="36"/>
       <c r="E3" s="11"/>
       <c r="F3" s="22"/>
-      <c r="G3" s="67"/>
+      <c r="G3" s="51"/>
       <c r="H3" s="25"/>
       <c r="I3" s="22"/>
       <c r="J3" s="22"/>
-      <c r="K3" s="47"/>
+      <c r="K3" s="33"/>
     </row>
     <row r="4" spans="1:11" ht="17">
-      <c r="A4" s="148" t="s">
+      <c r="A4" s="158" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="149"/>
-      <c r="C4" s="80"/>
-      <c r="D4" s="68"/>
+      <c r="B4" s="159"/>
+      <c r="C4" s="131"/>
+      <c r="D4" s="52"/>
       <c r="E4" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="F4" s="63"/>
-      <c r="G4" s="64"/>
+      <c r="F4" s="47"/>
+      <c r="G4" s="48"/>
       <c r="H4" s="15"/>
       <c r="I4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="95"/>
-      <c r="K4" s="96"/>
+      <c r="J4" s="144"/>
+      <c r="K4" s="115"/>
     </row>
     <row r="5" spans="1:11" ht="18.5">
-      <c r="A5" s="150" t="s">
+      <c r="A5" s="145" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="151"/>
-      <c r="C5" s="81"/>
+      <c r="B5" s="146"/>
+      <c r="C5" s="132"/>
       <c r="D5" s="14"/>
-      <c r="E5" s="102" t="s">
+      <c r="E5" s="122" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="103"/>
-      <c r="G5" s="104"/>
+      <c r="F5" s="123"/>
+      <c r="G5" s="124"/>
       <c r="H5" s="22"/>
       <c r="I5" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="J5" s="105"/>
-      <c r="K5" s="96"/>
+      <c r="J5" s="125"/>
+      <c r="K5" s="115"/>
     </row>
     <row r="6" spans="1:11" ht="15.5">
-      <c r="A6" s="79"/>
-      <c r="B6" s="80"/>
-      <c r="C6" s="152"/>
+      <c r="A6" s="130"/>
+      <c r="B6" s="131"/>
+      <c r="C6" s="147"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="153" t="s">
+      <c r="E6" s="148" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="80"/>
-      <c r="G6" s="154"/>
-      <c r="H6" s="62"/>
+      <c r="F6" s="131"/>
+      <c r="G6" s="149"/>
+      <c r="H6" s="46"/>
       <c r="I6" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="J6" s="108">
+      <c r="J6" s="127">
         <v>1230</v>
       </c>
-      <c r="K6" s="96"/>
+      <c r="K6" s="115"/>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="46"/>
+      <c r="A7" s="32"/>
       <c r="B7" s="22"/>
       <c r="C7" s="22"/>
       <c r="D7" s="22"/>
@@ -2658,52 +2649,52 @@
       <c r="H7" s="22"/>
       <c r="I7" s="22"/>
       <c r="J7" s="22"/>
-      <c r="K7" s="47"/>
+      <c r="K7" s="33"/>
     </row>
     <row r="8" spans="1:11" ht="15.5">
-      <c r="A8" s="122" t="s">
+      <c r="A8" s="107" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="72" t="s">
+      <c r="B8" s="56" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="124" t="s">
+      <c r="C8" s="109" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="125"/>
-      <c r="E8" s="126"/>
+      <c r="D8" s="110"/>
+      <c r="E8" s="111"/>
       <c r="F8" s="14"/>
-      <c r="G8" s="127" t="s">
+      <c r="G8" s="112" t="s">
         <v>12</v>
       </c>
-      <c r="H8" s="93"/>
+      <c r="H8" s="113"/>
       <c r="I8" s="14"/>
-      <c r="J8" s="128" t="s">
+      <c r="J8" s="114" t="s">
         <v>13</v>
       </c>
-      <c r="K8" s="96"/>
+      <c r="K8" s="115"/>
     </row>
     <row r="9" spans="1:11" ht="17">
-      <c r="A9" s="123"/>
-      <c r="B9" s="73" t="s">
+      <c r="A9" s="108"/>
+      <c r="B9" s="57" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="129" t="s">
+      <c r="C9" s="116" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="94"/>
-      <c r="E9" s="114"/>
+      <c r="D9" s="72"/>
+      <c r="E9" s="81"/>
       <c r="F9" s="22"/>
-      <c r="G9" s="113">
+      <c r="G9" s="87">
         <v>1</v>
       </c>
-      <c r="H9" s="114"/>
+      <c r="H9" s="81"/>
       <c r="I9" s="22"/>
-      <c r="J9" s="115"/>
-      <c r="K9" s="107"/>
+      <c r="J9" s="88"/>
+      <c r="K9" s="89"/>
     </row>
     <row r="10" spans="1:11">
-      <c r="A10" s="46"/>
+      <c r="A10" s="32"/>
       <c r="B10" s="22"/>
       <c r="C10" s="22"/>
       <c r="D10" s="22"/>
@@ -2713,340 +2704,340 @@
       <c r="H10" s="19"/>
       <c r="I10" s="19"/>
       <c r="J10" s="22"/>
-      <c r="K10" s="48"/>
+      <c r="K10" s="34"/>
     </row>
     <row r="11" spans="1:11" ht="18.5">
-      <c r="A11" s="116" t="s">
+      <c r="A11" s="90" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="117"/>
-      <c r="C11" s="117"/>
-      <c r="D11" s="117"/>
-      <c r="E11" s="118"/>
-      <c r="F11" s="119"/>
-      <c r="G11" s="117"/>
-      <c r="H11" s="117"/>
-      <c r="I11" s="117"/>
-      <c r="J11" s="117"/>
-      <c r="K11" s="120"/>
+      <c r="B11" s="91"/>
+      <c r="C11" s="91"/>
+      <c r="D11" s="91"/>
+      <c r="E11" s="92"/>
+      <c r="F11" s="93"/>
+      <c r="G11" s="91"/>
+      <c r="H11" s="91"/>
+      <c r="I11" s="91"/>
+      <c r="J11" s="91"/>
+      <c r="K11" s="94"/>
     </row>
     <row r="12" spans="1:11" ht="12.5" customHeight="1">
-      <c r="A12" s="121" t="s">
+      <c r="A12" s="95" t="s">
         <v>23</v>
       </c>
-      <c r="B12" s="99"/>
-      <c r="C12" s="99"/>
-      <c r="D12" s="99"/>
-      <c r="E12" s="114"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="44"/>
-      <c r="H12" s="49"/>
-      <c r="I12" s="45"/>
-      <c r="J12" s="130"/>
-      <c r="K12" s="131"/>
+      <c r="B12" s="96"/>
+      <c r="C12" s="96"/>
+      <c r="D12" s="96"/>
+      <c r="E12" s="81"/>
+      <c r="F12" s="59"/>
+      <c r="G12" s="31"/>
+      <c r="H12" s="60"/>
+      <c r="I12" s="31"/>
+      <c r="J12" s="117"/>
+      <c r="K12" s="118"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="100"/>
-      <c r="B13" s="94"/>
-      <c r="C13" s="94"/>
-      <c r="D13" s="94"/>
-      <c r="E13" s="101"/>
+      <c r="A13" s="97"/>
+      <c r="B13" s="72"/>
+      <c r="C13" s="72"/>
+      <c r="D13" s="72"/>
+      <c r="E13" s="73"/>
       <c r="F13" s="27"/>
-      <c r="G13" s="29"/>
-      <c r="H13" s="30"/>
+      <c r="G13" s="61"/>
+      <c r="H13" s="62"/>
       <c r="I13" s="2"/>
-      <c r="J13" s="130"/>
-      <c r="K13" s="131"/>
+      <c r="J13" s="117"/>
+      <c r="K13" s="118"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="155" t="str">
+      <c r="A14" s="98" t="str">
         <f>""&amp;A12&amp;""</f>
         <v>GOFEMM20052025002</v>
       </c>
-      <c r="B14" s="156"/>
-      <c r="C14" s="156"/>
-      <c r="D14" s="156"/>
-      <c r="E14" s="157"/>
+      <c r="B14" s="99"/>
+      <c r="C14" s="99"/>
+      <c r="D14" s="99"/>
+      <c r="E14" s="100"/>
       <c r="F14" s="27"/>
-      <c r="G14" s="30"/>
-      <c r="H14" s="30"/>
+      <c r="G14" s="62"/>
+      <c r="H14" s="62"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="130"/>
-      <c r="K14" s="131"/>
+      <c r="J14" s="117"/>
+      <c r="K14" s="118"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="158"/>
-      <c r="B15" s="159"/>
-      <c r="C15" s="159"/>
-      <c r="D15" s="159"/>
-      <c r="E15" s="160"/>
+      <c r="A15" s="101"/>
+      <c r="B15" s="102"/>
+      <c r="C15" s="102"/>
+      <c r="D15" s="102"/>
+      <c r="E15" s="103"/>
       <c r="F15" s="27"/>
-      <c r="G15" s="30"/>
-      <c r="H15" s="30"/>
+      <c r="G15" s="62"/>
+      <c r="H15" s="62"/>
       <c r="I15" s="2"/>
-      <c r="J15" s="130"/>
-      <c r="K15" s="131"/>
+      <c r="J15" s="117"/>
+      <c r="K15" s="118"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="158"/>
-      <c r="B16" s="159"/>
-      <c r="C16" s="159"/>
-      <c r="D16" s="159"/>
-      <c r="E16" s="160"/>
-      <c r="F16" s="31"/>
-      <c r="G16" s="30"/>
-      <c r="H16" s="30"/>
+      <c r="A16" s="101"/>
+      <c r="B16" s="102"/>
+      <c r="C16" s="102"/>
+      <c r="D16" s="102"/>
+      <c r="E16" s="103"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="62"/>
+      <c r="H16" s="62"/>
       <c r="I16" s="2"/>
-      <c r="J16" s="130"/>
-      <c r="K16" s="131"/>
+      <c r="J16" s="117"/>
+      <c r="K16" s="118"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="158"/>
-      <c r="B17" s="159"/>
-      <c r="C17" s="159"/>
-      <c r="D17" s="159"/>
-      <c r="E17" s="160"/>
+      <c r="A17" s="101"/>
+      <c r="B17" s="102"/>
+      <c r="C17" s="102"/>
+      <c r="D17" s="102"/>
+      <c r="E17" s="103"/>
       <c r="F17" s="27"/>
-      <c r="G17" s="30"/>
-      <c r="H17" s="30"/>
+      <c r="G17" s="62"/>
+      <c r="H17" s="62"/>
       <c r="I17" s="2"/>
-      <c r="J17" s="130"/>
-      <c r="K17" s="131"/>
+      <c r="J17" s="117"/>
+      <c r="K17" s="118"/>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="158"/>
-      <c r="B18" s="159"/>
-      <c r="C18" s="159"/>
-      <c r="D18" s="159"/>
-      <c r="E18" s="160"/>
+      <c r="A18" s="101"/>
+      <c r="B18" s="102"/>
+      <c r="C18" s="102"/>
+      <c r="D18" s="102"/>
+      <c r="E18" s="103"/>
       <c r="F18" s="27"/>
-      <c r="G18" s="30"/>
-      <c r="H18" s="30"/>
+      <c r="G18" s="62"/>
+      <c r="H18" s="62"/>
       <c r="I18" s="8"/>
-      <c r="J18" s="130"/>
-      <c r="K18" s="131"/>
+      <c r="J18" s="117"/>
+      <c r="K18" s="118"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="161"/>
-      <c r="B19" s="162"/>
-      <c r="C19" s="162"/>
-      <c r="D19" s="162"/>
-      <c r="E19" s="163"/>
-      <c r="F19" s="32"/>
-      <c r="G19" s="30"/>
-      <c r="H19" s="30"/>
-      <c r="I19" s="28"/>
-      <c r="J19" s="130"/>
-      <c r="K19" s="131"/>
-    </row>
-    <row r="20" spans="1:11" ht="13">
-      <c r="A20" s="46"/>
+      <c r="A19" s="104"/>
+      <c r="B19" s="105"/>
+      <c r="C19" s="105"/>
+      <c r="D19" s="105"/>
+      <c r="E19" s="106"/>
+      <c r="F19" s="63"/>
+      <c r="G19" s="62"/>
+      <c r="H19" s="62"/>
+      <c r="I19" s="27"/>
+      <c r="J19" s="117"/>
+      <c r="K19" s="118"/>
+    </row>
+    <row r="20" spans="1:11">
+      <c r="A20" s="32"/>
       <c r="B20" s="22"/>
       <c r="C20" s="22"/>
       <c r="D20" s="22"/>
       <c r="E20" s="22"/>
-      <c r="F20" s="32"/>
-      <c r="G20" s="50"/>
-      <c r="H20" s="30"/>
-      <c r="I20" s="28"/>
-      <c r="J20" s="130"/>
-      <c r="K20" s="131"/>
+      <c r="F20" s="63"/>
+      <c r="G20" s="64"/>
+      <c r="H20" s="62"/>
+      <c r="I20" s="27"/>
+      <c r="J20" s="117"/>
+      <c r="K20" s="118"/>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="46"/>
+      <c r="A21" s="32"/>
       <c r="B21" s="22"/>
       <c r="C21" s="22"/>
       <c r="D21" s="22"/>
-      <c r="E21" s="51"/>
-      <c r="F21" s="32"/>
-      <c r="G21" s="30"/>
-      <c r="H21" s="30"/>
-      <c r="I21" s="28"/>
-      <c r="J21" s="130"/>
-      <c r="K21" s="131"/>
+      <c r="E21" s="35"/>
+      <c r="F21" s="63"/>
+      <c r="G21" s="62"/>
+      <c r="H21" s="62"/>
+      <c r="I21" s="27"/>
+      <c r="J21" s="117"/>
+      <c r="K21" s="118"/>
     </row>
     <row r="22" spans="1:11">
-      <c r="A22" s="46"/>
+      <c r="A22" s="32"/>
       <c r="B22" s="22"/>
       <c r="C22" s="22"/>
       <c r="D22" s="22"/>
-      <c r="E22" s="51"/>
-      <c r="F22" s="32"/>
-      <c r="G22" s="30"/>
-      <c r="H22" s="30"/>
-      <c r="I22" s="28"/>
-      <c r="J22" s="130"/>
-      <c r="K22" s="131"/>
+      <c r="E22" s="35"/>
+      <c r="F22" s="63"/>
+      <c r="G22" s="62"/>
+      <c r="H22" s="62"/>
+      <c r="I22" s="27"/>
+      <c r="J22" s="117"/>
+      <c r="K22" s="118"/>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="46"/>
+      <c r="A23" s="32"/>
       <c r="B23" s="22"/>
       <c r="C23" s="22"/>
       <c r="D23" s="22"/>
       <c r="E23" s="22"/>
-      <c r="F23" s="33"/>
+      <c r="F23" s="2"/>
       <c r="G23" s="27"/>
       <c r="H23" s="27"/>
-      <c r="I23" s="28"/>
-      <c r="J23" s="130"/>
-      <c r="K23" s="131"/>
+      <c r="I23" s="27"/>
+      <c r="J23" s="117"/>
+      <c r="K23" s="118"/>
     </row>
     <row r="24" spans="1:11">
-      <c r="A24" s="46"/>
+      <c r="A24" s="32"/>
       <c r="B24" s="22"/>
       <c r="C24" s="22"/>
       <c r="D24" s="22"/>
       <c r="E24" s="22"/>
-      <c r="F24" s="33"/>
-      <c r="G24" s="33"/>
-      <c r="H24" s="33"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
       <c r="I24" s="2"/>
-      <c r="J24" s="130"/>
-      <c r="K24" s="131"/>
+      <c r="J24" s="117"/>
+      <c r="K24" s="118"/>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="46"/>
+      <c r="A25" s="32"/>
       <c r="B25" s="22"/>
       <c r="C25" s="22"/>
       <c r="D25" s="22"/>
       <c r="E25" s="22"/>
-      <c r="F25" s="34"/>
-      <c r="G25" s="31"/>
-      <c r="H25" s="31"/>
+      <c r="F25" s="65"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="8"/>
       <c r="I25" s="9"/>
-      <c r="J25" s="130"/>
-      <c r="K25" s="131"/>
+      <c r="J25" s="117"/>
+      <c r="K25" s="118"/>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="109"/>
-      <c r="B26" s="98"/>
-      <c r="C26" s="98"/>
-      <c r="D26" s="98"/>
-      <c r="E26" s="110"/>
-      <c r="F26" s="35"/>
-      <c r="G26" s="36"/>
-      <c r="H26" s="31"/>
+      <c r="A26" s="83"/>
+      <c r="B26" s="80"/>
+      <c r="C26" s="80"/>
+      <c r="D26" s="80"/>
+      <c r="E26" s="84"/>
+      <c r="F26" s="66"/>
+      <c r="G26" s="67"/>
+      <c r="H26" s="8"/>
       <c r="I26" s="9"/>
-      <c r="J26" s="130"/>
-      <c r="K26" s="131"/>
+      <c r="J26" s="117"/>
+      <c r="K26" s="118"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="98"/>
-      <c r="B27" s="98"/>
-      <c r="C27" s="98"/>
-      <c r="D27" s="98"/>
-      <c r="E27" s="110"/>
-      <c r="F27" s="37"/>
-      <c r="G27" s="36"/>
-      <c r="H27" s="31"/>
+      <c r="A27" s="80"/>
+      <c r="B27" s="80"/>
+      <c r="C27" s="80"/>
+      <c r="D27" s="80"/>
+      <c r="E27" s="84"/>
+      <c r="F27" s="68"/>
+      <c r="G27" s="67"/>
+      <c r="H27" s="8"/>
       <c r="I27" s="9"/>
-      <c r="J27" s="130"/>
-      <c r="K27" s="131"/>
+      <c r="J27" s="117"/>
+      <c r="K27" s="118"/>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="98"/>
-      <c r="B28" s="98"/>
-      <c r="C28" s="98"/>
-      <c r="D28" s="98"/>
-      <c r="E28" s="110"/>
-      <c r="F28" s="37"/>
-      <c r="G28" s="36"/>
-      <c r="H28" s="31"/>
+      <c r="A28" s="80"/>
+      <c r="B28" s="80"/>
+      <c r="C28" s="80"/>
+      <c r="D28" s="80"/>
+      <c r="E28" s="84"/>
+      <c r="F28" s="68"/>
+      <c r="G28" s="67"/>
+      <c r="H28" s="8"/>
       <c r="I28" s="9"/>
-      <c r="J28" s="130"/>
-      <c r="K28" s="131"/>
+      <c r="J28" s="117"/>
+      <c r="K28" s="118"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="98"/>
-      <c r="B29" s="98"/>
-      <c r="C29" s="98"/>
-      <c r="D29" s="98"/>
-      <c r="E29" s="110"/>
-      <c r="F29" s="38"/>
-      <c r="G29" s="39"/>
-      <c r="H29" s="34"/>
+      <c r="A29" s="80"/>
+      <c r="B29" s="80"/>
+      <c r="C29" s="80"/>
+      <c r="D29" s="80"/>
+      <c r="E29" s="84"/>
+      <c r="F29" s="69"/>
+      <c r="G29" s="70"/>
+      <c r="H29" s="65"/>
       <c r="I29" s="23"/>
-      <c r="J29" s="130"/>
-      <c r="K29" s="131"/>
+      <c r="J29" s="117"/>
+      <c r="K29" s="118"/>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="111"/>
-      <c r="B30" s="111"/>
-      <c r="C30" s="111"/>
-      <c r="D30" s="111"/>
-      <c r="E30" s="112"/>
-      <c r="F30" s="65"/>
+      <c r="A30" s="85"/>
+      <c r="B30" s="85"/>
+      <c r="C30" s="85"/>
+      <c r="D30" s="85"/>
+      <c r="E30" s="86"/>
+      <c r="F30" s="49"/>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
-      <c r="J30" s="130"/>
-      <c r="K30" s="131"/>
+      <c r="J30" s="117"/>
+      <c r="K30" s="118"/>
     </row>
     <row r="31" spans="1:11" ht="15.5">
-      <c r="A31" s="132" t="s">
+      <c r="A31" s="71" t="s">
         <v>17</v>
       </c>
-      <c r="B31" s="94"/>
-      <c r="C31" s="101"/>
-      <c r="D31" s="66"/>
-      <c r="E31" s="133"/>
-      <c r="F31" s="134"/>
-      <c r="G31" s="134"/>
-      <c r="H31" s="134"/>
-      <c r="I31" s="135" t="s">
+      <c r="B31" s="72"/>
+      <c r="C31" s="73"/>
+      <c r="D31" s="50"/>
+      <c r="E31" s="74"/>
+      <c r="F31" s="75"/>
+      <c r="G31" s="75"/>
+      <c r="H31" s="75"/>
+      <c r="I31" s="76" t="s">
         <v>18</v>
       </c>
-      <c r="J31" s="136"/>
-      <c r="K31" s="137"/>
+      <c r="J31" s="77"/>
+      <c r="K31" s="78"/>
     </row>
     <row r="32" spans="1:11">
-      <c r="A32" s="53"/>
-      <c r="B32" s="70"/>
+      <c r="A32" s="37"/>
+      <c r="B32" s="54"/>
       <c r="C32" s="4"/>
-      <c r="D32" s="54"/>
+      <c r="D32" s="38"/>
       <c r="E32" s="3"/>
-      <c r="F32" s="138"/>
-      <c r="G32" s="98"/>
-      <c r="H32" s="114"/>
-      <c r="I32" s="138"/>
-      <c r="J32" s="98"/>
-      <c r="K32" s="139"/>
+      <c r="F32" s="79"/>
+      <c r="G32" s="80"/>
+      <c r="H32" s="81"/>
+      <c r="I32" s="79"/>
+      <c r="J32" s="80"/>
+      <c r="K32" s="82"/>
     </row>
     <row r="33" spans="1:11">
-      <c r="A33" s="55"/>
-      <c r="B33" s="61"/>
-      <c r="C33" s="57"/>
-      <c r="D33" s="58"/>
-      <c r="E33" s="59"/>
-      <c r="F33" s="56"/>
-      <c r="G33" s="56"/>
-      <c r="H33" s="60"/>
-      <c r="I33" s="56"/>
-      <c r="J33" s="56"/>
-      <c r="K33" s="61"/>
+      <c r="A33" s="39"/>
+      <c r="B33" s="45"/>
+      <c r="C33" s="41"/>
+      <c r="D33" s="42"/>
+      <c r="E33" s="43"/>
+      <c r="F33" s="40"/>
+      <c r="G33" s="40"/>
+      <c r="H33" s="44"/>
+      <c r="I33" s="40"/>
+      <c r="J33" s="40"/>
+      <c r="K33" s="45"/>
     </row>
     <row r="34" spans="1:11">
-      <c r="A34" s="42"/>
-      <c r="B34" s="42"/>
-      <c r="C34" s="42"/>
-      <c r="D34" s="42"/>
-      <c r="E34" s="42"/>
+      <c r="A34" s="30"/>
+      <c r="B34" s="30"/>
+      <c r="C34" s="30"/>
+      <c r="D34" s="30"/>
+      <c r="E34" s="30"/>
     </row>
     <row r="35" spans="1:11">
-      <c r="A35" s="42"/>
-      <c r="B35" s="42"/>
-      <c r="C35" s="42"/>
-      <c r="D35" s="42"/>
-      <c r="E35" s="42"/>
+      <c r="A35" s="30"/>
+      <c r="B35" s="30"/>
+      <c r="C35" s="30"/>
+      <c r="D35" s="30"/>
+      <c r="E35" s="30"/>
     </row>
     <row r="36" spans="1:11">
-      <c r="A36" s="42"/>
+      <c r="A36" s="30"/>
     </row>
     <row r="37" spans="1:11">
-      <c r="A37" s="42"/>
+      <c r="A37" s="30"/>
     </row>
     <row r="38" spans="1:11">
-      <c r="A38" s="42"/>
+      <c r="A38" s="30"/>
     </row>
     <row r="45" spans="1:11" ht="15.5">
       <c r="J45" s="5"/>
@@ -3089,16 +3080,27 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="A26:E30"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="E31:H31"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="E1:G2"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="J4:K4"/>
     <mergeCell ref="A14:E19"/>
     <mergeCell ref="A5:C6"/>
     <mergeCell ref="E5:G5"/>
@@ -3115,27 +3117,16 @@
     <mergeCell ref="A11:E11"/>
     <mergeCell ref="F11:K11"/>
     <mergeCell ref="A12:E13"/>
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="E1:G2"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="A26:E30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="E31:H31"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J30:K30"/>
   </mergeCells>
   <conditionalFormatting sqref="F12:G15 I12 F17:F22 G17:G19 G21:G22">
     <cfRule type="expression" dxfId="3" priority="1">

</xml_diff>

<commit_message>
feat: add exportation of out zone data workbook, also some improvements
</commit_message>
<xml_diff>
--- a/dummy-content/ECHEC-RETOUR_CLIENT-CASABLANCA.xlsx
+++ b/dummy-content/ECHEC-RETOUR_CLIENT-CASABLANCA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User1\Desktop\GoFleet-Enhancer\dummy-content\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65E33A46-2CCE-473D-A1E8-442A141F2726}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEC0E857-1BC1-4997-AA17-053272EDFA2F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12110" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1403,24 +1403,66 @@
     <xf numFmtId="0" fontId="15" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="5" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
@@ -1428,10 +1470,10 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="11" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1444,8 +1486,6 @@
     <xf numFmtId="0" fontId="21" fillId="12" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="24" fillId="3" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1469,11 +1509,9 @@
     <xf numFmtId="0" fontId="8" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1483,67 +1521,20 @@
     <xf numFmtId="0" fontId="15" fillId="15" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="5" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="20" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="19" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="17" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1558,6 +1549,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="19" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1892,37 +1892,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.5" customHeight="1">
-      <c r="A1" s="128"/>
-      <c r="B1" s="129"/>
-      <c r="C1" s="129"/>
+      <c r="A1" s="73"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
       <c r="D1" s="53"/>
-      <c r="E1" s="133" t="s">
+      <c r="E1" s="78" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="134"/>
-      <c r="G1" s="135"/>
+      <c r="F1" s="79"/>
+      <c r="G1" s="80"/>
       <c r="H1" s="29"/>
-      <c r="I1" s="139" t="s">
+      <c r="I1" s="84" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="140"/>
-      <c r="K1" s="141"/>
+      <c r="J1" s="85"/>
+      <c r="K1" s="86"/>
     </row>
     <row r="2" spans="1:11" ht="15.5">
-      <c r="A2" s="130"/>
-      <c r="B2" s="131"/>
-      <c r="C2" s="132"/>
+      <c r="A2" s="75"/>
+      <c r="B2" s="76"/>
+      <c r="C2" s="77"/>
       <c r="D2" s="53"/>
-      <c r="E2" s="136"/>
-      <c r="F2" s="137"/>
-      <c r="G2" s="138"/>
+      <c r="E2" s="81"/>
+      <c r="F2" s="82"/>
+      <c r="G2" s="83"/>
       <c r="H2" s="15"/>
-      <c r="I2" s="142">
+      <c r="I2" s="87">
         <f ca="1">TODAY()</f>
-        <v>45811</v>
-      </c>
-      <c r="J2" s="137"/>
-      <c r="K2" s="138"/>
+        <v>45833</v>
+      </c>
+      <c r="J2" s="82"/>
+      <c r="K2" s="83"/>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="32"/>
@@ -1938,11 +1938,11 @@
       <c r="K3" s="33"/>
     </row>
     <row r="4" spans="1:11" ht="17">
-      <c r="A4" s="143" t="s">
+      <c r="A4" s="88" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="113"/>
-      <c r="C4" s="72"/>
+      <c r="B4" s="89"/>
+      <c r="C4" s="90"/>
       <c r="D4" s="52"/>
       <c r="E4" s="16" t="s">
         <v>21</v>
@@ -1953,46 +1953,46 @@
       <c r="I4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="144"/>
-      <c r="K4" s="115"/>
+      <c r="J4" s="91"/>
+      <c r="K4" s="92"/>
     </row>
     <row r="5" spans="1:11" ht="18.5">
-      <c r="A5" s="121" t="s">
+      <c r="A5" s="93" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="80"/>
-      <c r="C5" s="96"/>
+      <c r="B5" s="94"/>
+      <c r="C5" s="95"/>
       <c r="D5" s="14"/>
-      <c r="E5" s="122" t="s">
+      <c r="E5" s="98" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="123"/>
-      <c r="G5" s="124"/>
+      <c r="F5" s="99"/>
+      <c r="G5" s="100"/>
       <c r="H5" s="22"/>
       <c r="I5" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="J5" s="125"/>
-      <c r="K5" s="115"/>
+      <c r="J5" s="101"/>
+      <c r="K5" s="92"/>
     </row>
     <row r="6" spans="1:11" ht="15.5">
-      <c r="A6" s="97"/>
-      <c r="B6" s="72"/>
-      <c r="C6" s="73"/>
+      <c r="A6" s="96"/>
+      <c r="B6" s="90"/>
+      <c r="C6" s="97"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="126" t="s">
+      <c r="E6" s="102" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="72"/>
-      <c r="G6" s="89"/>
+      <c r="F6" s="90"/>
+      <c r="G6" s="103"/>
       <c r="H6" s="46"/>
       <c r="I6" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="J6" s="127">
+      <c r="J6" s="104">
         <v>1230</v>
       </c>
-      <c r="K6" s="115"/>
+      <c r="K6" s="92"/>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="32"/>
@@ -2008,46 +2008,46 @@
       <c r="K7" s="33"/>
     </row>
     <row r="8" spans="1:11" ht="15.5">
-      <c r="A8" s="107" t="s">
+      <c r="A8" s="127" t="s">
         <v>9</v>
       </c>
       <c r="B8" s="56" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="109" t="s">
+      <c r="C8" s="129" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="110"/>
-      <c r="E8" s="111"/>
+      <c r="D8" s="130"/>
+      <c r="E8" s="131"/>
       <c r="F8" s="14"/>
-      <c r="G8" s="112" t="s">
+      <c r="G8" s="132" t="s">
         <v>12</v>
       </c>
-      <c r="H8" s="113"/>
+      <c r="H8" s="89"/>
       <c r="I8" s="14"/>
-      <c r="J8" s="114" t="s">
+      <c r="J8" s="133" t="s">
         <v>13</v>
       </c>
-      <c r="K8" s="115"/>
+      <c r="K8" s="92"/>
     </row>
     <row r="9" spans="1:11" ht="17">
-      <c r="A9" s="108"/>
+      <c r="A9" s="128"/>
       <c r="B9" s="57" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="116" t="s">
+      <c r="C9" s="134" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="72"/>
-      <c r="E9" s="81"/>
+      <c r="D9" s="90"/>
+      <c r="E9" s="110"/>
       <c r="F9" s="22"/>
-      <c r="G9" s="87">
+      <c r="G9" s="109">
         <v>1</v>
       </c>
-      <c r="H9" s="81"/>
+      <c r="H9" s="110"/>
       <c r="I9" s="22"/>
-      <c r="J9" s="88"/>
-      <c r="K9" s="89"/>
+      <c r="J9" s="111"/>
+      <c r="K9" s="103"/>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="32"/>
@@ -2063,128 +2063,128 @@
       <c r="K10" s="34"/>
     </row>
     <row r="11" spans="1:11" ht="18.5">
-      <c r="A11" s="90" t="s">
+      <c r="A11" s="112" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="91"/>
-      <c r="C11" s="91"/>
-      <c r="D11" s="91"/>
-      <c r="E11" s="92"/>
-      <c r="F11" s="93"/>
-      <c r="G11" s="91"/>
-      <c r="H11" s="91"/>
-      <c r="I11" s="91"/>
-      <c r="J11" s="91"/>
-      <c r="K11" s="94"/>
+      <c r="B11" s="113"/>
+      <c r="C11" s="113"/>
+      <c r="D11" s="113"/>
+      <c r="E11" s="114"/>
+      <c r="F11" s="115"/>
+      <c r="G11" s="113"/>
+      <c r="H11" s="113"/>
+      <c r="I11" s="113"/>
+      <c r="J11" s="113"/>
+      <c r="K11" s="116"/>
     </row>
     <row r="12" spans="1:11">
-      <c r="A12" s="95" t="s">
+      <c r="A12" s="117" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="96"/>
-      <c r="C12" s="96"/>
-      <c r="D12" s="96"/>
-      <c r="E12" s="81"/>
+      <c r="B12" s="95"/>
+      <c r="C12" s="95"/>
+      <c r="D12" s="95"/>
+      <c r="E12" s="110"/>
       <c r="F12" s="59"/>
       <c r="G12" s="31"/>
       <c r="H12" s="60"/>
       <c r="I12" s="31"/>
-      <c r="J12" s="117"/>
-      <c r="K12" s="118"/>
+      <c r="J12" s="135"/>
+      <c r="K12" s="136"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="97"/>
-      <c r="B13" s="72"/>
-      <c r="C13" s="72"/>
-      <c r="D13" s="72"/>
-      <c r="E13" s="73"/>
+      <c r="A13" s="96"/>
+      <c r="B13" s="90"/>
+      <c r="C13" s="90"/>
+      <c r="D13" s="90"/>
+      <c r="E13" s="97"/>
       <c r="F13" s="27"/>
       <c r="G13" s="61"/>
       <c r="H13" s="62"/>
       <c r="I13" s="2"/>
-      <c r="J13" s="119"/>
-      <c r="K13" s="120"/>
+      <c r="J13" s="71"/>
+      <c r="K13" s="72"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="98" t="str">
+      <c r="A14" s="118" t="str">
         <f>"*"&amp;A12&amp;"*"</f>
         <v>*GOFEMM20052025001*</v>
       </c>
-      <c r="B14" s="99"/>
-      <c r="C14" s="99"/>
-      <c r="D14" s="99"/>
-      <c r="E14" s="100"/>
+      <c r="B14" s="119"/>
+      <c r="C14" s="119"/>
+      <c r="D14" s="119"/>
+      <c r="E14" s="120"/>
       <c r="F14" s="27"/>
       <c r="G14" s="62"/>
       <c r="H14" s="62"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="119"/>
-      <c r="K14" s="120"/>
+      <c r="J14" s="71"/>
+      <c r="K14" s="72"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="101"/>
-      <c r="B15" s="102"/>
-      <c r="C15" s="102"/>
-      <c r="D15" s="102"/>
-      <c r="E15" s="103"/>
+      <c r="A15" s="121"/>
+      <c r="B15" s="122"/>
+      <c r="C15" s="122"/>
+      <c r="D15" s="122"/>
+      <c r="E15" s="123"/>
       <c r="F15" s="27"/>
       <c r="G15" s="62"/>
       <c r="H15" s="62"/>
       <c r="I15" s="2"/>
-      <c r="J15" s="119"/>
-      <c r="K15" s="120"/>
+      <c r="J15" s="71"/>
+      <c r="K15" s="72"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="101"/>
-      <c r="B16" s="102"/>
-      <c r="C16" s="102"/>
-      <c r="D16" s="102"/>
-      <c r="E16" s="103"/>
+      <c r="A16" s="121"/>
+      <c r="B16" s="122"/>
+      <c r="C16" s="122"/>
+      <c r="D16" s="122"/>
+      <c r="E16" s="123"/>
       <c r="F16" s="8"/>
       <c r="G16" s="62"/>
       <c r="H16" s="62"/>
       <c r="I16" s="2"/>
-      <c r="J16" s="119"/>
-      <c r="K16" s="120"/>
+      <c r="J16" s="71"/>
+      <c r="K16" s="72"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="101"/>
-      <c r="B17" s="102"/>
-      <c r="C17" s="102"/>
-      <c r="D17" s="102"/>
-      <c r="E17" s="103"/>
+      <c r="A17" s="121"/>
+      <c r="B17" s="122"/>
+      <c r="C17" s="122"/>
+      <c r="D17" s="122"/>
+      <c r="E17" s="123"/>
       <c r="F17" s="27"/>
       <c r="G17" s="62"/>
       <c r="H17" s="62"/>
       <c r="I17" s="2"/>
-      <c r="J17" s="119"/>
-      <c r="K17" s="120"/>
+      <c r="J17" s="71"/>
+      <c r="K17" s="72"/>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="101"/>
-      <c r="B18" s="102"/>
-      <c r="C18" s="102"/>
-      <c r="D18" s="102"/>
-      <c r="E18" s="103"/>
+      <c r="A18" s="121"/>
+      <c r="B18" s="122"/>
+      <c r="C18" s="122"/>
+      <c r="D18" s="122"/>
+      <c r="E18" s="123"/>
       <c r="F18" s="27"/>
       <c r="G18" s="62"/>
       <c r="H18" s="62"/>
       <c r="I18" s="8"/>
-      <c r="J18" s="119"/>
-      <c r="K18" s="120"/>
+      <c r="J18" s="71"/>
+      <c r="K18" s="72"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="104"/>
-      <c r="B19" s="105"/>
-      <c r="C19" s="105"/>
-      <c r="D19" s="105"/>
-      <c r="E19" s="106"/>
+      <c r="A19" s="124"/>
+      <c r="B19" s="125"/>
+      <c r="C19" s="125"/>
+      <c r="D19" s="125"/>
+      <c r="E19" s="126"/>
       <c r="F19" s="63"/>
       <c r="G19" s="62"/>
       <c r="H19" s="62"/>
       <c r="I19" s="27"/>
-      <c r="J19" s="119"/>
-      <c r="K19" s="120"/>
+      <c r="J19" s="71"/>
+      <c r="K19" s="72"/>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="32"/>
@@ -2196,8 +2196,8 @@
       <c r="G20" s="64"/>
       <c r="H20" s="62"/>
       <c r="I20" s="27"/>
-      <c r="J20" s="119"/>
-      <c r="K20" s="120"/>
+      <c r="J20" s="71"/>
+      <c r="K20" s="72"/>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="32"/>
@@ -2209,8 +2209,8 @@
       <c r="G21" s="62"/>
       <c r="H21" s="62"/>
       <c r="I21" s="27"/>
-      <c r="J21" s="119"/>
-      <c r="K21" s="120"/>
+      <c r="J21" s="71"/>
+      <c r="K21" s="72"/>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="32"/>
@@ -2222,8 +2222,8 @@
       <c r="G22" s="62"/>
       <c r="H22" s="62"/>
       <c r="I22" s="27"/>
-      <c r="J22" s="119"/>
-      <c r="K22" s="120"/>
+      <c r="J22" s="71"/>
+      <c r="K22" s="72"/>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="32"/>
@@ -2235,8 +2235,8 @@
       <c r="G23" s="27"/>
       <c r="H23" s="27"/>
       <c r="I23" s="27"/>
-      <c r="J23" s="119"/>
-      <c r="K23" s="120"/>
+      <c r="J23" s="71"/>
+      <c r="K23" s="72"/>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" s="32"/>
@@ -2248,8 +2248,8 @@
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
-      <c r="J24" s="119"/>
-      <c r="K24" s="120"/>
+      <c r="J24" s="71"/>
+      <c r="K24" s="72"/>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="32"/>
@@ -2261,90 +2261,90 @@
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
       <c r="I25" s="9"/>
-      <c r="J25" s="119"/>
-      <c r="K25" s="120"/>
+      <c r="J25" s="71"/>
+      <c r="K25" s="72"/>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="83"/>
-      <c r="B26" s="80"/>
-      <c r="C26" s="80"/>
-      <c r="D26" s="80"/>
-      <c r="E26" s="84"/>
+      <c r="A26" s="105"/>
+      <c r="B26" s="94"/>
+      <c r="C26" s="94"/>
+      <c r="D26" s="94"/>
+      <c r="E26" s="106"/>
       <c r="F26" s="66"/>
       <c r="G26" s="67"/>
       <c r="H26" s="8"/>
       <c r="I26" s="9"/>
-      <c r="J26" s="119"/>
-      <c r="K26" s="120"/>
+      <c r="J26" s="71"/>
+      <c r="K26" s="72"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="80"/>
-      <c r="B27" s="80"/>
-      <c r="C27" s="80"/>
-      <c r="D27" s="80"/>
-      <c r="E27" s="84"/>
+      <c r="A27" s="94"/>
+      <c r="B27" s="94"/>
+      <c r="C27" s="94"/>
+      <c r="D27" s="94"/>
+      <c r="E27" s="106"/>
       <c r="F27" s="68"/>
       <c r="G27" s="67"/>
       <c r="H27" s="8"/>
       <c r="I27" s="9"/>
-      <c r="J27" s="119"/>
-      <c r="K27" s="120"/>
+      <c r="J27" s="71"/>
+      <c r="K27" s="72"/>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="80"/>
-      <c r="B28" s="80"/>
-      <c r="C28" s="80"/>
-      <c r="D28" s="80"/>
-      <c r="E28" s="84"/>
+      <c r="A28" s="94"/>
+      <c r="B28" s="94"/>
+      <c r="C28" s="94"/>
+      <c r="D28" s="94"/>
+      <c r="E28" s="106"/>
       <c r="F28" s="68"/>
       <c r="G28" s="67"/>
       <c r="H28" s="8"/>
       <c r="I28" s="9"/>
-      <c r="J28" s="119"/>
-      <c r="K28" s="120"/>
+      <c r="J28" s="71"/>
+      <c r="K28" s="72"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="80"/>
-      <c r="B29" s="80"/>
-      <c r="C29" s="80"/>
-      <c r="D29" s="80"/>
-      <c r="E29" s="84"/>
+      <c r="A29" s="94"/>
+      <c r="B29" s="94"/>
+      <c r="C29" s="94"/>
+      <c r="D29" s="94"/>
+      <c r="E29" s="106"/>
       <c r="F29" s="69"/>
       <c r="G29" s="70"/>
       <c r="H29" s="65"/>
       <c r="I29" s="23"/>
-      <c r="J29" s="119"/>
-      <c r="K29" s="120"/>
+      <c r="J29" s="71"/>
+      <c r="K29" s="72"/>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="85"/>
-      <c r="B30" s="85"/>
-      <c r="C30" s="85"/>
-      <c r="D30" s="85"/>
-      <c r="E30" s="86"/>
+      <c r="A30" s="107"/>
+      <c r="B30" s="107"/>
+      <c r="C30" s="107"/>
+      <c r="D30" s="107"/>
+      <c r="E30" s="108"/>
       <c r="F30" s="49"/>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
-      <c r="J30" s="119"/>
-      <c r="K30" s="120"/>
+      <c r="J30" s="71"/>
+      <c r="K30" s="72"/>
     </row>
     <row r="31" spans="1:11" ht="15.5">
-      <c r="A31" s="71" t="s">
+      <c r="A31" s="137" t="s">
         <v>17</v>
       </c>
-      <c r="B31" s="72"/>
-      <c r="C31" s="73"/>
+      <c r="B31" s="90"/>
+      <c r="C31" s="97"/>
       <c r="D31" s="50"/>
-      <c r="E31" s="74"/>
-      <c r="F31" s="75"/>
-      <c r="G31" s="75"/>
-      <c r="H31" s="75"/>
-      <c r="I31" s="76" t="s">
+      <c r="E31" s="138"/>
+      <c r="F31" s="139"/>
+      <c r="G31" s="139"/>
+      <c r="H31" s="139"/>
+      <c r="I31" s="140" t="s">
         <v>18</v>
       </c>
-      <c r="J31" s="77"/>
-      <c r="K31" s="78"/>
+      <c r="J31" s="141"/>
+      <c r="K31" s="142"/>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" s="37"/>
@@ -2352,12 +2352,12 @@
       <c r="C32" s="4"/>
       <c r="D32" s="38"/>
       <c r="E32" s="3"/>
-      <c r="F32" s="79"/>
-      <c r="G32" s="80"/>
-      <c r="H32" s="81"/>
-      <c r="I32" s="79"/>
-      <c r="J32" s="80"/>
-      <c r="K32" s="82"/>
+      <c r="F32" s="143"/>
+      <c r="G32" s="94"/>
+      <c r="H32" s="110"/>
+      <c r="I32" s="143"/>
+      <c r="J32" s="94"/>
+      <c r="K32" s="144"/>
     </row>
     <row r="33" spans="1:11">
       <c r="A33" s="39"/>
@@ -2436,32 +2436,11 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J30:K30"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="E1:G2"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="A5:C6"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="E6:G6"/>
-    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="E31:H31"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="I32:K32"/>
     <mergeCell ref="A26:E30"/>
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="J9:K9"/>
@@ -2478,11 +2457,32 @@
     <mergeCell ref="J13:K13"/>
     <mergeCell ref="J14:K14"/>
     <mergeCell ref="J15:K15"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="E31:H31"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="A5:C6"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="E1:G2"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J30:K30"/>
   </mergeCells>
   <conditionalFormatting sqref="F12:G15 I12 F17:F22 G17:G19 G21:G22">
     <cfRule type="expression" dxfId="7" priority="1">
@@ -2534,39 +2534,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.5" customHeight="1">
-      <c r="A1" s="128" t="s">
+      <c r="A1" s="73" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="129"/>
-      <c r="C1" s="150"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="145"/>
       <c r="D1" s="58"/>
-      <c r="E1" s="152" t="s">
+      <c r="E1" s="147" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="153"/>
-      <c r="G1" s="154"/>
+      <c r="F1" s="148"/>
+      <c r="G1" s="149"/>
       <c r="H1" s="29"/>
-      <c r="I1" s="139" t="s">
+      <c r="I1" s="84" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="140"/>
-      <c r="K1" s="141"/>
+      <c r="J1" s="85"/>
+      <c r="K1" s="86"/>
     </row>
     <row r="2" spans="1:11" ht="15.5">
-      <c r="A2" s="130"/>
-      <c r="B2" s="131"/>
-      <c r="C2" s="151"/>
+      <c r="A2" s="75"/>
+      <c r="B2" s="76"/>
+      <c r="C2" s="146"/>
       <c r="D2" s="52"/>
-      <c r="E2" s="155"/>
-      <c r="F2" s="156"/>
-      <c r="G2" s="157"/>
+      <c r="E2" s="150"/>
+      <c r="F2" s="151"/>
+      <c r="G2" s="152"/>
       <c r="H2" s="15"/>
-      <c r="I2" s="142">
+      <c r="I2" s="87">
         <f ca="1">TODAY()</f>
-        <v>45811</v>
-      </c>
-      <c r="J2" s="137"/>
-      <c r="K2" s="138"/>
+        <v>45833</v>
+      </c>
+      <c r="J2" s="82"/>
+      <c r="K2" s="83"/>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="32"/>
@@ -2582,11 +2582,11 @@
       <c r="K3" s="33"/>
     </row>
     <row r="4" spans="1:11" ht="17">
-      <c r="A4" s="158" t="s">
+      <c r="A4" s="153" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="159"/>
-      <c r="C4" s="131"/>
+      <c r="B4" s="154"/>
+      <c r="C4" s="76"/>
       <c r="D4" s="52"/>
       <c r="E4" s="26" t="s">
         <v>21</v>
@@ -2597,46 +2597,46 @@
       <c r="I4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="144"/>
-      <c r="K4" s="115"/>
+      <c r="J4" s="91"/>
+      <c r="K4" s="92"/>
     </row>
     <row r="5" spans="1:11" ht="18.5">
-      <c r="A5" s="145" t="s">
+      <c r="A5" s="155" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="146"/>
-      <c r="C5" s="132"/>
+      <c r="B5" s="156"/>
+      <c r="C5" s="77"/>
       <c r="D5" s="14"/>
-      <c r="E5" s="122" t="s">
+      <c r="E5" s="98" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="123"/>
-      <c r="G5" s="124"/>
+      <c r="F5" s="99"/>
+      <c r="G5" s="100"/>
       <c r="H5" s="22"/>
       <c r="I5" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="J5" s="125"/>
-      <c r="K5" s="115"/>
+      <c r="J5" s="101"/>
+      <c r="K5" s="92"/>
     </row>
     <row r="6" spans="1:11" ht="15.5">
-      <c r="A6" s="130"/>
-      <c r="B6" s="131"/>
-      <c r="C6" s="147"/>
+      <c r="A6" s="75"/>
+      <c r="B6" s="76"/>
+      <c r="C6" s="157"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="148" t="s">
+      <c r="E6" s="158" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="131"/>
-      <c r="G6" s="149"/>
+      <c r="F6" s="76"/>
+      <c r="G6" s="159"/>
       <c r="H6" s="46"/>
       <c r="I6" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="J6" s="127">
+      <c r="J6" s="104">
         <v>1230</v>
       </c>
-      <c r="K6" s="115"/>
+      <c r="K6" s="92"/>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="32"/>
@@ -2652,46 +2652,46 @@
       <c r="K7" s="33"/>
     </row>
     <row r="8" spans="1:11" ht="15.5">
-      <c r="A8" s="107" t="s">
+      <c r="A8" s="127" t="s">
         <v>9</v>
       </c>
       <c r="B8" s="56" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="109" t="s">
+      <c r="C8" s="129" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="110"/>
-      <c r="E8" s="111"/>
+      <c r="D8" s="130"/>
+      <c r="E8" s="131"/>
       <c r="F8" s="14"/>
-      <c r="G8" s="112" t="s">
+      <c r="G8" s="132" t="s">
         <v>12</v>
       </c>
-      <c r="H8" s="113"/>
+      <c r="H8" s="89"/>
       <c r="I8" s="14"/>
-      <c r="J8" s="114" t="s">
+      <c r="J8" s="133" t="s">
         <v>13</v>
       </c>
-      <c r="K8" s="115"/>
+      <c r="K8" s="92"/>
     </row>
     <row r="9" spans="1:11" ht="17">
-      <c r="A9" s="108"/>
+      <c r="A9" s="128"/>
       <c r="B9" s="57" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="116" t="s">
+      <c r="C9" s="134" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="72"/>
-      <c r="E9" s="81"/>
+      <c r="D9" s="90"/>
+      <c r="E9" s="110"/>
       <c r="F9" s="22"/>
-      <c r="G9" s="87">
+      <c r="G9" s="109">
         <v>1</v>
       </c>
-      <c r="H9" s="81"/>
+      <c r="H9" s="110"/>
       <c r="I9" s="22"/>
-      <c r="J9" s="88"/>
-      <c r="K9" s="89"/>
+      <c r="J9" s="111"/>
+      <c r="K9" s="103"/>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="32"/>
@@ -2707,128 +2707,128 @@
       <c r="K10" s="34"/>
     </row>
     <row r="11" spans="1:11" ht="18.5">
-      <c r="A11" s="90" t="s">
+      <c r="A11" s="112" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="91"/>
-      <c r="C11" s="91"/>
-      <c r="D11" s="91"/>
-      <c r="E11" s="92"/>
-      <c r="F11" s="93"/>
-      <c r="G11" s="91"/>
-      <c r="H11" s="91"/>
-      <c r="I11" s="91"/>
-      <c r="J11" s="91"/>
-      <c r="K11" s="94"/>
+      <c r="B11" s="113"/>
+      <c r="C11" s="113"/>
+      <c r="D11" s="113"/>
+      <c r="E11" s="114"/>
+      <c r="F11" s="115"/>
+      <c r="G11" s="113"/>
+      <c r="H11" s="113"/>
+      <c r="I11" s="113"/>
+      <c r="J11" s="113"/>
+      <c r="K11" s="116"/>
     </row>
     <row r="12" spans="1:11" ht="12.5" customHeight="1">
-      <c r="A12" s="95" t="s">
+      <c r="A12" s="117" t="s">
         <v>23</v>
       </c>
-      <c r="B12" s="96"/>
-      <c r="C12" s="96"/>
-      <c r="D12" s="96"/>
-      <c r="E12" s="81"/>
+      <c r="B12" s="95"/>
+      <c r="C12" s="95"/>
+      <c r="D12" s="95"/>
+      <c r="E12" s="110"/>
       <c r="F12" s="59"/>
       <c r="G12" s="31"/>
       <c r="H12" s="60"/>
       <c r="I12" s="31"/>
-      <c r="J12" s="117"/>
-      <c r="K12" s="118"/>
+      <c r="J12" s="135"/>
+      <c r="K12" s="136"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="97"/>
-      <c r="B13" s="72"/>
-      <c r="C13" s="72"/>
-      <c r="D13" s="72"/>
-      <c r="E13" s="73"/>
+      <c r="A13" s="96"/>
+      <c r="B13" s="90"/>
+      <c r="C13" s="90"/>
+      <c r="D13" s="90"/>
+      <c r="E13" s="97"/>
       <c r="F13" s="27"/>
       <c r="G13" s="61"/>
       <c r="H13" s="62"/>
       <c r="I13" s="2"/>
-      <c r="J13" s="117"/>
-      <c r="K13" s="118"/>
+      <c r="J13" s="135"/>
+      <c r="K13" s="136"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="98" t="str">
-        <f>""&amp;A12&amp;""</f>
-        <v>GOFEMM20052025002</v>
-      </c>
-      <c r="B14" s="99"/>
-      <c r="C14" s="99"/>
-      <c r="D14" s="99"/>
-      <c r="E14" s="100"/>
+      <c r="A14" s="118" t="str">
+        <f>"*"&amp;A12&amp;"*"</f>
+        <v>*GOFEMM20052025002*</v>
+      </c>
+      <c r="B14" s="119"/>
+      <c r="C14" s="119"/>
+      <c r="D14" s="119"/>
+      <c r="E14" s="120"/>
       <c r="F14" s="27"/>
       <c r="G14" s="62"/>
       <c r="H14" s="62"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="117"/>
-      <c r="K14" s="118"/>
+      <c r="J14" s="135"/>
+      <c r="K14" s="136"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="101"/>
-      <c r="B15" s="102"/>
-      <c r="C15" s="102"/>
-      <c r="D15" s="102"/>
-      <c r="E15" s="103"/>
+      <c r="A15" s="121"/>
+      <c r="B15" s="122"/>
+      <c r="C15" s="122"/>
+      <c r="D15" s="122"/>
+      <c r="E15" s="123"/>
       <c r="F15" s="27"/>
       <c r="G15" s="62"/>
       <c r="H15" s="62"/>
       <c r="I15" s="2"/>
-      <c r="J15" s="117"/>
-      <c r="K15" s="118"/>
+      <c r="J15" s="135"/>
+      <c r="K15" s="136"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="101"/>
-      <c r="B16" s="102"/>
-      <c r="C16" s="102"/>
-      <c r="D16" s="102"/>
-      <c r="E16" s="103"/>
+      <c r="A16" s="121"/>
+      <c r="B16" s="122"/>
+      <c r="C16" s="122"/>
+      <c r="D16" s="122"/>
+      <c r="E16" s="123"/>
       <c r="F16" s="8"/>
       <c r="G16" s="62"/>
       <c r="H16" s="62"/>
       <c r="I16" s="2"/>
-      <c r="J16" s="117"/>
-      <c r="K16" s="118"/>
+      <c r="J16" s="135"/>
+      <c r="K16" s="136"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="101"/>
-      <c r="B17" s="102"/>
-      <c r="C17" s="102"/>
-      <c r="D17" s="102"/>
-      <c r="E17" s="103"/>
+      <c r="A17" s="121"/>
+      <c r="B17" s="122"/>
+      <c r="C17" s="122"/>
+      <c r="D17" s="122"/>
+      <c r="E17" s="123"/>
       <c r="F17" s="27"/>
       <c r="G17" s="62"/>
       <c r="H17" s="62"/>
       <c r="I17" s="2"/>
-      <c r="J17" s="117"/>
-      <c r="K17" s="118"/>
+      <c r="J17" s="135"/>
+      <c r="K17" s="136"/>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="101"/>
-      <c r="B18" s="102"/>
-      <c r="C18" s="102"/>
-      <c r="D18" s="102"/>
-      <c r="E18" s="103"/>
+      <c r="A18" s="121"/>
+      <c r="B18" s="122"/>
+      <c r="C18" s="122"/>
+      <c r="D18" s="122"/>
+      <c r="E18" s="123"/>
       <c r="F18" s="27"/>
       <c r="G18" s="62"/>
       <c r="H18" s="62"/>
       <c r="I18" s="8"/>
-      <c r="J18" s="117"/>
-      <c r="K18" s="118"/>
+      <c r="J18" s="135"/>
+      <c r="K18" s="136"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="104"/>
-      <c r="B19" s="105"/>
-      <c r="C19" s="105"/>
-      <c r="D19" s="105"/>
-      <c r="E19" s="106"/>
+      <c r="A19" s="124"/>
+      <c r="B19" s="125"/>
+      <c r="C19" s="125"/>
+      <c r="D19" s="125"/>
+      <c r="E19" s="126"/>
       <c r="F19" s="63"/>
       <c r="G19" s="62"/>
       <c r="H19" s="62"/>
       <c r="I19" s="27"/>
-      <c r="J19" s="117"/>
-      <c r="K19" s="118"/>
+      <c r="J19" s="135"/>
+      <c r="K19" s="136"/>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="32"/>
@@ -2840,8 +2840,8 @@
       <c r="G20" s="64"/>
       <c r="H20" s="62"/>
       <c r="I20" s="27"/>
-      <c r="J20" s="117"/>
-      <c r="K20" s="118"/>
+      <c r="J20" s="135"/>
+      <c r="K20" s="136"/>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="32"/>
@@ -2853,8 +2853,8 @@
       <c r="G21" s="62"/>
       <c r="H21" s="62"/>
       <c r="I21" s="27"/>
-      <c r="J21" s="117"/>
-      <c r="K21" s="118"/>
+      <c r="J21" s="135"/>
+      <c r="K21" s="136"/>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="32"/>
@@ -2866,8 +2866,8 @@
       <c r="G22" s="62"/>
       <c r="H22" s="62"/>
       <c r="I22" s="27"/>
-      <c r="J22" s="117"/>
-      <c r="K22" s="118"/>
+      <c r="J22" s="135"/>
+      <c r="K22" s="136"/>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="32"/>
@@ -2879,8 +2879,8 @@
       <c r="G23" s="27"/>
       <c r="H23" s="27"/>
       <c r="I23" s="27"/>
-      <c r="J23" s="117"/>
-      <c r="K23" s="118"/>
+      <c r="J23" s="135"/>
+      <c r="K23" s="136"/>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" s="32"/>
@@ -2892,8 +2892,8 @@
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
-      <c r="J24" s="117"/>
-      <c r="K24" s="118"/>
+      <c r="J24" s="135"/>
+      <c r="K24" s="136"/>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="32"/>
@@ -2905,90 +2905,90 @@
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
       <c r="I25" s="9"/>
-      <c r="J25" s="117"/>
-      <c r="K25" s="118"/>
+      <c r="J25" s="135"/>
+      <c r="K25" s="136"/>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="83"/>
-      <c r="B26" s="80"/>
-      <c r="C26" s="80"/>
-      <c r="D26" s="80"/>
-      <c r="E26" s="84"/>
+      <c r="A26" s="105"/>
+      <c r="B26" s="94"/>
+      <c r="C26" s="94"/>
+      <c r="D26" s="94"/>
+      <c r="E26" s="106"/>
       <c r="F26" s="66"/>
       <c r="G26" s="67"/>
       <c r="H26" s="8"/>
       <c r="I26" s="9"/>
-      <c r="J26" s="117"/>
-      <c r="K26" s="118"/>
+      <c r="J26" s="135"/>
+      <c r="K26" s="136"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="80"/>
-      <c r="B27" s="80"/>
-      <c r="C27" s="80"/>
-      <c r="D27" s="80"/>
-      <c r="E27" s="84"/>
+      <c r="A27" s="94"/>
+      <c r="B27" s="94"/>
+      <c r="C27" s="94"/>
+      <c r="D27" s="94"/>
+      <c r="E27" s="106"/>
       <c r="F27" s="68"/>
       <c r="G27" s="67"/>
       <c r="H27" s="8"/>
       <c r="I27" s="9"/>
-      <c r="J27" s="117"/>
-      <c r="K27" s="118"/>
+      <c r="J27" s="135"/>
+      <c r="K27" s="136"/>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="80"/>
-      <c r="B28" s="80"/>
-      <c r="C28" s="80"/>
-      <c r="D28" s="80"/>
-      <c r="E28" s="84"/>
+      <c r="A28" s="94"/>
+      <c r="B28" s="94"/>
+      <c r="C28" s="94"/>
+      <c r="D28" s="94"/>
+      <c r="E28" s="106"/>
       <c r="F28" s="68"/>
       <c r="G28" s="67"/>
       <c r="H28" s="8"/>
       <c r="I28" s="9"/>
-      <c r="J28" s="117"/>
-      <c r="K28" s="118"/>
+      <c r="J28" s="135"/>
+      <c r="K28" s="136"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="80"/>
-      <c r="B29" s="80"/>
-      <c r="C29" s="80"/>
-      <c r="D29" s="80"/>
-      <c r="E29" s="84"/>
+      <c r="A29" s="94"/>
+      <c r="B29" s="94"/>
+      <c r="C29" s="94"/>
+      <c r="D29" s="94"/>
+      <c r="E29" s="106"/>
       <c r="F29" s="69"/>
       <c r="G29" s="70"/>
       <c r="H29" s="65"/>
       <c r="I29" s="23"/>
-      <c r="J29" s="117"/>
-      <c r="K29" s="118"/>
+      <c r="J29" s="135"/>
+      <c r="K29" s="136"/>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="85"/>
-      <c r="B30" s="85"/>
-      <c r="C30" s="85"/>
-      <c r="D30" s="85"/>
-      <c r="E30" s="86"/>
+      <c r="A30" s="107"/>
+      <c r="B30" s="107"/>
+      <c r="C30" s="107"/>
+      <c r="D30" s="107"/>
+      <c r="E30" s="108"/>
       <c r="F30" s="49"/>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
-      <c r="J30" s="117"/>
-      <c r="K30" s="118"/>
+      <c r="J30" s="135"/>
+      <c r="K30" s="136"/>
     </row>
     <row r="31" spans="1:11" ht="15.5">
-      <c r="A31" s="71" t="s">
+      <c r="A31" s="137" t="s">
         <v>17</v>
       </c>
-      <c r="B31" s="72"/>
-      <c r="C31" s="73"/>
+      <c r="B31" s="90"/>
+      <c r="C31" s="97"/>
       <c r="D31" s="50"/>
-      <c r="E31" s="74"/>
-      <c r="F31" s="75"/>
-      <c r="G31" s="75"/>
-      <c r="H31" s="75"/>
-      <c r="I31" s="76" t="s">
+      <c r="E31" s="138"/>
+      <c r="F31" s="139"/>
+      <c r="G31" s="139"/>
+      <c r="H31" s="139"/>
+      <c r="I31" s="140" t="s">
         <v>18</v>
       </c>
-      <c r="J31" s="77"/>
-      <c r="K31" s="78"/>
+      <c r="J31" s="141"/>
+      <c r="K31" s="142"/>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" s="37"/>
@@ -2996,12 +2996,12 @@
       <c r="C32" s="4"/>
       <c r="D32" s="38"/>
       <c r="E32" s="3"/>
-      <c r="F32" s="79"/>
-      <c r="G32" s="80"/>
-      <c r="H32" s="81"/>
-      <c r="I32" s="79"/>
-      <c r="J32" s="80"/>
-      <c r="K32" s="82"/>
+      <c r="F32" s="143"/>
+      <c r="G32" s="94"/>
+      <c r="H32" s="110"/>
+      <c r="I32" s="143"/>
+      <c r="J32" s="94"/>
+      <c r="K32" s="144"/>
     </row>
     <row r="33" spans="1:11">
       <c r="A33" s="39"/>
@@ -3080,27 +3080,16 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="E1:G2"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="A26:E30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="E31:H31"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J30:K30"/>
     <mergeCell ref="A14:E19"/>
     <mergeCell ref="A5:C6"/>
     <mergeCell ref="E5:G5"/>
@@ -3117,16 +3106,27 @@
     <mergeCell ref="A11:E11"/>
     <mergeCell ref="F11:K11"/>
     <mergeCell ref="A12:E13"/>
-    <mergeCell ref="A26:E30"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="E31:H31"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="E1:G2"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J26:K26"/>
   </mergeCells>
   <conditionalFormatting sqref="F12:G15 I12 F17:F22 G17:G19 G21:G22">
     <cfRule type="expression" dxfId="3" priority="1">

</xml_diff>

<commit_message>
feat: add rabat branch
</commit_message>
<xml_diff>
--- a/dummy-content/ECHEC-RETOUR_CLIENT-CASABLANCA.xlsx
+++ b/dummy-content/ECHEC-RETOUR_CLIENT-CASABLANCA.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User1\Desktop\GoFleet-Enhancer\dummy-content\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UNK\Desktop\GoFleet-Enhancer\dummy-content\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEC0E857-1BC1-4997-AA17-053272EDFA2F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1B4C9ED-1BAA-4ECD-9F77-33AFFD184B73}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12110" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ECHEC CASA" sheetId="5" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="23">
   <si>
     <t>ECHEC DE LIVRAISON</t>
   </si>
@@ -33,9 +33,6 @@
   </si>
   <si>
     <t>N° Expedition</t>
-  </si>
-  <si>
-    <t>GO FLEET CASABLANCA</t>
   </si>
   <si>
     <t>ENTREPOT MARJANE MALL</t>
@@ -55,9 +52,6 @@
   </si>
   <si>
     <t>Chauffeur</t>
-  </si>
-  <si>
-    <t>MAROUANE NOUAHY</t>
   </si>
   <si>
     <t>Nombre de palettes</t>
@@ -94,6 +88,9 @@
   </si>
   <si>
     <t>GOFEMM20052025002</t>
+  </si>
+  <si>
+    <t>GO FLEET RABAT</t>
   </si>
 </sst>
 </file>
@@ -1403,66 +1400,24 @@
     <xf numFmtId="0" fontId="15" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="5" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
@@ -1470,10 +1425,10 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="11" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1486,6 +1441,8 @@
     <xf numFmtId="0" fontId="21" fillId="12" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="24" fillId="3" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1509,9 +1466,11 @@
     <xf numFmtId="0" fontId="8" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1521,20 +1480,67 @@
     <xf numFmtId="0" fontId="15" fillId="15" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="5" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="19" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="17" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1549,15 +1555,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="20" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="19" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1662,6 +1659,72 @@
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
     <mruColors>
       <color rgb="FF003399"/>
     </mruColors>
@@ -1879,50 +1942,50 @@
     <tabColor rgb="FF003399"/>
   </sheetPr>
   <dimension ref="A1:K67"/>
-  <sheetFormatPr defaultRowHeight="12.5"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
-    <col min="1" max="1" width="23.54296875" style="28" customWidth="1"/>
-    <col min="2" max="2" width="13.26953125" style="28" customWidth="1"/>
-    <col min="3" max="3" width="4.90625" style="28" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="8.7265625" style="28"/>
-    <col min="5" max="5" width="29.81640625" style="28" customWidth="1"/>
-    <col min="6" max="9" width="14.54296875" style="28" customWidth="1"/>
-    <col min="10" max="10" width="8.7265625" style="28"/>
-    <col min="11" max="11" width="17.453125" style="28" customWidth="1"/>
+    <col min="1" max="1" width="23.5703125" style="28" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" style="28" customWidth="1"/>
+    <col min="3" max="3" width="4.85546875" style="28" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="8.7109375" style="28"/>
+    <col min="5" max="5" width="29.85546875" style="28" customWidth="1"/>
+    <col min="6" max="9" width="14.5703125" style="28" customWidth="1"/>
+    <col min="10" max="10" width="8.7109375" style="28"/>
+    <col min="11" max="11" width="17.42578125" style="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.5" customHeight="1">
-      <c r="A1" s="73"/>
-      <c r="B1" s="74"/>
-      <c r="C1" s="74"/>
+    <row r="1" spans="1:11" ht="15.6" customHeight="1">
+      <c r="A1" s="128"/>
+      <c r="B1" s="129"/>
+      <c r="C1" s="129"/>
       <c r="D1" s="53"/>
-      <c r="E1" s="78" t="s">
+      <c r="E1" s="133" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="79"/>
-      <c r="G1" s="80"/>
+      <c r="F1" s="134"/>
+      <c r="G1" s="135"/>
       <c r="H1" s="29"/>
-      <c r="I1" s="84" t="s">
+      <c r="I1" s="139" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="85"/>
-      <c r="K1" s="86"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.5">
-      <c r="A2" s="75"/>
-      <c r="B2" s="76"/>
-      <c r="C2" s="77"/>
+      <c r="J1" s="140"/>
+      <c r="K1" s="141"/>
+    </row>
+    <row r="2" spans="1:11" ht="15.75">
+      <c r="A2" s="130"/>
+      <c r="B2" s="131"/>
+      <c r="C2" s="132"/>
       <c r="D2" s="53"/>
-      <c r="E2" s="81"/>
-      <c r="F2" s="82"/>
-      <c r="G2" s="83"/>
+      <c r="E2" s="136"/>
+      <c r="F2" s="137"/>
+      <c r="G2" s="138"/>
       <c r="H2" s="15"/>
-      <c r="I2" s="87">
+      <c r="I2" s="142">
         <f ca="1">TODAY()</f>
-        <v>45833</v>
-      </c>
-      <c r="J2" s="82"/>
-      <c r="K2" s="83"/>
+        <v>45864</v>
+      </c>
+      <c r="J2" s="137"/>
+      <c r="K2" s="138"/>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="32"/>
@@ -1937,15 +2000,15 @@
       <c r="J3" s="22"/>
       <c r="K3" s="33"/>
     </row>
-    <row r="4" spans="1:11" ht="17">
-      <c r="A4" s="88" t="s">
+    <row r="4" spans="1:11" ht="17.25">
+      <c r="A4" s="143" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="89"/>
-      <c r="C4" s="90"/>
+      <c r="B4" s="113"/>
+      <c r="C4" s="72"/>
       <c r="D4" s="52"/>
       <c r="E4" s="16" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="55"/>
@@ -1953,46 +2016,46 @@
       <c r="I4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="91"/>
-      <c r="K4" s="92"/>
-    </row>
-    <row r="5" spans="1:11" ht="18.5">
-      <c r="A5" s="93" t="s">
+      <c r="J4" s="144"/>
+      <c r="K4" s="115"/>
+    </row>
+    <row r="5" spans="1:11" ht="18.75">
+      <c r="A5" s="121" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="80"/>
+      <c r="C5" s="96"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="122" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="94"/>
-      <c r="C5" s="95"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="98" t="s">
-        <v>5</v>
-      </c>
-      <c r="F5" s="99"/>
-      <c r="G5" s="100"/>
+      <c r="F5" s="123"/>
+      <c r="G5" s="124"/>
       <c r="H5" s="22"/>
       <c r="I5" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="J5" s="125"/>
+      <c r="K5" s="115"/>
+    </row>
+    <row r="6" spans="1:11" ht="15.75">
+      <c r="A6" s="97"/>
+      <c r="B6" s="72"/>
+      <c r="C6" s="73"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="126" t="s">
         <v>6</v>
       </c>
-      <c r="J5" s="101"/>
-      <c r="K5" s="92"/>
-    </row>
-    <row r="6" spans="1:11" ht="15.5">
-      <c r="A6" s="96"/>
-      <c r="B6" s="90"/>
-      <c r="C6" s="97"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="102" t="s">
-        <v>7</v>
-      </c>
-      <c r="F6" s="90"/>
-      <c r="G6" s="103"/>
+      <c r="F6" s="72"/>
+      <c r="G6" s="89"/>
       <c r="H6" s="46"/>
       <c r="I6" s="21" t="s">
-        <v>8</v>
-      </c>
-      <c r="J6" s="104">
+        <v>7</v>
+      </c>
+      <c r="J6" s="127">
         <v>1230</v>
       </c>
-      <c r="K6" s="92"/>
+      <c r="K6" s="115"/>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="32"/>
@@ -2007,47 +2070,45 @@
       <c r="J7" s="22"/>
       <c r="K7" s="33"/>
     </row>
-    <row r="8" spans="1:11" ht="15.5">
-      <c r="A8" s="127" t="s">
+    <row r="8" spans="1:11" ht="15.75">
+      <c r="A8" s="107" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="56" t="s">
+      <c r="C8" s="109"/>
+      <c r="D8" s="110"/>
+      <c r="E8" s="111"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="112" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="129" t="s">
+      <c r="H8" s="113"/>
+      <c r="I8" s="14"/>
+      <c r="J8" s="114" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="130"/>
-      <c r="E8" s="131"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="132" t="s">
+      <c r="K8" s="115"/>
+    </row>
+    <row r="9" spans="1:11" ht="17.25">
+      <c r="A9" s="108"/>
+      <c r="B9" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="H8" s="89"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="133" t="s">
+      <c r="C9" s="116" t="s">
         <v>13</v>
       </c>
-      <c r="K8" s="92"/>
-    </row>
-    <row r="9" spans="1:11" ht="17">
-      <c r="A9" s="128"/>
-      <c r="B9" s="57" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9" s="134" t="s">
-        <v>15</v>
-      </c>
-      <c r="D9" s="90"/>
-      <c r="E9" s="110"/>
+      <c r="D9" s="72"/>
+      <c r="E9" s="81"/>
       <c r="F9" s="22"/>
-      <c r="G9" s="109">
+      <c r="G9" s="87">
         <v>1</v>
       </c>
-      <c r="H9" s="110"/>
+      <c r="H9" s="81"/>
       <c r="I9" s="22"/>
-      <c r="J9" s="111"/>
-      <c r="K9" s="103"/>
+      <c r="J9" s="88"/>
+      <c r="K9" s="89"/>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="32"/>
@@ -2062,129 +2123,129 @@
       <c r="J10" s="22"/>
       <c r="K10" s="34"/>
     </row>
-    <row r="11" spans="1:11" ht="18.5">
-      <c r="A11" s="112" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="113"/>
-      <c r="C11" s="113"/>
-      <c r="D11" s="113"/>
-      <c r="E11" s="114"/>
-      <c r="F11" s="115"/>
-      <c r="G11" s="113"/>
-      <c r="H11" s="113"/>
-      <c r="I11" s="113"/>
-      <c r="J11" s="113"/>
-      <c r="K11" s="116"/>
+    <row r="11" spans="1:11" ht="18.75">
+      <c r="A11" s="90" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="91"/>
+      <c r="C11" s="91"/>
+      <c r="D11" s="91"/>
+      <c r="E11" s="92"/>
+      <c r="F11" s="93"/>
+      <c r="G11" s="91"/>
+      <c r="H11" s="91"/>
+      <c r="I11" s="91"/>
+      <c r="J11" s="91"/>
+      <c r="K11" s="94"/>
     </row>
     <row r="12" spans="1:11">
-      <c r="A12" s="117" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" s="95"/>
-      <c r="C12" s="95"/>
-      <c r="D12" s="95"/>
-      <c r="E12" s="110"/>
+      <c r="A12" s="95" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="96"/>
+      <c r="C12" s="96"/>
+      <c r="D12" s="96"/>
+      <c r="E12" s="81"/>
       <c r="F12" s="59"/>
       <c r="G12" s="31"/>
       <c r="H12" s="60"/>
       <c r="I12" s="31"/>
-      <c r="J12" s="135"/>
-      <c r="K12" s="136"/>
+      <c r="J12" s="117"/>
+      <c r="K12" s="118"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="96"/>
-      <c r="B13" s="90"/>
-      <c r="C13" s="90"/>
-      <c r="D13" s="90"/>
-      <c r="E13" s="97"/>
+      <c r="A13" s="97"/>
+      <c r="B13" s="72"/>
+      <c r="C13" s="72"/>
+      <c r="D13" s="72"/>
+      <c r="E13" s="73"/>
       <c r="F13" s="27"/>
       <c r="G13" s="61"/>
       <c r="H13" s="62"/>
       <c r="I13" s="2"/>
-      <c r="J13" s="71"/>
-      <c r="K13" s="72"/>
+      <c r="J13" s="119"/>
+      <c r="K13" s="120"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="118" t="str">
+      <c r="A14" s="98" t="str">
         <f>"*"&amp;A12&amp;"*"</f>
         <v>*GOFEMM20052025001*</v>
       </c>
-      <c r="B14" s="119"/>
-      <c r="C14" s="119"/>
-      <c r="D14" s="119"/>
-      <c r="E14" s="120"/>
+      <c r="B14" s="99"/>
+      <c r="C14" s="99"/>
+      <c r="D14" s="99"/>
+      <c r="E14" s="100"/>
       <c r="F14" s="27"/>
       <c r="G14" s="62"/>
       <c r="H14" s="62"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="71"/>
-      <c r="K14" s="72"/>
+      <c r="J14" s="119"/>
+      <c r="K14" s="120"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="121"/>
-      <c r="B15" s="122"/>
-      <c r="C15" s="122"/>
-      <c r="D15" s="122"/>
-      <c r="E15" s="123"/>
+      <c r="A15" s="101"/>
+      <c r="B15" s="102"/>
+      <c r="C15" s="102"/>
+      <c r="D15" s="102"/>
+      <c r="E15" s="103"/>
       <c r="F15" s="27"/>
       <c r="G15" s="62"/>
       <c r="H15" s="62"/>
       <c r="I15" s="2"/>
-      <c r="J15" s="71"/>
-      <c r="K15" s="72"/>
+      <c r="J15" s="119"/>
+      <c r="K15" s="120"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="121"/>
-      <c r="B16" s="122"/>
-      <c r="C16" s="122"/>
-      <c r="D16" s="122"/>
-      <c r="E16" s="123"/>
+      <c r="A16" s="101"/>
+      <c r="B16" s="102"/>
+      <c r="C16" s="102"/>
+      <c r="D16" s="102"/>
+      <c r="E16" s="103"/>
       <c r="F16" s="8"/>
       <c r="G16" s="62"/>
       <c r="H16" s="62"/>
       <c r="I16" s="2"/>
-      <c r="J16" s="71"/>
-      <c r="K16" s="72"/>
+      <c r="J16" s="119"/>
+      <c r="K16" s="120"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="121"/>
-      <c r="B17" s="122"/>
-      <c r="C17" s="122"/>
-      <c r="D17" s="122"/>
-      <c r="E17" s="123"/>
+      <c r="A17" s="101"/>
+      <c r="B17" s="102"/>
+      <c r="C17" s="102"/>
+      <c r="D17" s="102"/>
+      <c r="E17" s="103"/>
       <c r="F17" s="27"/>
       <c r="G17" s="62"/>
       <c r="H17" s="62"/>
       <c r="I17" s="2"/>
-      <c r="J17" s="71"/>
-      <c r="K17" s="72"/>
+      <c r="J17" s="119"/>
+      <c r="K17" s="120"/>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="121"/>
-      <c r="B18" s="122"/>
-      <c r="C18" s="122"/>
-      <c r="D18" s="122"/>
-      <c r="E18" s="123"/>
+      <c r="A18" s="101"/>
+      <c r="B18" s="102"/>
+      <c r="C18" s="102"/>
+      <c r="D18" s="102"/>
+      <c r="E18" s="103"/>
       <c r="F18" s="27"/>
       <c r="G18" s="62"/>
       <c r="H18" s="62"/>
       <c r="I18" s="8"/>
-      <c r="J18" s="71"/>
-      <c r="K18" s="72"/>
+      <c r="J18" s="119"/>
+      <c r="K18" s="120"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="124"/>
-      <c r="B19" s="125"/>
-      <c r="C19" s="125"/>
-      <c r="D19" s="125"/>
-      <c r="E19" s="126"/>
+      <c r="A19" s="104"/>
+      <c r="B19" s="105"/>
+      <c r="C19" s="105"/>
+      <c r="D19" s="105"/>
+      <c r="E19" s="106"/>
       <c r="F19" s="63"/>
       <c r="G19" s="62"/>
       <c r="H19" s="62"/>
       <c r="I19" s="27"/>
-      <c r="J19" s="71"/>
-      <c r="K19" s="72"/>
+      <c r="J19" s="119"/>
+      <c r="K19" s="120"/>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="32"/>
@@ -2196,8 +2257,8 @@
       <c r="G20" s="64"/>
       <c r="H20" s="62"/>
       <c r="I20" s="27"/>
-      <c r="J20" s="71"/>
-      <c r="K20" s="72"/>
+      <c r="J20" s="119"/>
+      <c r="K20" s="120"/>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="32"/>
@@ -2209,8 +2270,8 @@
       <c r="G21" s="62"/>
       <c r="H21" s="62"/>
       <c r="I21" s="27"/>
-      <c r="J21" s="71"/>
-      <c r="K21" s="72"/>
+      <c r="J21" s="119"/>
+      <c r="K21" s="120"/>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="32"/>
@@ -2222,8 +2283,8 @@
       <c r="G22" s="62"/>
       <c r="H22" s="62"/>
       <c r="I22" s="27"/>
-      <c r="J22" s="71"/>
-      <c r="K22" s="72"/>
+      <c r="J22" s="119"/>
+      <c r="K22" s="120"/>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="32"/>
@@ -2235,8 +2296,8 @@
       <c r="G23" s="27"/>
       <c r="H23" s="27"/>
       <c r="I23" s="27"/>
-      <c r="J23" s="71"/>
-      <c r="K23" s="72"/>
+      <c r="J23" s="119"/>
+      <c r="K23" s="120"/>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" s="32"/>
@@ -2248,8 +2309,8 @@
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
-      <c r="J24" s="71"/>
-      <c r="K24" s="72"/>
+      <c r="J24" s="119"/>
+      <c r="K24" s="120"/>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="32"/>
@@ -2261,90 +2322,90 @@
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
       <c r="I25" s="9"/>
-      <c r="J25" s="71"/>
-      <c r="K25" s="72"/>
+      <c r="J25" s="119"/>
+      <c r="K25" s="120"/>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="105"/>
-      <c r="B26" s="94"/>
-      <c r="C26" s="94"/>
-      <c r="D26" s="94"/>
-      <c r="E26" s="106"/>
+      <c r="A26" s="83"/>
+      <c r="B26" s="80"/>
+      <c r="C26" s="80"/>
+      <c r="D26" s="80"/>
+      <c r="E26" s="84"/>
       <c r="F26" s="66"/>
       <c r="G26" s="67"/>
       <c r="H26" s="8"/>
       <c r="I26" s="9"/>
-      <c r="J26" s="71"/>
-      <c r="K26" s="72"/>
+      <c r="J26" s="119"/>
+      <c r="K26" s="120"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="94"/>
-      <c r="B27" s="94"/>
-      <c r="C27" s="94"/>
-      <c r="D27" s="94"/>
-      <c r="E27" s="106"/>
+      <c r="A27" s="80"/>
+      <c r="B27" s="80"/>
+      <c r="C27" s="80"/>
+      <c r="D27" s="80"/>
+      <c r="E27" s="84"/>
       <c r="F27" s="68"/>
       <c r="G27" s="67"/>
       <c r="H27" s="8"/>
       <c r="I27" s="9"/>
-      <c r="J27" s="71"/>
-      <c r="K27" s="72"/>
+      <c r="J27" s="119"/>
+      <c r="K27" s="120"/>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="94"/>
-      <c r="B28" s="94"/>
-      <c r="C28" s="94"/>
-      <c r="D28" s="94"/>
-      <c r="E28" s="106"/>
+      <c r="A28" s="80"/>
+      <c r="B28" s="80"/>
+      <c r="C28" s="80"/>
+      <c r="D28" s="80"/>
+      <c r="E28" s="84"/>
       <c r="F28" s="68"/>
       <c r="G28" s="67"/>
       <c r="H28" s="8"/>
       <c r="I28" s="9"/>
-      <c r="J28" s="71"/>
-      <c r="K28" s="72"/>
+      <c r="J28" s="119"/>
+      <c r="K28" s="120"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="94"/>
-      <c r="B29" s="94"/>
-      <c r="C29" s="94"/>
-      <c r="D29" s="94"/>
-      <c r="E29" s="106"/>
+      <c r="A29" s="80"/>
+      <c r="B29" s="80"/>
+      <c r="C29" s="80"/>
+      <c r="D29" s="80"/>
+      <c r="E29" s="84"/>
       <c r="F29" s="69"/>
       <c r="G29" s="70"/>
       <c r="H29" s="65"/>
       <c r="I29" s="23"/>
-      <c r="J29" s="71"/>
-      <c r="K29" s="72"/>
+      <c r="J29" s="119"/>
+      <c r="K29" s="120"/>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="107"/>
-      <c r="B30" s="107"/>
-      <c r="C30" s="107"/>
-      <c r="D30" s="107"/>
-      <c r="E30" s="108"/>
+      <c r="A30" s="85"/>
+      <c r="B30" s="85"/>
+      <c r="C30" s="85"/>
+      <c r="D30" s="85"/>
+      <c r="E30" s="86"/>
       <c r="F30" s="49"/>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
-      <c r="J30" s="71"/>
-      <c r="K30" s="72"/>
-    </row>
-    <row r="31" spans="1:11" ht="15.5">
-      <c r="A31" s="137" t="s">
-        <v>17</v>
-      </c>
-      <c r="B31" s="90"/>
-      <c r="C31" s="97"/>
+      <c r="J30" s="119"/>
+      <c r="K30" s="120"/>
+    </row>
+    <row r="31" spans="1:11" ht="15.75">
+      <c r="A31" s="71" t="s">
+        <v>15</v>
+      </c>
+      <c r="B31" s="72"/>
+      <c r="C31" s="73"/>
       <c r="D31" s="50"/>
-      <c r="E31" s="138"/>
-      <c r="F31" s="139"/>
-      <c r="G31" s="139"/>
-      <c r="H31" s="139"/>
-      <c r="I31" s="140" t="s">
-        <v>18</v>
-      </c>
-      <c r="J31" s="141"/>
-      <c r="K31" s="142"/>
+      <c r="E31" s="74"/>
+      <c r="F31" s="75"/>
+      <c r="G31" s="75"/>
+      <c r="H31" s="75"/>
+      <c r="I31" s="76" t="s">
+        <v>16</v>
+      </c>
+      <c r="J31" s="77"/>
+      <c r="K31" s="78"/>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" s="37"/>
@@ -2352,12 +2413,12 @@
       <c r="C32" s="4"/>
       <c r="D32" s="38"/>
       <c r="E32" s="3"/>
-      <c r="F32" s="143"/>
-      <c r="G32" s="94"/>
-      <c r="H32" s="110"/>
-      <c r="I32" s="143"/>
-      <c r="J32" s="94"/>
-      <c r="K32" s="144"/>
+      <c r="F32" s="79"/>
+      <c r="G32" s="80"/>
+      <c r="H32" s="81"/>
+      <c r="I32" s="79"/>
+      <c r="J32" s="80"/>
+      <c r="K32" s="82"/>
     </row>
     <row r="33" spans="1:11">
       <c r="A33" s="39"/>
@@ -2395,40 +2456,40 @@
     <row r="38" spans="1:11">
       <c r="A38" s="30"/>
     </row>
-    <row r="45" spans="1:11" ht="15.5">
+    <row r="45" spans="1:11" ht="15.75">
       <c r="J45" s="5"/>
     </row>
-    <row r="46" spans="1:11" ht="13">
+    <row r="46" spans="1:11">
       <c r="J46" s="6"/>
     </row>
-    <row r="47" spans="1:11" ht="15.5">
+    <row r="47" spans="1:11" ht="15.75">
       <c r="J47" s="5"/>
     </row>
-    <row r="48" spans="1:11" ht="13">
+    <row r="48" spans="1:11">
       <c r="J48" s="6"/>
     </row>
-    <row r="49" spans="10:10" ht="15.5">
+    <row r="49" spans="10:10" ht="15.75">
       <c r="J49" s="5"/>
     </row>
-    <row r="50" spans="10:10" ht="13">
+    <row r="50" spans="10:10">
       <c r="J50" s="6"/>
     </row>
-    <row r="51" spans="10:10" ht="15.5">
+    <row r="51" spans="10:10" ht="15.75">
       <c r="J51" s="5"/>
     </row>
-    <row r="52" spans="10:10" ht="13">
+    <row r="52" spans="10:10">
       <c r="J52" s="6"/>
     </row>
-    <row r="53" spans="10:10" ht="15.5">
+    <row r="53" spans="10:10" ht="15.75">
       <c r="J53" s="5"/>
     </row>
-    <row r="54" spans="10:10" ht="13">
+    <row r="54" spans="10:10">
       <c r="J54" s="6"/>
     </row>
-    <row r="55" spans="10:10" ht="15.5">
+    <row r="55" spans="10:10" ht="15.75">
       <c r="J55" s="5"/>
     </row>
-    <row r="56" spans="10:10" ht="13">
+    <row r="56" spans="10:10">
       <c r="J56" s="6"/>
     </row>
     <row r="67" spans="11:11">
@@ -2436,11 +2497,32 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="E31:H31"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="E1:G2"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="A5:C6"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="J6:K6"/>
     <mergeCell ref="A26:E30"/>
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="J9:K9"/>
@@ -2457,32 +2539,11 @@
     <mergeCell ref="J13:K13"/>
     <mergeCell ref="J14:K14"/>
     <mergeCell ref="J15:K15"/>
-    <mergeCell ref="A5:C6"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="E6:G6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="E1:G2"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="E31:H31"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="I32:K32"/>
   </mergeCells>
   <conditionalFormatting sqref="F12:G15 I12 F17:F22 G17:G19 G21:G22">
     <cfRule type="expression" dxfId="7" priority="1">
@@ -2519,54 +2580,54 @@
     <tabColor theme="9" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:K67"/>
-  <sheetFormatPr defaultRowHeight="12.5"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
-    <col min="1" max="1" width="23.54296875" style="28" customWidth="1"/>
-    <col min="2" max="2" width="13.26953125" style="28" customWidth="1"/>
-    <col min="3" max="3" width="4.90625" style="28" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="8.7265625" style="28"/>
-    <col min="5" max="5" width="30.26953125" style="28" customWidth="1"/>
-    <col min="6" max="6" width="16.54296875" style="28" customWidth="1"/>
-    <col min="7" max="8" width="15.54296875" style="28" customWidth="1"/>
-    <col min="9" max="9" width="13.7265625" style="28" customWidth="1"/>
-    <col min="10" max="10" width="9.81640625" style="28" customWidth="1"/>
-    <col min="11" max="11" width="16.1796875" style="28" customWidth="1"/>
+    <col min="1" max="1" width="23.5703125" style="28" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" style="28" customWidth="1"/>
+    <col min="3" max="3" width="4.85546875" style="28" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="8.7109375" style="28"/>
+    <col min="5" max="5" width="30.28515625" style="28" customWidth="1"/>
+    <col min="6" max="6" width="16.5703125" style="28" customWidth="1"/>
+    <col min="7" max="8" width="15.5703125" style="28" customWidth="1"/>
+    <col min="9" max="9" width="13.7109375" style="28" customWidth="1"/>
+    <col min="10" max="10" width="9.85546875" style="28" customWidth="1"/>
+    <col min="11" max="11" width="16.140625" style="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.5" customHeight="1">
-      <c r="A1" s="73" t="s">
-        <v>19</v>
-      </c>
-      <c r="B1" s="74"/>
-      <c r="C1" s="145"/>
+    <row r="1" spans="1:11" ht="15.6" customHeight="1">
+      <c r="A1" s="128" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="129"/>
+      <c r="C1" s="150"/>
       <c r="D1" s="58"/>
-      <c r="E1" s="147" t="s">
-        <v>20</v>
-      </c>
-      <c r="F1" s="148"/>
-      <c r="G1" s="149"/>
+      <c r="E1" s="152" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" s="153"/>
+      <c r="G1" s="154"/>
       <c r="H1" s="29"/>
-      <c r="I1" s="84" t="s">
+      <c r="I1" s="139" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="85"/>
-      <c r="K1" s="86"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.5">
-      <c r="A2" s="75"/>
-      <c r="B2" s="76"/>
-      <c r="C2" s="146"/>
+      <c r="J1" s="140"/>
+      <c r="K1" s="141"/>
+    </row>
+    <row r="2" spans="1:11" ht="15.75">
+      <c r="A2" s="130"/>
+      <c r="B2" s="131"/>
+      <c r="C2" s="151"/>
       <c r="D2" s="52"/>
-      <c r="E2" s="150"/>
-      <c r="F2" s="151"/>
-      <c r="G2" s="152"/>
+      <c r="E2" s="155"/>
+      <c r="F2" s="156"/>
+      <c r="G2" s="157"/>
       <c r="H2" s="15"/>
-      <c r="I2" s="87">
+      <c r="I2" s="142">
         <f ca="1">TODAY()</f>
-        <v>45833</v>
-      </c>
-      <c r="J2" s="82"/>
-      <c r="K2" s="83"/>
+        <v>45864</v>
+      </c>
+      <c r="J2" s="137"/>
+      <c r="K2" s="138"/>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="32"/>
@@ -2581,15 +2642,15 @@
       <c r="J3" s="22"/>
       <c r="K3" s="33"/>
     </row>
-    <row r="4" spans="1:11" ht="17">
-      <c r="A4" s="153" t="s">
+    <row r="4" spans="1:11" ht="17.25">
+      <c r="A4" s="158" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="154"/>
-      <c r="C4" s="76"/>
+      <c r="B4" s="159"/>
+      <c r="C4" s="131"/>
       <c r="D4" s="52"/>
       <c r="E4" s="26" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F4" s="47"/>
       <c r="G4" s="48"/>
@@ -2597,46 +2658,46 @@
       <c r="I4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="91"/>
-      <c r="K4" s="92"/>
-    </row>
-    <row r="5" spans="1:11" ht="18.5">
-      <c r="A5" s="155" t="s">
+      <c r="J4" s="144"/>
+      <c r="K4" s="115"/>
+    </row>
+    <row r="5" spans="1:11" ht="18.75">
+      <c r="A5" s="145" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="146"/>
+      <c r="C5" s="132"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="122" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="156"/>
-      <c r="C5" s="77"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="98" t="s">
-        <v>5</v>
-      </c>
-      <c r="F5" s="99"/>
-      <c r="G5" s="100"/>
+      <c r="F5" s="123"/>
+      <c r="G5" s="124"/>
       <c r="H5" s="22"/>
       <c r="I5" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="J5" s="125"/>
+      <c r="K5" s="115"/>
+    </row>
+    <row r="6" spans="1:11" ht="15.75">
+      <c r="A6" s="130"/>
+      <c r="B6" s="131"/>
+      <c r="C6" s="147"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="148" t="s">
         <v>6</v>
       </c>
-      <c r="J5" s="101"/>
-      <c r="K5" s="92"/>
-    </row>
-    <row r="6" spans="1:11" ht="15.5">
-      <c r="A6" s="75"/>
-      <c r="B6" s="76"/>
-      <c r="C6" s="157"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="158" t="s">
-        <v>7</v>
-      </c>
-      <c r="F6" s="76"/>
-      <c r="G6" s="159"/>
+      <c r="F6" s="131"/>
+      <c r="G6" s="149"/>
       <c r="H6" s="46"/>
       <c r="I6" s="21" t="s">
-        <v>8</v>
-      </c>
-      <c r="J6" s="104">
+        <v>7</v>
+      </c>
+      <c r="J6" s="127">
         <v>1230</v>
       </c>
-      <c r="K6" s="92"/>
+      <c r="K6" s="115"/>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="32"/>
@@ -2651,47 +2712,45 @@
       <c r="J7" s="22"/>
       <c r="K7" s="33"/>
     </row>
-    <row r="8" spans="1:11" ht="15.5">
-      <c r="A8" s="127" t="s">
+    <row r="8" spans="1:11" ht="15.75">
+      <c r="A8" s="107" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="56" t="s">
+      <c r="C8" s="109"/>
+      <c r="D8" s="110"/>
+      <c r="E8" s="111"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="112" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="129" t="s">
+      <c r="H8" s="113"/>
+      <c r="I8" s="14"/>
+      <c r="J8" s="114" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="130"/>
-      <c r="E8" s="131"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="132" t="s">
+      <c r="K8" s="115"/>
+    </row>
+    <row r="9" spans="1:11" ht="17.25">
+      <c r="A9" s="108"/>
+      <c r="B9" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="H8" s="89"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="133" t="s">
+      <c r="C9" s="116" t="s">
         <v>13</v>
       </c>
-      <c r="K8" s="92"/>
-    </row>
-    <row r="9" spans="1:11" ht="17">
-      <c r="A9" s="128"/>
-      <c r="B9" s="57" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9" s="134" t="s">
-        <v>15</v>
-      </c>
-      <c r="D9" s="90"/>
-      <c r="E9" s="110"/>
+      <c r="D9" s="72"/>
+      <c r="E9" s="81"/>
       <c r="F9" s="22"/>
-      <c r="G9" s="109">
+      <c r="G9" s="87">
         <v>1</v>
       </c>
-      <c r="H9" s="110"/>
+      <c r="H9" s="81"/>
       <c r="I9" s="22"/>
-      <c r="J9" s="111"/>
-      <c r="K9" s="103"/>
+      <c r="J9" s="88"/>
+      <c r="K9" s="89"/>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="32"/>
@@ -2706,129 +2765,129 @@
       <c r="J10" s="22"/>
       <c r="K10" s="34"/>
     </row>
-    <row r="11" spans="1:11" ht="18.5">
-      <c r="A11" s="112" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="113"/>
-      <c r="C11" s="113"/>
-      <c r="D11" s="113"/>
-      <c r="E11" s="114"/>
-      <c r="F11" s="115"/>
-      <c r="G11" s="113"/>
-      <c r="H11" s="113"/>
-      <c r="I11" s="113"/>
-      <c r="J11" s="113"/>
-      <c r="K11" s="116"/>
-    </row>
-    <row r="12" spans="1:11" ht="12.5" customHeight="1">
-      <c r="A12" s="117" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" s="95"/>
-      <c r="C12" s="95"/>
-      <c r="D12" s="95"/>
-      <c r="E12" s="110"/>
+    <row r="11" spans="1:11" ht="18.75">
+      <c r="A11" s="90" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="91"/>
+      <c r="C11" s="91"/>
+      <c r="D11" s="91"/>
+      <c r="E11" s="92"/>
+      <c r="F11" s="93"/>
+      <c r="G11" s="91"/>
+      <c r="H11" s="91"/>
+      <c r="I11" s="91"/>
+      <c r="J11" s="91"/>
+      <c r="K11" s="94"/>
+    </row>
+    <row r="12" spans="1:11" ht="12.6" customHeight="1">
+      <c r="A12" s="95" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="96"/>
+      <c r="C12" s="96"/>
+      <c r="D12" s="96"/>
+      <c r="E12" s="81"/>
       <c r="F12" s="59"/>
       <c r="G12" s="31"/>
       <c r="H12" s="60"/>
       <c r="I12" s="31"/>
-      <c r="J12" s="135"/>
-      <c r="K12" s="136"/>
+      <c r="J12" s="117"/>
+      <c r="K12" s="118"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="96"/>
-      <c r="B13" s="90"/>
-      <c r="C13" s="90"/>
-      <c r="D13" s="90"/>
-      <c r="E13" s="97"/>
+      <c r="A13" s="97"/>
+      <c r="B13" s="72"/>
+      <c r="C13" s="72"/>
+      <c r="D13" s="72"/>
+      <c r="E13" s="73"/>
       <c r="F13" s="27"/>
       <c r="G13" s="61"/>
       <c r="H13" s="62"/>
       <c r="I13" s="2"/>
-      <c r="J13" s="135"/>
-      <c r="K13" s="136"/>
+      <c r="J13" s="117"/>
+      <c r="K13" s="118"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="118" t="str">
+      <c r="A14" s="98" t="str">
         <f>"*"&amp;A12&amp;"*"</f>
         <v>*GOFEMM20052025002*</v>
       </c>
-      <c r="B14" s="119"/>
-      <c r="C14" s="119"/>
-      <c r="D14" s="119"/>
-      <c r="E14" s="120"/>
+      <c r="B14" s="99"/>
+      <c r="C14" s="99"/>
+      <c r="D14" s="99"/>
+      <c r="E14" s="100"/>
       <c r="F14" s="27"/>
       <c r="G14" s="62"/>
       <c r="H14" s="62"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="135"/>
-      <c r="K14" s="136"/>
+      <c r="J14" s="117"/>
+      <c r="K14" s="118"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="121"/>
-      <c r="B15" s="122"/>
-      <c r="C15" s="122"/>
-      <c r="D15" s="122"/>
-      <c r="E15" s="123"/>
+      <c r="A15" s="101"/>
+      <c r="B15" s="102"/>
+      <c r="C15" s="102"/>
+      <c r="D15" s="102"/>
+      <c r="E15" s="103"/>
       <c r="F15" s="27"/>
       <c r="G15" s="62"/>
       <c r="H15" s="62"/>
       <c r="I15" s="2"/>
-      <c r="J15" s="135"/>
-      <c r="K15" s="136"/>
+      <c r="J15" s="117"/>
+      <c r="K15" s="118"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="121"/>
-      <c r="B16" s="122"/>
-      <c r="C16" s="122"/>
-      <c r="D16" s="122"/>
-      <c r="E16" s="123"/>
+      <c r="A16" s="101"/>
+      <c r="B16" s="102"/>
+      <c r="C16" s="102"/>
+      <c r="D16" s="102"/>
+      <c r="E16" s="103"/>
       <c r="F16" s="8"/>
       <c r="G16" s="62"/>
       <c r="H16" s="62"/>
       <c r="I16" s="2"/>
-      <c r="J16" s="135"/>
-      <c r="K16" s="136"/>
+      <c r="J16" s="117"/>
+      <c r="K16" s="118"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="121"/>
-      <c r="B17" s="122"/>
-      <c r="C17" s="122"/>
-      <c r="D17" s="122"/>
-      <c r="E17" s="123"/>
+      <c r="A17" s="101"/>
+      <c r="B17" s="102"/>
+      <c r="C17" s="102"/>
+      <c r="D17" s="102"/>
+      <c r="E17" s="103"/>
       <c r="F17" s="27"/>
       <c r="G17" s="62"/>
       <c r="H17" s="62"/>
       <c r="I17" s="2"/>
-      <c r="J17" s="135"/>
-      <c r="K17" s="136"/>
+      <c r="J17" s="117"/>
+      <c r="K17" s="118"/>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="121"/>
-      <c r="B18" s="122"/>
-      <c r="C18" s="122"/>
-      <c r="D18" s="122"/>
-      <c r="E18" s="123"/>
+      <c r="A18" s="101"/>
+      <c r="B18" s="102"/>
+      <c r="C18" s="102"/>
+      <c r="D18" s="102"/>
+      <c r="E18" s="103"/>
       <c r="F18" s="27"/>
       <c r="G18" s="62"/>
       <c r="H18" s="62"/>
       <c r="I18" s="8"/>
-      <c r="J18" s="135"/>
-      <c r="K18" s="136"/>
+      <c r="J18" s="117"/>
+      <c r="K18" s="118"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="124"/>
-      <c r="B19" s="125"/>
-      <c r="C19" s="125"/>
-      <c r="D19" s="125"/>
-      <c r="E19" s="126"/>
+      <c r="A19" s="104"/>
+      <c r="B19" s="105"/>
+      <c r="C19" s="105"/>
+      <c r="D19" s="105"/>
+      <c r="E19" s="106"/>
       <c r="F19" s="63"/>
       <c r="G19" s="62"/>
       <c r="H19" s="62"/>
       <c r="I19" s="27"/>
-      <c r="J19" s="135"/>
-      <c r="K19" s="136"/>
+      <c r="J19" s="117"/>
+      <c r="K19" s="118"/>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="32"/>
@@ -2840,8 +2899,8 @@
       <c r="G20" s="64"/>
       <c r="H20" s="62"/>
       <c r="I20" s="27"/>
-      <c r="J20" s="135"/>
-      <c r="K20" s="136"/>
+      <c r="J20" s="117"/>
+      <c r="K20" s="118"/>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="32"/>
@@ -2853,8 +2912,8 @@
       <c r="G21" s="62"/>
       <c r="H21" s="62"/>
       <c r="I21" s="27"/>
-      <c r="J21" s="135"/>
-      <c r="K21" s="136"/>
+      <c r="J21" s="117"/>
+      <c r="K21" s="118"/>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="32"/>
@@ -2866,8 +2925,8 @@
       <c r="G22" s="62"/>
       <c r="H22" s="62"/>
       <c r="I22" s="27"/>
-      <c r="J22" s="135"/>
-      <c r="K22" s="136"/>
+      <c r="J22" s="117"/>
+      <c r="K22" s="118"/>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="32"/>
@@ -2879,8 +2938,8 @@
       <c r="G23" s="27"/>
       <c r="H23" s="27"/>
       <c r="I23" s="27"/>
-      <c r="J23" s="135"/>
-      <c r="K23" s="136"/>
+      <c r="J23" s="117"/>
+      <c r="K23" s="118"/>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" s="32"/>
@@ -2892,8 +2951,8 @@
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
-      <c r="J24" s="135"/>
-      <c r="K24" s="136"/>
+      <c r="J24" s="117"/>
+      <c r="K24" s="118"/>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="32"/>
@@ -2905,90 +2964,90 @@
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
       <c r="I25" s="9"/>
-      <c r="J25" s="135"/>
-      <c r="K25" s="136"/>
+      <c r="J25" s="117"/>
+      <c r="K25" s="118"/>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="105"/>
-      <c r="B26" s="94"/>
-      <c r="C26" s="94"/>
-      <c r="D26" s="94"/>
-      <c r="E26" s="106"/>
+      <c r="A26" s="83"/>
+      <c r="B26" s="80"/>
+      <c r="C26" s="80"/>
+      <c r="D26" s="80"/>
+      <c r="E26" s="84"/>
       <c r="F26" s="66"/>
       <c r="G26" s="67"/>
       <c r="H26" s="8"/>
       <c r="I26" s="9"/>
-      <c r="J26" s="135"/>
-      <c r="K26" s="136"/>
+      <c r="J26" s="117"/>
+      <c r="K26" s="118"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="94"/>
-      <c r="B27" s="94"/>
-      <c r="C27" s="94"/>
-      <c r="D27" s="94"/>
-      <c r="E27" s="106"/>
+      <c r="A27" s="80"/>
+      <c r="B27" s="80"/>
+      <c r="C27" s="80"/>
+      <c r="D27" s="80"/>
+      <c r="E27" s="84"/>
       <c r="F27" s="68"/>
       <c r="G27" s="67"/>
       <c r="H27" s="8"/>
       <c r="I27" s="9"/>
-      <c r="J27" s="135"/>
-      <c r="K27" s="136"/>
+      <c r="J27" s="117"/>
+      <c r="K27" s="118"/>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="94"/>
-      <c r="B28" s="94"/>
-      <c r="C28" s="94"/>
-      <c r="D28" s="94"/>
-      <c r="E28" s="106"/>
+      <c r="A28" s="80"/>
+      <c r="B28" s="80"/>
+      <c r="C28" s="80"/>
+      <c r="D28" s="80"/>
+      <c r="E28" s="84"/>
       <c r="F28" s="68"/>
       <c r="G28" s="67"/>
       <c r="H28" s="8"/>
       <c r="I28" s="9"/>
-      <c r="J28" s="135"/>
-      <c r="K28" s="136"/>
+      <c r="J28" s="117"/>
+      <c r="K28" s="118"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="94"/>
-      <c r="B29" s="94"/>
-      <c r="C29" s="94"/>
-      <c r="D29" s="94"/>
-      <c r="E29" s="106"/>
+      <c r="A29" s="80"/>
+      <c r="B29" s="80"/>
+      <c r="C29" s="80"/>
+      <c r="D29" s="80"/>
+      <c r="E29" s="84"/>
       <c r="F29" s="69"/>
       <c r="G29" s="70"/>
       <c r="H29" s="65"/>
       <c r="I29" s="23"/>
-      <c r="J29" s="135"/>
-      <c r="K29" s="136"/>
+      <c r="J29" s="117"/>
+      <c r="K29" s="118"/>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="107"/>
-      <c r="B30" s="107"/>
-      <c r="C30" s="107"/>
-      <c r="D30" s="107"/>
-      <c r="E30" s="108"/>
+      <c r="A30" s="85"/>
+      <c r="B30" s="85"/>
+      <c r="C30" s="85"/>
+      <c r="D30" s="85"/>
+      <c r="E30" s="86"/>
       <c r="F30" s="49"/>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
-      <c r="J30" s="135"/>
-      <c r="K30" s="136"/>
-    </row>
-    <row r="31" spans="1:11" ht="15.5">
-      <c r="A31" s="137" t="s">
-        <v>17</v>
-      </c>
-      <c r="B31" s="90"/>
-      <c r="C31" s="97"/>
+      <c r="J30" s="117"/>
+      <c r="K30" s="118"/>
+    </row>
+    <row r="31" spans="1:11" ht="15.75">
+      <c r="A31" s="71" t="s">
+        <v>15</v>
+      </c>
+      <c r="B31" s="72"/>
+      <c r="C31" s="73"/>
       <c r="D31" s="50"/>
-      <c r="E31" s="138"/>
-      <c r="F31" s="139"/>
-      <c r="G31" s="139"/>
-      <c r="H31" s="139"/>
-      <c r="I31" s="140" t="s">
-        <v>18</v>
-      </c>
-      <c r="J31" s="141"/>
-      <c r="K31" s="142"/>
+      <c r="E31" s="74"/>
+      <c r="F31" s="75"/>
+      <c r="G31" s="75"/>
+      <c r="H31" s="75"/>
+      <c r="I31" s="76" t="s">
+        <v>16</v>
+      </c>
+      <c r="J31" s="77"/>
+      <c r="K31" s="78"/>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" s="37"/>
@@ -2996,12 +3055,12 @@
       <c r="C32" s="4"/>
       <c r="D32" s="38"/>
       <c r="E32" s="3"/>
-      <c r="F32" s="143"/>
-      <c r="G32" s="94"/>
-      <c r="H32" s="110"/>
-      <c r="I32" s="143"/>
-      <c r="J32" s="94"/>
-      <c r="K32" s="144"/>
+      <c r="F32" s="79"/>
+      <c r="G32" s="80"/>
+      <c r="H32" s="81"/>
+      <c r="I32" s="79"/>
+      <c r="J32" s="80"/>
+      <c r="K32" s="82"/>
     </row>
     <row r="33" spans="1:11">
       <c r="A33" s="39"/>
@@ -3039,40 +3098,40 @@
     <row r="38" spans="1:11">
       <c r="A38" s="30"/>
     </row>
-    <row r="45" spans="1:11" ht="15.5">
+    <row r="45" spans="1:11" ht="15.75">
       <c r="J45" s="5"/>
     </row>
-    <row r="46" spans="1:11" ht="13">
+    <row r="46" spans="1:11">
       <c r="J46" s="6"/>
     </row>
-    <row r="47" spans="1:11" ht="15.5">
+    <row r="47" spans="1:11" ht="15.75">
       <c r="J47" s="5"/>
     </row>
-    <row r="48" spans="1:11" ht="13">
+    <row r="48" spans="1:11">
       <c r="J48" s="6"/>
     </row>
-    <row r="49" spans="10:10" ht="15.5">
+    <row r="49" spans="10:10" ht="15.75">
       <c r="J49" s="5"/>
     </row>
-    <row r="50" spans="10:10" ht="13">
+    <row r="50" spans="10:10">
       <c r="J50" s="6"/>
     </row>
-    <row r="51" spans="10:10" ht="15.5">
+    <row r="51" spans="10:10" ht="15.75">
       <c r="J51" s="5"/>
     </row>
-    <row r="52" spans="10:10" ht="13">
+    <row r="52" spans="10:10">
       <c r="J52" s="6"/>
     </row>
-    <row r="53" spans="10:10" ht="15.5">
+    <row r="53" spans="10:10" ht="15.75">
       <c r="J53" s="5"/>
     </row>
-    <row r="54" spans="10:10" ht="13">
+    <row r="54" spans="10:10">
       <c r="J54" s="6"/>
     </row>
-    <row r="55" spans="10:10" ht="15.5">
+    <row r="55" spans="10:10" ht="15.75">
       <c r="J55" s="5"/>
     </row>
-    <row r="56" spans="10:10" ht="13">
+    <row r="56" spans="10:10">
       <c r="J56" s="6"/>
     </row>
     <row r="67" spans="11:11">
@@ -3080,16 +3139,27 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="A26:E30"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="E31:H31"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="E1:G2"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="J4:K4"/>
     <mergeCell ref="A14:E19"/>
     <mergeCell ref="A5:C6"/>
     <mergeCell ref="E5:G5"/>
@@ -3106,27 +3176,16 @@
     <mergeCell ref="A11:E11"/>
     <mergeCell ref="F11:K11"/>
     <mergeCell ref="A12:E13"/>
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="E1:G2"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="A26:E30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="E31:H31"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J30:K30"/>
   </mergeCells>
   <conditionalFormatting sqref="F12:G15 I12 F17:F22 G17:G19 G21:G22">
     <cfRule type="expression" dxfId="3" priority="1">

</xml_diff>

<commit_message>
feat: add fes  branch
</commit_message>
<xml_diff>
--- a/dummy-content/ECHEC-RETOUR_CLIENT-CASABLANCA.xlsx
+++ b/dummy-content/ECHEC-RETOUR_CLIENT-CASABLANCA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UNK\Desktop\GoFleet-Enhancer\dummy-content\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1B4C9ED-1BAA-4ECD-9F77-33AFFD184B73}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{879B84F3-3B23-4C58-A575-ACF97916BF11}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ECHEC CASA" sheetId="5" r:id="rId1"/>
@@ -90,7 +90,7 @@
     <t>GOFEMM20052025002</t>
   </si>
   <si>
-    <t>GO FLEET RABAT</t>
+    <t>GO FLEET FES</t>
   </si>
 </sst>
 </file>
@@ -1400,24 +1400,66 @@
     <xf numFmtId="0" fontId="15" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="5" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
@@ -1425,10 +1467,10 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="11" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1441,8 +1483,6 @@
     <xf numFmtId="0" fontId="21" fillId="12" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="24" fillId="3" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1466,11 +1506,9 @@
     <xf numFmtId="0" fontId="8" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1480,67 +1518,20 @@
     <xf numFmtId="0" fontId="15" fillId="15" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="5" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="20" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="19" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="17" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1555,6 +1546,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="19" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1955,37 +1955,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.6" customHeight="1">
-      <c r="A1" s="128"/>
-      <c r="B1" s="129"/>
-      <c r="C1" s="129"/>
+      <c r="A1" s="73"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
       <c r="D1" s="53"/>
-      <c r="E1" s="133" t="s">
+      <c r="E1" s="78" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="134"/>
-      <c r="G1" s="135"/>
+      <c r="F1" s="79"/>
+      <c r="G1" s="80"/>
       <c r="H1" s="29"/>
-      <c r="I1" s="139" t="s">
+      <c r="I1" s="84" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="140"/>
-      <c r="K1" s="141"/>
+      <c r="J1" s="85"/>
+      <c r="K1" s="86"/>
     </row>
     <row r="2" spans="1:11" ht="15.75">
-      <c r="A2" s="130"/>
-      <c r="B2" s="131"/>
-      <c r="C2" s="132"/>
+      <c r="A2" s="75"/>
+      <c r="B2" s="76"/>
+      <c r="C2" s="77"/>
       <c r="D2" s="53"/>
-      <c r="E2" s="136"/>
-      <c r="F2" s="137"/>
-      <c r="G2" s="138"/>
+      <c r="E2" s="81"/>
+      <c r="F2" s="82"/>
+      <c r="G2" s="83"/>
       <c r="H2" s="15"/>
-      <c r="I2" s="142">
+      <c r="I2" s="87">
         <f ca="1">TODAY()</f>
         <v>45864</v>
       </c>
-      <c r="J2" s="137"/>
-      <c r="K2" s="138"/>
+      <c r="J2" s="82"/>
+      <c r="K2" s="83"/>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="32"/>
@@ -2001,11 +2001,11 @@
       <c r="K3" s="33"/>
     </row>
     <row r="4" spans="1:11" ht="17.25">
-      <c r="A4" s="143" t="s">
+      <c r="A4" s="88" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="113"/>
-      <c r="C4" s="72"/>
+      <c r="B4" s="89"/>
+      <c r="C4" s="90"/>
       <c r="D4" s="52"/>
       <c r="E4" s="16" t="s">
         <v>19</v>
@@ -2016,46 +2016,46 @@
       <c r="I4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="144"/>
-      <c r="K4" s="115"/>
+      <c r="J4" s="91"/>
+      <c r="K4" s="92"/>
     </row>
     <row r="5" spans="1:11" ht="18.75">
-      <c r="A5" s="121" t="s">
+      <c r="A5" s="93" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="80"/>
-      <c r="C5" s="96"/>
+      <c r="B5" s="94"/>
+      <c r="C5" s="95"/>
       <c r="D5" s="14"/>
-      <c r="E5" s="122" t="s">
+      <c r="E5" s="98" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="123"/>
-      <c r="G5" s="124"/>
+      <c r="F5" s="99"/>
+      <c r="G5" s="100"/>
       <c r="H5" s="22"/>
       <c r="I5" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="J5" s="125"/>
-      <c r="K5" s="115"/>
+      <c r="J5" s="101"/>
+      <c r="K5" s="92"/>
     </row>
     <row r="6" spans="1:11" ht="15.75">
-      <c r="A6" s="97"/>
-      <c r="B6" s="72"/>
-      <c r="C6" s="73"/>
+      <c r="A6" s="96"/>
+      <c r="B6" s="90"/>
+      <c r="C6" s="97"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="126" t="s">
+      <c r="E6" s="102" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="72"/>
-      <c r="G6" s="89"/>
+      <c r="F6" s="90"/>
+      <c r="G6" s="103"/>
       <c r="H6" s="46"/>
       <c r="I6" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="127">
+      <c r="J6" s="104">
         <v>1230</v>
       </c>
-      <c r="K6" s="115"/>
+      <c r="K6" s="92"/>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="32"/>
@@ -2071,44 +2071,44 @@
       <c r="K7" s="33"/>
     </row>
     <row r="8" spans="1:11" ht="15.75">
-      <c r="A8" s="107" t="s">
+      <c r="A8" s="127" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="109"/>
-      <c r="D8" s="110"/>
-      <c r="E8" s="111"/>
+      <c r="C8" s="129"/>
+      <c r="D8" s="130"/>
+      <c r="E8" s="131"/>
       <c r="F8" s="14"/>
-      <c r="G8" s="112" t="s">
+      <c r="G8" s="132" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="113"/>
+      <c r="H8" s="89"/>
       <c r="I8" s="14"/>
-      <c r="J8" s="114" t="s">
+      <c r="J8" s="133" t="s">
         <v>11</v>
       </c>
-      <c r="K8" s="115"/>
+      <c r="K8" s="92"/>
     </row>
     <row r="9" spans="1:11" ht="17.25">
-      <c r="A9" s="108"/>
+      <c r="A9" s="128"/>
       <c r="B9" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="116" t="s">
+      <c r="C9" s="134" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="72"/>
-      <c r="E9" s="81"/>
+      <c r="D9" s="90"/>
+      <c r="E9" s="110"/>
       <c r="F9" s="22"/>
-      <c r="G9" s="87">
+      <c r="G9" s="109">
         <v>1</v>
       </c>
-      <c r="H9" s="81"/>
+      <c r="H9" s="110"/>
       <c r="I9" s="22"/>
-      <c r="J9" s="88"/>
-      <c r="K9" s="89"/>
+      <c r="J9" s="111"/>
+      <c r="K9" s="103"/>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="32"/>
@@ -2124,128 +2124,128 @@
       <c r="K10" s="34"/>
     </row>
     <row r="11" spans="1:11" ht="18.75">
-      <c r="A11" s="90" t="s">
+      <c r="A11" s="112" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="91"/>
-      <c r="C11" s="91"/>
-      <c r="D11" s="91"/>
-      <c r="E11" s="92"/>
-      <c r="F11" s="93"/>
-      <c r="G11" s="91"/>
-      <c r="H11" s="91"/>
-      <c r="I11" s="91"/>
-      <c r="J11" s="91"/>
-      <c r="K11" s="94"/>
+      <c r="B11" s="113"/>
+      <c r="C11" s="113"/>
+      <c r="D11" s="113"/>
+      <c r="E11" s="114"/>
+      <c r="F11" s="115"/>
+      <c r="G11" s="113"/>
+      <c r="H11" s="113"/>
+      <c r="I11" s="113"/>
+      <c r="J11" s="113"/>
+      <c r="K11" s="116"/>
     </row>
     <row r="12" spans="1:11">
-      <c r="A12" s="95" t="s">
+      <c r="A12" s="117" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="96"/>
-      <c r="C12" s="96"/>
-      <c r="D12" s="96"/>
-      <c r="E12" s="81"/>
+      <c r="B12" s="95"/>
+      <c r="C12" s="95"/>
+      <c r="D12" s="95"/>
+      <c r="E12" s="110"/>
       <c r="F12" s="59"/>
       <c r="G12" s="31"/>
       <c r="H12" s="60"/>
       <c r="I12" s="31"/>
-      <c r="J12" s="117"/>
-      <c r="K12" s="118"/>
+      <c r="J12" s="135"/>
+      <c r="K12" s="136"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="97"/>
-      <c r="B13" s="72"/>
-      <c r="C13" s="72"/>
-      <c r="D13" s="72"/>
-      <c r="E13" s="73"/>
+      <c r="A13" s="96"/>
+      <c r="B13" s="90"/>
+      <c r="C13" s="90"/>
+      <c r="D13" s="90"/>
+      <c r="E13" s="97"/>
       <c r="F13" s="27"/>
       <c r="G13" s="61"/>
       <c r="H13" s="62"/>
       <c r="I13" s="2"/>
-      <c r="J13" s="119"/>
-      <c r="K13" s="120"/>
+      <c r="J13" s="71"/>
+      <c r="K13" s="72"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="98" t="str">
+      <c r="A14" s="118" t="str">
         <f>"*"&amp;A12&amp;"*"</f>
         <v>*GOFEMM20052025001*</v>
       </c>
-      <c r="B14" s="99"/>
-      <c r="C14" s="99"/>
-      <c r="D14" s="99"/>
-      <c r="E14" s="100"/>
+      <c r="B14" s="119"/>
+      <c r="C14" s="119"/>
+      <c r="D14" s="119"/>
+      <c r="E14" s="120"/>
       <c r="F14" s="27"/>
       <c r="G14" s="62"/>
       <c r="H14" s="62"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="119"/>
-      <c r="K14" s="120"/>
+      <c r="J14" s="71"/>
+      <c r="K14" s="72"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="101"/>
-      <c r="B15" s="102"/>
-      <c r="C15" s="102"/>
-      <c r="D15" s="102"/>
-      <c r="E15" s="103"/>
+      <c r="A15" s="121"/>
+      <c r="B15" s="122"/>
+      <c r="C15" s="122"/>
+      <c r="D15" s="122"/>
+      <c r="E15" s="123"/>
       <c r="F15" s="27"/>
       <c r="G15" s="62"/>
       <c r="H15" s="62"/>
       <c r="I15" s="2"/>
-      <c r="J15" s="119"/>
-      <c r="K15" s="120"/>
+      <c r="J15" s="71"/>
+      <c r="K15" s="72"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="101"/>
-      <c r="B16" s="102"/>
-      <c r="C16" s="102"/>
-      <c r="D16" s="102"/>
-      <c r="E16" s="103"/>
+      <c r="A16" s="121"/>
+      <c r="B16" s="122"/>
+      <c r="C16" s="122"/>
+      <c r="D16" s="122"/>
+      <c r="E16" s="123"/>
       <c r="F16" s="8"/>
       <c r="G16" s="62"/>
       <c r="H16" s="62"/>
       <c r="I16" s="2"/>
-      <c r="J16" s="119"/>
-      <c r="K16" s="120"/>
+      <c r="J16" s="71"/>
+      <c r="K16" s="72"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="101"/>
-      <c r="B17" s="102"/>
-      <c r="C17" s="102"/>
-      <c r="D17" s="102"/>
-      <c r="E17" s="103"/>
+      <c r="A17" s="121"/>
+      <c r="B17" s="122"/>
+      <c r="C17" s="122"/>
+      <c r="D17" s="122"/>
+      <c r="E17" s="123"/>
       <c r="F17" s="27"/>
       <c r="G17" s="62"/>
       <c r="H17" s="62"/>
       <c r="I17" s="2"/>
-      <c r="J17" s="119"/>
-      <c r="K17" s="120"/>
+      <c r="J17" s="71"/>
+      <c r="K17" s="72"/>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="101"/>
-      <c r="B18" s="102"/>
-      <c r="C18" s="102"/>
-      <c r="D18" s="102"/>
-      <c r="E18" s="103"/>
+      <c r="A18" s="121"/>
+      <c r="B18" s="122"/>
+      <c r="C18" s="122"/>
+      <c r="D18" s="122"/>
+      <c r="E18" s="123"/>
       <c r="F18" s="27"/>
       <c r="G18" s="62"/>
       <c r="H18" s="62"/>
       <c r="I18" s="8"/>
-      <c r="J18" s="119"/>
-      <c r="K18" s="120"/>
+      <c r="J18" s="71"/>
+      <c r="K18" s="72"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="104"/>
-      <c r="B19" s="105"/>
-      <c r="C19" s="105"/>
-      <c r="D19" s="105"/>
-      <c r="E19" s="106"/>
+      <c r="A19" s="124"/>
+      <c r="B19" s="125"/>
+      <c r="C19" s="125"/>
+      <c r="D19" s="125"/>
+      <c r="E19" s="126"/>
       <c r="F19" s="63"/>
       <c r="G19" s="62"/>
       <c r="H19" s="62"/>
       <c r="I19" s="27"/>
-      <c r="J19" s="119"/>
-      <c r="K19" s="120"/>
+      <c r="J19" s="71"/>
+      <c r="K19" s="72"/>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="32"/>
@@ -2257,8 +2257,8 @@
       <c r="G20" s="64"/>
       <c r="H20" s="62"/>
       <c r="I20" s="27"/>
-      <c r="J20" s="119"/>
-      <c r="K20" s="120"/>
+      <c r="J20" s="71"/>
+      <c r="K20" s="72"/>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="32"/>
@@ -2270,8 +2270,8 @@
       <c r="G21" s="62"/>
       <c r="H21" s="62"/>
       <c r="I21" s="27"/>
-      <c r="J21" s="119"/>
-      <c r="K21" s="120"/>
+      <c r="J21" s="71"/>
+      <c r="K21" s="72"/>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="32"/>
@@ -2283,8 +2283,8 @@
       <c r="G22" s="62"/>
       <c r="H22" s="62"/>
       <c r="I22" s="27"/>
-      <c r="J22" s="119"/>
-      <c r="K22" s="120"/>
+      <c r="J22" s="71"/>
+      <c r="K22" s="72"/>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="32"/>
@@ -2296,8 +2296,8 @@
       <c r="G23" s="27"/>
       <c r="H23" s="27"/>
       <c r="I23" s="27"/>
-      <c r="J23" s="119"/>
-      <c r="K23" s="120"/>
+      <c r="J23" s="71"/>
+      <c r="K23" s="72"/>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" s="32"/>
@@ -2309,8 +2309,8 @@
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
-      <c r="J24" s="119"/>
-      <c r="K24" s="120"/>
+      <c r="J24" s="71"/>
+      <c r="K24" s="72"/>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="32"/>
@@ -2322,90 +2322,90 @@
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
       <c r="I25" s="9"/>
-      <c r="J25" s="119"/>
-      <c r="K25" s="120"/>
+      <c r="J25" s="71"/>
+      <c r="K25" s="72"/>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="83"/>
-      <c r="B26" s="80"/>
-      <c r="C26" s="80"/>
-      <c r="D26" s="80"/>
-      <c r="E26" s="84"/>
+      <c r="A26" s="105"/>
+      <c r="B26" s="94"/>
+      <c r="C26" s="94"/>
+      <c r="D26" s="94"/>
+      <c r="E26" s="106"/>
       <c r="F26" s="66"/>
       <c r="G26" s="67"/>
       <c r="H26" s="8"/>
       <c r="I26" s="9"/>
-      <c r="J26" s="119"/>
-      <c r="K26" s="120"/>
+      <c r="J26" s="71"/>
+      <c r="K26" s="72"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="80"/>
-      <c r="B27" s="80"/>
-      <c r="C27" s="80"/>
-      <c r="D27" s="80"/>
-      <c r="E27" s="84"/>
+      <c r="A27" s="94"/>
+      <c r="B27" s="94"/>
+      <c r="C27" s="94"/>
+      <c r="D27" s="94"/>
+      <c r="E27" s="106"/>
       <c r="F27" s="68"/>
       <c r="G27" s="67"/>
       <c r="H27" s="8"/>
       <c r="I27" s="9"/>
-      <c r="J27" s="119"/>
-      <c r="K27" s="120"/>
+      <c r="J27" s="71"/>
+      <c r="K27" s="72"/>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="80"/>
-      <c r="B28" s="80"/>
-      <c r="C28" s="80"/>
-      <c r="D28" s="80"/>
-      <c r="E28" s="84"/>
+      <c r="A28" s="94"/>
+      <c r="B28" s="94"/>
+      <c r="C28" s="94"/>
+      <c r="D28" s="94"/>
+      <c r="E28" s="106"/>
       <c r="F28" s="68"/>
       <c r="G28" s="67"/>
       <c r="H28" s="8"/>
       <c r="I28" s="9"/>
-      <c r="J28" s="119"/>
-      <c r="K28" s="120"/>
+      <c r="J28" s="71"/>
+      <c r="K28" s="72"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="80"/>
-      <c r="B29" s="80"/>
-      <c r="C29" s="80"/>
-      <c r="D29" s="80"/>
-      <c r="E29" s="84"/>
+      <c r="A29" s="94"/>
+      <c r="B29" s="94"/>
+      <c r="C29" s="94"/>
+      <c r="D29" s="94"/>
+      <c r="E29" s="106"/>
       <c r="F29" s="69"/>
       <c r="G29" s="70"/>
       <c r="H29" s="65"/>
       <c r="I29" s="23"/>
-      <c r="J29" s="119"/>
-      <c r="K29" s="120"/>
+      <c r="J29" s="71"/>
+      <c r="K29" s="72"/>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="85"/>
-      <c r="B30" s="85"/>
-      <c r="C30" s="85"/>
-      <c r="D30" s="85"/>
-      <c r="E30" s="86"/>
+      <c r="A30" s="107"/>
+      <c r="B30" s="107"/>
+      <c r="C30" s="107"/>
+      <c r="D30" s="107"/>
+      <c r="E30" s="108"/>
       <c r="F30" s="49"/>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
-      <c r="J30" s="119"/>
-      <c r="K30" s="120"/>
+      <c r="J30" s="71"/>
+      <c r="K30" s="72"/>
     </row>
     <row r="31" spans="1:11" ht="15.75">
-      <c r="A31" s="71" t="s">
+      <c r="A31" s="137" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="72"/>
-      <c r="C31" s="73"/>
+      <c r="B31" s="90"/>
+      <c r="C31" s="97"/>
       <c r="D31" s="50"/>
-      <c r="E31" s="74"/>
-      <c r="F31" s="75"/>
-      <c r="G31" s="75"/>
-      <c r="H31" s="75"/>
-      <c r="I31" s="76" t="s">
+      <c r="E31" s="138"/>
+      <c r="F31" s="139"/>
+      <c r="G31" s="139"/>
+      <c r="H31" s="139"/>
+      <c r="I31" s="140" t="s">
         <v>16</v>
       </c>
-      <c r="J31" s="77"/>
-      <c r="K31" s="78"/>
+      <c r="J31" s="141"/>
+      <c r="K31" s="142"/>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" s="37"/>
@@ -2413,12 +2413,12 @@
       <c r="C32" s="4"/>
       <c r="D32" s="38"/>
       <c r="E32" s="3"/>
-      <c r="F32" s="79"/>
-      <c r="G32" s="80"/>
-      <c r="H32" s="81"/>
-      <c r="I32" s="79"/>
-      <c r="J32" s="80"/>
-      <c r="K32" s="82"/>
+      <c r="F32" s="143"/>
+      <c r="G32" s="94"/>
+      <c r="H32" s="110"/>
+      <c r="I32" s="143"/>
+      <c r="J32" s="94"/>
+      <c r="K32" s="144"/>
     </row>
     <row r="33" spans="1:11">
       <c r="A33" s="39"/>
@@ -2497,32 +2497,11 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J30:K30"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="E1:G2"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="A5:C6"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="E6:G6"/>
-    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="E31:H31"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="I32:K32"/>
     <mergeCell ref="A26:E30"/>
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="J9:K9"/>
@@ -2539,11 +2518,32 @@
     <mergeCell ref="J13:K13"/>
     <mergeCell ref="J14:K14"/>
     <mergeCell ref="J15:K15"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="E31:H31"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="A5:C6"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="E1:G2"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J30:K30"/>
   </mergeCells>
   <conditionalFormatting sqref="F12:G15 I12 F17:F22 G17:G19 G21:G22">
     <cfRule type="expression" dxfId="7" priority="1">
@@ -2595,39 +2595,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.6" customHeight="1">
-      <c r="A1" s="128" t="s">
+      <c r="A1" s="73" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="129"/>
-      <c r="C1" s="150"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="145"/>
       <c r="D1" s="58"/>
-      <c r="E1" s="152" t="s">
+      <c r="E1" s="147" t="s">
         <v>18</v>
       </c>
-      <c r="F1" s="153"/>
-      <c r="G1" s="154"/>
+      <c r="F1" s="148"/>
+      <c r="G1" s="149"/>
       <c r="H1" s="29"/>
-      <c r="I1" s="139" t="s">
+      <c r="I1" s="84" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="140"/>
-      <c r="K1" s="141"/>
+      <c r="J1" s="85"/>
+      <c r="K1" s="86"/>
     </row>
     <row r="2" spans="1:11" ht="15.75">
-      <c r="A2" s="130"/>
-      <c r="B2" s="131"/>
-      <c r="C2" s="151"/>
+      <c r="A2" s="75"/>
+      <c r="B2" s="76"/>
+      <c r="C2" s="146"/>
       <c r="D2" s="52"/>
-      <c r="E2" s="155"/>
-      <c r="F2" s="156"/>
-      <c r="G2" s="157"/>
+      <c r="E2" s="150"/>
+      <c r="F2" s="151"/>
+      <c r="G2" s="152"/>
       <c r="H2" s="15"/>
-      <c r="I2" s="142">
+      <c r="I2" s="87">
         <f ca="1">TODAY()</f>
         <v>45864</v>
       </c>
-      <c r="J2" s="137"/>
-      <c r="K2" s="138"/>
+      <c r="J2" s="82"/>
+      <c r="K2" s="83"/>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="32"/>
@@ -2643,11 +2643,11 @@
       <c r="K3" s="33"/>
     </row>
     <row r="4" spans="1:11" ht="17.25">
-      <c r="A4" s="158" t="s">
+      <c r="A4" s="153" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="159"/>
-      <c r="C4" s="131"/>
+      <c r="B4" s="154"/>
+      <c r="C4" s="76"/>
       <c r="D4" s="52"/>
       <c r="E4" s="26" t="s">
         <v>19</v>
@@ -2658,46 +2658,46 @@
       <c r="I4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="144"/>
-      <c r="K4" s="115"/>
+      <c r="J4" s="91"/>
+      <c r="K4" s="92"/>
     </row>
     <row r="5" spans="1:11" ht="18.75">
-      <c r="A5" s="145" t="s">
+      <c r="A5" s="155" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="146"/>
-      <c r="C5" s="132"/>
+      <c r="B5" s="156"/>
+      <c r="C5" s="77"/>
       <c r="D5" s="14"/>
-      <c r="E5" s="122" t="s">
+      <c r="E5" s="98" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="123"/>
-      <c r="G5" s="124"/>
+      <c r="F5" s="99"/>
+      <c r="G5" s="100"/>
       <c r="H5" s="22"/>
       <c r="I5" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="J5" s="125"/>
-      <c r="K5" s="115"/>
+      <c r="J5" s="101"/>
+      <c r="K5" s="92"/>
     </row>
     <row r="6" spans="1:11" ht="15.75">
-      <c r="A6" s="130"/>
-      <c r="B6" s="131"/>
-      <c r="C6" s="147"/>
+      <c r="A6" s="75"/>
+      <c r="B6" s="76"/>
+      <c r="C6" s="157"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="148" t="s">
+      <c r="E6" s="158" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="131"/>
-      <c r="G6" s="149"/>
+      <c r="F6" s="76"/>
+      <c r="G6" s="159"/>
       <c r="H6" s="46"/>
       <c r="I6" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="127">
+      <c r="J6" s="104">
         <v>1230</v>
       </c>
-      <c r="K6" s="115"/>
+      <c r="K6" s="92"/>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="32"/>
@@ -2713,44 +2713,44 @@
       <c r="K7" s="33"/>
     </row>
     <row r="8" spans="1:11" ht="15.75">
-      <c r="A8" s="107" t="s">
+      <c r="A8" s="127" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="109"/>
-      <c r="D8" s="110"/>
-      <c r="E8" s="111"/>
+      <c r="C8" s="129"/>
+      <c r="D8" s="130"/>
+      <c r="E8" s="131"/>
       <c r="F8" s="14"/>
-      <c r="G8" s="112" t="s">
+      <c r="G8" s="132" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="113"/>
+      <c r="H8" s="89"/>
       <c r="I8" s="14"/>
-      <c r="J8" s="114" t="s">
+      <c r="J8" s="133" t="s">
         <v>11</v>
       </c>
-      <c r="K8" s="115"/>
+      <c r="K8" s="92"/>
     </row>
     <row r="9" spans="1:11" ht="17.25">
-      <c r="A9" s="108"/>
+      <c r="A9" s="128"/>
       <c r="B9" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="116" t="s">
+      <c r="C9" s="134" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="72"/>
-      <c r="E9" s="81"/>
+      <c r="D9" s="90"/>
+      <c r="E9" s="110"/>
       <c r="F9" s="22"/>
-      <c r="G9" s="87">
+      <c r="G9" s="109">
         <v>1</v>
       </c>
-      <c r="H9" s="81"/>
+      <c r="H9" s="110"/>
       <c r="I9" s="22"/>
-      <c r="J9" s="88"/>
-      <c r="K9" s="89"/>
+      <c r="J9" s="111"/>
+      <c r="K9" s="103"/>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="32"/>
@@ -2766,128 +2766,128 @@
       <c r="K10" s="34"/>
     </row>
     <row r="11" spans="1:11" ht="18.75">
-      <c r="A11" s="90" t="s">
+      <c r="A11" s="112" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="91"/>
-      <c r="C11" s="91"/>
-      <c r="D11" s="91"/>
-      <c r="E11" s="92"/>
-      <c r="F11" s="93"/>
-      <c r="G11" s="91"/>
-      <c r="H11" s="91"/>
-      <c r="I11" s="91"/>
-      <c r="J11" s="91"/>
-      <c r="K11" s="94"/>
+      <c r="B11" s="113"/>
+      <c r="C11" s="113"/>
+      <c r="D11" s="113"/>
+      <c r="E11" s="114"/>
+      <c r="F11" s="115"/>
+      <c r="G11" s="113"/>
+      <c r="H11" s="113"/>
+      <c r="I11" s="113"/>
+      <c r="J11" s="113"/>
+      <c r="K11" s="116"/>
     </row>
     <row r="12" spans="1:11" ht="12.6" customHeight="1">
-      <c r="A12" s="95" t="s">
+      <c r="A12" s="117" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="96"/>
-      <c r="C12" s="96"/>
-      <c r="D12" s="96"/>
-      <c r="E12" s="81"/>
+      <c r="B12" s="95"/>
+      <c r="C12" s="95"/>
+      <c r="D12" s="95"/>
+      <c r="E12" s="110"/>
       <c r="F12" s="59"/>
       <c r="G12" s="31"/>
       <c r="H12" s="60"/>
       <c r="I12" s="31"/>
-      <c r="J12" s="117"/>
-      <c r="K12" s="118"/>
+      <c r="J12" s="135"/>
+      <c r="K12" s="136"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="97"/>
-      <c r="B13" s="72"/>
-      <c r="C13" s="72"/>
-      <c r="D13" s="72"/>
-      <c r="E13" s="73"/>
+      <c r="A13" s="96"/>
+      <c r="B13" s="90"/>
+      <c r="C13" s="90"/>
+      <c r="D13" s="90"/>
+      <c r="E13" s="97"/>
       <c r="F13" s="27"/>
       <c r="G13" s="61"/>
       <c r="H13" s="62"/>
       <c r="I13" s="2"/>
-      <c r="J13" s="117"/>
-      <c r="K13" s="118"/>
+      <c r="J13" s="135"/>
+      <c r="K13" s="136"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="98" t="str">
+      <c r="A14" s="118" t="str">
         <f>"*"&amp;A12&amp;"*"</f>
         <v>*GOFEMM20052025002*</v>
       </c>
-      <c r="B14" s="99"/>
-      <c r="C14" s="99"/>
-      <c r="D14" s="99"/>
-      <c r="E14" s="100"/>
+      <c r="B14" s="119"/>
+      <c r="C14" s="119"/>
+      <c r="D14" s="119"/>
+      <c r="E14" s="120"/>
       <c r="F14" s="27"/>
       <c r="G14" s="62"/>
       <c r="H14" s="62"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="117"/>
-      <c r="K14" s="118"/>
+      <c r="J14" s="135"/>
+      <c r="K14" s="136"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="101"/>
-      <c r="B15" s="102"/>
-      <c r="C15" s="102"/>
-      <c r="D15" s="102"/>
-      <c r="E15" s="103"/>
+      <c r="A15" s="121"/>
+      <c r="B15" s="122"/>
+      <c r="C15" s="122"/>
+      <c r="D15" s="122"/>
+      <c r="E15" s="123"/>
       <c r="F15" s="27"/>
       <c r="G15" s="62"/>
       <c r="H15" s="62"/>
       <c r="I15" s="2"/>
-      <c r="J15" s="117"/>
-      <c r="K15" s="118"/>
+      <c r="J15" s="135"/>
+      <c r="K15" s="136"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="101"/>
-      <c r="B16" s="102"/>
-      <c r="C16" s="102"/>
-      <c r="D16" s="102"/>
-      <c r="E16" s="103"/>
+      <c r="A16" s="121"/>
+      <c r="B16" s="122"/>
+      <c r="C16" s="122"/>
+      <c r="D16" s="122"/>
+      <c r="E16" s="123"/>
       <c r="F16" s="8"/>
       <c r="G16" s="62"/>
       <c r="H16" s="62"/>
       <c r="I16" s="2"/>
-      <c r="J16" s="117"/>
-      <c r="K16" s="118"/>
+      <c r="J16" s="135"/>
+      <c r="K16" s="136"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="101"/>
-      <c r="B17" s="102"/>
-      <c r="C17" s="102"/>
-      <c r="D17" s="102"/>
-      <c r="E17" s="103"/>
+      <c r="A17" s="121"/>
+      <c r="B17" s="122"/>
+      <c r="C17" s="122"/>
+      <c r="D17" s="122"/>
+      <c r="E17" s="123"/>
       <c r="F17" s="27"/>
       <c r="G17" s="62"/>
       <c r="H17" s="62"/>
       <c r="I17" s="2"/>
-      <c r="J17" s="117"/>
-      <c r="K17" s="118"/>
+      <c r="J17" s="135"/>
+      <c r="K17" s="136"/>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="101"/>
-      <c r="B18" s="102"/>
-      <c r="C18" s="102"/>
-      <c r="D18" s="102"/>
-      <c r="E18" s="103"/>
+      <c r="A18" s="121"/>
+      <c r="B18" s="122"/>
+      <c r="C18" s="122"/>
+      <c r="D18" s="122"/>
+      <c r="E18" s="123"/>
       <c r="F18" s="27"/>
       <c r="G18" s="62"/>
       <c r="H18" s="62"/>
       <c r="I18" s="8"/>
-      <c r="J18" s="117"/>
-      <c r="K18" s="118"/>
+      <c r="J18" s="135"/>
+      <c r="K18" s="136"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="104"/>
-      <c r="B19" s="105"/>
-      <c r="C19" s="105"/>
-      <c r="D19" s="105"/>
-      <c r="E19" s="106"/>
+      <c r="A19" s="124"/>
+      <c r="B19" s="125"/>
+      <c r="C19" s="125"/>
+      <c r="D19" s="125"/>
+      <c r="E19" s="126"/>
       <c r="F19" s="63"/>
       <c r="G19" s="62"/>
       <c r="H19" s="62"/>
       <c r="I19" s="27"/>
-      <c r="J19" s="117"/>
-      <c r="K19" s="118"/>
+      <c r="J19" s="135"/>
+      <c r="K19" s="136"/>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="32"/>
@@ -2899,8 +2899,8 @@
       <c r="G20" s="64"/>
       <c r="H20" s="62"/>
       <c r="I20" s="27"/>
-      <c r="J20" s="117"/>
-      <c r="K20" s="118"/>
+      <c r="J20" s="135"/>
+      <c r="K20" s="136"/>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="32"/>
@@ -2912,8 +2912,8 @@
       <c r="G21" s="62"/>
       <c r="H21" s="62"/>
       <c r="I21" s="27"/>
-      <c r="J21" s="117"/>
-      <c r="K21" s="118"/>
+      <c r="J21" s="135"/>
+      <c r="K21" s="136"/>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="32"/>
@@ -2925,8 +2925,8 @@
       <c r="G22" s="62"/>
       <c r="H22" s="62"/>
       <c r="I22" s="27"/>
-      <c r="J22" s="117"/>
-      <c r="K22" s="118"/>
+      <c r="J22" s="135"/>
+      <c r="K22" s="136"/>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="32"/>
@@ -2938,8 +2938,8 @@
       <c r="G23" s="27"/>
       <c r="H23" s="27"/>
       <c r="I23" s="27"/>
-      <c r="J23" s="117"/>
-      <c r="K23" s="118"/>
+      <c r="J23" s="135"/>
+      <c r="K23" s="136"/>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" s="32"/>
@@ -2951,8 +2951,8 @@
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
-      <c r="J24" s="117"/>
-      <c r="K24" s="118"/>
+      <c r="J24" s="135"/>
+      <c r="K24" s="136"/>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="32"/>
@@ -2964,90 +2964,90 @@
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
       <c r="I25" s="9"/>
-      <c r="J25" s="117"/>
-      <c r="K25" s="118"/>
+      <c r="J25" s="135"/>
+      <c r="K25" s="136"/>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="83"/>
-      <c r="B26" s="80"/>
-      <c r="C26" s="80"/>
-      <c r="D26" s="80"/>
-      <c r="E26" s="84"/>
+      <c r="A26" s="105"/>
+      <c r="B26" s="94"/>
+      <c r="C26" s="94"/>
+      <c r="D26" s="94"/>
+      <c r="E26" s="106"/>
       <c r="F26" s="66"/>
       <c r="G26" s="67"/>
       <c r="H26" s="8"/>
       <c r="I26" s="9"/>
-      <c r="J26" s="117"/>
-      <c r="K26" s="118"/>
+      <c r="J26" s="135"/>
+      <c r="K26" s="136"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="80"/>
-      <c r="B27" s="80"/>
-      <c r="C27" s="80"/>
-      <c r="D27" s="80"/>
-      <c r="E27" s="84"/>
+      <c r="A27" s="94"/>
+      <c r="B27" s="94"/>
+      <c r="C27" s="94"/>
+      <c r="D27" s="94"/>
+      <c r="E27" s="106"/>
       <c r="F27" s="68"/>
       <c r="G27" s="67"/>
       <c r="H27" s="8"/>
       <c r="I27" s="9"/>
-      <c r="J27" s="117"/>
-      <c r="K27" s="118"/>
+      <c r="J27" s="135"/>
+      <c r="K27" s="136"/>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="80"/>
-      <c r="B28" s="80"/>
-      <c r="C28" s="80"/>
-      <c r="D28" s="80"/>
-      <c r="E28" s="84"/>
+      <c r="A28" s="94"/>
+      <c r="B28" s="94"/>
+      <c r="C28" s="94"/>
+      <c r="D28" s="94"/>
+      <c r="E28" s="106"/>
       <c r="F28" s="68"/>
       <c r="G28" s="67"/>
       <c r="H28" s="8"/>
       <c r="I28" s="9"/>
-      <c r="J28" s="117"/>
-      <c r="K28" s="118"/>
+      <c r="J28" s="135"/>
+      <c r="K28" s="136"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="80"/>
-      <c r="B29" s="80"/>
-      <c r="C29" s="80"/>
-      <c r="D29" s="80"/>
-      <c r="E29" s="84"/>
+      <c r="A29" s="94"/>
+      <c r="B29" s="94"/>
+      <c r="C29" s="94"/>
+      <c r="D29" s="94"/>
+      <c r="E29" s="106"/>
       <c r="F29" s="69"/>
       <c r="G29" s="70"/>
       <c r="H29" s="65"/>
       <c r="I29" s="23"/>
-      <c r="J29" s="117"/>
-      <c r="K29" s="118"/>
+      <c r="J29" s="135"/>
+      <c r="K29" s="136"/>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="85"/>
-      <c r="B30" s="85"/>
-      <c r="C30" s="85"/>
-      <c r="D30" s="85"/>
-      <c r="E30" s="86"/>
+      <c r="A30" s="107"/>
+      <c r="B30" s="107"/>
+      <c r="C30" s="107"/>
+      <c r="D30" s="107"/>
+      <c r="E30" s="108"/>
       <c r="F30" s="49"/>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
-      <c r="J30" s="117"/>
-      <c r="K30" s="118"/>
+      <c r="J30" s="135"/>
+      <c r="K30" s="136"/>
     </row>
     <row r="31" spans="1:11" ht="15.75">
-      <c r="A31" s="71" t="s">
+      <c r="A31" s="137" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="72"/>
-      <c r="C31" s="73"/>
+      <c r="B31" s="90"/>
+      <c r="C31" s="97"/>
       <c r="D31" s="50"/>
-      <c r="E31" s="74"/>
-      <c r="F31" s="75"/>
-      <c r="G31" s="75"/>
-      <c r="H31" s="75"/>
-      <c r="I31" s="76" t="s">
+      <c r="E31" s="138"/>
+      <c r="F31" s="139"/>
+      <c r="G31" s="139"/>
+      <c r="H31" s="139"/>
+      <c r="I31" s="140" t="s">
         <v>16</v>
       </c>
-      <c r="J31" s="77"/>
-      <c r="K31" s="78"/>
+      <c r="J31" s="141"/>
+      <c r="K31" s="142"/>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" s="37"/>
@@ -3055,12 +3055,12 @@
       <c r="C32" s="4"/>
       <c r="D32" s="38"/>
       <c r="E32" s="3"/>
-      <c r="F32" s="79"/>
-      <c r="G32" s="80"/>
-      <c r="H32" s="81"/>
-      <c r="I32" s="79"/>
-      <c r="J32" s="80"/>
-      <c r="K32" s="82"/>
+      <c r="F32" s="143"/>
+      <c r="G32" s="94"/>
+      <c r="H32" s="110"/>
+      <c r="I32" s="143"/>
+      <c r="J32" s="94"/>
+      <c r="K32" s="144"/>
     </row>
     <row r="33" spans="1:11">
       <c r="A33" s="39"/>
@@ -3139,27 +3139,16 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="E1:G2"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="A26:E30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="E31:H31"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J30:K30"/>
     <mergeCell ref="A14:E19"/>
     <mergeCell ref="A5:C6"/>
     <mergeCell ref="E5:G5"/>
@@ -3176,16 +3165,27 @@
     <mergeCell ref="A11:E11"/>
     <mergeCell ref="F11:K11"/>
     <mergeCell ref="A12:E13"/>
-    <mergeCell ref="A26:E30"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="E31:H31"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="E1:G2"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J26:K26"/>
   </mergeCells>
   <conditionalFormatting sqref="F12:G15 I12 F17:F22 G17:G19 G21:G22">
     <cfRule type="expression" dxfId="3" priority="1">

</xml_diff>

<commit_message>
feat: add meknes  branch
</commit_message>
<xml_diff>
--- a/dummy-content/ECHEC-RETOUR_CLIENT-CASABLANCA.xlsx
+++ b/dummy-content/ECHEC-RETOUR_CLIENT-CASABLANCA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UNK\Desktop\GoFleet-Enhancer\dummy-content\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{879B84F3-3B23-4C58-A575-ACF97916BF11}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4EC71F9-E2CC-4694-BB7B-C5BBE004612B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ECHEC CASA" sheetId="5" r:id="rId1"/>
@@ -90,7 +90,7 @@
     <t>GOFEMM20052025002</t>
   </si>
   <si>
-    <t>GO FLEET FES</t>
+    <t>GO FLEET MEKNES</t>
   </si>
 </sst>
 </file>
@@ -1400,66 +1400,24 @@
     <xf numFmtId="0" fontId="15" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="5" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
@@ -1467,10 +1425,10 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="11" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1483,6 +1441,8 @@
     <xf numFmtId="0" fontId="21" fillId="12" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="24" fillId="3" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1506,9 +1466,11 @@
     <xf numFmtId="0" fontId="8" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1518,20 +1480,67 @@
     <xf numFmtId="0" fontId="15" fillId="15" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="5" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="19" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="17" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1546,15 +1555,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="20" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="19" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1955,37 +1955,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.6" customHeight="1">
-      <c r="A1" s="73"/>
-      <c r="B1" s="74"/>
-      <c r="C1" s="74"/>
+      <c r="A1" s="128"/>
+      <c r="B1" s="129"/>
+      <c r="C1" s="129"/>
       <c r="D1" s="53"/>
-      <c r="E1" s="78" t="s">
+      <c r="E1" s="133" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="79"/>
-      <c r="G1" s="80"/>
+      <c r="F1" s="134"/>
+      <c r="G1" s="135"/>
       <c r="H1" s="29"/>
-      <c r="I1" s="84" t="s">
+      <c r="I1" s="139" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="85"/>
-      <c r="K1" s="86"/>
+      <c r="J1" s="140"/>
+      <c r="K1" s="141"/>
     </row>
     <row r="2" spans="1:11" ht="15.75">
-      <c r="A2" s="75"/>
-      <c r="B2" s="76"/>
-      <c r="C2" s="77"/>
+      <c r="A2" s="130"/>
+      <c r="B2" s="131"/>
+      <c r="C2" s="132"/>
       <c r="D2" s="53"/>
-      <c r="E2" s="81"/>
-      <c r="F2" s="82"/>
-      <c r="G2" s="83"/>
+      <c r="E2" s="136"/>
+      <c r="F2" s="137"/>
+      <c r="G2" s="138"/>
       <c r="H2" s="15"/>
-      <c r="I2" s="87">
+      <c r="I2" s="142">
         <f ca="1">TODAY()</f>
         <v>45864</v>
       </c>
-      <c r="J2" s="82"/>
-      <c r="K2" s="83"/>
+      <c r="J2" s="137"/>
+      <c r="K2" s="138"/>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="32"/>
@@ -2001,11 +2001,11 @@
       <c r="K3" s="33"/>
     </row>
     <row r="4" spans="1:11" ht="17.25">
-      <c r="A4" s="88" t="s">
+      <c r="A4" s="143" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="89"/>
-      <c r="C4" s="90"/>
+      <c r="B4" s="113"/>
+      <c r="C4" s="72"/>
       <c r="D4" s="52"/>
       <c r="E4" s="16" t="s">
         <v>19</v>
@@ -2016,46 +2016,46 @@
       <c r="I4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="91"/>
-      <c r="K4" s="92"/>
+      <c r="J4" s="144"/>
+      <c r="K4" s="115"/>
     </row>
     <row r="5" spans="1:11" ht="18.75">
-      <c r="A5" s="93" t="s">
+      <c r="A5" s="121" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="94"/>
-      <c r="C5" s="95"/>
+      <c r="B5" s="80"/>
+      <c r="C5" s="96"/>
       <c r="D5" s="14"/>
-      <c r="E5" s="98" t="s">
+      <c r="E5" s="122" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="99"/>
-      <c r="G5" s="100"/>
+      <c r="F5" s="123"/>
+      <c r="G5" s="124"/>
       <c r="H5" s="22"/>
       <c r="I5" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="J5" s="101"/>
-      <c r="K5" s="92"/>
+      <c r="J5" s="125"/>
+      <c r="K5" s="115"/>
     </row>
     <row r="6" spans="1:11" ht="15.75">
-      <c r="A6" s="96"/>
-      <c r="B6" s="90"/>
-      <c r="C6" s="97"/>
+      <c r="A6" s="97"/>
+      <c r="B6" s="72"/>
+      <c r="C6" s="73"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="102" t="s">
+      <c r="E6" s="126" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="90"/>
-      <c r="G6" s="103"/>
+      <c r="F6" s="72"/>
+      <c r="G6" s="89"/>
       <c r="H6" s="46"/>
       <c r="I6" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="104">
+      <c r="J6" s="127">
         <v>1230</v>
       </c>
-      <c r="K6" s="92"/>
+      <c r="K6" s="115"/>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="32"/>
@@ -2071,44 +2071,44 @@
       <c r="K7" s="33"/>
     </row>
     <row r="8" spans="1:11" ht="15.75">
-      <c r="A8" s="127" t="s">
+      <c r="A8" s="107" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="129"/>
-      <c r="D8" s="130"/>
-      <c r="E8" s="131"/>
+      <c r="C8" s="109"/>
+      <c r="D8" s="110"/>
+      <c r="E8" s="111"/>
       <c r="F8" s="14"/>
-      <c r="G8" s="132" t="s">
+      <c r="G8" s="112" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="89"/>
+      <c r="H8" s="113"/>
       <c r="I8" s="14"/>
-      <c r="J8" s="133" t="s">
+      <c r="J8" s="114" t="s">
         <v>11</v>
       </c>
-      <c r="K8" s="92"/>
+      <c r="K8" s="115"/>
     </row>
     <row r="9" spans="1:11" ht="17.25">
-      <c r="A9" s="128"/>
+      <c r="A9" s="108"/>
       <c r="B9" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="134" t="s">
+      <c r="C9" s="116" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="90"/>
-      <c r="E9" s="110"/>
+      <c r="D9" s="72"/>
+      <c r="E9" s="81"/>
       <c r="F9" s="22"/>
-      <c r="G9" s="109">
+      <c r="G9" s="87">
         <v>1</v>
       </c>
-      <c r="H9" s="110"/>
+      <c r="H9" s="81"/>
       <c r="I9" s="22"/>
-      <c r="J9" s="111"/>
-      <c r="K9" s="103"/>
+      <c r="J9" s="88"/>
+      <c r="K9" s="89"/>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="32"/>
@@ -2124,128 +2124,128 @@
       <c r="K10" s="34"/>
     </row>
     <row r="11" spans="1:11" ht="18.75">
-      <c r="A11" s="112" t="s">
+      <c r="A11" s="90" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="113"/>
-      <c r="C11" s="113"/>
-      <c r="D11" s="113"/>
-      <c r="E11" s="114"/>
-      <c r="F11" s="115"/>
-      <c r="G11" s="113"/>
-      <c r="H11" s="113"/>
-      <c r="I11" s="113"/>
-      <c r="J11" s="113"/>
-      <c r="K11" s="116"/>
+      <c r="B11" s="91"/>
+      <c r="C11" s="91"/>
+      <c r="D11" s="91"/>
+      <c r="E11" s="92"/>
+      <c r="F11" s="93"/>
+      <c r="G11" s="91"/>
+      <c r="H11" s="91"/>
+      <c r="I11" s="91"/>
+      <c r="J11" s="91"/>
+      <c r="K11" s="94"/>
     </row>
     <row r="12" spans="1:11">
-      <c r="A12" s="117" t="s">
+      <c r="A12" s="95" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="95"/>
-      <c r="C12" s="95"/>
-      <c r="D12" s="95"/>
-      <c r="E12" s="110"/>
+      <c r="B12" s="96"/>
+      <c r="C12" s="96"/>
+      <c r="D12" s="96"/>
+      <c r="E12" s="81"/>
       <c r="F12" s="59"/>
       <c r="G12" s="31"/>
       <c r="H12" s="60"/>
       <c r="I12" s="31"/>
-      <c r="J12" s="135"/>
-      <c r="K12" s="136"/>
+      <c r="J12" s="117"/>
+      <c r="K12" s="118"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="96"/>
-      <c r="B13" s="90"/>
-      <c r="C13" s="90"/>
-      <c r="D13" s="90"/>
-      <c r="E13" s="97"/>
+      <c r="A13" s="97"/>
+      <c r="B13" s="72"/>
+      <c r="C13" s="72"/>
+      <c r="D13" s="72"/>
+      <c r="E13" s="73"/>
       <c r="F13" s="27"/>
       <c r="G13" s="61"/>
       <c r="H13" s="62"/>
       <c r="I13" s="2"/>
-      <c r="J13" s="71"/>
-      <c r="K13" s="72"/>
+      <c r="J13" s="119"/>
+      <c r="K13" s="120"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="118" t="str">
+      <c r="A14" s="98" t="str">
         <f>"*"&amp;A12&amp;"*"</f>
         <v>*GOFEMM20052025001*</v>
       </c>
-      <c r="B14" s="119"/>
-      <c r="C14" s="119"/>
-      <c r="D14" s="119"/>
-      <c r="E14" s="120"/>
+      <c r="B14" s="99"/>
+      <c r="C14" s="99"/>
+      <c r="D14" s="99"/>
+      <c r="E14" s="100"/>
       <c r="F14" s="27"/>
       <c r="G14" s="62"/>
       <c r="H14" s="62"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="71"/>
-      <c r="K14" s="72"/>
+      <c r="J14" s="119"/>
+      <c r="K14" s="120"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="121"/>
-      <c r="B15" s="122"/>
-      <c r="C15" s="122"/>
-      <c r="D15" s="122"/>
-      <c r="E15" s="123"/>
+      <c r="A15" s="101"/>
+      <c r="B15" s="102"/>
+      <c r="C15" s="102"/>
+      <c r="D15" s="102"/>
+      <c r="E15" s="103"/>
       <c r="F15" s="27"/>
       <c r="G15" s="62"/>
       <c r="H15" s="62"/>
       <c r="I15" s="2"/>
-      <c r="J15" s="71"/>
-      <c r="K15" s="72"/>
+      <c r="J15" s="119"/>
+      <c r="K15" s="120"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="121"/>
-      <c r="B16" s="122"/>
-      <c r="C16" s="122"/>
-      <c r="D16" s="122"/>
-      <c r="E16" s="123"/>
+      <c r="A16" s="101"/>
+      <c r="B16" s="102"/>
+      <c r="C16" s="102"/>
+      <c r="D16" s="102"/>
+      <c r="E16" s="103"/>
       <c r="F16" s="8"/>
       <c r="G16" s="62"/>
       <c r="H16" s="62"/>
       <c r="I16" s="2"/>
-      <c r="J16" s="71"/>
-      <c r="K16" s="72"/>
+      <c r="J16" s="119"/>
+      <c r="K16" s="120"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="121"/>
-      <c r="B17" s="122"/>
-      <c r="C17" s="122"/>
-      <c r="D17" s="122"/>
-      <c r="E17" s="123"/>
+      <c r="A17" s="101"/>
+      <c r="B17" s="102"/>
+      <c r="C17" s="102"/>
+      <c r="D17" s="102"/>
+      <c r="E17" s="103"/>
       <c r="F17" s="27"/>
       <c r="G17" s="62"/>
       <c r="H17" s="62"/>
       <c r="I17" s="2"/>
-      <c r="J17" s="71"/>
-      <c r="K17" s="72"/>
+      <c r="J17" s="119"/>
+      <c r="K17" s="120"/>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="121"/>
-      <c r="B18" s="122"/>
-      <c r="C18" s="122"/>
-      <c r="D18" s="122"/>
-      <c r="E18" s="123"/>
+      <c r="A18" s="101"/>
+      <c r="B18" s="102"/>
+      <c r="C18" s="102"/>
+      <c r="D18" s="102"/>
+      <c r="E18" s="103"/>
       <c r="F18" s="27"/>
       <c r="G18" s="62"/>
       <c r="H18" s="62"/>
       <c r="I18" s="8"/>
-      <c r="J18" s="71"/>
-      <c r="K18" s="72"/>
+      <c r="J18" s="119"/>
+      <c r="K18" s="120"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="124"/>
-      <c r="B19" s="125"/>
-      <c r="C19" s="125"/>
-      <c r="D19" s="125"/>
-      <c r="E19" s="126"/>
+      <c r="A19" s="104"/>
+      <c r="B19" s="105"/>
+      <c r="C19" s="105"/>
+      <c r="D19" s="105"/>
+      <c r="E19" s="106"/>
       <c r="F19" s="63"/>
       <c r="G19" s="62"/>
       <c r="H19" s="62"/>
       <c r="I19" s="27"/>
-      <c r="J19" s="71"/>
-      <c r="K19" s="72"/>
+      <c r="J19" s="119"/>
+      <c r="K19" s="120"/>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="32"/>
@@ -2257,8 +2257,8 @@
       <c r="G20" s="64"/>
       <c r="H20" s="62"/>
       <c r="I20" s="27"/>
-      <c r="J20" s="71"/>
-      <c r="K20" s="72"/>
+      <c r="J20" s="119"/>
+      <c r="K20" s="120"/>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="32"/>
@@ -2270,8 +2270,8 @@
       <c r="G21" s="62"/>
       <c r="H21" s="62"/>
       <c r="I21" s="27"/>
-      <c r="J21" s="71"/>
-      <c r="K21" s="72"/>
+      <c r="J21" s="119"/>
+      <c r="K21" s="120"/>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="32"/>
@@ -2283,8 +2283,8 @@
       <c r="G22" s="62"/>
       <c r="H22" s="62"/>
       <c r="I22" s="27"/>
-      <c r="J22" s="71"/>
-      <c r="K22" s="72"/>
+      <c r="J22" s="119"/>
+      <c r="K22" s="120"/>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="32"/>
@@ -2296,8 +2296,8 @@
       <c r="G23" s="27"/>
       <c r="H23" s="27"/>
       <c r="I23" s="27"/>
-      <c r="J23" s="71"/>
-      <c r="K23" s="72"/>
+      <c r="J23" s="119"/>
+      <c r="K23" s="120"/>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" s="32"/>
@@ -2309,8 +2309,8 @@
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
-      <c r="J24" s="71"/>
-      <c r="K24" s="72"/>
+      <c r="J24" s="119"/>
+      <c r="K24" s="120"/>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="32"/>
@@ -2322,90 +2322,90 @@
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
       <c r="I25" s="9"/>
-      <c r="J25" s="71"/>
-      <c r="K25" s="72"/>
+      <c r="J25" s="119"/>
+      <c r="K25" s="120"/>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="105"/>
-      <c r="B26" s="94"/>
-      <c r="C26" s="94"/>
-      <c r="D26" s="94"/>
-      <c r="E26" s="106"/>
+      <c r="A26" s="83"/>
+      <c r="B26" s="80"/>
+      <c r="C26" s="80"/>
+      <c r="D26" s="80"/>
+      <c r="E26" s="84"/>
       <c r="F26" s="66"/>
       <c r="G26" s="67"/>
       <c r="H26" s="8"/>
       <c r="I26" s="9"/>
-      <c r="J26" s="71"/>
-      <c r="K26" s="72"/>
+      <c r="J26" s="119"/>
+      <c r="K26" s="120"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="94"/>
-      <c r="B27" s="94"/>
-      <c r="C27" s="94"/>
-      <c r="D27" s="94"/>
-      <c r="E27" s="106"/>
+      <c r="A27" s="80"/>
+      <c r="B27" s="80"/>
+      <c r="C27" s="80"/>
+      <c r="D27" s="80"/>
+      <c r="E27" s="84"/>
       <c r="F27" s="68"/>
       <c r="G27" s="67"/>
       <c r="H27" s="8"/>
       <c r="I27" s="9"/>
-      <c r="J27" s="71"/>
-      <c r="K27" s="72"/>
+      <c r="J27" s="119"/>
+      <c r="K27" s="120"/>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="94"/>
-      <c r="B28" s="94"/>
-      <c r="C28" s="94"/>
-      <c r="D28" s="94"/>
-      <c r="E28" s="106"/>
+      <c r="A28" s="80"/>
+      <c r="B28" s="80"/>
+      <c r="C28" s="80"/>
+      <c r="D28" s="80"/>
+      <c r="E28" s="84"/>
       <c r="F28" s="68"/>
       <c r="G28" s="67"/>
       <c r="H28" s="8"/>
       <c r="I28" s="9"/>
-      <c r="J28" s="71"/>
-      <c r="K28" s="72"/>
+      <c r="J28" s="119"/>
+      <c r="K28" s="120"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="94"/>
-      <c r="B29" s="94"/>
-      <c r="C29" s="94"/>
-      <c r="D29" s="94"/>
-      <c r="E29" s="106"/>
+      <c r="A29" s="80"/>
+      <c r="B29" s="80"/>
+      <c r="C29" s="80"/>
+      <c r="D29" s="80"/>
+      <c r="E29" s="84"/>
       <c r="F29" s="69"/>
       <c r="G29" s="70"/>
       <c r="H29" s="65"/>
       <c r="I29" s="23"/>
-      <c r="J29" s="71"/>
-      <c r="K29" s="72"/>
+      <c r="J29" s="119"/>
+      <c r="K29" s="120"/>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="107"/>
-      <c r="B30" s="107"/>
-      <c r="C30" s="107"/>
-      <c r="D30" s="107"/>
-      <c r="E30" s="108"/>
+      <c r="A30" s="85"/>
+      <c r="B30" s="85"/>
+      <c r="C30" s="85"/>
+      <c r="D30" s="85"/>
+      <c r="E30" s="86"/>
       <c r="F30" s="49"/>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
-      <c r="J30" s="71"/>
-      <c r="K30" s="72"/>
+      <c r="J30" s="119"/>
+      <c r="K30" s="120"/>
     </row>
     <row r="31" spans="1:11" ht="15.75">
-      <c r="A31" s="137" t="s">
+      <c r="A31" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="90"/>
-      <c r="C31" s="97"/>
+      <c r="B31" s="72"/>
+      <c r="C31" s="73"/>
       <c r="D31" s="50"/>
-      <c r="E31" s="138"/>
-      <c r="F31" s="139"/>
-      <c r="G31" s="139"/>
-      <c r="H31" s="139"/>
-      <c r="I31" s="140" t="s">
+      <c r="E31" s="74"/>
+      <c r="F31" s="75"/>
+      <c r="G31" s="75"/>
+      <c r="H31" s="75"/>
+      <c r="I31" s="76" t="s">
         <v>16</v>
       </c>
-      <c r="J31" s="141"/>
-      <c r="K31" s="142"/>
+      <c r="J31" s="77"/>
+      <c r="K31" s="78"/>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" s="37"/>
@@ -2413,12 +2413,12 @@
       <c r="C32" s="4"/>
       <c r="D32" s="38"/>
       <c r="E32" s="3"/>
-      <c r="F32" s="143"/>
-      <c r="G32" s="94"/>
-      <c r="H32" s="110"/>
-      <c r="I32" s="143"/>
-      <c r="J32" s="94"/>
-      <c r="K32" s="144"/>
+      <c r="F32" s="79"/>
+      <c r="G32" s="80"/>
+      <c r="H32" s="81"/>
+      <c r="I32" s="79"/>
+      <c r="J32" s="80"/>
+      <c r="K32" s="82"/>
     </row>
     <row r="33" spans="1:11">
       <c r="A33" s="39"/>
@@ -2497,11 +2497,32 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="E31:H31"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="E1:G2"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="A5:C6"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="J6:K6"/>
     <mergeCell ref="A26:E30"/>
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="J9:K9"/>
@@ -2518,32 +2539,11 @@
     <mergeCell ref="J13:K13"/>
     <mergeCell ref="J14:K14"/>
     <mergeCell ref="J15:K15"/>
-    <mergeCell ref="A5:C6"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="E6:G6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="E1:G2"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="E31:H31"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="I32:K32"/>
   </mergeCells>
   <conditionalFormatting sqref="F12:G15 I12 F17:F22 G17:G19 G21:G22">
     <cfRule type="expression" dxfId="7" priority="1">
@@ -2595,39 +2595,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.6" customHeight="1">
-      <c r="A1" s="73" t="s">
+      <c r="A1" s="128" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="74"/>
-      <c r="C1" s="145"/>
+      <c r="B1" s="129"/>
+      <c r="C1" s="150"/>
       <c r="D1" s="58"/>
-      <c r="E1" s="147" t="s">
+      <c r="E1" s="152" t="s">
         <v>18</v>
       </c>
-      <c r="F1" s="148"/>
-      <c r="G1" s="149"/>
+      <c r="F1" s="153"/>
+      <c r="G1" s="154"/>
       <c r="H1" s="29"/>
-      <c r="I1" s="84" t="s">
+      <c r="I1" s="139" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="85"/>
-      <c r="K1" s="86"/>
+      <c r="J1" s="140"/>
+      <c r="K1" s="141"/>
     </row>
     <row r="2" spans="1:11" ht="15.75">
-      <c r="A2" s="75"/>
-      <c r="B2" s="76"/>
-      <c r="C2" s="146"/>
+      <c r="A2" s="130"/>
+      <c r="B2" s="131"/>
+      <c r="C2" s="151"/>
       <c r="D2" s="52"/>
-      <c r="E2" s="150"/>
-      <c r="F2" s="151"/>
-      <c r="G2" s="152"/>
+      <c r="E2" s="155"/>
+      <c r="F2" s="156"/>
+      <c r="G2" s="157"/>
       <c r="H2" s="15"/>
-      <c r="I2" s="87">
+      <c r="I2" s="142">
         <f ca="1">TODAY()</f>
         <v>45864</v>
       </c>
-      <c r="J2" s="82"/>
-      <c r="K2" s="83"/>
+      <c r="J2" s="137"/>
+      <c r="K2" s="138"/>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="32"/>
@@ -2643,11 +2643,11 @@
       <c r="K3" s="33"/>
     </row>
     <row r="4" spans="1:11" ht="17.25">
-      <c r="A4" s="153" t="s">
+      <c r="A4" s="158" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="154"/>
-      <c r="C4" s="76"/>
+      <c r="B4" s="159"/>
+      <c r="C4" s="131"/>
       <c r="D4" s="52"/>
       <c r="E4" s="26" t="s">
         <v>19</v>
@@ -2658,46 +2658,46 @@
       <c r="I4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="91"/>
-      <c r="K4" s="92"/>
+      <c r="J4" s="144"/>
+      <c r="K4" s="115"/>
     </row>
     <row r="5" spans="1:11" ht="18.75">
-      <c r="A5" s="155" t="s">
+      <c r="A5" s="145" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="156"/>
-      <c r="C5" s="77"/>
+      <c r="B5" s="146"/>
+      <c r="C5" s="132"/>
       <c r="D5" s="14"/>
-      <c r="E5" s="98" t="s">
+      <c r="E5" s="122" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="99"/>
-      <c r="G5" s="100"/>
+      <c r="F5" s="123"/>
+      <c r="G5" s="124"/>
       <c r="H5" s="22"/>
       <c r="I5" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="J5" s="101"/>
-      <c r="K5" s="92"/>
+      <c r="J5" s="125"/>
+      <c r="K5" s="115"/>
     </row>
     <row r="6" spans="1:11" ht="15.75">
-      <c r="A6" s="75"/>
-      <c r="B6" s="76"/>
-      <c r="C6" s="157"/>
+      <c r="A6" s="130"/>
+      <c r="B6" s="131"/>
+      <c r="C6" s="147"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="158" t="s">
+      <c r="E6" s="148" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="76"/>
-      <c r="G6" s="159"/>
+      <c r="F6" s="131"/>
+      <c r="G6" s="149"/>
       <c r="H6" s="46"/>
       <c r="I6" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="104">
+      <c r="J6" s="127">
         <v>1230</v>
       </c>
-      <c r="K6" s="92"/>
+      <c r="K6" s="115"/>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="32"/>
@@ -2713,44 +2713,44 @@
       <c r="K7" s="33"/>
     </row>
     <row r="8" spans="1:11" ht="15.75">
-      <c r="A8" s="127" t="s">
+      <c r="A8" s="107" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="129"/>
-      <c r="D8" s="130"/>
-      <c r="E8" s="131"/>
+      <c r="C8" s="109"/>
+      <c r="D8" s="110"/>
+      <c r="E8" s="111"/>
       <c r="F8" s="14"/>
-      <c r="G8" s="132" t="s">
+      <c r="G8" s="112" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="89"/>
+      <c r="H8" s="113"/>
       <c r="I8" s="14"/>
-      <c r="J8" s="133" t="s">
+      <c r="J8" s="114" t="s">
         <v>11</v>
       </c>
-      <c r="K8" s="92"/>
+      <c r="K8" s="115"/>
     </row>
     <row r="9" spans="1:11" ht="17.25">
-      <c r="A9" s="128"/>
+      <c r="A9" s="108"/>
       <c r="B9" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="134" t="s">
+      <c r="C9" s="116" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="90"/>
-      <c r="E9" s="110"/>
+      <c r="D9" s="72"/>
+      <c r="E9" s="81"/>
       <c r="F9" s="22"/>
-      <c r="G9" s="109">
+      <c r="G9" s="87">
         <v>1</v>
       </c>
-      <c r="H9" s="110"/>
+      <c r="H9" s="81"/>
       <c r="I9" s="22"/>
-      <c r="J9" s="111"/>
-      <c r="K9" s="103"/>
+      <c r="J9" s="88"/>
+      <c r="K9" s="89"/>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="32"/>
@@ -2766,128 +2766,128 @@
       <c r="K10" s="34"/>
     </row>
     <row r="11" spans="1:11" ht="18.75">
-      <c r="A11" s="112" t="s">
+      <c r="A11" s="90" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="113"/>
-      <c r="C11" s="113"/>
-      <c r="D11" s="113"/>
-      <c r="E11" s="114"/>
-      <c r="F11" s="115"/>
-      <c r="G11" s="113"/>
-      <c r="H11" s="113"/>
-      <c r="I11" s="113"/>
-      <c r="J11" s="113"/>
-      <c r="K11" s="116"/>
+      <c r="B11" s="91"/>
+      <c r="C11" s="91"/>
+      <c r="D11" s="91"/>
+      <c r="E11" s="92"/>
+      <c r="F11" s="93"/>
+      <c r="G11" s="91"/>
+      <c r="H11" s="91"/>
+      <c r="I11" s="91"/>
+      <c r="J11" s="91"/>
+      <c r="K11" s="94"/>
     </row>
     <row r="12" spans="1:11" ht="12.6" customHeight="1">
-      <c r="A12" s="117" t="s">
+      <c r="A12" s="95" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="95"/>
-      <c r="C12" s="95"/>
-      <c r="D12" s="95"/>
-      <c r="E12" s="110"/>
+      <c r="B12" s="96"/>
+      <c r="C12" s="96"/>
+      <c r="D12" s="96"/>
+      <c r="E12" s="81"/>
       <c r="F12" s="59"/>
       <c r="G12" s="31"/>
       <c r="H12" s="60"/>
       <c r="I12" s="31"/>
-      <c r="J12" s="135"/>
-      <c r="K12" s="136"/>
+      <c r="J12" s="117"/>
+      <c r="K12" s="118"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="96"/>
-      <c r="B13" s="90"/>
-      <c r="C13" s="90"/>
-      <c r="D13" s="90"/>
-      <c r="E13" s="97"/>
+      <c r="A13" s="97"/>
+      <c r="B13" s="72"/>
+      <c r="C13" s="72"/>
+      <c r="D13" s="72"/>
+      <c r="E13" s="73"/>
       <c r="F13" s="27"/>
       <c r="G13" s="61"/>
       <c r="H13" s="62"/>
       <c r="I13" s="2"/>
-      <c r="J13" s="135"/>
-      <c r="K13" s="136"/>
+      <c r="J13" s="117"/>
+      <c r="K13" s="118"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="118" t="str">
+      <c r="A14" s="98" t="str">
         <f>"*"&amp;A12&amp;"*"</f>
         <v>*GOFEMM20052025002*</v>
       </c>
-      <c r="B14" s="119"/>
-      <c r="C14" s="119"/>
-      <c r="D14" s="119"/>
-      <c r="E14" s="120"/>
+      <c r="B14" s="99"/>
+      <c r="C14" s="99"/>
+      <c r="D14" s="99"/>
+      <c r="E14" s="100"/>
       <c r="F14" s="27"/>
       <c r="G14" s="62"/>
       <c r="H14" s="62"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="135"/>
-      <c r="K14" s="136"/>
+      <c r="J14" s="117"/>
+      <c r="K14" s="118"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="121"/>
-      <c r="B15" s="122"/>
-      <c r="C15" s="122"/>
-      <c r="D15" s="122"/>
-      <c r="E15" s="123"/>
+      <c r="A15" s="101"/>
+      <c r="B15" s="102"/>
+      <c r="C15" s="102"/>
+      <c r="D15" s="102"/>
+      <c r="E15" s="103"/>
       <c r="F15" s="27"/>
       <c r="G15" s="62"/>
       <c r="H15" s="62"/>
       <c r="I15" s="2"/>
-      <c r="J15" s="135"/>
-      <c r="K15" s="136"/>
+      <c r="J15" s="117"/>
+      <c r="K15" s="118"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="121"/>
-      <c r="B16" s="122"/>
-      <c r="C16" s="122"/>
-      <c r="D16" s="122"/>
-      <c r="E16" s="123"/>
+      <c r="A16" s="101"/>
+      <c r="B16" s="102"/>
+      <c r="C16" s="102"/>
+      <c r="D16" s="102"/>
+      <c r="E16" s="103"/>
       <c r="F16" s="8"/>
       <c r="G16" s="62"/>
       <c r="H16" s="62"/>
       <c r="I16" s="2"/>
-      <c r="J16" s="135"/>
-      <c r="K16" s="136"/>
+      <c r="J16" s="117"/>
+      <c r="K16" s="118"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="121"/>
-      <c r="B17" s="122"/>
-      <c r="C17" s="122"/>
-      <c r="D17" s="122"/>
-      <c r="E17" s="123"/>
+      <c r="A17" s="101"/>
+      <c r="B17" s="102"/>
+      <c r="C17" s="102"/>
+      <c r="D17" s="102"/>
+      <c r="E17" s="103"/>
       <c r="F17" s="27"/>
       <c r="G17" s="62"/>
       <c r="H17" s="62"/>
       <c r="I17" s="2"/>
-      <c r="J17" s="135"/>
-      <c r="K17" s="136"/>
+      <c r="J17" s="117"/>
+      <c r="K17" s="118"/>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="121"/>
-      <c r="B18" s="122"/>
-      <c r="C18" s="122"/>
-      <c r="D18" s="122"/>
-      <c r="E18" s="123"/>
+      <c r="A18" s="101"/>
+      <c r="B18" s="102"/>
+      <c r="C18" s="102"/>
+      <c r="D18" s="102"/>
+      <c r="E18" s="103"/>
       <c r="F18" s="27"/>
       <c r="G18" s="62"/>
       <c r="H18" s="62"/>
       <c r="I18" s="8"/>
-      <c r="J18" s="135"/>
-      <c r="K18" s="136"/>
+      <c r="J18" s="117"/>
+      <c r="K18" s="118"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="124"/>
-      <c r="B19" s="125"/>
-      <c r="C19" s="125"/>
-      <c r="D19" s="125"/>
-      <c r="E19" s="126"/>
+      <c r="A19" s="104"/>
+      <c r="B19" s="105"/>
+      <c r="C19" s="105"/>
+      <c r="D19" s="105"/>
+      <c r="E19" s="106"/>
       <c r="F19" s="63"/>
       <c r="G19" s="62"/>
       <c r="H19" s="62"/>
       <c r="I19" s="27"/>
-      <c r="J19" s="135"/>
-      <c r="K19" s="136"/>
+      <c r="J19" s="117"/>
+      <c r="K19" s="118"/>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="32"/>
@@ -2899,8 +2899,8 @@
       <c r="G20" s="64"/>
       <c r="H20" s="62"/>
       <c r="I20" s="27"/>
-      <c r="J20" s="135"/>
-      <c r="K20" s="136"/>
+      <c r="J20" s="117"/>
+      <c r="K20" s="118"/>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="32"/>
@@ -2912,8 +2912,8 @@
       <c r="G21" s="62"/>
       <c r="H21" s="62"/>
       <c r="I21" s="27"/>
-      <c r="J21" s="135"/>
-      <c r="K21" s="136"/>
+      <c r="J21" s="117"/>
+      <c r="K21" s="118"/>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="32"/>
@@ -2925,8 +2925,8 @@
       <c r="G22" s="62"/>
       <c r="H22" s="62"/>
       <c r="I22" s="27"/>
-      <c r="J22" s="135"/>
-      <c r="K22" s="136"/>
+      <c r="J22" s="117"/>
+      <c r="K22" s="118"/>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="32"/>
@@ -2938,8 +2938,8 @@
       <c r="G23" s="27"/>
       <c r="H23" s="27"/>
       <c r="I23" s="27"/>
-      <c r="J23" s="135"/>
-      <c r="K23" s="136"/>
+      <c r="J23" s="117"/>
+      <c r="K23" s="118"/>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" s="32"/>
@@ -2951,8 +2951,8 @@
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
-      <c r="J24" s="135"/>
-      <c r="K24" s="136"/>
+      <c r="J24" s="117"/>
+      <c r="K24" s="118"/>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="32"/>
@@ -2964,90 +2964,90 @@
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
       <c r="I25" s="9"/>
-      <c r="J25" s="135"/>
-      <c r="K25" s="136"/>
+      <c r="J25" s="117"/>
+      <c r="K25" s="118"/>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="105"/>
-      <c r="B26" s="94"/>
-      <c r="C26" s="94"/>
-      <c r="D26" s="94"/>
-      <c r="E26" s="106"/>
+      <c r="A26" s="83"/>
+      <c r="B26" s="80"/>
+      <c r="C26" s="80"/>
+      <c r="D26" s="80"/>
+      <c r="E26" s="84"/>
       <c r="F26" s="66"/>
       <c r="G26" s="67"/>
       <c r="H26" s="8"/>
       <c r="I26" s="9"/>
-      <c r="J26" s="135"/>
-      <c r="K26" s="136"/>
+      <c r="J26" s="117"/>
+      <c r="K26" s="118"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="94"/>
-      <c r="B27" s="94"/>
-      <c r="C27" s="94"/>
-      <c r="D27" s="94"/>
-      <c r="E27" s="106"/>
+      <c r="A27" s="80"/>
+      <c r="B27" s="80"/>
+      <c r="C27" s="80"/>
+      <c r="D27" s="80"/>
+      <c r="E27" s="84"/>
       <c r="F27" s="68"/>
       <c r="G27" s="67"/>
       <c r="H27" s="8"/>
       <c r="I27" s="9"/>
-      <c r="J27" s="135"/>
-      <c r="K27" s="136"/>
+      <c r="J27" s="117"/>
+      <c r="K27" s="118"/>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="94"/>
-      <c r="B28" s="94"/>
-      <c r="C28" s="94"/>
-      <c r="D28" s="94"/>
-      <c r="E28" s="106"/>
+      <c r="A28" s="80"/>
+      <c r="B28" s="80"/>
+      <c r="C28" s="80"/>
+      <c r="D28" s="80"/>
+      <c r="E28" s="84"/>
       <c r="F28" s="68"/>
       <c r="G28" s="67"/>
       <c r="H28" s="8"/>
       <c r="I28" s="9"/>
-      <c r="J28" s="135"/>
-      <c r="K28" s="136"/>
+      <c r="J28" s="117"/>
+      <c r="K28" s="118"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="94"/>
-      <c r="B29" s="94"/>
-      <c r="C29" s="94"/>
-      <c r="D29" s="94"/>
-      <c r="E29" s="106"/>
+      <c r="A29" s="80"/>
+      <c r="B29" s="80"/>
+      <c r="C29" s="80"/>
+      <c r="D29" s="80"/>
+      <c r="E29" s="84"/>
       <c r="F29" s="69"/>
       <c r="G29" s="70"/>
       <c r="H29" s="65"/>
       <c r="I29" s="23"/>
-      <c r="J29" s="135"/>
-      <c r="K29" s="136"/>
+      <c r="J29" s="117"/>
+      <c r="K29" s="118"/>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="107"/>
-      <c r="B30" s="107"/>
-      <c r="C30" s="107"/>
-      <c r="D30" s="107"/>
-      <c r="E30" s="108"/>
+      <c r="A30" s="85"/>
+      <c r="B30" s="85"/>
+      <c r="C30" s="85"/>
+      <c r="D30" s="85"/>
+      <c r="E30" s="86"/>
       <c r="F30" s="49"/>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
-      <c r="J30" s="135"/>
-      <c r="K30" s="136"/>
+      <c r="J30" s="117"/>
+      <c r="K30" s="118"/>
     </row>
     <row r="31" spans="1:11" ht="15.75">
-      <c r="A31" s="137" t="s">
+      <c r="A31" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="90"/>
-      <c r="C31" s="97"/>
+      <c r="B31" s="72"/>
+      <c r="C31" s="73"/>
       <c r="D31" s="50"/>
-      <c r="E31" s="138"/>
-      <c r="F31" s="139"/>
-      <c r="G31" s="139"/>
-      <c r="H31" s="139"/>
-      <c r="I31" s="140" t="s">
+      <c r="E31" s="74"/>
+      <c r="F31" s="75"/>
+      <c r="G31" s="75"/>
+      <c r="H31" s="75"/>
+      <c r="I31" s="76" t="s">
         <v>16</v>
       </c>
-      <c r="J31" s="141"/>
-      <c r="K31" s="142"/>
+      <c r="J31" s="77"/>
+      <c r="K31" s="78"/>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" s="37"/>
@@ -3055,12 +3055,12 @@
       <c r="C32" s="4"/>
       <c r="D32" s="38"/>
       <c r="E32" s="3"/>
-      <c r="F32" s="143"/>
-      <c r="G32" s="94"/>
-      <c r="H32" s="110"/>
-      <c r="I32" s="143"/>
-      <c r="J32" s="94"/>
-      <c r="K32" s="144"/>
+      <c r="F32" s="79"/>
+      <c r="G32" s="80"/>
+      <c r="H32" s="81"/>
+      <c r="I32" s="79"/>
+      <c r="J32" s="80"/>
+      <c r="K32" s="82"/>
     </row>
     <row r="33" spans="1:11">
       <c r="A33" s="39"/>
@@ -3139,16 +3139,27 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="A26:E30"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="E31:H31"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="E1:G2"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="J4:K4"/>
     <mergeCell ref="A14:E19"/>
     <mergeCell ref="A5:C6"/>
     <mergeCell ref="E5:G5"/>
@@ -3165,27 +3176,16 @@
     <mergeCell ref="A11:E11"/>
     <mergeCell ref="F11:K11"/>
     <mergeCell ref="A12:E13"/>
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="E1:G2"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="A26:E30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="E31:H31"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J30:K30"/>
   </mergeCells>
   <conditionalFormatting sqref="F12:G15 I12 F17:F22 G17:G19 G21:G22">
     <cfRule type="expression" dxfId="3" priority="1">

</xml_diff>

<commit_message>
feat: add tanger  branch
</commit_message>
<xml_diff>
--- a/dummy-content/ECHEC-RETOUR_CLIENT-CASABLANCA.xlsx
+++ b/dummy-content/ECHEC-RETOUR_CLIENT-CASABLANCA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UNK\Desktop\GoFleet-Enhancer\dummy-content\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4EC71F9-E2CC-4694-BB7B-C5BBE004612B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{221F0FBB-6A08-4A4B-8B1B-C1F1090C05E5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -90,7 +90,7 @@
     <t>GOFEMM20052025002</t>
   </si>
   <si>
-    <t>GO FLEET MEKNES</t>
+    <t>GO FLEET TANGER</t>
   </si>
 </sst>
 </file>
@@ -1400,24 +1400,66 @@
     <xf numFmtId="0" fontId="15" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="5" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
@@ -1425,10 +1467,10 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="11" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1441,8 +1483,6 @@
     <xf numFmtId="0" fontId="21" fillId="12" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="24" fillId="3" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1466,11 +1506,9 @@
     <xf numFmtId="0" fontId="8" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1480,67 +1518,20 @@
     <xf numFmtId="0" fontId="15" fillId="15" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="5" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="20" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="19" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="17" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1555,6 +1546,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="19" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1955,37 +1955,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.6" customHeight="1">
-      <c r="A1" s="128"/>
-      <c r="B1" s="129"/>
-      <c r="C1" s="129"/>
+      <c r="A1" s="73"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
       <c r="D1" s="53"/>
-      <c r="E1" s="133" t="s">
+      <c r="E1" s="78" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="134"/>
-      <c r="G1" s="135"/>
+      <c r="F1" s="79"/>
+      <c r="G1" s="80"/>
       <c r="H1" s="29"/>
-      <c r="I1" s="139" t="s">
+      <c r="I1" s="84" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="140"/>
-      <c r="K1" s="141"/>
+      <c r="J1" s="85"/>
+      <c r="K1" s="86"/>
     </row>
     <row r="2" spans="1:11" ht="15.75">
-      <c r="A2" s="130"/>
-      <c r="B2" s="131"/>
-      <c r="C2" s="132"/>
+      <c r="A2" s="75"/>
+      <c r="B2" s="76"/>
+      <c r="C2" s="77"/>
       <c r="D2" s="53"/>
-      <c r="E2" s="136"/>
-      <c r="F2" s="137"/>
-      <c r="G2" s="138"/>
+      <c r="E2" s="81"/>
+      <c r="F2" s="82"/>
+      <c r="G2" s="83"/>
       <c r="H2" s="15"/>
-      <c r="I2" s="142">
+      <c r="I2" s="87">
         <f ca="1">TODAY()</f>
         <v>45864</v>
       </c>
-      <c r="J2" s="137"/>
-      <c r="K2" s="138"/>
+      <c r="J2" s="82"/>
+      <c r="K2" s="83"/>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="32"/>
@@ -2001,11 +2001,11 @@
       <c r="K3" s="33"/>
     </row>
     <row r="4" spans="1:11" ht="17.25">
-      <c r="A4" s="143" t="s">
+      <c r="A4" s="88" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="113"/>
-      <c r="C4" s="72"/>
+      <c r="B4" s="89"/>
+      <c r="C4" s="90"/>
       <c r="D4" s="52"/>
       <c r="E4" s="16" t="s">
         <v>19</v>
@@ -2016,46 +2016,46 @@
       <c r="I4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="144"/>
-      <c r="K4" s="115"/>
+      <c r="J4" s="91"/>
+      <c r="K4" s="92"/>
     </row>
     <row r="5" spans="1:11" ht="18.75">
-      <c r="A5" s="121" t="s">
+      <c r="A5" s="93" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="80"/>
-      <c r="C5" s="96"/>
+      <c r="B5" s="94"/>
+      <c r="C5" s="95"/>
       <c r="D5" s="14"/>
-      <c r="E5" s="122" t="s">
+      <c r="E5" s="98" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="123"/>
-      <c r="G5" s="124"/>
+      <c r="F5" s="99"/>
+      <c r="G5" s="100"/>
       <c r="H5" s="22"/>
       <c r="I5" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="J5" s="125"/>
-      <c r="K5" s="115"/>
+      <c r="J5" s="101"/>
+      <c r="K5" s="92"/>
     </row>
     <row r="6" spans="1:11" ht="15.75">
-      <c r="A6" s="97"/>
-      <c r="B6" s="72"/>
-      <c r="C6" s="73"/>
+      <c r="A6" s="96"/>
+      <c r="B6" s="90"/>
+      <c r="C6" s="97"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="126" t="s">
+      <c r="E6" s="102" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="72"/>
-      <c r="G6" s="89"/>
+      <c r="F6" s="90"/>
+      <c r="G6" s="103"/>
       <c r="H6" s="46"/>
       <c r="I6" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="127">
+      <c r="J6" s="104">
         <v>1230</v>
       </c>
-      <c r="K6" s="115"/>
+      <c r="K6" s="92"/>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="32"/>
@@ -2071,44 +2071,44 @@
       <c r="K7" s="33"/>
     </row>
     <row r="8" spans="1:11" ht="15.75">
-      <c r="A8" s="107" t="s">
+      <c r="A8" s="127" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="109"/>
-      <c r="D8" s="110"/>
-      <c r="E8" s="111"/>
+      <c r="C8" s="129"/>
+      <c r="D8" s="130"/>
+      <c r="E8" s="131"/>
       <c r="F8" s="14"/>
-      <c r="G8" s="112" t="s">
+      <c r="G8" s="132" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="113"/>
+      <c r="H8" s="89"/>
       <c r="I8" s="14"/>
-      <c r="J8" s="114" t="s">
+      <c r="J8" s="133" t="s">
         <v>11</v>
       </c>
-      <c r="K8" s="115"/>
+      <c r="K8" s="92"/>
     </row>
     <row r="9" spans="1:11" ht="17.25">
-      <c r="A9" s="108"/>
+      <c r="A9" s="128"/>
       <c r="B9" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="116" t="s">
+      <c r="C9" s="134" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="72"/>
-      <c r="E9" s="81"/>
+      <c r="D9" s="90"/>
+      <c r="E9" s="110"/>
       <c r="F9" s="22"/>
-      <c r="G9" s="87">
+      <c r="G9" s="109">
         <v>1</v>
       </c>
-      <c r="H9" s="81"/>
+      <c r="H9" s="110"/>
       <c r="I9" s="22"/>
-      <c r="J9" s="88"/>
-      <c r="K9" s="89"/>
+      <c r="J9" s="111"/>
+      <c r="K9" s="103"/>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="32"/>
@@ -2124,128 +2124,128 @@
       <c r="K10" s="34"/>
     </row>
     <row r="11" spans="1:11" ht="18.75">
-      <c r="A11" s="90" t="s">
+      <c r="A11" s="112" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="91"/>
-      <c r="C11" s="91"/>
-      <c r="D11" s="91"/>
-      <c r="E11" s="92"/>
-      <c r="F11" s="93"/>
-      <c r="G11" s="91"/>
-      <c r="H11" s="91"/>
-      <c r="I11" s="91"/>
-      <c r="J11" s="91"/>
-      <c r="K11" s="94"/>
+      <c r="B11" s="113"/>
+      <c r="C11" s="113"/>
+      <c r="D11" s="113"/>
+      <c r="E11" s="114"/>
+      <c r="F11" s="115"/>
+      <c r="G11" s="113"/>
+      <c r="H11" s="113"/>
+      <c r="I11" s="113"/>
+      <c r="J11" s="113"/>
+      <c r="K11" s="116"/>
     </row>
     <row r="12" spans="1:11">
-      <c r="A12" s="95" t="s">
+      <c r="A12" s="117" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="96"/>
-      <c r="C12" s="96"/>
-      <c r="D12" s="96"/>
-      <c r="E12" s="81"/>
+      <c r="B12" s="95"/>
+      <c r="C12" s="95"/>
+      <c r="D12" s="95"/>
+      <c r="E12" s="110"/>
       <c r="F12" s="59"/>
       <c r="G12" s="31"/>
       <c r="H12" s="60"/>
       <c r="I12" s="31"/>
-      <c r="J12" s="117"/>
-      <c r="K12" s="118"/>
+      <c r="J12" s="135"/>
+      <c r="K12" s="136"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="97"/>
-      <c r="B13" s="72"/>
-      <c r="C13" s="72"/>
-      <c r="D13" s="72"/>
-      <c r="E13" s="73"/>
+      <c r="A13" s="96"/>
+      <c r="B13" s="90"/>
+      <c r="C13" s="90"/>
+      <c r="D13" s="90"/>
+      <c r="E13" s="97"/>
       <c r="F13" s="27"/>
       <c r="G13" s="61"/>
       <c r="H13" s="62"/>
       <c r="I13" s="2"/>
-      <c r="J13" s="119"/>
-      <c r="K13" s="120"/>
+      <c r="J13" s="71"/>
+      <c r="K13" s="72"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="98" t="str">
+      <c r="A14" s="118" t="str">
         <f>"*"&amp;A12&amp;"*"</f>
         <v>*GOFEMM20052025001*</v>
       </c>
-      <c r="B14" s="99"/>
-      <c r="C14" s="99"/>
-      <c r="D14" s="99"/>
-      <c r="E14" s="100"/>
+      <c r="B14" s="119"/>
+      <c r="C14" s="119"/>
+      <c r="D14" s="119"/>
+      <c r="E14" s="120"/>
       <c r="F14" s="27"/>
       <c r="G14" s="62"/>
       <c r="H14" s="62"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="119"/>
-      <c r="K14" s="120"/>
+      <c r="J14" s="71"/>
+      <c r="K14" s="72"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="101"/>
-      <c r="B15" s="102"/>
-      <c r="C15" s="102"/>
-      <c r="D15" s="102"/>
-      <c r="E15" s="103"/>
+      <c r="A15" s="121"/>
+      <c r="B15" s="122"/>
+      <c r="C15" s="122"/>
+      <c r="D15" s="122"/>
+      <c r="E15" s="123"/>
       <c r="F15" s="27"/>
       <c r="G15" s="62"/>
       <c r="H15" s="62"/>
       <c r="I15" s="2"/>
-      <c r="J15" s="119"/>
-      <c r="K15" s="120"/>
+      <c r="J15" s="71"/>
+      <c r="K15" s="72"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="101"/>
-      <c r="B16" s="102"/>
-      <c r="C16" s="102"/>
-      <c r="D16" s="102"/>
-      <c r="E16" s="103"/>
+      <c r="A16" s="121"/>
+      <c r="B16" s="122"/>
+      <c r="C16" s="122"/>
+      <c r="D16" s="122"/>
+      <c r="E16" s="123"/>
       <c r="F16" s="8"/>
       <c r="G16" s="62"/>
       <c r="H16" s="62"/>
       <c r="I16" s="2"/>
-      <c r="J16" s="119"/>
-      <c r="K16" s="120"/>
+      <c r="J16" s="71"/>
+      <c r="K16" s="72"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="101"/>
-      <c r="B17" s="102"/>
-      <c r="C17" s="102"/>
-      <c r="D17" s="102"/>
-      <c r="E17" s="103"/>
+      <c r="A17" s="121"/>
+      <c r="B17" s="122"/>
+      <c r="C17" s="122"/>
+      <c r="D17" s="122"/>
+      <c r="E17" s="123"/>
       <c r="F17" s="27"/>
       <c r="G17" s="62"/>
       <c r="H17" s="62"/>
       <c r="I17" s="2"/>
-      <c r="J17" s="119"/>
-      <c r="K17" s="120"/>
+      <c r="J17" s="71"/>
+      <c r="K17" s="72"/>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="101"/>
-      <c r="B18" s="102"/>
-      <c r="C18" s="102"/>
-      <c r="D18" s="102"/>
-      <c r="E18" s="103"/>
+      <c r="A18" s="121"/>
+      <c r="B18" s="122"/>
+      <c r="C18" s="122"/>
+      <c r="D18" s="122"/>
+      <c r="E18" s="123"/>
       <c r="F18" s="27"/>
       <c r="G18" s="62"/>
       <c r="H18" s="62"/>
       <c r="I18" s="8"/>
-      <c r="J18" s="119"/>
-      <c r="K18" s="120"/>
+      <c r="J18" s="71"/>
+      <c r="K18" s="72"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="104"/>
-      <c r="B19" s="105"/>
-      <c r="C19" s="105"/>
-      <c r="D19" s="105"/>
-      <c r="E19" s="106"/>
+      <c r="A19" s="124"/>
+      <c r="B19" s="125"/>
+      <c r="C19" s="125"/>
+      <c r="D19" s="125"/>
+      <c r="E19" s="126"/>
       <c r="F19" s="63"/>
       <c r="G19" s="62"/>
       <c r="H19" s="62"/>
       <c r="I19" s="27"/>
-      <c r="J19" s="119"/>
-      <c r="K19" s="120"/>
+      <c r="J19" s="71"/>
+      <c r="K19" s="72"/>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="32"/>
@@ -2257,8 +2257,8 @@
       <c r="G20" s="64"/>
       <c r="H20" s="62"/>
       <c r="I20" s="27"/>
-      <c r="J20" s="119"/>
-      <c r="K20" s="120"/>
+      <c r="J20" s="71"/>
+      <c r="K20" s="72"/>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="32"/>
@@ -2270,8 +2270,8 @@
       <c r="G21" s="62"/>
       <c r="H21" s="62"/>
       <c r="I21" s="27"/>
-      <c r="J21" s="119"/>
-      <c r="K21" s="120"/>
+      <c r="J21" s="71"/>
+      <c r="K21" s="72"/>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="32"/>
@@ -2283,8 +2283,8 @@
       <c r="G22" s="62"/>
       <c r="H22" s="62"/>
       <c r="I22" s="27"/>
-      <c r="J22" s="119"/>
-      <c r="K22" s="120"/>
+      <c r="J22" s="71"/>
+      <c r="K22" s="72"/>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="32"/>
@@ -2296,8 +2296,8 @@
       <c r="G23" s="27"/>
       <c r="H23" s="27"/>
       <c r="I23" s="27"/>
-      <c r="J23" s="119"/>
-      <c r="K23" s="120"/>
+      <c r="J23" s="71"/>
+      <c r="K23" s="72"/>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" s="32"/>
@@ -2309,8 +2309,8 @@
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
-      <c r="J24" s="119"/>
-      <c r="K24" s="120"/>
+      <c r="J24" s="71"/>
+      <c r="K24" s="72"/>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="32"/>
@@ -2322,90 +2322,90 @@
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
       <c r="I25" s="9"/>
-      <c r="J25" s="119"/>
-      <c r="K25" s="120"/>
+      <c r="J25" s="71"/>
+      <c r="K25" s="72"/>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="83"/>
-      <c r="B26" s="80"/>
-      <c r="C26" s="80"/>
-      <c r="D26" s="80"/>
-      <c r="E26" s="84"/>
+      <c r="A26" s="105"/>
+      <c r="B26" s="94"/>
+      <c r="C26" s="94"/>
+      <c r="D26" s="94"/>
+      <c r="E26" s="106"/>
       <c r="F26" s="66"/>
       <c r="G26" s="67"/>
       <c r="H26" s="8"/>
       <c r="I26" s="9"/>
-      <c r="J26" s="119"/>
-      <c r="K26" s="120"/>
+      <c r="J26" s="71"/>
+      <c r="K26" s="72"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="80"/>
-      <c r="B27" s="80"/>
-      <c r="C27" s="80"/>
-      <c r="D27" s="80"/>
-      <c r="E27" s="84"/>
+      <c r="A27" s="94"/>
+      <c r="B27" s="94"/>
+      <c r="C27" s="94"/>
+      <c r="D27" s="94"/>
+      <c r="E27" s="106"/>
       <c r="F27" s="68"/>
       <c r="G27" s="67"/>
       <c r="H27" s="8"/>
       <c r="I27" s="9"/>
-      <c r="J27" s="119"/>
-      <c r="K27" s="120"/>
+      <c r="J27" s="71"/>
+      <c r="K27" s="72"/>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="80"/>
-      <c r="B28" s="80"/>
-      <c r="C28" s="80"/>
-      <c r="D28" s="80"/>
-      <c r="E28" s="84"/>
+      <c r="A28" s="94"/>
+      <c r="B28" s="94"/>
+      <c r="C28" s="94"/>
+      <c r="D28" s="94"/>
+      <c r="E28" s="106"/>
       <c r="F28" s="68"/>
       <c r="G28" s="67"/>
       <c r="H28" s="8"/>
       <c r="I28" s="9"/>
-      <c r="J28" s="119"/>
-      <c r="K28" s="120"/>
+      <c r="J28" s="71"/>
+      <c r="K28" s="72"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="80"/>
-      <c r="B29" s="80"/>
-      <c r="C29" s="80"/>
-      <c r="D29" s="80"/>
-      <c r="E29" s="84"/>
+      <c r="A29" s="94"/>
+      <c r="B29" s="94"/>
+      <c r="C29" s="94"/>
+      <c r="D29" s="94"/>
+      <c r="E29" s="106"/>
       <c r="F29" s="69"/>
       <c r="G29" s="70"/>
       <c r="H29" s="65"/>
       <c r="I29" s="23"/>
-      <c r="J29" s="119"/>
-      <c r="K29" s="120"/>
+      <c r="J29" s="71"/>
+      <c r="K29" s="72"/>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="85"/>
-      <c r="B30" s="85"/>
-      <c r="C30" s="85"/>
-      <c r="D30" s="85"/>
-      <c r="E30" s="86"/>
+      <c r="A30" s="107"/>
+      <c r="B30" s="107"/>
+      <c r="C30" s="107"/>
+      <c r="D30" s="107"/>
+      <c r="E30" s="108"/>
       <c r="F30" s="49"/>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
-      <c r="J30" s="119"/>
-      <c r="K30" s="120"/>
+      <c r="J30" s="71"/>
+      <c r="K30" s="72"/>
     </row>
     <row r="31" spans="1:11" ht="15.75">
-      <c r="A31" s="71" t="s">
+      <c r="A31" s="137" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="72"/>
-      <c r="C31" s="73"/>
+      <c r="B31" s="90"/>
+      <c r="C31" s="97"/>
       <c r="D31" s="50"/>
-      <c r="E31" s="74"/>
-      <c r="F31" s="75"/>
-      <c r="G31" s="75"/>
-      <c r="H31" s="75"/>
-      <c r="I31" s="76" t="s">
+      <c r="E31" s="138"/>
+      <c r="F31" s="139"/>
+      <c r="G31" s="139"/>
+      <c r="H31" s="139"/>
+      <c r="I31" s="140" t="s">
         <v>16</v>
       </c>
-      <c r="J31" s="77"/>
-      <c r="K31" s="78"/>
+      <c r="J31" s="141"/>
+      <c r="K31" s="142"/>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" s="37"/>
@@ -2413,12 +2413,12 @@
       <c r="C32" s="4"/>
       <c r="D32" s="38"/>
       <c r="E32" s="3"/>
-      <c r="F32" s="79"/>
-      <c r="G32" s="80"/>
-      <c r="H32" s="81"/>
-      <c r="I32" s="79"/>
-      <c r="J32" s="80"/>
-      <c r="K32" s="82"/>
+      <c r="F32" s="143"/>
+      <c r="G32" s="94"/>
+      <c r="H32" s="110"/>
+      <c r="I32" s="143"/>
+      <c r="J32" s="94"/>
+      <c r="K32" s="144"/>
     </row>
     <row r="33" spans="1:11">
       <c r="A33" s="39"/>
@@ -2497,32 +2497,11 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J30:K30"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="E1:G2"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="A5:C6"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="E6:G6"/>
-    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="E31:H31"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="I32:K32"/>
     <mergeCell ref="A26:E30"/>
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="J9:K9"/>
@@ -2539,11 +2518,32 @@
     <mergeCell ref="J13:K13"/>
     <mergeCell ref="J14:K14"/>
     <mergeCell ref="J15:K15"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="E31:H31"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="A5:C6"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="E1:G2"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J30:K30"/>
   </mergeCells>
   <conditionalFormatting sqref="F12:G15 I12 F17:F22 G17:G19 G21:G22">
     <cfRule type="expression" dxfId="7" priority="1">
@@ -2595,39 +2595,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.6" customHeight="1">
-      <c r="A1" s="128" t="s">
+      <c r="A1" s="73" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="129"/>
-      <c r="C1" s="150"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="145"/>
       <c r="D1" s="58"/>
-      <c r="E1" s="152" t="s">
+      <c r="E1" s="147" t="s">
         <v>18</v>
       </c>
-      <c r="F1" s="153"/>
-      <c r="G1" s="154"/>
+      <c r="F1" s="148"/>
+      <c r="G1" s="149"/>
       <c r="H1" s="29"/>
-      <c r="I1" s="139" t="s">
+      <c r="I1" s="84" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="140"/>
-      <c r="K1" s="141"/>
+      <c r="J1" s="85"/>
+      <c r="K1" s="86"/>
     </row>
     <row r="2" spans="1:11" ht="15.75">
-      <c r="A2" s="130"/>
-      <c r="B2" s="131"/>
-      <c r="C2" s="151"/>
+      <c r="A2" s="75"/>
+      <c r="B2" s="76"/>
+      <c r="C2" s="146"/>
       <c r="D2" s="52"/>
-      <c r="E2" s="155"/>
-      <c r="F2" s="156"/>
-      <c r="G2" s="157"/>
+      <c r="E2" s="150"/>
+      <c r="F2" s="151"/>
+      <c r="G2" s="152"/>
       <c r="H2" s="15"/>
-      <c r="I2" s="142">
+      <c r="I2" s="87">
         <f ca="1">TODAY()</f>
         <v>45864</v>
       </c>
-      <c r="J2" s="137"/>
-      <c r="K2" s="138"/>
+      <c r="J2" s="82"/>
+      <c r="K2" s="83"/>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="32"/>
@@ -2643,11 +2643,11 @@
       <c r="K3" s="33"/>
     </row>
     <row r="4" spans="1:11" ht="17.25">
-      <c r="A4" s="158" t="s">
+      <c r="A4" s="153" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="159"/>
-      <c r="C4" s="131"/>
+      <c r="B4" s="154"/>
+      <c r="C4" s="76"/>
       <c r="D4" s="52"/>
       <c r="E4" s="26" t="s">
         <v>19</v>
@@ -2658,46 +2658,46 @@
       <c r="I4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="144"/>
-      <c r="K4" s="115"/>
+      <c r="J4" s="91"/>
+      <c r="K4" s="92"/>
     </row>
     <row r="5" spans="1:11" ht="18.75">
-      <c r="A5" s="145" t="s">
+      <c r="A5" s="155" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="146"/>
-      <c r="C5" s="132"/>
+      <c r="B5" s="156"/>
+      <c r="C5" s="77"/>
       <c r="D5" s="14"/>
-      <c r="E5" s="122" t="s">
+      <c r="E5" s="98" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="123"/>
-      <c r="G5" s="124"/>
+      <c r="F5" s="99"/>
+      <c r="G5" s="100"/>
       <c r="H5" s="22"/>
       <c r="I5" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="J5" s="125"/>
-      <c r="K5" s="115"/>
+      <c r="J5" s="101"/>
+      <c r="K5" s="92"/>
     </row>
     <row r="6" spans="1:11" ht="15.75">
-      <c r="A6" s="130"/>
-      <c r="B6" s="131"/>
-      <c r="C6" s="147"/>
+      <c r="A6" s="75"/>
+      <c r="B6" s="76"/>
+      <c r="C6" s="157"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="148" t="s">
+      <c r="E6" s="158" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="131"/>
-      <c r="G6" s="149"/>
+      <c r="F6" s="76"/>
+      <c r="G6" s="159"/>
       <c r="H6" s="46"/>
       <c r="I6" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="127">
+      <c r="J6" s="104">
         <v>1230</v>
       </c>
-      <c r="K6" s="115"/>
+      <c r="K6" s="92"/>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="32"/>
@@ -2713,44 +2713,44 @@
       <c r="K7" s="33"/>
     </row>
     <row r="8" spans="1:11" ht="15.75">
-      <c r="A8" s="107" t="s">
+      <c r="A8" s="127" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="109"/>
-      <c r="D8" s="110"/>
-      <c r="E8" s="111"/>
+      <c r="C8" s="129"/>
+      <c r="D8" s="130"/>
+      <c r="E8" s="131"/>
       <c r="F8" s="14"/>
-      <c r="G8" s="112" t="s">
+      <c r="G8" s="132" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="113"/>
+      <c r="H8" s="89"/>
       <c r="I8" s="14"/>
-      <c r="J8" s="114" t="s">
+      <c r="J8" s="133" t="s">
         <v>11</v>
       </c>
-      <c r="K8" s="115"/>
+      <c r="K8" s="92"/>
     </row>
     <row r="9" spans="1:11" ht="17.25">
-      <c r="A9" s="108"/>
+      <c r="A9" s="128"/>
       <c r="B9" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="116" t="s">
+      <c r="C9" s="134" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="72"/>
-      <c r="E9" s="81"/>
+      <c r="D9" s="90"/>
+      <c r="E9" s="110"/>
       <c r="F9" s="22"/>
-      <c r="G9" s="87">
+      <c r="G9" s="109">
         <v>1</v>
       </c>
-      <c r="H9" s="81"/>
+      <c r="H9" s="110"/>
       <c r="I9" s="22"/>
-      <c r="J9" s="88"/>
-      <c r="K9" s="89"/>
+      <c r="J9" s="111"/>
+      <c r="K9" s="103"/>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="32"/>
@@ -2766,128 +2766,128 @@
       <c r="K10" s="34"/>
     </row>
     <row r="11" spans="1:11" ht="18.75">
-      <c r="A11" s="90" t="s">
+      <c r="A11" s="112" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="91"/>
-      <c r="C11" s="91"/>
-      <c r="D11" s="91"/>
-      <c r="E11" s="92"/>
-      <c r="F11" s="93"/>
-      <c r="G11" s="91"/>
-      <c r="H11" s="91"/>
-      <c r="I11" s="91"/>
-      <c r="J11" s="91"/>
-      <c r="K11" s="94"/>
+      <c r="B11" s="113"/>
+      <c r="C11" s="113"/>
+      <c r="D11" s="113"/>
+      <c r="E11" s="114"/>
+      <c r="F11" s="115"/>
+      <c r="G11" s="113"/>
+      <c r="H11" s="113"/>
+      <c r="I11" s="113"/>
+      <c r="J11" s="113"/>
+      <c r="K11" s="116"/>
     </row>
     <row r="12" spans="1:11" ht="12.6" customHeight="1">
-      <c r="A12" s="95" t="s">
+      <c r="A12" s="117" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="96"/>
-      <c r="C12" s="96"/>
-      <c r="D12" s="96"/>
-      <c r="E12" s="81"/>
+      <c r="B12" s="95"/>
+      <c r="C12" s="95"/>
+      <c r="D12" s="95"/>
+      <c r="E12" s="110"/>
       <c r="F12" s="59"/>
       <c r="G12" s="31"/>
       <c r="H12" s="60"/>
       <c r="I12" s="31"/>
-      <c r="J12" s="117"/>
-      <c r="K12" s="118"/>
+      <c r="J12" s="135"/>
+      <c r="K12" s="136"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="97"/>
-      <c r="B13" s="72"/>
-      <c r="C13" s="72"/>
-      <c r="D13" s="72"/>
-      <c r="E13" s="73"/>
+      <c r="A13" s="96"/>
+      <c r="B13" s="90"/>
+      <c r="C13" s="90"/>
+      <c r="D13" s="90"/>
+      <c r="E13" s="97"/>
       <c r="F13" s="27"/>
       <c r="G13" s="61"/>
       <c r="H13" s="62"/>
       <c r="I13" s="2"/>
-      <c r="J13" s="117"/>
-      <c r="K13" s="118"/>
+      <c r="J13" s="135"/>
+      <c r="K13" s="136"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="98" t="str">
+      <c r="A14" s="118" t="str">
         <f>"*"&amp;A12&amp;"*"</f>
         <v>*GOFEMM20052025002*</v>
       </c>
-      <c r="B14" s="99"/>
-      <c r="C14" s="99"/>
-      <c r="D14" s="99"/>
-      <c r="E14" s="100"/>
+      <c r="B14" s="119"/>
+      <c r="C14" s="119"/>
+      <c r="D14" s="119"/>
+      <c r="E14" s="120"/>
       <c r="F14" s="27"/>
       <c r="G14" s="62"/>
       <c r="H14" s="62"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="117"/>
-      <c r="K14" s="118"/>
+      <c r="J14" s="135"/>
+      <c r="K14" s="136"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="101"/>
-      <c r="B15" s="102"/>
-      <c r="C15" s="102"/>
-      <c r="D15" s="102"/>
-      <c r="E15" s="103"/>
+      <c r="A15" s="121"/>
+      <c r="B15" s="122"/>
+      <c r="C15" s="122"/>
+      <c r="D15" s="122"/>
+      <c r="E15" s="123"/>
       <c r="F15" s="27"/>
       <c r="G15" s="62"/>
       <c r="H15" s="62"/>
       <c r="I15" s="2"/>
-      <c r="J15" s="117"/>
-      <c r="K15" s="118"/>
+      <c r="J15" s="135"/>
+      <c r="K15" s="136"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="101"/>
-      <c r="B16" s="102"/>
-      <c r="C16" s="102"/>
-      <c r="D16" s="102"/>
-      <c r="E16" s="103"/>
+      <c r="A16" s="121"/>
+      <c r="B16" s="122"/>
+      <c r="C16" s="122"/>
+      <c r="D16" s="122"/>
+      <c r="E16" s="123"/>
       <c r="F16" s="8"/>
       <c r="G16" s="62"/>
       <c r="H16" s="62"/>
       <c r="I16" s="2"/>
-      <c r="J16" s="117"/>
-      <c r="K16" s="118"/>
+      <c r="J16" s="135"/>
+      <c r="K16" s="136"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="101"/>
-      <c r="B17" s="102"/>
-      <c r="C17" s="102"/>
-      <c r="D17" s="102"/>
-      <c r="E17" s="103"/>
+      <c r="A17" s="121"/>
+      <c r="B17" s="122"/>
+      <c r="C17" s="122"/>
+      <c r="D17" s="122"/>
+      <c r="E17" s="123"/>
       <c r="F17" s="27"/>
       <c r="G17" s="62"/>
       <c r="H17" s="62"/>
       <c r="I17" s="2"/>
-      <c r="J17" s="117"/>
-      <c r="K17" s="118"/>
+      <c r="J17" s="135"/>
+      <c r="K17" s="136"/>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="101"/>
-      <c r="B18" s="102"/>
-      <c r="C18" s="102"/>
-      <c r="D18" s="102"/>
-      <c r="E18" s="103"/>
+      <c r="A18" s="121"/>
+      <c r="B18" s="122"/>
+      <c r="C18" s="122"/>
+      <c r="D18" s="122"/>
+      <c r="E18" s="123"/>
       <c r="F18" s="27"/>
       <c r="G18" s="62"/>
       <c r="H18" s="62"/>
       <c r="I18" s="8"/>
-      <c r="J18" s="117"/>
-      <c r="K18" s="118"/>
+      <c r="J18" s="135"/>
+      <c r="K18" s="136"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="104"/>
-      <c r="B19" s="105"/>
-      <c r="C19" s="105"/>
-      <c r="D19" s="105"/>
-      <c r="E19" s="106"/>
+      <c r="A19" s="124"/>
+      <c r="B19" s="125"/>
+      <c r="C19" s="125"/>
+      <c r="D19" s="125"/>
+      <c r="E19" s="126"/>
       <c r="F19" s="63"/>
       <c r="G19" s="62"/>
       <c r="H19" s="62"/>
       <c r="I19" s="27"/>
-      <c r="J19" s="117"/>
-      <c r="K19" s="118"/>
+      <c r="J19" s="135"/>
+      <c r="K19" s="136"/>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="32"/>
@@ -2899,8 +2899,8 @@
       <c r="G20" s="64"/>
       <c r="H20" s="62"/>
       <c r="I20" s="27"/>
-      <c r="J20" s="117"/>
-      <c r="K20" s="118"/>
+      <c r="J20" s="135"/>
+      <c r="K20" s="136"/>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="32"/>
@@ -2912,8 +2912,8 @@
       <c r="G21" s="62"/>
       <c r="H21" s="62"/>
       <c r="I21" s="27"/>
-      <c r="J21" s="117"/>
-      <c r="K21" s="118"/>
+      <c r="J21" s="135"/>
+      <c r="K21" s="136"/>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="32"/>
@@ -2925,8 +2925,8 @@
       <c r="G22" s="62"/>
       <c r="H22" s="62"/>
       <c r="I22" s="27"/>
-      <c r="J22" s="117"/>
-      <c r="K22" s="118"/>
+      <c r="J22" s="135"/>
+      <c r="K22" s="136"/>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="32"/>
@@ -2938,8 +2938,8 @@
       <c r="G23" s="27"/>
       <c r="H23" s="27"/>
       <c r="I23" s="27"/>
-      <c r="J23" s="117"/>
-      <c r="K23" s="118"/>
+      <c r="J23" s="135"/>
+      <c r="K23" s="136"/>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" s="32"/>
@@ -2951,8 +2951,8 @@
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
-      <c r="J24" s="117"/>
-      <c r="K24" s="118"/>
+      <c r="J24" s="135"/>
+      <c r="K24" s="136"/>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="32"/>
@@ -2964,90 +2964,90 @@
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
       <c r="I25" s="9"/>
-      <c r="J25" s="117"/>
-      <c r="K25" s="118"/>
+      <c r="J25" s="135"/>
+      <c r="K25" s="136"/>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="83"/>
-      <c r="B26" s="80"/>
-      <c r="C26" s="80"/>
-      <c r="D26" s="80"/>
-      <c r="E26" s="84"/>
+      <c r="A26" s="105"/>
+      <c r="B26" s="94"/>
+      <c r="C26" s="94"/>
+      <c r="D26" s="94"/>
+      <c r="E26" s="106"/>
       <c r="F26" s="66"/>
       <c r="G26" s="67"/>
       <c r="H26" s="8"/>
       <c r="I26" s="9"/>
-      <c r="J26" s="117"/>
-      <c r="K26" s="118"/>
+      <c r="J26" s="135"/>
+      <c r="K26" s="136"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="80"/>
-      <c r="B27" s="80"/>
-      <c r="C27" s="80"/>
-      <c r="D27" s="80"/>
-      <c r="E27" s="84"/>
+      <c r="A27" s="94"/>
+      <c r="B27" s="94"/>
+      <c r="C27" s="94"/>
+      <c r="D27" s="94"/>
+      <c r="E27" s="106"/>
       <c r="F27" s="68"/>
       <c r="G27" s="67"/>
       <c r="H27" s="8"/>
       <c r="I27" s="9"/>
-      <c r="J27" s="117"/>
-      <c r="K27" s="118"/>
+      <c r="J27" s="135"/>
+      <c r="K27" s="136"/>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="80"/>
-      <c r="B28" s="80"/>
-      <c r="C28" s="80"/>
-      <c r="D28" s="80"/>
-      <c r="E28" s="84"/>
+      <c r="A28" s="94"/>
+      <c r="B28" s="94"/>
+      <c r="C28" s="94"/>
+      <c r="D28" s="94"/>
+      <c r="E28" s="106"/>
       <c r="F28" s="68"/>
       <c r="G28" s="67"/>
       <c r="H28" s="8"/>
       <c r="I28" s="9"/>
-      <c r="J28" s="117"/>
-      <c r="K28" s="118"/>
+      <c r="J28" s="135"/>
+      <c r="K28" s="136"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="80"/>
-      <c r="B29" s="80"/>
-      <c r="C29" s="80"/>
-      <c r="D29" s="80"/>
-      <c r="E29" s="84"/>
+      <c r="A29" s="94"/>
+      <c r="B29" s="94"/>
+      <c r="C29" s="94"/>
+      <c r="D29" s="94"/>
+      <c r="E29" s="106"/>
       <c r="F29" s="69"/>
       <c r="G29" s="70"/>
       <c r="H29" s="65"/>
       <c r="I29" s="23"/>
-      <c r="J29" s="117"/>
-      <c r="K29" s="118"/>
+      <c r="J29" s="135"/>
+      <c r="K29" s="136"/>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="85"/>
-      <c r="B30" s="85"/>
-      <c r="C30" s="85"/>
-      <c r="D30" s="85"/>
-      <c r="E30" s="86"/>
+      <c r="A30" s="107"/>
+      <c r="B30" s="107"/>
+      <c r="C30" s="107"/>
+      <c r="D30" s="107"/>
+      <c r="E30" s="108"/>
       <c r="F30" s="49"/>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
-      <c r="J30" s="117"/>
-      <c r="K30" s="118"/>
+      <c r="J30" s="135"/>
+      <c r="K30" s="136"/>
     </row>
     <row r="31" spans="1:11" ht="15.75">
-      <c r="A31" s="71" t="s">
+      <c r="A31" s="137" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="72"/>
-      <c r="C31" s="73"/>
+      <c r="B31" s="90"/>
+      <c r="C31" s="97"/>
       <c r="D31" s="50"/>
-      <c r="E31" s="74"/>
-      <c r="F31" s="75"/>
-      <c r="G31" s="75"/>
-      <c r="H31" s="75"/>
-      <c r="I31" s="76" t="s">
+      <c r="E31" s="138"/>
+      <c r="F31" s="139"/>
+      <c r="G31" s="139"/>
+      <c r="H31" s="139"/>
+      <c r="I31" s="140" t="s">
         <v>16</v>
       </c>
-      <c r="J31" s="77"/>
-      <c r="K31" s="78"/>
+      <c r="J31" s="141"/>
+      <c r="K31" s="142"/>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" s="37"/>
@@ -3055,12 +3055,12 @@
       <c r="C32" s="4"/>
       <c r="D32" s="38"/>
       <c r="E32" s="3"/>
-      <c r="F32" s="79"/>
-      <c r="G32" s="80"/>
-      <c r="H32" s="81"/>
-      <c r="I32" s="79"/>
-      <c r="J32" s="80"/>
-      <c r="K32" s="82"/>
+      <c r="F32" s="143"/>
+      <c r="G32" s="94"/>
+      <c r="H32" s="110"/>
+      <c r="I32" s="143"/>
+      <c r="J32" s="94"/>
+      <c r="K32" s="144"/>
     </row>
     <row r="33" spans="1:11">
       <c r="A33" s="39"/>
@@ -3139,27 +3139,16 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="E1:G2"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="A26:E30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="E31:H31"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J30:K30"/>
     <mergeCell ref="A14:E19"/>
     <mergeCell ref="A5:C6"/>
     <mergeCell ref="E5:G5"/>
@@ -3176,16 +3165,27 @@
     <mergeCell ref="A11:E11"/>
     <mergeCell ref="F11:K11"/>
     <mergeCell ref="A12:E13"/>
-    <mergeCell ref="A26:E30"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="E31:H31"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="E1:G2"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J26:K26"/>
   </mergeCells>
   <conditionalFormatting sqref="F12:G15 I12 F17:F22 G17:G19 G21:G22">
     <cfRule type="expression" dxfId="3" priority="1">

</xml_diff>

<commit_message>
add all changes for tanger
</commit_message>
<xml_diff>
--- a/dummy-content/ECHEC-RETOUR_CLIENT-CASABLANCA.xlsx
+++ b/dummy-content/ECHEC-RETOUR_CLIENT-CASABLANCA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UNK\Desktop\GoFleet-Enhancer\dummy-content\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{221F0FBB-6A08-4A4B-8B1B-C1F1090C05E5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FC134E7-FCF8-49FB-A7D3-F1C93F7432BA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -84,13 +84,13 @@
     <t xml:space="preserve">                                                       Destination</t>
   </si>
   <si>
-    <t>GOFEMM20052025001</t>
+    <t>GO FLEET TANGER</t>
   </si>
   <si>
-    <t>GOFEMM20052025002</t>
+    <t>GTGEMM20052025001</t>
   </si>
   <si>
-    <t>GO FLEET TANGER</t>
+    <t>GTGEMM20052025002</t>
   </si>
 </sst>
 </file>
@@ -1400,66 +1400,24 @@
     <xf numFmtId="0" fontId="15" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="5" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
@@ -1467,10 +1425,10 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="11" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1483,6 +1441,8 @@
     <xf numFmtId="0" fontId="21" fillId="12" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="24" fillId="3" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1506,9 +1466,11 @@
     <xf numFmtId="0" fontId="8" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1518,20 +1480,67 @@
     <xf numFmtId="0" fontId="15" fillId="15" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="5" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="19" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="17" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1546,15 +1555,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="20" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="19" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1955,37 +1955,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.6" customHeight="1">
-      <c r="A1" s="73"/>
-      <c r="B1" s="74"/>
-      <c r="C1" s="74"/>
+      <c r="A1" s="128"/>
+      <c r="B1" s="129"/>
+      <c r="C1" s="129"/>
       <c r="D1" s="53"/>
-      <c r="E1" s="78" t="s">
+      <c r="E1" s="133" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="79"/>
-      <c r="G1" s="80"/>
+      <c r="F1" s="134"/>
+      <c r="G1" s="135"/>
       <c r="H1" s="29"/>
-      <c r="I1" s="84" t="s">
+      <c r="I1" s="139" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="85"/>
-      <c r="K1" s="86"/>
+      <c r="J1" s="140"/>
+      <c r="K1" s="141"/>
     </row>
     <row r="2" spans="1:11" ht="15.75">
-      <c r="A2" s="75"/>
-      <c r="B2" s="76"/>
-      <c r="C2" s="77"/>
+      <c r="A2" s="130"/>
+      <c r="B2" s="131"/>
+      <c r="C2" s="132"/>
       <c r="D2" s="53"/>
-      <c r="E2" s="81"/>
-      <c r="F2" s="82"/>
-      <c r="G2" s="83"/>
+      <c r="E2" s="136"/>
+      <c r="F2" s="137"/>
+      <c r="G2" s="138"/>
       <c r="H2" s="15"/>
-      <c r="I2" s="87">
+      <c r="I2" s="142">
         <f ca="1">TODAY()</f>
-        <v>45864</v>
-      </c>
-      <c r="J2" s="82"/>
-      <c r="K2" s="83"/>
+        <v>45865</v>
+      </c>
+      <c r="J2" s="137"/>
+      <c r="K2" s="138"/>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="32"/>
@@ -2001,11 +2001,11 @@
       <c r="K3" s="33"/>
     </row>
     <row r="4" spans="1:11" ht="17.25">
-      <c r="A4" s="88" t="s">
+      <c r="A4" s="143" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="89"/>
-      <c r="C4" s="90"/>
+      <c r="B4" s="113"/>
+      <c r="C4" s="72"/>
       <c r="D4" s="52"/>
       <c r="E4" s="16" t="s">
         <v>19</v>
@@ -2016,46 +2016,46 @@
       <c r="I4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="91"/>
-      <c r="K4" s="92"/>
+      <c r="J4" s="144"/>
+      <c r="K4" s="115"/>
     </row>
     <row r="5" spans="1:11" ht="18.75">
-      <c r="A5" s="93" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="94"/>
-      <c r="C5" s="95"/>
+      <c r="A5" s="121" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="80"/>
+      <c r="C5" s="96"/>
       <c r="D5" s="14"/>
-      <c r="E5" s="98" t="s">
+      <c r="E5" s="122" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="99"/>
-      <c r="G5" s="100"/>
+      <c r="F5" s="123"/>
+      <c r="G5" s="124"/>
       <c r="H5" s="22"/>
       <c r="I5" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="J5" s="101"/>
-      <c r="K5" s="92"/>
+      <c r="J5" s="125"/>
+      <c r="K5" s="115"/>
     </row>
     <row r="6" spans="1:11" ht="15.75">
-      <c r="A6" s="96"/>
-      <c r="B6" s="90"/>
-      <c r="C6" s="97"/>
+      <c r="A6" s="97"/>
+      <c r="B6" s="72"/>
+      <c r="C6" s="73"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="102" t="s">
+      <c r="E6" s="126" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="90"/>
-      <c r="G6" s="103"/>
+      <c r="F6" s="72"/>
+      <c r="G6" s="89"/>
       <c r="H6" s="46"/>
       <c r="I6" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="104">
+      <c r="J6" s="127">
         <v>1230</v>
       </c>
-      <c r="K6" s="92"/>
+      <c r="K6" s="115"/>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="32"/>
@@ -2071,44 +2071,44 @@
       <c r="K7" s="33"/>
     </row>
     <row r="8" spans="1:11" ht="15.75">
-      <c r="A8" s="127" t="s">
+      <c r="A8" s="107" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="129"/>
-      <c r="D8" s="130"/>
-      <c r="E8" s="131"/>
+      <c r="C8" s="109"/>
+      <c r="D8" s="110"/>
+      <c r="E8" s="111"/>
       <c r="F8" s="14"/>
-      <c r="G8" s="132" t="s">
+      <c r="G8" s="112" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="89"/>
+      <c r="H8" s="113"/>
       <c r="I8" s="14"/>
-      <c r="J8" s="133" t="s">
+      <c r="J8" s="114" t="s">
         <v>11</v>
       </c>
-      <c r="K8" s="92"/>
+      <c r="K8" s="115"/>
     </row>
     <row r="9" spans="1:11" ht="17.25">
-      <c r="A9" s="128"/>
+      <c r="A9" s="108"/>
       <c r="B9" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="134" t="s">
+      <c r="C9" s="116" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="90"/>
-      <c r="E9" s="110"/>
+      <c r="D9" s="72"/>
+      <c r="E9" s="81"/>
       <c r="F9" s="22"/>
-      <c r="G9" s="109">
+      <c r="G9" s="87">
         <v>1</v>
       </c>
-      <c r="H9" s="110"/>
+      <c r="H9" s="81"/>
       <c r="I9" s="22"/>
-      <c r="J9" s="111"/>
-      <c r="K9" s="103"/>
+      <c r="J9" s="88"/>
+      <c r="K9" s="89"/>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="32"/>
@@ -2124,128 +2124,128 @@
       <c r="K10" s="34"/>
     </row>
     <row r="11" spans="1:11" ht="18.75">
-      <c r="A11" s="112" t="s">
+      <c r="A11" s="90" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="113"/>
-      <c r="C11" s="113"/>
-      <c r="D11" s="113"/>
-      <c r="E11" s="114"/>
-      <c r="F11" s="115"/>
-      <c r="G11" s="113"/>
-      <c r="H11" s="113"/>
-      <c r="I11" s="113"/>
-      <c r="J11" s="113"/>
-      <c r="K11" s="116"/>
+      <c r="B11" s="91"/>
+      <c r="C11" s="91"/>
+      <c r="D11" s="91"/>
+      <c r="E11" s="92"/>
+      <c r="F11" s="93"/>
+      <c r="G11" s="91"/>
+      <c r="H11" s="91"/>
+      <c r="I11" s="91"/>
+      <c r="J11" s="91"/>
+      <c r="K11" s="94"/>
     </row>
     <row r="12" spans="1:11">
-      <c r="A12" s="117" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" s="95"/>
-      <c r="C12" s="95"/>
-      <c r="D12" s="95"/>
-      <c r="E12" s="110"/>
+      <c r="A12" s="95" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="96"/>
+      <c r="C12" s="96"/>
+      <c r="D12" s="96"/>
+      <c r="E12" s="81"/>
       <c r="F12" s="59"/>
       <c r="G12" s="31"/>
       <c r="H12" s="60"/>
       <c r="I12" s="31"/>
-      <c r="J12" s="135"/>
-      <c r="K12" s="136"/>
+      <c r="J12" s="117"/>
+      <c r="K12" s="118"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="96"/>
-      <c r="B13" s="90"/>
-      <c r="C13" s="90"/>
-      <c r="D13" s="90"/>
-      <c r="E13" s="97"/>
+      <c r="A13" s="97"/>
+      <c r="B13" s="72"/>
+      <c r="C13" s="72"/>
+      <c r="D13" s="72"/>
+      <c r="E13" s="73"/>
       <c r="F13" s="27"/>
       <c r="G13" s="61"/>
       <c r="H13" s="62"/>
       <c r="I13" s="2"/>
-      <c r="J13" s="71"/>
-      <c r="K13" s="72"/>
+      <c r="J13" s="119"/>
+      <c r="K13" s="120"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="118" t="str">
+      <c r="A14" s="98" t="str">
         <f>"*"&amp;A12&amp;"*"</f>
-        <v>*GOFEMM20052025001*</v>
-      </c>
-      <c r="B14" s="119"/>
-      <c r="C14" s="119"/>
-      <c r="D14" s="119"/>
-      <c r="E14" s="120"/>
+        <v>*GTGEMM20052025001*</v>
+      </c>
+      <c r="B14" s="99"/>
+      <c r="C14" s="99"/>
+      <c r="D14" s="99"/>
+      <c r="E14" s="100"/>
       <c r="F14" s="27"/>
       <c r="G14" s="62"/>
       <c r="H14" s="62"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="71"/>
-      <c r="K14" s="72"/>
+      <c r="J14" s="119"/>
+      <c r="K14" s="120"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="121"/>
-      <c r="B15" s="122"/>
-      <c r="C15" s="122"/>
-      <c r="D15" s="122"/>
-      <c r="E15" s="123"/>
+      <c r="A15" s="101"/>
+      <c r="B15" s="102"/>
+      <c r="C15" s="102"/>
+      <c r="D15" s="102"/>
+      <c r="E15" s="103"/>
       <c r="F15" s="27"/>
       <c r="G15" s="62"/>
       <c r="H15" s="62"/>
       <c r="I15" s="2"/>
-      <c r="J15" s="71"/>
-      <c r="K15" s="72"/>
+      <c r="J15" s="119"/>
+      <c r="K15" s="120"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="121"/>
-      <c r="B16" s="122"/>
-      <c r="C16" s="122"/>
-      <c r="D16" s="122"/>
-      <c r="E16" s="123"/>
+      <c r="A16" s="101"/>
+      <c r="B16" s="102"/>
+      <c r="C16" s="102"/>
+      <c r="D16" s="102"/>
+      <c r="E16" s="103"/>
       <c r="F16" s="8"/>
       <c r="G16" s="62"/>
       <c r="H16" s="62"/>
       <c r="I16" s="2"/>
-      <c r="J16" s="71"/>
-      <c r="K16" s="72"/>
+      <c r="J16" s="119"/>
+      <c r="K16" s="120"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="121"/>
-      <c r="B17" s="122"/>
-      <c r="C17" s="122"/>
-      <c r="D17" s="122"/>
-      <c r="E17" s="123"/>
+      <c r="A17" s="101"/>
+      <c r="B17" s="102"/>
+      <c r="C17" s="102"/>
+      <c r="D17" s="102"/>
+      <c r="E17" s="103"/>
       <c r="F17" s="27"/>
       <c r="G17" s="62"/>
       <c r="H17" s="62"/>
       <c r="I17" s="2"/>
-      <c r="J17" s="71"/>
-      <c r="K17" s="72"/>
+      <c r="J17" s="119"/>
+      <c r="K17" s="120"/>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="121"/>
-      <c r="B18" s="122"/>
-      <c r="C18" s="122"/>
-      <c r="D18" s="122"/>
-      <c r="E18" s="123"/>
+      <c r="A18" s="101"/>
+      <c r="B18" s="102"/>
+      <c r="C18" s="102"/>
+      <c r="D18" s="102"/>
+      <c r="E18" s="103"/>
       <c r="F18" s="27"/>
       <c r="G18" s="62"/>
       <c r="H18" s="62"/>
       <c r="I18" s="8"/>
-      <c r="J18" s="71"/>
-      <c r="K18" s="72"/>
+      <c r="J18" s="119"/>
+      <c r="K18" s="120"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="124"/>
-      <c r="B19" s="125"/>
-      <c r="C19" s="125"/>
-      <c r="D19" s="125"/>
-      <c r="E19" s="126"/>
+      <c r="A19" s="104"/>
+      <c r="B19" s="105"/>
+      <c r="C19" s="105"/>
+      <c r="D19" s="105"/>
+      <c r="E19" s="106"/>
       <c r="F19" s="63"/>
       <c r="G19" s="62"/>
       <c r="H19" s="62"/>
       <c r="I19" s="27"/>
-      <c r="J19" s="71"/>
-      <c r="K19" s="72"/>
+      <c r="J19" s="119"/>
+      <c r="K19" s="120"/>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="32"/>
@@ -2257,8 +2257,8 @@
       <c r="G20" s="64"/>
       <c r="H20" s="62"/>
       <c r="I20" s="27"/>
-      <c r="J20" s="71"/>
-      <c r="K20" s="72"/>
+      <c r="J20" s="119"/>
+      <c r="K20" s="120"/>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="32"/>
@@ -2270,8 +2270,8 @@
       <c r="G21" s="62"/>
       <c r="H21" s="62"/>
       <c r="I21" s="27"/>
-      <c r="J21" s="71"/>
-      <c r="K21" s="72"/>
+      <c r="J21" s="119"/>
+      <c r="K21" s="120"/>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="32"/>
@@ -2283,8 +2283,8 @@
       <c r="G22" s="62"/>
       <c r="H22" s="62"/>
       <c r="I22" s="27"/>
-      <c r="J22" s="71"/>
-      <c r="K22" s="72"/>
+      <c r="J22" s="119"/>
+      <c r="K22" s="120"/>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="32"/>
@@ -2296,8 +2296,8 @@
       <c r="G23" s="27"/>
       <c r="H23" s="27"/>
       <c r="I23" s="27"/>
-      <c r="J23" s="71"/>
-      <c r="K23" s="72"/>
+      <c r="J23" s="119"/>
+      <c r="K23" s="120"/>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" s="32"/>
@@ -2309,8 +2309,8 @@
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
-      <c r="J24" s="71"/>
-      <c r="K24" s="72"/>
+      <c r="J24" s="119"/>
+      <c r="K24" s="120"/>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="32"/>
@@ -2322,90 +2322,90 @@
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
       <c r="I25" s="9"/>
-      <c r="J25" s="71"/>
-      <c r="K25" s="72"/>
+      <c r="J25" s="119"/>
+      <c r="K25" s="120"/>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="105"/>
-      <c r="B26" s="94"/>
-      <c r="C26" s="94"/>
-      <c r="D26" s="94"/>
-      <c r="E26" s="106"/>
+      <c r="A26" s="83"/>
+      <c r="B26" s="80"/>
+      <c r="C26" s="80"/>
+      <c r="D26" s="80"/>
+      <c r="E26" s="84"/>
       <c r="F26" s="66"/>
       <c r="G26" s="67"/>
       <c r="H26" s="8"/>
       <c r="I26" s="9"/>
-      <c r="J26" s="71"/>
-      <c r="K26" s="72"/>
+      <c r="J26" s="119"/>
+      <c r="K26" s="120"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="94"/>
-      <c r="B27" s="94"/>
-      <c r="C27" s="94"/>
-      <c r="D27" s="94"/>
-      <c r="E27" s="106"/>
+      <c r="A27" s="80"/>
+      <c r="B27" s="80"/>
+      <c r="C27" s="80"/>
+      <c r="D27" s="80"/>
+      <c r="E27" s="84"/>
       <c r="F27" s="68"/>
       <c r="G27" s="67"/>
       <c r="H27" s="8"/>
       <c r="I27" s="9"/>
-      <c r="J27" s="71"/>
-      <c r="K27" s="72"/>
+      <c r="J27" s="119"/>
+      <c r="K27" s="120"/>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="94"/>
-      <c r="B28" s="94"/>
-      <c r="C28" s="94"/>
-      <c r="D28" s="94"/>
-      <c r="E28" s="106"/>
+      <c r="A28" s="80"/>
+      <c r="B28" s="80"/>
+      <c r="C28" s="80"/>
+      <c r="D28" s="80"/>
+      <c r="E28" s="84"/>
       <c r="F28" s="68"/>
       <c r="G28" s="67"/>
       <c r="H28" s="8"/>
       <c r="I28" s="9"/>
-      <c r="J28" s="71"/>
-      <c r="K28" s="72"/>
+      <c r="J28" s="119"/>
+      <c r="K28" s="120"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="94"/>
-      <c r="B29" s="94"/>
-      <c r="C29" s="94"/>
-      <c r="D29" s="94"/>
-      <c r="E29" s="106"/>
+      <c r="A29" s="80"/>
+      <c r="B29" s="80"/>
+      <c r="C29" s="80"/>
+      <c r="D29" s="80"/>
+      <c r="E29" s="84"/>
       <c r="F29" s="69"/>
       <c r="G29" s="70"/>
       <c r="H29" s="65"/>
       <c r="I29" s="23"/>
-      <c r="J29" s="71"/>
-      <c r="K29" s="72"/>
+      <c r="J29" s="119"/>
+      <c r="K29" s="120"/>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="107"/>
-      <c r="B30" s="107"/>
-      <c r="C30" s="107"/>
-      <c r="D30" s="107"/>
-      <c r="E30" s="108"/>
+      <c r="A30" s="85"/>
+      <c r="B30" s="85"/>
+      <c r="C30" s="85"/>
+      <c r="D30" s="85"/>
+      <c r="E30" s="86"/>
       <c r="F30" s="49"/>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
-      <c r="J30" s="71"/>
-      <c r="K30" s="72"/>
+      <c r="J30" s="119"/>
+      <c r="K30" s="120"/>
     </row>
     <row r="31" spans="1:11" ht="15.75">
-      <c r="A31" s="137" t="s">
+      <c r="A31" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="90"/>
-      <c r="C31" s="97"/>
+      <c r="B31" s="72"/>
+      <c r="C31" s="73"/>
       <c r="D31" s="50"/>
-      <c r="E31" s="138"/>
-      <c r="F31" s="139"/>
-      <c r="G31" s="139"/>
-      <c r="H31" s="139"/>
-      <c r="I31" s="140" t="s">
+      <c r="E31" s="74"/>
+      <c r="F31" s="75"/>
+      <c r="G31" s="75"/>
+      <c r="H31" s="75"/>
+      <c r="I31" s="76" t="s">
         <v>16</v>
       </c>
-      <c r="J31" s="141"/>
-      <c r="K31" s="142"/>
+      <c r="J31" s="77"/>
+      <c r="K31" s="78"/>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" s="37"/>
@@ -2413,12 +2413,12 @@
       <c r="C32" s="4"/>
       <c r="D32" s="38"/>
       <c r="E32" s="3"/>
-      <c r="F32" s="143"/>
-      <c r="G32" s="94"/>
-      <c r="H32" s="110"/>
-      <c r="I32" s="143"/>
-      <c r="J32" s="94"/>
-      <c r="K32" s="144"/>
+      <c r="F32" s="79"/>
+      <c r="G32" s="80"/>
+      <c r="H32" s="81"/>
+      <c r="I32" s="79"/>
+      <c r="J32" s="80"/>
+      <c r="K32" s="82"/>
     </row>
     <row r="33" spans="1:11">
       <c r="A33" s="39"/>
@@ -2497,11 +2497,32 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="E31:H31"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="E1:G2"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="A5:C6"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="J6:K6"/>
     <mergeCell ref="A26:E30"/>
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="J9:K9"/>
@@ -2518,32 +2539,11 @@
     <mergeCell ref="J13:K13"/>
     <mergeCell ref="J14:K14"/>
     <mergeCell ref="J15:K15"/>
-    <mergeCell ref="A5:C6"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="E6:G6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="E1:G2"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="E31:H31"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="I32:K32"/>
   </mergeCells>
   <conditionalFormatting sqref="F12:G15 I12 F17:F22 G17:G19 G21:G22">
     <cfRule type="expression" dxfId="7" priority="1">
@@ -2595,39 +2595,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.6" customHeight="1">
-      <c r="A1" s="73" t="s">
+      <c r="A1" s="128" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="74"/>
-      <c r="C1" s="145"/>
+      <c r="B1" s="129"/>
+      <c r="C1" s="150"/>
       <c r="D1" s="58"/>
-      <c r="E1" s="147" t="s">
+      <c r="E1" s="152" t="s">
         <v>18</v>
       </c>
-      <c r="F1" s="148"/>
-      <c r="G1" s="149"/>
+      <c r="F1" s="153"/>
+      <c r="G1" s="154"/>
       <c r="H1" s="29"/>
-      <c r="I1" s="84" t="s">
+      <c r="I1" s="139" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="85"/>
-      <c r="K1" s="86"/>
+      <c r="J1" s="140"/>
+      <c r="K1" s="141"/>
     </row>
     <row r="2" spans="1:11" ht="15.75">
-      <c r="A2" s="75"/>
-      <c r="B2" s="76"/>
-      <c r="C2" s="146"/>
+      <c r="A2" s="130"/>
+      <c r="B2" s="131"/>
+      <c r="C2" s="151"/>
       <c r="D2" s="52"/>
-      <c r="E2" s="150"/>
-      <c r="F2" s="151"/>
-      <c r="G2" s="152"/>
+      <c r="E2" s="155"/>
+      <c r="F2" s="156"/>
+      <c r="G2" s="157"/>
       <c r="H2" s="15"/>
-      <c r="I2" s="87">
+      <c r="I2" s="142">
         <f ca="1">TODAY()</f>
-        <v>45864</v>
-      </c>
-      <c r="J2" s="82"/>
-      <c r="K2" s="83"/>
+        <v>45865</v>
+      </c>
+      <c r="J2" s="137"/>
+      <c r="K2" s="138"/>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="32"/>
@@ -2643,11 +2643,11 @@
       <c r="K3" s="33"/>
     </row>
     <row r="4" spans="1:11" ht="17.25">
-      <c r="A4" s="153" t="s">
+      <c r="A4" s="158" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="154"/>
-      <c r="C4" s="76"/>
+      <c r="B4" s="159"/>
+      <c r="C4" s="131"/>
       <c r="D4" s="52"/>
       <c r="E4" s="26" t="s">
         <v>19</v>
@@ -2658,46 +2658,46 @@
       <c r="I4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="91"/>
-      <c r="K4" s="92"/>
+      <c r="J4" s="144"/>
+      <c r="K4" s="115"/>
     </row>
     <row r="5" spans="1:11" ht="18.75">
-      <c r="A5" s="155" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="156"/>
-      <c r="C5" s="77"/>
+      <c r="A5" s="145" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="146"/>
+      <c r="C5" s="132"/>
       <c r="D5" s="14"/>
-      <c r="E5" s="98" t="s">
+      <c r="E5" s="122" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="99"/>
-      <c r="G5" s="100"/>
+      <c r="F5" s="123"/>
+      <c r="G5" s="124"/>
       <c r="H5" s="22"/>
       <c r="I5" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="J5" s="101"/>
-      <c r="K5" s="92"/>
+      <c r="J5" s="125"/>
+      <c r="K5" s="115"/>
     </row>
     <row r="6" spans="1:11" ht="15.75">
-      <c r="A6" s="75"/>
-      <c r="B6" s="76"/>
-      <c r="C6" s="157"/>
+      <c r="A6" s="130"/>
+      <c r="B6" s="131"/>
+      <c r="C6" s="147"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="158" t="s">
+      <c r="E6" s="148" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="76"/>
-      <c r="G6" s="159"/>
+      <c r="F6" s="131"/>
+      <c r="G6" s="149"/>
       <c r="H6" s="46"/>
       <c r="I6" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="104">
+      <c r="J6" s="127">
         <v>1230</v>
       </c>
-      <c r="K6" s="92"/>
+      <c r="K6" s="115"/>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="32"/>
@@ -2713,44 +2713,44 @@
       <c r="K7" s="33"/>
     </row>
     <row r="8" spans="1:11" ht="15.75">
-      <c r="A8" s="127" t="s">
+      <c r="A8" s="107" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="129"/>
-      <c r="D8" s="130"/>
-      <c r="E8" s="131"/>
+      <c r="C8" s="109"/>
+      <c r="D8" s="110"/>
+      <c r="E8" s="111"/>
       <c r="F8" s="14"/>
-      <c r="G8" s="132" t="s">
+      <c r="G8" s="112" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="89"/>
+      <c r="H8" s="113"/>
       <c r="I8" s="14"/>
-      <c r="J8" s="133" t="s">
+      <c r="J8" s="114" t="s">
         <v>11</v>
       </c>
-      <c r="K8" s="92"/>
+      <c r="K8" s="115"/>
     </row>
     <row r="9" spans="1:11" ht="17.25">
-      <c r="A9" s="128"/>
+      <c r="A9" s="108"/>
       <c r="B9" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="134" t="s">
+      <c r="C9" s="116" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="90"/>
-      <c r="E9" s="110"/>
+      <c r="D9" s="72"/>
+      <c r="E9" s="81"/>
       <c r="F9" s="22"/>
-      <c r="G9" s="109">
+      <c r="G9" s="87">
         <v>1</v>
       </c>
-      <c r="H9" s="110"/>
+      <c r="H9" s="81"/>
       <c r="I9" s="22"/>
-      <c r="J9" s="111"/>
-      <c r="K9" s="103"/>
+      <c r="J9" s="88"/>
+      <c r="K9" s="89"/>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="32"/>
@@ -2766,128 +2766,128 @@
       <c r="K10" s="34"/>
     </row>
     <row r="11" spans="1:11" ht="18.75">
-      <c r="A11" s="112" t="s">
+      <c r="A11" s="90" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="113"/>
-      <c r="C11" s="113"/>
-      <c r="D11" s="113"/>
-      <c r="E11" s="114"/>
-      <c r="F11" s="115"/>
-      <c r="G11" s="113"/>
-      <c r="H11" s="113"/>
-      <c r="I11" s="113"/>
-      <c r="J11" s="113"/>
-      <c r="K11" s="116"/>
+      <c r="B11" s="91"/>
+      <c r="C11" s="91"/>
+      <c r="D11" s="91"/>
+      <c r="E11" s="92"/>
+      <c r="F11" s="93"/>
+      <c r="G11" s="91"/>
+      <c r="H11" s="91"/>
+      <c r="I11" s="91"/>
+      <c r="J11" s="91"/>
+      <c r="K11" s="94"/>
     </row>
     <row r="12" spans="1:11" ht="12.6" customHeight="1">
-      <c r="A12" s="117" t="s">
-        <v>21</v>
-      </c>
-      <c r="B12" s="95"/>
-      <c r="C12" s="95"/>
-      <c r="D12" s="95"/>
-      <c r="E12" s="110"/>
+      <c r="A12" s="95" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="96"/>
+      <c r="C12" s="96"/>
+      <c r="D12" s="96"/>
+      <c r="E12" s="81"/>
       <c r="F12" s="59"/>
       <c r="G12" s="31"/>
       <c r="H12" s="60"/>
       <c r="I12" s="31"/>
-      <c r="J12" s="135"/>
-      <c r="K12" s="136"/>
+      <c r="J12" s="117"/>
+      <c r="K12" s="118"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="96"/>
-      <c r="B13" s="90"/>
-      <c r="C13" s="90"/>
-      <c r="D13" s="90"/>
-      <c r="E13" s="97"/>
+      <c r="A13" s="97"/>
+      <c r="B13" s="72"/>
+      <c r="C13" s="72"/>
+      <c r="D13" s="72"/>
+      <c r="E13" s="73"/>
       <c r="F13" s="27"/>
       <c r="G13" s="61"/>
       <c r="H13" s="62"/>
       <c r="I13" s="2"/>
-      <c r="J13" s="135"/>
-      <c r="K13" s="136"/>
+      <c r="J13" s="117"/>
+      <c r="K13" s="118"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="118" t="str">
+      <c r="A14" s="98" t="str">
         <f>"*"&amp;A12&amp;"*"</f>
-        <v>*GOFEMM20052025002*</v>
-      </c>
-      <c r="B14" s="119"/>
-      <c r="C14" s="119"/>
-      <c r="D14" s="119"/>
-      <c r="E14" s="120"/>
+        <v>*GTGEMM20052025002*</v>
+      </c>
+      <c r="B14" s="99"/>
+      <c r="C14" s="99"/>
+      <c r="D14" s="99"/>
+      <c r="E14" s="100"/>
       <c r="F14" s="27"/>
       <c r="G14" s="62"/>
       <c r="H14" s="62"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="135"/>
-      <c r="K14" s="136"/>
+      <c r="J14" s="117"/>
+      <c r="K14" s="118"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="121"/>
-      <c r="B15" s="122"/>
-      <c r="C15" s="122"/>
-      <c r="D15" s="122"/>
-      <c r="E15" s="123"/>
+      <c r="A15" s="101"/>
+      <c r="B15" s="102"/>
+      <c r="C15" s="102"/>
+      <c r="D15" s="102"/>
+      <c r="E15" s="103"/>
       <c r="F15" s="27"/>
       <c r="G15" s="62"/>
       <c r="H15" s="62"/>
       <c r="I15" s="2"/>
-      <c r="J15" s="135"/>
-      <c r="K15" s="136"/>
+      <c r="J15" s="117"/>
+      <c r="K15" s="118"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="121"/>
-      <c r="B16" s="122"/>
-      <c r="C16" s="122"/>
-      <c r="D16" s="122"/>
-      <c r="E16" s="123"/>
+      <c r="A16" s="101"/>
+      <c r="B16" s="102"/>
+      <c r="C16" s="102"/>
+      <c r="D16" s="102"/>
+      <c r="E16" s="103"/>
       <c r="F16" s="8"/>
       <c r="G16" s="62"/>
       <c r="H16" s="62"/>
       <c r="I16" s="2"/>
-      <c r="J16" s="135"/>
-      <c r="K16" s="136"/>
+      <c r="J16" s="117"/>
+      <c r="K16" s="118"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="121"/>
-      <c r="B17" s="122"/>
-      <c r="C17" s="122"/>
-      <c r="D17" s="122"/>
-      <c r="E17" s="123"/>
+      <c r="A17" s="101"/>
+      <c r="B17" s="102"/>
+      <c r="C17" s="102"/>
+      <c r="D17" s="102"/>
+      <c r="E17" s="103"/>
       <c r="F17" s="27"/>
       <c r="G17" s="62"/>
       <c r="H17" s="62"/>
       <c r="I17" s="2"/>
-      <c r="J17" s="135"/>
-      <c r="K17" s="136"/>
+      <c r="J17" s="117"/>
+      <c r="K17" s="118"/>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="121"/>
-      <c r="B18" s="122"/>
-      <c r="C18" s="122"/>
-      <c r="D18" s="122"/>
-      <c r="E18" s="123"/>
+      <c r="A18" s="101"/>
+      <c r="B18" s="102"/>
+      <c r="C18" s="102"/>
+      <c r="D18" s="102"/>
+      <c r="E18" s="103"/>
       <c r="F18" s="27"/>
       <c r="G18" s="62"/>
       <c r="H18" s="62"/>
       <c r="I18" s="8"/>
-      <c r="J18" s="135"/>
-      <c r="K18" s="136"/>
+      <c r="J18" s="117"/>
+      <c r="K18" s="118"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="124"/>
-      <c r="B19" s="125"/>
-      <c r="C19" s="125"/>
-      <c r="D19" s="125"/>
-      <c r="E19" s="126"/>
+      <c r="A19" s="104"/>
+      <c r="B19" s="105"/>
+      <c r="C19" s="105"/>
+      <c r="D19" s="105"/>
+      <c r="E19" s="106"/>
       <c r="F19" s="63"/>
       <c r="G19" s="62"/>
       <c r="H19" s="62"/>
       <c r="I19" s="27"/>
-      <c r="J19" s="135"/>
-      <c r="K19" s="136"/>
+      <c r="J19" s="117"/>
+      <c r="K19" s="118"/>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="32"/>
@@ -2899,8 +2899,8 @@
       <c r="G20" s="64"/>
       <c r="H20" s="62"/>
       <c r="I20" s="27"/>
-      <c r="J20" s="135"/>
-      <c r="K20" s="136"/>
+      <c r="J20" s="117"/>
+      <c r="K20" s="118"/>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="32"/>
@@ -2912,8 +2912,8 @@
       <c r="G21" s="62"/>
       <c r="H21" s="62"/>
       <c r="I21" s="27"/>
-      <c r="J21" s="135"/>
-      <c r="K21" s="136"/>
+      <c r="J21" s="117"/>
+      <c r="K21" s="118"/>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="32"/>
@@ -2925,8 +2925,8 @@
       <c r="G22" s="62"/>
       <c r="H22" s="62"/>
       <c r="I22" s="27"/>
-      <c r="J22" s="135"/>
-      <c r="K22" s="136"/>
+      <c r="J22" s="117"/>
+      <c r="K22" s="118"/>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="32"/>
@@ -2938,8 +2938,8 @@
       <c r="G23" s="27"/>
       <c r="H23" s="27"/>
       <c r="I23" s="27"/>
-      <c r="J23" s="135"/>
-      <c r="K23" s="136"/>
+      <c r="J23" s="117"/>
+      <c r="K23" s="118"/>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" s="32"/>
@@ -2951,8 +2951,8 @@
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
-      <c r="J24" s="135"/>
-      <c r="K24" s="136"/>
+      <c r="J24" s="117"/>
+      <c r="K24" s="118"/>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="32"/>
@@ -2964,90 +2964,90 @@
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
       <c r="I25" s="9"/>
-      <c r="J25" s="135"/>
-      <c r="K25" s="136"/>
+      <c r="J25" s="117"/>
+      <c r="K25" s="118"/>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="105"/>
-      <c r="B26" s="94"/>
-      <c r="C26" s="94"/>
-      <c r="D26" s="94"/>
-      <c r="E26" s="106"/>
+      <c r="A26" s="83"/>
+      <c r="B26" s="80"/>
+      <c r="C26" s="80"/>
+      <c r="D26" s="80"/>
+      <c r="E26" s="84"/>
       <c r="F26" s="66"/>
       <c r="G26" s="67"/>
       <c r="H26" s="8"/>
       <c r="I26" s="9"/>
-      <c r="J26" s="135"/>
-      <c r="K26" s="136"/>
+      <c r="J26" s="117"/>
+      <c r="K26" s="118"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="94"/>
-      <c r="B27" s="94"/>
-      <c r="C27" s="94"/>
-      <c r="D27" s="94"/>
-      <c r="E27" s="106"/>
+      <c r="A27" s="80"/>
+      <c r="B27" s="80"/>
+      <c r="C27" s="80"/>
+      <c r="D27" s="80"/>
+      <c r="E27" s="84"/>
       <c r="F27" s="68"/>
       <c r="G27" s="67"/>
       <c r="H27" s="8"/>
       <c r="I27" s="9"/>
-      <c r="J27" s="135"/>
-      <c r="K27" s="136"/>
+      <c r="J27" s="117"/>
+      <c r="K27" s="118"/>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="94"/>
-      <c r="B28" s="94"/>
-      <c r="C28" s="94"/>
-      <c r="D28" s="94"/>
-      <c r="E28" s="106"/>
+      <c r="A28" s="80"/>
+      <c r="B28" s="80"/>
+      <c r="C28" s="80"/>
+      <c r="D28" s="80"/>
+      <c r="E28" s="84"/>
       <c r="F28" s="68"/>
       <c r="G28" s="67"/>
       <c r="H28" s="8"/>
       <c r="I28" s="9"/>
-      <c r="J28" s="135"/>
-      <c r="K28" s="136"/>
+      <c r="J28" s="117"/>
+      <c r="K28" s="118"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="94"/>
-      <c r="B29" s="94"/>
-      <c r="C29" s="94"/>
-      <c r="D29" s="94"/>
-      <c r="E29" s="106"/>
+      <c r="A29" s="80"/>
+      <c r="B29" s="80"/>
+      <c r="C29" s="80"/>
+      <c r="D29" s="80"/>
+      <c r="E29" s="84"/>
       <c r="F29" s="69"/>
       <c r="G29" s="70"/>
       <c r="H29" s="65"/>
       <c r="I29" s="23"/>
-      <c r="J29" s="135"/>
-      <c r="K29" s="136"/>
+      <c r="J29" s="117"/>
+      <c r="K29" s="118"/>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="107"/>
-      <c r="B30" s="107"/>
-      <c r="C30" s="107"/>
-      <c r="D30" s="107"/>
-      <c r="E30" s="108"/>
+      <c r="A30" s="85"/>
+      <c r="B30" s="85"/>
+      <c r="C30" s="85"/>
+      <c r="D30" s="85"/>
+      <c r="E30" s="86"/>
       <c r="F30" s="49"/>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
-      <c r="J30" s="135"/>
-      <c r="K30" s="136"/>
+      <c r="J30" s="117"/>
+      <c r="K30" s="118"/>
     </row>
     <row r="31" spans="1:11" ht="15.75">
-      <c r="A31" s="137" t="s">
+      <c r="A31" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="90"/>
-      <c r="C31" s="97"/>
+      <c r="B31" s="72"/>
+      <c r="C31" s="73"/>
       <c r="D31" s="50"/>
-      <c r="E31" s="138"/>
-      <c r="F31" s="139"/>
-      <c r="G31" s="139"/>
-      <c r="H31" s="139"/>
-      <c r="I31" s="140" t="s">
+      <c r="E31" s="74"/>
+      <c r="F31" s="75"/>
+      <c r="G31" s="75"/>
+      <c r="H31" s="75"/>
+      <c r="I31" s="76" t="s">
         <v>16</v>
       </c>
-      <c r="J31" s="141"/>
-      <c r="K31" s="142"/>
+      <c r="J31" s="77"/>
+      <c r="K31" s="78"/>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" s="37"/>
@@ -3055,12 +3055,12 @@
       <c r="C32" s="4"/>
       <c r="D32" s="38"/>
       <c r="E32" s="3"/>
-      <c r="F32" s="143"/>
-      <c r="G32" s="94"/>
-      <c r="H32" s="110"/>
-      <c r="I32" s="143"/>
-      <c r="J32" s="94"/>
-      <c r="K32" s="144"/>
+      <c r="F32" s="79"/>
+      <c r="G32" s="80"/>
+      <c r="H32" s="81"/>
+      <c r="I32" s="79"/>
+      <c r="J32" s="80"/>
+      <c r="K32" s="82"/>
     </row>
     <row r="33" spans="1:11">
       <c r="A33" s="39"/>
@@ -3139,16 +3139,27 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="A26:E30"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="E31:H31"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="E1:G2"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="J4:K4"/>
     <mergeCell ref="A14:E19"/>
     <mergeCell ref="A5:C6"/>
     <mergeCell ref="E5:G5"/>
@@ -3165,27 +3176,16 @@
     <mergeCell ref="A11:E11"/>
     <mergeCell ref="F11:K11"/>
     <mergeCell ref="A12:E13"/>
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="E1:G2"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="A26:E30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="E31:H31"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J30:K30"/>
   </mergeCells>
   <conditionalFormatting sqref="F12:G15 I12 F17:F22 G17:G19 G21:G22">
     <cfRule type="expression" dxfId="3" priority="1">

</xml_diff>

<commit_message>
fix: add all changes to fes
</commit_message>
<xml_diff>
--- a/dummy-content/ECHEC-RETOUR_CLIENT-CASABLANCA.xlsx
+++ b/dummy-content/ECHEC-RETOUR_CLIENT-CASABLANCA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UNK\Desktop\GoFleet-Enhancer\dummy-content\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{879B84F3-3B23-4C58-A575-ACF97916BF11}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{878AB693-0D6A-49B7-9D58-7F1BA4C62B5F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -84,13 +84,13 @@
     <t xml:space="preserve">                                                       Destination</t>
   </si>
   <si>
-    <t>GOFEMM20052025001</t>
+    <t>GO FLEET FES</t>
   </si>
   <si>
-    <t>GOFEMM20052025002</t>
+    <t>GFSEMM20052025001</t>
   </si>
   <si>
-    <t>GO FLEET FES</t>
+    <t>GFSEMM20052025002</t>
   </si>
 </sst>
 </file>
@@ -1400,66 +1400,24 @@
     <xf numFmtId="0" fontId="15" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="5" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
@@ -1467,10 +1425,10 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="11" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1483,6 +1441,8 @@
     <xf numFmtId="0" fontId="21" fillId="12" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="24" fillId="3" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1506,9 +1466,11 @@
     <xf numFmtId="0" fontId="8" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1518,20 +1480,67 @@
     <xf numFmtId="0" fontId="15" fillId="15" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="5" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="19" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="17" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1546,15 +1555,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="20" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="19" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1955,37 +1955,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.6" customHeight="1">
-      <c r="A1" s="73"/>
-      <c r="B1" s="74"/>
-      <c r="C1" s="74"/>
+      <c r="A1" s="128"/>
+      <c r="B1" s="129"/>
+      <c r="C1" s="129"/>
       <c r="D1" s="53"/>
-      <c r="E1" s="78" t="s">
+      <c r="E1" s="133" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="79"/>
-      <c r="G1" s="80"/>
+      <c r="F1" s="134"/>
+      <c r="G1" s="135"/>
       <c r="H1" s="29"/>
-      <c r="I1" s="84" t="s">
+      <c r="I1" s="139" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="85"/>
-      <c r="K1" s="86"/>
+      <c r="J1" s="140"/>
+      <c r="K1" s="141"/>
     </row>
     <row r="2" spans="1:11" ht="15.75">
-      <c r="A2" s="75"/>
-      <c r="B2" s="76"/>
-      <c r="C2" s="77"/>
+      <c r="A2" s="130"/>
+      <c r="B2" s="131"/>
+      <c r="C2" s="132"/>
       <c r="D2" s="53"/>
-      <c r="E2" s="81"/>
-      <c r="F2" s="82"/>
-      <c r="G2" s="83"/>
+      <c r="E2" s="136"/>
+      <c r="F2" s="137"/>
+      <c r="G2" s="138"/>
       <c r="H2" s="15"/>
-      <c r="I2" s="87">
+      <c r="I2" s="142">
         <f ca="1">TODAY()</f>
-        <v>45864</v>
-      </c>
-      <c r="J2" s="82"/>
-      <c r="K2" s="83"/>
+        <v>45865</v>
+      </c>
+      <c r="J2" s="137"/>
+      <c r="K2" s="138"/>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="32"/>
@@ -2001,11 +2001,11 @@
       <c r="K3" s="33"/>
     </row>
     <row r="4" spans="1:11" ht="17.25">
-      <c r="A4" s="88" t="s">
+      <c r="A4" s="143" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="89"/>
-      <c r="C4" s="90"/>
+      <c r="B4" s="113"/>
+      <c r="C4" s="72"/>
       <c r="D4" s="52"/>
       <c r="E4" s="16" t="s">
         <v>19</v>
@@ -2016,46 +2016,46 @@
       <c r="I4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="91"/>
-      <c r="K4" s="92"/>
+      <c r="J4" s="144"/>
+      <c r="K4" s="115"/>
     </row>
     <row r="5" spans="1:11" ht="18.75">
-      <c r="A5" s="93" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="94"/>
-      <c r="C5" s="95"/>
+      <c r="A5" s="121" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="80"/>
+      <c r="C5" s="96"/>
       <c r="D5" s="14"/>
-      <c r="E5" s="98" t="s">
+      <c r="E5" s="122" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="99"/>
-      <c r="G5" s="100"/>
+      <c r="F5" s="123"/>
+      <c r="G5" s="124"/>
       <c r="H5" s="22"/>
       <c r="I5" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="J5" s="101"/>
-      <c r="K5" s="92"/>
+      <c r="J5" s="125"/>
+      <c r="K5" s="115"/>
     </row>
     <row r="6" spans="1:11" ht="15.75">
-      <c r="A6" s="96"/>
-      <c r="B6" s="90"/>
-      <c r="C6" s="97"/>
+      <c r="A6" s="97"/>
+      <c r="B6" s="72"/>
+      <c r="C6" s="73"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="102" t="s">
+      <c r="E6" s="126" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="90"/>
-      <c r="G6" s="103"/>
+      <c r="F6" s="72"/>
+      <c r="G6" s="89"/>
       <c r="H6" s="46"/>
       <c r="I6" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="104">
+      <c r="J6" s="127">
         <v>1230</v>
       </c>
-      <c r="K6" s="92"/>
+      <c r="K6" s="115"/>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="32"/>
@@ -2071,44 +2071,44 @@
       <c r="K7" s="33"/>
     </row>
     <row r="8" spans="1:11" ht="15.75">
-      <c r="A8" s="127" t="s">
+      <c r="A8" s="107" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="129"/>
-      <c r="D8" s="130"/>
-      <c r="E8" s="131"/>
+      <c r="C8" s="109"/>
+      <c r="D8" s="110"/>
+      <c r="E8" s="111"/>
       <c r="F8" s="14"/>
-      <c r="G8" s="132" t="s">
+      <c r="G8" s="112" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="89"/>
+      <c r="H8" s="113"/>
       <c r="I8" s="14"/>
-      <c r="J8" s="133" t="s">
+      <c r="J8" s="114" t="s">
         <v>11</v>
       </c>
-      <c r="K8" s="92"/>
+      <c r="K8" s="115"/>
     </row>
     <row r="9" spans="1:11" ht="17.25">
-      <c r="A9" s="128"/>
+      <c r="A9" s="108"/>
       <c r="B9" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="134" t="s">
+      <c r="C9" s="116" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="90"/>
-      <c r="E9" s="110"/>
+      <c r="D9" s="72"/>
+      <c r="E9" s="81"/>
       <c r="F9" s="22"/>
-      <c r="G9" s="109">
+      <c r="G9" s="87">
         <v>1</v>
       </c>
-      <c r="H9" s="110"/>
+      <c r="H9" s="81"/>
       <c r="I9" s="22"/>
-      <c r="J9" s="111"/>
-      <c r="K9" s="103"/>
+      <c r="J9" s="88"/>
+      <c r="K9" s="89"/>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="32"/>
@@ -2124,128 +2124,128 @@
       <c r="K10" s="34"/>
     </row>
     <row r="11" spans="1:11" ht="18.75">
-      <c r="A11" s="112" t="s">
+      <c r="A11" s="90" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="113"/>
-      <c r="C11" s="113"/>
-      <c r="D11" s="113"/>
-      <c r="E11" s="114"/>
-      <c r="F11" s="115"/>
-      <c r="G11" s="113"/>
-      <c r="H11" s="113"/>
-      <c r="I11" s="113"/>
-      <c r="J11" s="113"/>
-      <c r="K11" s="116"/>
+      <c r="B11" s="91"/>
+      <c r="C11" s="91"/>
+      <c r="D11" s="91"/>
+      <c r="E11" s="92"/>
+      <c r="F11" s="93"/>
+      <c r="G11" s="91"/>
+      <c r="H11" s="91"/>
+      <c r="I11" s="91"/>
+      <c r="J11" s="91"/>
+      <c r="K11" s="94"/>
     </row>
     <row r="12" spans="1:11">
-      <c r="A12" s="117" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" s="95"/>
-      <c r="C12" s="95"/>
-      <c r="D12" s="95"/>
-      <c r="E12" s="110"/>
+      <c r="A12" s="95" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="96"/>
+      <c r="C12" s="96"/>
+      <c r="D12" s="96"/>
+      <c r="E12" s="81"/>
       <c r="F12" s="59"/>
       <c r="G12" s="31"/>
       <c r="H12" s="60"/>
       <c r="I12" s="31"/>
-      <c r="J12" s="135"/>
-      <c r="K12" s="136"/>
+      <c r="J12" s="117"/>
+      <c r="K12" s="118"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="96"/>
-      <c r="B13" s="90"/>
-      <c r="C13" s="90"/>
-      <c r="D13" s="90"/>
-      <c r="E13" s="97"/>
+      <c r="A13" s="97"/>
+      <c r="B13" s="72"/>
+      <c r="C13" s="72"/>
+      <c r="D13" s="72"/>
+      <c r="E13" s="73"/>
       <c r="F13" s="27"/>
       <c r="G13" s="61"/>
       <c r="H13" s="62"/>
       <c r="I13" s="2"/>
-      <c r="J13" s="71"/>
-      <c r="K13" s="72"/>
+      <c r="J13" s="119"/>
+      <c r="K13" s="120"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="118" t="str">
+      <c r="A14" s="98" t="str">
         <f>"*"&amp;A12&amp;"*"</f>
-        <v>*GOFEMM20052025001*</v>
-      </c>
-      <c r="B14" s="119"/>
-      <c r="C14" s="119"/>
-      <c r="D14" s="119"/>
-      <c r="E14" s="120"/>
+        <v>*GFSEMM20052025001*</v>
+      </c>
+      <c r="B14" s="99"/>
+      <c r="C14" s="99"/>
+      <c r="D14" s="99"/>
+      <c r="E14" s="100"/>
       <c r="F14" s="27"/>
       <c r="G14" s="62"/>
       <c r="H14" s="62"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="71"/>
-      <c r="K14" s="72"/>
+      <c r="J14" s="119"/>
+      <c r="K14" s="120"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="121"/>
-      <c r="B15" s="122"/>
-      <c r="C15" s="122"/>
-      <c r="D15" s="122"/>
-      <c r="E15" s="123"/>
+      <c r="A15" s="101"/>
+      <c r="B15" s="102"/>
+      <c r="C15" s="102"/>
+      <c r="D15" s="102"/>
+      <c r="E15" s="103"/>
       <c r="F15" s="27"/>
       <c r="G15" s="62"/>
       <c r="H15" s="62"/>
       <c r="I15" s="2"/>
-      <c r="J15" s="71"/>
-      <c r="K15" s="72"/>
+      <c r="J15" s="119"/>
+      <c r="K15" s="120"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="121"/>
-      <c r="B16" s="122"/>
-      <c r="C16" s="122"/>
-      <c r="D16" s="122"/>
-      <c r="E16" s="123"/>
+      <c r="A16" s="101"/>
+      <c r="B16" s="102"/>
+      <c r="C16" s="102"/>
+      <c r="D16" s="102"/>
+      <c r="E16" s="103"/>
       <c r="F16" s="8"/>
       <c r="G16" s="62"/>
       <c r="H16" s="62"/>
       <c r="I16" s="2"/>
-      <c r="J16" s="71"/>
-      <c r="K16" s="72"/>
+      <c r="J16" s="119"/>
+      <c r="K16" s="120"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="121"/>
-      <c r="B17" s="122"/>
-      <c r="C17" s="122"/>
-      <c r="D17" s="122"/>
-      <c r="E17" s="123"/>
+      <c r="A17" s="101"/>
+      <c r="B17" s="102"/>
+      <c r="C17" s="102"/>
+      <c r="D17" s="102"/>
+      <c r="E17" s="103"/>
       <c r="F17" s="27"/>
       <c r="G17" s="62"/>
       <c r="H17" s="62"/>
       <c r="I17" s="2"/>
-      <c r="J17" s="71"/>
-      <c r="K17" s="72"/>
+      <c r="J17" s="119"/>
+      <c r="K17" s="120"/>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="121"/>
-      <c r="B18" s="122"/>
-      <c r="C18" s="122"/>
-      <c r="D18" s="122"/>
-      <c r="E18" s="123"/>
+      <c r="A18" s="101"/>
+      <c r="B18" s="102"/>
+      <c r="C18" s="102"/>
+      <c r="D18" s="102"/>
+      <c r="E18" s="103"/>
       <c r="F18" s="27"/>
       <c r="G18" s="62"/>
       <c r="H18" s="62"/>
       <c r="I18" s="8"/>
-      <c r="J18" s="71"/>
-      <c r="K18" s="72"/>
+      <c r="J18" s="119"/>
+      <c r="K18" s="120"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="124"/>
-      <c r="B19" s="125"/>
-      <c r="C19" s="125"/>
-      <c r="D19" s="125"/>
-      <c r="E19" s="126"/>
+      <c r="A19" s="104"/>
+      <c r="B19" s="105"/>
+      <c r="C19" s="105"/>
+      <c r="D19" s="105"/>
+      <c r="E19" s="106"/>
       <c r="F19" s="63"/>
       <c r="G19" s="62"/>
       <c r="H19" s="62"/>
       <c r="I19" s="27"/>
-      <c r="J19" s="71"/>
-      <c r="K19" s="72"/>
+      <c r="J19" s="119"/>
+      <c r="K19" s="120"/>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="32"/>
@@ -2257,8 +2257,8 @@
       <c r="G20" s="64"/>
       <c r="H20" s="62"/>
       <c r="I20" s="27"/>
-      <c r="J20" s="71"/>
-      <c r="K20" s="72"/>
+      <c r="J20" s="119"/>
+      <c r="K20" s="120"/>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="32"/>
@@ -2270,8 +2270,8 @@
       <c r="G21" s="62"/>
       <c r="H21" s="62"/>
       <c r="I21" s="27"/>
-      <c r="J21" s="71"/>
-      <c r="K21" s="72"/>
+      <c r="J21" s="119"/>
+      <c r="K21" s="120"/>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="32"/>
@@ -2283,8 +2283,8 @@
       <c r="G22" s="62"/>
       <c r="H22" s="62"/>
       <c r="I22" s="27"/>
-      <c r="J22" s="71"/>
-      <c r="K22" s="72"/>
+      <c r="J22" s="119"/>
+      <c r="K22" s="120"/>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="32"/>
@@ -2296,8 +2296,8 @@
       <c r="G23" s="27"/>
       <c r="H23" s="27"/>
       <c r="I23" s="27"/>
-      <c r="J23" s="71"/>
-      <c r="K23" s="72"/>
+      <c r="J23" s="119"/>
+      <c r="K23" s="120"/>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" s="32"/>
@@ -2309,8 +2309,8 @@
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
-      <c r="J24" s="71"/>
-      <c r="K24" s="72"/>
+      <c r="J24" s="119"/>
+      <c r="K24" s="120"/>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="32"/>
@@ -2322,90 +2322,90 @@
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
       <c r="I25" s="9"/>
-      <c r="J25" s="71"/>
-      <c r="K25" s="72"/>
+      <c r="J25" s="119"/>
+      <c r="K25" s="120"/>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="105"/>
-      <c r="B26" s="94"/>
-      <c r="C26" s="94"/>
-      <c r="D26" s="94"/>
-      <c r="E26" s="106"/>
+      <c r="A26" s="83"/>
+      <c r="B26" s="80"/>
+      <c r="C26" s="80"/>
+      <c r="D26" s="80"/>
+      <c r="E26" s="84"/>
       <c r="F26" s="66"/>
       <c r="G26" s="67"/>
       <c r="H26" s="8"/>
       <c r="I26" s="9"/>
-      <c r="J26" s="71"/>
-      <c r="K26" s="72"/>
+      <c r="J26" s="119"/>
+      <c r="K26" s="120"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="94"/>
-      <c r="B27" s="94"/>
-      <c r="C27" s="94"/>
-      <c r="D27" s="94"/>
-      <c r="E27" s="106"/>
+      <c r="A27" s="80"/>
+      <c r="B27" s="80"/>
+      <c r="C27" s="80"/>
+      <c r="D27" s="80"/>
+      <c r="E27" s="84"/>
       <c r="F27" s="68"/>
       <c r="G27" s="67"/>
       <c r="H27" s="8"/>
       <c r="I27" s="9"/>
-      <c r="J27" s="71"/>
-      <c r="K27" s="72"/>
+      <c r="J27" s="119"/>
+      <c r="K27" s="120"/>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="94"/>
-      <c r="B28" s="94"/>
-      <c r="C28" s="94"/>
-      <c r="D28" s="94"/>
-      <c r="E28" s="106"/>
+      <c r="A28" s="80"/>
+      <c r="B28" s="80"/>
+      <c r="C28" s="80"/>
+      <c r="D28" s="80"/>
+      <c r="E28" s="84"/>
       <c r="F28" s="68"/>
       <c r="G28" s="67"/>
       <c r="H28" s="8"/>
       <c r="I28" s="9"/>
-      <c r="J28" s="71"/>
-      <c r="K28" s="72"/>
+      <c r="J28" s="119"/>
+      <c r="K28" s="120"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="94"/>
-      <c r="B29" s="94"/>
-      <c r="C29" s="94"/>
-      <c r="D29" s="94"/>
-      <c r="E29" s="106"/>
+      <c r="A29" s="80"/>
+      <c r="B29" s="80"/>
+      <c r="C29" s="80"/>
+      <c r="D29" s="80"/>
+      <c r="E29" s="84"/>
       <c r="F29" s="69"/>
       <c r="G29" s="70"/>
       <c r="H29" s="65"/>
       <c r="I29" s="23"/>
-      <c r="J29" s="71"/>
-      <c r="K29" s="72"/>
+      <c r="J29" s="119"/>
+      <c r="K29" s="120"/>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="107"/>
-      <c r="B30" s="107"/>
-      <c r="C30" s="107"/>
-      <c r="D30" s="107"/>
-      <c r="E30" s="108"/>
+      <c r="A30" s="85"/>
+      <c r="B30" s="85"/>
+      <c r="C30" s="85"/>
+      <c r="D30" s="85"/>
+      <c r="E30" s="86"/>
       <c r="F30" s="49"/>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
-      <c r="J30" s="71"/>
-      <c r="K30" s="72"/>
+      <c r="J30" s="119"/>
+      <c r="K30" s="120"/>
     </row>
     <row r="31" spans="1:11" ht="15.75">
-      <c r="A31" s="137" t="s">
+      <c r="A31" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="90"/>
-      <c r="C31" s="97"/>
+      <c r="B31" s="72"/>
+      <c r="C31" s="73"/>
       <c r="D31" s="50"/>
-      <c r="E31" s="138"/>
-      <c r="F31" s="139"/>
-      <c r="G31" s="139"/>
-      <c r="H31" s="139"/>
-      <c r="I31" s="140" t="s">
+      <c r="E31" s="74"/>
+      <c r="F31" s="75"/>
+      <c r="G31" s="75"/>
+      <c r="H31" s="75"/>
+      <c r="I31" s="76" t="s">
         <v>16</v>
       </c>
-      <c r="J31" s="141"/>
-      <c r="K31" s="142"/>
+      <c r="J31" s="77"/>
+      <c r="K31" s="78"/>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" s="37"/>
@@ -2413,12 +2413,12 @@
       <c r="C32" s="4"/>
       <c r="D32" s="38"/>
       <c r="E32" s="3"/>
-      <c r="F32" s="143"/>
-      <c r="G32" s="94"/>
-      <c r="H32" s="110"/>
-      <c r="I32" s="143"/>
-      <c r="J32" s="94"/>
-      <c r="K32" s="144"/>
+      <c r="F32" s="79"/>
+      <c r="G32" s="80"/>
+      <c r="H32" s="81"/>
+      <c r="I32" s="79"/>
+      <c r="J32" s="80"/>
+      <c r="K32" s="82"/>
     </row>
     <row r="33" spans="1:11">
       <c r="A33" s="39"/>
@@ -2497,11 +2497,32 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="E31:H31"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="E1:G2"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="A5:C6"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="J6:K6"/>
     <mergeCell ref="A26:E30"/>
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="J9:K9"/>
@@ -2518,32 +2539,11 @@
     <mergeCell ref="J13:K13"/>
     <mergeCell ref="J14:K14"/>
     <mergeCell ref="J15:K15"/>
-    <mergeCell ref="A5:C6"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="E6:G6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="E1:G2"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="E31:H31"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="I32:K32"/>
   </mergeCells>
   <conditionalFormatting sqref="F12:G15 I12 F17:F22 G17:G19 G21:G22">
     <cfRule type="expression" dxfId="7" priority="1">
@@ -2595,39 +2595,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.6" customHeight="1">
-      <c r="A1" s="73" t="s">
+      <c r="A1" s="128" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="74"/>
-      <c r="C1" s="145"/>
+      <c r="B1" s="129"/>
+      <c r="C1" s="150"/>
       <c r="D1" s="58"/>
-      <c r="E1" s="147" t="s">
+      <c r="E1" s="152" t="s">
         <v>18</v>
       </c>
-      <c r="F1" s="148"/>
-      <c r="G1" s="149"/>
+      <c r="F1" s="153"/>
+      <c r="G1" s="154"/>
       <c r="H1" s="29"/>
-      <c r="I1" s="84" t="s">
+      <c r="I1" s="139" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="85"/>
-      <c r="K1" s="86"/>
+      <c r="J1" s="140"/>
+      <c r="K1" s="141"/>
     </row>
     <row r="2" spans="1:11" ht="15.75">
-      <c r="A2" s="75"/>
-      <c r="B2" s="76"/>
-      <c r="C2" s="146"/>
+      <c r="A2" s="130"/>
+      <c r="B2" s="131"/>
+      <c r="C2" s="151"/>
       <c r="D2" s="52"/>
-      <c r="E2" s="150"/>
-      <c r="F2" s="151"/>
-      <c r="G2" s="152"/>
+      <c r="E2" s="155"/>
+      <c r="F2" s="156"/>
+      <c r="G2" s="157"/>
       <c r="H2" s="15"/>
-      <c r="I2" s="87">
+      <c r="I2" s="142">
         <f ca="1">TODAY()</f>
-        <v>45864</v>
-      </c>
-      <c r="J2" s="82"/>
-      <c r="K2" s="83"/>
+        <v>45865</v>
+      </c>
+      <c r="J2" s="137"/>
+      <c r="K2" s="138"/>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="32"/>
@@ -2643,11 +2643,11 @@
       <c r="K3" s="33"/>
     </row>
     <row r="4" spans="1:11" ht="17.25">
-      <c r="A4" s="153" t="s">
+      <c r="A4" s="158" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="154"/>
-      <c r="C4" s="76"/>
+      <c r="B4" s="159"/>
+      <c r="C4" s="131"/>
       <c r="D4" s="52"/>
       <c r="E4" s="26" t="s">
         <v>19</v>
@@ -2658,46 +2658,46 @@
       <c r="I4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="91"/>
-      <c r="K4" s="92"/>
+      <c r="J4" s="144"/>
+      <c r="K4" s="115"/>
     </row>
     <row r="5" spans="1:11" ht="18.75">
-      <c r="A5" s="155" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="156"/>
-      <c r="C5" s="77"/>
+      <c r="A5" s="145" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="146"/>
+      <c r="C5" s="132"/>
       <c r="D5" s="14"/>
-      <c r="E5" s="98" t="s">
+      <c r="E5" s="122" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="99"/>
-      <c r="G5" s="100"/>
+      <c r="F5" s="123"/>
+      <c r="G5" s="124"/>
       <c r="H5" s="22"/>
       <c r="I5" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="J5" s="101"/>
-      <c r="K5" s="92"/>
+      <c r="J5" s="125"/>
+      <c r="K5" s="115"/>
     </row>
     <row r="6" spans="1:11" ht="15.75">
-      <c r="A6" s="75"/>
-      <c r="B6" s="76"/>
-      <c r="C6" s="157"/>
+      <c r="A6" s="130"/>
+      <c r="B6" s="131"/>
+      <c r="C6" s="147"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="158" t="s">
+      <c r="E6" s="148" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="76"/>
-      <c r="G6" s="159"/>
+      <c r="F6" s="131"/>
+      <c r="G6" s="149"/>
       <c r="H6" s="46"/>
       <c r="I6" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="104">
+      <c r="J6" s="127">
         <v>1230</v>
       </c>
-      <c r="K6" s="92"/>
+      <c r="K6" s="115"/>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="32"/>
@@ -2713,44 +2713,44 @@
       <c r="K7" s="33"/>
     </row>
     <row r="8" spans="1:11" ht="15.75">
-      <c r="A8" s="127" t="s">
+      <c r="A8" s="107" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="129"/>
-      <c r="D8" s="130"/>
-      <c r="E8" s="131"/>
+      <c r="C8" s="109"/>
+      <c r="D8" s="110"/>
+      <c r="E8" s="111"/>
       <c r="F8" s="14"/>
-      <c r="G8" s="132" t="s">
+      <c r="G8" s="112" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="89"/>
+      <c r="H8" s="113"/>
       <c r="I8" s="14"/>
-      <c r="J8" s="133" t="s">
+      <c r="J8" s="114" t="s">
         <v>11</v>
       </c>
-      <c r="K8" s="92"/>
+      <c r="K8" s="115"/>
     </row>
     <row r="9" spans="1:11" ht="17.25">
-      <c r="A9" s="128"/>
+      <c r="A9" s="108"/>
       <c r="B9" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="134" t="s">
+      <c r="C9" s="116" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="90"/>
-      <c r="E9" s="110"/>
+      <c r="D9" s="72"/>
+      <c r="E9" s="81"/>
       <c r="F9" s="22"/>
-      <c r="G9" s="109">
+      <c r="G9" s="87">
         <v>1</v>
       </c>
-      <c r="H9" s="110"/>
+      <c r="H9" s="81"/>
       <c r="I9" s="22"/>
-      <c r="J9" s="111"/>
-      <c r="K9" s="103"/>
+      <c r="J9" s="88"/>
+      <c r="K9" s="89"/>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="32"/>
@@ -2766,128 +2766,128 @@
       <c r="K10" s="34"/>
     </row>
     <row r="11" spans="1:11" ht="18.75">
-      <c r="A11" s="112" t="s">
+      <c r="A11" s="90" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="113"/>
-      <c r="C11" s="113"/>
-      <c r="D11" s="113"/>
-      <c r="E11" s="114"/>
-      <c r="F11" s="115"/>
-      <c r="G11" s="113"/>
-      <c r="H11" s="113"/>
-      <c r="I11" s="113"/>
-      <c r="J11" s="113"/>
-      <c r="K11" s="116"/>
+      <c r="B11" s="91"/>
+      <c r="C11" s="91"/>
+      <c r="D11" s="91"/>
+      <c r="E11" s="92"/>
+      <c r="F11" s="93"/>
+      <c r="G11" s="91"/>
+      <c r="H11" s="91"/>
+      <c r="I11" s="91"/>
+      <c r="J11" s="91"/>
+      <c r="K11" s="94"/>
     </row>
     <row r="12" spans="1:11" ht="12.6" customHeight="1">
-      <c r="A12" s="117" t="s">
-        <v>21</v>
-      </c>
-      <c r="B12" s="95"/>
-      <c r="C12" s="95"/>
-      <c r="D12" s="95"/>
-      <c r="E12" s="110"/>
+      <c r="A12" s="95" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="96"/>
+      <c r="C12" s="96"/>
+      <c r="D12" s="96"/>
+      <c r="E12" s="81"/>
       <c r="F12" s="59"/>
       <c r="G12" s="31"/>
       <c r="H12" s="60"/>
       <c r="I12" s="31"/>
-      <c r="J12" s="135"/>
-      <c r="K12" s="136"/>
+      <c r="J12" s="117"/>
+      <c r="K12" s="118"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="96"/>
-      <c r="B13" s="90"/>
-      <c r="C13" s="90"/>
-      <c r="D13" s="90"/>
-      <c r="E13" s="97"/>
+      <c r="A13" s="97"/>
+      <c r="B13" s="72"/>
+      <c r="C13" s="72"/>
+      <c r="D13" s="72"/>
+      <c r="E13" s="73"/>
       <c r="F13" s="27"/>
       <c r="G13" s="61"/>
       <c r="H13" s="62"/>
       <c r="I13" s="2"/>
-      <c r="J13" s="135"/>
-      <c r="K13" s="136"/>
+      <c r="J13" s="117"/>
+      <c r="K13" s="118"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="118" t="str">
+      <c r="A14" s="98" t="str">
         <f>"*"&amp;A12&amp;"*"</f>
-        <v>*GOFEMM20052025002*</v>
-      </c>
-      <c r="B14" s="119"/>
-      <c r="C14" s="119"/>
-      <c r="D14" s="119"/>
-      <c r="E14" s="120"/>
+        <v>*GFSEMM20052025002*</v>
+      </c>
+      <c r="B14" s="99"/>
+      <c r="C14" s="99"/>
+      <c r="D14" s="99"/>
+      <c r="E14" s="100"/>
       <c r="F14" s="27"/>
       <c r="G14" s="62"/>
       <c r="H14" s="62"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="135"/>
-      <c r="K14" s="136"/>
+      <c r="J14" s="117"/>
+      <c r="K14" s="118"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="121"/>
-      <c r="B15" s="122"/>
-      <c r="C15" s="122"/>
-      <c r="D15" s="122"/>
-      <c r="E15" s="123"/>
+      <c r="A15" s="101"/>
+      <c r="B15" s="102"/>
+      <c r="C15" s="102"/>
+      <c r="D15" s="102"/>
+      <c r="E15" s="103"/>
       <c r="F15" s="27"/>
       <c r="G15" s="62"/>
       <c r="H15" s="62"/>
       <c r="I15" s="2"/>
-      <c r="J15" s="135"/>
-      <c r="K15" s="136"/>
+      <c r="J15" s="117"/>
+      <c r="K15" s="118"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="121"/>
-      <c r="B16" s="122"/>
-      <c r="C16" s="122"/>
-      <c r="D16" s="122"/>
-      <c r="E16" s="123"/>
+      <c r="A16" s="101"/>
+      <c r="B16" s="102"/>
+      <c r="C16" s="102"/>
+      <c r="D16" s="102"/>
+      <c r="E16" s="103"/>
       <c r="F16" s="8"/>
       <c r="G16" s="62"/>
       <c r="H16" s="62"/>
       <c r="I16" s="2"/>
-      <c r="J16" s="135"/>
-      <c r="K16" s="136"/>
+      <c r="J16" s="117"/>
+      <c r="K16" s="118"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="121"/>
-      <c r="B17" s="122"/>
-      <c r="C17" s="122"/>
-      <c r="D17" s="122"/>
-      <c r="E17" s="123"/>
+      <c r="A17" s="101"/>
+      <c r="B17" s="102"/>
+      <c r="C17" s="102"/>
+      <c r="D17" s="102"/>
+      <c r="E17" s="103"/>
       <c r="F17" s="27"/>
       <c r="G17" s="62"/>
       <c r="H17" s="62"/>
       <c r="I17" s="2"/>
-      <c r="J17" s="135"/>
-      <c r="K17" s="136"/>
+      <c r="J17" s="117"/>
+      <c r="K17" s="118"/>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="121"/>
-      <c r="B18" s="122"/>
-      <c r="C18" s="122"/>
-      <c r="D18" s="122"/>
-      <c r="E18" s="123"/>
+      <c r="A18" s="101"/>
+      <c r="B18" s="102"/>
+      <c r="C18" s="102"/>
+      <c r="D18" s="102"/>
+      <c r="E18" s="103"/>
       <c r="F18" s="27"/>
       <c r="G18" s="62"/>
       <c r="H18" s="62"/>
       <c r="I18" s="8"/>
-      <c r="J18" s="135"/>
-      <c r="K18" s="136"/>
+      <c r="J18" s="117"/>
+      <c r="K18" s="118"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="124"/>
-      <c r="B19" s="125"/>
-      <c r="C19" s="125"/>
-      <c r="D19" s="125"/>
-      <c r="E19" s="126"/>
+      <c r="A19" s="104"/>
+      <c r="B19" s="105"/>
+      <c r="C19" s="105"/>
+      <c r="D19" s="105"/>
+      <c r="E19" s="106"/>
       <c r="F19" s="63"/>
       <c r="G19" s="62"/>
       <c r="H19" s="62"/>
       <c r="I19" s="27"/>
-      <c r="J19" s="135"/>
-      <c r="K19" s="136"/>
+      <c r="J19" s="117"/>
+      <c r="K19" s="118"/>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="32"/>
@@ -2899,8 +2899,8 @@
       <c r="G20" s="64"/>
       <c r="H20" s="62"/>
       <c r="I20" s="27"/>
-      <c r="J20" s="135"/>
-      <c r="K20" s="136"/>
+      <c r="J20" s="117"/>
+      <c r="K20" s="118"/>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="32"/>
@@ -2912,8 +2912,8 @@
       <c r="G21" s="62"/>
       <c r="H21" s="62"/>
       <c r="I21" s="27"/>
-      <c r="J21" s="135"/>
-      <c r="K21" s="136"/>
+      <c r="J21" s="117"/>
+      <c r="K21" s="118"/>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="32"/>
@@ -2925,8 +2925,8 @@
       <c r="G22" s="62"/>
       <c r="H22" s="62"/>
       <c r="I22" s="27"/>
-      <c r="J22" s="135"/>
-      <c r="K22" s="136"/>
+      <c r="J22" s="117"/>
+      <c r="K22" s="118"/>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="32"/>
@@ -2938,8 +2938,8 @@
       <c r="G23" s="27"/>
       <c r="H23" s="27"/>
       <c r="I23" s="27"/>
-      <c r="J23" s="135"/>
-      <c r="K23" s="136"/>
+      <c r="J23" s="117"/>
+      <c r="K23" s="118"/>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" s="32"/>
@@ -2951,8 +2951,8 @@
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
-      <c r="J24" s="135"/>
-      <c r="K24" s="136"/>
+      <c r="J24" s="117"/>
+      <c r="K24" s="118"/>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="32"/>
@@ -2964,90 +2964,90 @@
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
       <c r="I25" s="9"/>
-      <c r="J25" s="135"/>
-      <c r="K25" s="136"/>
+      <c r="J25" s="117"/>
+      <c r="K25" s="118"/>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="105"/>
-      <c r="B26" s="94"/>
-      <c r="C26" s="94"/>
-      <c r="D26" s="94"/>
-      <c r="E26" s="106"/>
+      <c r="A26" s="83"/>
+      <c r="B26" s="80"/>
+      <c r="C26" s="80"/>
+      <c r="D26" s="80"/>
+      <c r="E26" s="84"/>
       <c r="F26" s="66"/>
       <c r="G26" s="67"/>
       <c r="H26" s="8"/>
       <c r="I26" s="9"/>
-      <c r="J26" s="135"/>
-      <c r="K26" s="136"/>
+      <c r="J26" s="117"/>
+      <c r="K26" s="118"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="94"/>
-      <c r="B27" s="94"/>
-      <c r="C27" s="94"/>
-      <c r="D27" s="94"/>
-      <c r="E27" s="106"/>
+      <c r="A27" s="80"/>
+      <c r="B27" s="80"/>
+      <c r="C27" s="80"/>
+      <c r="D27" s="80"/>
+      <c r="E27" s="84"/>
       <c r="F27" s="68"/>
       <c r="G27" s="67"/>
       <c r="H27" s="8"/>
       <c r="I27" s="9"/>
-      <c r="J27" s="135"/>
-      <c r="K27" s="136"/>
+      <c r="J27" s="117"/>
+      <c r="K27" s="118"/>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="94"/>
-      <c r="B28" s="94"/>
-      <c r="C28" s="94"/>
-      <c r="D28" s="94"/>
-      <c r="E28" s="106"/>
+      <c r="A28" s="80"/>
+      <c r="B28" s="80"/>
+      <c r="C28" s="80"/>
+      <c r="D28" s="80"/>
+      <c r="E28" s="84"/>
       <c r="F28" s="68"/>
       <c r="G28" s="67"/>
       <c r="H28" s="8"/>
       <c r="I28" s="9"/>
-      <c r="J28" s="135"/>
-      <c r="K28" s="136"/>
+      <c r="J28" s="117"/>
+      <c r="K28" s="118"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="94"/>
-      <c r="B29" s="94"/>
-      <c r="C29" s="94"/>
-      <c r="D29" s="94"/>
-      <c r="E29" s="106"/>
+      <c r="A29" s="80"/>
+      <c r="B29" s="80"/>
+      <c r="C29" s="80"/>
+      <c r="D29" s="80"/>
+      <c r="E29" s="84"/>
       <c r="F29" s="69"/>
       <c r="G29" s="70"/>
       <c r="H29" s="65"/>
       <c r="I29" s="23"/>
-      <c r="J29" s="135"/>
-      <c r="K29" s="136"/>
+      <c r="J29" s="117"/>
+      <c r="K29" s="118"/>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="107"/>
-      <c r="B30" s="107"/>
-      <c r="C30" s="107"/>
-      <c r="D30" s="107"/>
-      <c r="E30" s="108"/>
+      <c r="A30" s="85"/>
+      <c r="B30" s="85"/>
+      <c r="C30" s="85"/>
+      <c r="D30" s="85"/>
+      <c r="E30" s="86"/>
       <c r="F30" s="49"/>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
-      <c r="J30" s="135"/>
-      <c r="K30" s="136"/>
+      <c r="J30" s="117"/>
+      <c r="K30" s="118"/>
     </row>
     <row r="31" spans="1:11" ht="15.75">
-      <c r="A31" s="137" t="s">
+      <c r="A31" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="90"/>
-      <c r="C31" s="97"/>
+      <c r="B31" s="72"/>
+      <c r="C31" s="73"/>
       <c r="D31" s="50"/>
-      <c r="E31" s="138"/>
-      <c r="F31" s="139"/>
-      <c r="G31" s="139"/>
-      <c r="H31" s="139"/>
-      <c r="I31" s="140" t="s">
+      <c r="E31" s="74"/>
+      <c r="F31" s="75"/>
+      <c r="G31" s="75"/>
+      <c r="H31" s="75"/>
+      <c r="I31" s="76" t="s">
         <v>16</v>
       </c>
-      <c r="J31" s="141"/>
-      <c r="K31" s="142"/>
+      <c r="J31" s="77"/>
+      <c r="K31" s="78"/>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" s="37"/>
@@ -3055,12 +3055,12 @@
       <c r="C32" s="4"/>
       <c r="D32" s="38"/>
       <c r="E32" s="3"/>
-      <c r="F32" s="143"/>
-      <c r="G32" s="94"/>
-      <c r="H32" s="110"/>
-      <c r="I32" s="143"/>
-      <c r="J32" s="94"/>
-      <c r="K32" s="144"/>
+      <c r="F32" s="79"/>
+      <c r="G32" s="80"/>
+      <c r="H32" s="81"/>
+      <c r="I32" s="79"/>
+      <c r="J32" s="80"/>
+      <c r="K32" s="82"/>
     </row>
     <row r="33" spans="1:11">
       <c r="A33" s="39"/>
@@ -3139,16 +3139,27 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="A26:E30"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="E31:H31"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="E1:G2"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="J4:K4"/>
     <mergeCell ref="A14:E19"/>
     <mergeCell ref="A5:C6"/>
     <mergeCell ref="E5:G5"/>
@@ -3165,27 +3176,16 @@
     <mergeCell ref="A11:E11"/>
     <mergeCell ref="F11:K11"/>
     <mergeCell ref="A12:E13"/>
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="E1:G2"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="A26:E30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="E31:H31"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J30:K30"/>
   </mergeCells>
   <conditionalFormatting sqref="F12:G15 I12 F17:F22 G17:G19 G21:G22">
     <cfRule type="expression" dxfId="3" priority="1">

</xml_diff>

<commit_message>
add all changes for meknes+ fix refused colis export
</commit_message>
<xml_diff>
--- a/dummy-content/ECHEC-RETOUR_CLIENT-CASABLANCA.xlsx
+++ b/dummy-content/ECHEC-RETOUR_CLIENT-CASABLANCA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UNK\Desktop\GoFleet-Enhancer\dummy-content\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4EC71F9-E2CC-4694-BB7B-C5BBE004612B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E01933D3-212F-4511-868A-E0BA5F38FCF0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ECHEC CASA" sheetId="5" r:id="rId1"/>
@@ -84,13 +84,13 @@
     <t xml:space="preserve">                                                       Destination</t>
   </si>
   <si>
-    <t>GOFEMM20052025001</t>
+    <t>GO FLEET MEKNES</t>
   </si>
   <si>
-    <t>GOFEMM20052025002</t>
+    <t>GMKEMM20052025001</t>
   </si>
   <si>
-    <t>GO FLEET MEKNES</t>
+    <t>GMKEMM20052025002</t>
   </si>
 </sst>
 </file>
@@ -1400,24 +1400,66 @@
     <xf numFmtId="0" fontId="15" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="5" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
@@ -1425,10 +1467,10 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="11" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1441,8 +1483,6 @@
     <xf numFmtId="0" fontId="21" fillId="12" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="24" fillId="3" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1466,11 +1506,9 @@
     <xf numFmtId="0" fontId="8" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1480,67 +1518,20 @@
     <xf numFmtId="0" fontId="15" fillId="15" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="5" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="20" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="19" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="17" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1555,6 +1546,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="19" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1955,37 +1955,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.6" customHeight="1">
-      <c r="A1" s="128"/>
-      <c r="B1" s="129"/>
-      <c r="C1" s="129"/>
+      <c r="A1" s="73"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
       <c r="D1" s="53"/>
-      <c r="E1" s="133" t="s">
+      <c r="E1" s="78" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="134"/>
-      <c r="G1" s="135"/>
+      <c r="F1" s="79"/>
+      <c r="G1" s="80"/>
       <c r="H1" s="29"/>
-      <c r="I1" s="139" t="s">
+      <c r="I1" s="84" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="140"/>
-      <c r="K1" s="141"/>
+      <c r="J1" s="85"/>
+      <c r="K1" s="86"/>
     </row>
     <row r="2" spans="1:11" ht="15.75">
-      <c r="A2" s="130"/>
-      <c r="B2" s="131"/>
-      <c r="C2" s="132"/>
+      <c r="A2" s="75"/>
+      <c r="B2" s="76"/>
+      <c r="C2" s="77"/>
       <c r="D2" s="53"/>
-      <c r="E2" s="136"/>
-      <c r="F2" s="137"/>
-      <c r="G2" s="138"/>
+      <c r="E2" s="81"/>
+      <c r="F2" s="82"/>
+      <c r="G2" s="83"/>
       <c r="H2" s="15"/>
-      <c r="I2" s="142">
+      <c r="I2" s="87">
         <f ca="1">TODAY()</f>
-        <v>45864</v>
-      </c>
-      <c r="J2" s="137"/>
-      <c r="K2" s="138"/>
+        <v>45865</v>
+      </c>
+      <c r="J2" s="82"/>
+      <c r="K2" s="83"/>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="32"/>
@@ -2001,11 +2001,11 @@
       <c r="K3" s="33"/>
     </row>
     <row r="4" spans="1:11" ht="17.25">
-      <c r="A4" s="143" t="s">
+      <c r="A4" s="88" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="113"/>
-      <c r="C4" s="72"/>
+      <c r="B4" s="89"/>
+      <c r="C4" s="90"/>
       <c r="D4" s="52"/>
       <c r="E4" s="16" t="s">
         <v>19</v>
@@ -2016,46 +2016,46 @@
       <c r="I4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="144"/>
-      <c r="K4" s="115"/>
+      <c r="J4" s="91"/>
+      <c r="K4" s="92"/>
     </row>
     <row r="5" spans="1:11" ht="18.75">
-      <c r="A5" s="121" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="80"/>
-      <c r="C5" s="96"/>
+      <c r="A5" s="93" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="94"/>
+      <c r="C5" s="95"/>
       <c r="D5" s="14"/>
-      <c r="E5" s="122" t="s">
+      <c r="E5" s="98" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="123"/>
-      <c r="G5" s="124"/>
+      <c r="F5" s="99"/>
+      <c r="G5" s="100"/>
       <c r="H5" s="22"/>
       <c r="I5" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="J5" s="125"/>
-      <c r="K5" s="115"/>
+      <c r="J5" s="101"/>
+      <c r="K5" s="92"/>
     </row>
     <row r="6" spans="1:11" ht="15.75">
-      <c r="A6" s="97"/>
-      <c r="B6" s="72"/>
-      <c r="C6" s="73"/>
+      <c r="A6" s="96"/>
+      <c r="B6" s="90"/>
+      <c r="C6" s="97"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="126" t="s">
+      <c r="E6" s="102" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="72"/>
-      <c r="G6" s="89"/>
+      <c r="F6" s="90"/>
+      <c r="G6" s="103"/>
       <c r="H6" s="46"/>
       <c r="I6" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="127">
+      <c r="J6" s="104">
         <v>1230</v>
       </c>
-      <c r="K6" s="115"/>
+      <c r="K6" s="92"/>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="32"/>
@@ -2071,44 +2071,44 @@
       <c r="K7" s="33"/>
     </row>
     <row r="8" spans="1:11" ht="15.75">
-      <c r="A8" s="107" t="s">
+      <c r="A8" s="127" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="109"/>
-      <c r="D8" s="110"/>
-      <c r="E8" s="111"/>
+      <c r="C8" s="129"/>
+      <c r="D8" s="130"/>
+      <c r="E8" s="131"/>
       <c r="F8" s="14"/>
-      <c r="G8" s="112" t="s">
+      <c r="G8" s="132" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="113"/>
+      <c r="H8" s="89"/>
       <c r="I8" s="14"/>
-      <c r="J8" s="114" t="s">
+      <c r="J8" s="133" t="s">
         <v>11</v>
       </c>
-      <c r="K8" s="115"/>
+      <c r="K8" s="92"/>
     </row>
     <row r="9" spans="1:11" ht="17.25">
-      <c r="A9" s="108"/>
+      <c r="A9" s="128"/>
       <c r="B9" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="116" t="s">
+      <c r="C9" s="134" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="72"/>
-      <c r="E9" s="81"/>
+      <c r="D9" s="90"/>
+      <c r="E9" s="110"/>
       <c r="F9" s="22"/>
-      <c r="G9" s="87">
+      <c r="G9" s="109">
         <v>1</v>
       </c>
-      <c r="H9" s="81"/>
+      <c r="H9" s="110"/>
       <c r="I9" s="22"/>
-      <c r="J9" s="88"/>
-      <c r="K9" s="89"/>
+      <c r="J9" s="111"/>
+      <c r="K9" s="103"/>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="32"/>
@@ -2124,128 +2124,128 @@
       <c r="K10" s="34"/>
     </row>
     <row r="11" spans="1:11" ht="18.75">
-      <c r="A11" s="90" t="s">
+      <c r="A11" s="112" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="91"/>
-      <c r="C11" s="91"/>
-      <c r="D11" s="91"/>
-      <c r="E11" s="92"/>
-      <c r="F11" s="93"/>
-      <c r="G11" s="91"/>
-      <c r="H11" s="91"/>
-      <c r="I11" s="91"/>
-      <c r="J11" s="91"/>
-      <c r="K11" s="94"/>
+      <c r="B11" s="113"/>
+      <c r="C11" s="113"/>
+      <c r="D11" s="113"/>
+      <c r="E11" s="114"/>
+      <c r="F11" s="115"/>
+      <c r="G11" s="113"/>
+      <c r="H11" s="113"/>
+      <c r="I11" s="113"/>
+      <c r="J11" s="113"/>
+      <c r="K11" s="116"/>
     </row>
     <row r="12" spans="1:11">
-      <c r="A12" s="95" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" s="96"/>
-      <c r="C12" s="96"/>
-      <c r="D12" s="96"/>
-      <c r="E12" s="81"/>
+      <c r="A12" s="117" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="95"/>
+      <c r="C12" s="95"/>
+      <c r="D12" s="95"/>
+      <c r="E12" s="110"/>
       <c r="F12" s="59"/>
       <c r="G12" s="31"/>
       <c r="H12" s="60"/>
       <c r="I12" s="31"/>
-      <c r="J12" s="117"/>
-      <c r="K12" s="118"/>
+      <c r="J12" s="135"/>
+      <c r="K12" s="136"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="97"/>
-      <c r="B13" s="72"/>
-      <c r="C13" s="72"/>
-      <c r="D13" s="72"/>
-      <c r="E13" s="73"/>
+      <c r="A13" s="96"/>
+      <c r="B13" s="90"/>
+      <c r="C13" s="90"/>
+      <c r="D13" s="90"/>
+      <c r="E13" s="97"/>
       <c r="F13" s="27"/>
       <c r="G13" s="61"/>
       <c r="H13" s="62"/>
       <c r="I13" s="2"/>
-      <c r="J13" s="119"/>
-      <c r="K13" s="120"/>
+      <c r="J13" s="71"/>
+      <c r="K13" s="72"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="98" t="str">
+      <c r="A14" s="118" t="str">
         <f>"*"&amp;A12&amp;"*"</f>
-        <v>*GOFEMM20052025001*</v>
-      </c>
-      <c r="B14" s="99"/>
-      <c r="C14" s="99"/>
-      <c r="D14" s="99"/>
-      <c r="E14" s="100"/>
+        <v>*GMKEMM20052025001*</v>
+      </c>
+      <c r="B14" s="119"/>
+      <c r="C14" s="119"/>
+      <c r="D14" s="119"/>
+      <c r="E14" s="120"/>
       <c r="F14" s="27"/>
       <c r="G14" s="62"/>
       <c r="H14" s="62"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="119"/>
-      <c r="K14" s="120"/>
+      <c r="J14" s="71"/>
+      <c r="K14" s="72"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="101"/>
-      <c r="B15" s="102"/>
-      <c r="C15" s="102"/>
-      <c r="D15" s="102"/>
-      <c r="E15" s="103"/>
+      <c r="A15" s="121"/>
+      <c r="B15" s="122"/>
+      <c r="C15" s="122"/>
+      <c r="D15" s="122"/>
+      <c r="E15" s="123"/>
       <c r="F15" s="27"/>
       <c r="G15" s="62"/>
       <c r="H15" s="62"/>
       <c r="I15" s="2"/>
-      <c r="J15" s="119"/>
-      <c r="K15" s="120"/>
+      <c r="J15" s="71"/>
+      <c r="K15" s="72"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="101"/>
-      <c r="B16" s="102"/>
-      <c r="C16" s="102"/>
-      <c r="D16" s="102"/>
-      <c r="E16" s="103"/>
+      <c r="A16" s="121"/>
+      <c r="B16" s="122"/>
+      <c r="C16" s="122"/>
+      <c r="D16" s="122"/>
+      <c r="E16" s="123"/>
       <c r="F16" s="8"/>
       <c r="G16" s="62"/>
       <c r="H16" s="62"/>
       <c r="I16" s="2"/>
-      <c r="J16" s="119"/>
-      <c r="K16" s="120"/>
+      <c r="J16" s="71"/>
+      <c r="K16" s="72"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="101"/>
-      <c r="B17" s="102"/>
-      <c r="C17" s="102"/>
-      <c r="D17" s="102"/>
-      <c r="E17" s="103"/>
+      <c r="A17" s="121"/>
+      <c r="B17" s="122"/>
+      <c r="C17" s="122"/>
+      <c r="D17" s="122"/>
+      <c r="E17" s="123"/>
       <c r="F17" s="27"/>
       <c r="G17" s="62"/>
       <c r="H17" s="62"/>
       <c r="I17" s="2"/>
-      <c r="J17" s="119"/>
-      <c r="K17" s="120"/>
+      <c r="J17" s="71"/>
+      <c r="K17" s="72"/>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="101"/>
-      <c r="B18" s="102"/>
-      <c r="C18" s="102"/>
-      <c r="D18" s="102"/>
-      <c r="E18" s="103"/>
+      <c r="A18" s="121"/>
+      <c r="B18" s="122"/>
+      <c r="C18" s="122"/>
+      <c r="D18" s="122"/>
+      <c r="E18" s="123"/>
       <c r="F18" s="27"/>
       <c r="G18" s="62"/>
       <c r="H18" s="62"/>
       <c r="I18" s="8"/>
-      <c r="J18" s="119"/>
-      <c r="K18" s="120"/>
+      <c r="J18" s="71"/>
+      <c r="K18" s="72"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="104"/>
-      <c r="B19" s="105"/>
-      <c r="C19" s="105"/>
-      <c r="D19" s="105"/>
-      <c r="E19" s="106"/>
+      <c r="A19" s="124"/>
+      <c r="B19" s="125"/>
+      <c r="C19" s="125"/>
+      <c r="D19" s="125"/>
+      <c r="E19" s="126"/>
       <c r="F19" s="63"/>
       <c r="G19" s="62"/>
       <c r="H19" s="62"/>
       <c r="I19" s="27"/>
-      <c r="J19" s="119"/>
-      <c r="K19" s="120"/>
+      <c r="J19" s="71"/>
+      <c r="K19" s="72"/>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="32"/>
@@ -2257,8 +2257,8 @@
       <c r="G20" s="64"/>
       <c r="H20" s="62"/>
       <c r="I20" s="27"/>
-      <c r="J20" s="119"/>
-      <c r="K20" s="120"/>
+      <c r="J20" s="71"/>
+      <c r="K20" s="72"/>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="32"/>
@@ -2270,8 +2270,8 @@
       <c r="G21" s="62"/>
       <c r="H21" s="62"/>
       <c r="I21" s="27"/>
-      <c r="J21" s="119"/>
-      <c r="K21" s="120"/>
+      <c r="J21" s="71"/>
+      <c r="K21" s="72"/>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="32"/>
@@ -2283,8 +2283,8 @@
       <c r="G22" s="62"/>
       <c r="H22" s="62"/>
       <c r="I22" s="27"/>
-      <c r="J22" s="119"/>
-      <c r="K22" s="120"/>
+      <c r="J22" s="71"/>
+      <c r="K22" s="72"/>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="32"/>
@@ -2296,8 +2296,8 @@
       <c r="G23" s="27"/>
       <c r="H23" s="27"/>
       <c r="I23" s="27"/>
-      <c r="J23" s="119"/>
-      <c r="K23" s="120"/>
+      <c r="J23" s="71"/>
+      <c r="K23" s="72"/>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" s="32"/>
@@ -2309,8 +2309,8 @@
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
-      <c r="J24" s="119"/>
-      <c r="K24" s="120"/>
+      <c r="J24" s="71"/>
+      <c r="K24" s="72"/>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="32"/>
@@ -2322,90 +2322,90 @@
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
       <c r="I25" s="9"/>
-      <c r="J25" s="119"/>
-      <c r="K25" s="120"/>
+      <c r="J25" s="71"/>
+      <c r="K25" s="72"/>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="83"/>
-      <c r="B26" s="80"/>
-      <c r="C26" s="80"/>
-      <c r="D26" s="80"/>
-      <c r="E26" s="84"/>
+      <c r="A26" s="105"/>
+      <c r="B26" s="94"/>
+      <c r="C26" s="94"/>
+      <c r="D26" s="94"/>
+      <c r="E26" s="106"/>
       <c r="F26" s="66"/>
       <c r="G26" s="67"/>
       <c r="H26" s="8"/>
       <c r="I26" s="9"/>
-      <c r="J26" s="119"/>
-      <c r="K26" s="120"/>
+      <c r="J26" s="71"/>
+      <c r="K26" s="72"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="80"/>
-      <c r="B27" s="80"/>
-      <c r="C27" s="80"/>
-      <c r="D27" s="80"/>
-      <c r="E27" s="84"/>
+      <c r="A27" s="94"/>
+      <c r="B27" s="94"/>
+      <c r="C27" s="94"/>
+      <c r="D27" s="94"/>
+      <c r="E27" s="106"/>
       <c r="F27" s="68"/>
       <c r="G27" s="67"/>
       <c r="H27" s="8"/>
       <c r="I27" s="9"/>
-      <c r="J27" s="119"/>
-      <c r="K27" s="120"/>
+      <c r="J27" s="71"/>
+      <c r="K27" s="72"/>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="80"/>
-      <c r="B28" s="80"/>
-      <c r="C28" s="80"/>
-      <c r="D28" s="80"/>
-      <c r="E28" s="84"/>
+      <c r="A28" s="94"/>
+      <c r="B28" s="94"/>
+      <c r="C28" s="94"/>
+      <c r="D28" s="94"/>
+      <c r="E28" s="106"/>
       <c r="F28" s="68"/>
       <c r="G28" s="67"/>
       <c r="H28" s="8"/>
       <c r="I28" s="9"/>
-      <c r="J28" s="119"/>
-      <c r="K28" s="120"/>
+      <c r="J28" s="71"/>
+      <c r="K28" s="72"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="80"/>
-      <c r="B29" s="80"/>
-      <c r="C29" s="80"/>
-      <c r="D29" s="80"/>
-      <c r="E29" s="84"/>
+      <c r="A29" s="94"/>
+      <c r="B29" s="94"/>
+      <c r="C29" s="94"/>
+      <c r="D29" s="94"/>
+      <c r="E29" s="106"/>
       <c r="F29" s="69"/>
       <c r="G29" s="70"/>
       <c r="H29" s="65"/>
       <c r="I29" s="23"/>
-      <c r="J29" s="119"/>
-      <c r="K29" s="120"/>
+      <c r="J29" s="71"/>
+      <c r="K29" s="72"/>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="85"/>
-      <c r="B30" s="85"/>
-      <c r="C30" s="85"/>
-      <c r="D30" s="85"/>
-      <c r="E30" s="86"/>
+      <c r="A30" s="107"/>
+      <c r="B30" s="107"/>
+      <c r="C30" s="107"/>
+      <c r="D30" s="107"/>
+      <c r="E30" s="108"/>
       <c r="F30" s="49"/>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
-      <c r="J30" s="119"/>
-      <c r="K30" s="120"/>
+      <c r="J30" s="71"/>
+      <c r="K30" s="72"/>
     </row>
     <row r="31" spans="1:11" ht="15.75">
-      <c r="A31" s="71" t="s">
+      <c r="A31" s="137" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="72"/>
-      <c r="C31" s="73"/>
+      <c r="B31" s="90"/>
+      <c r="C31" s="97"/>
       <c r="D31" s="50"/>
-      <c r="E31" s="74"/>
-      <c r="F31" s="75"/>
-      <c r="G31" s="75"/>
-      <c r="H31" s="75"/>
-      <c r="I31" s="76" t="s">
+      <c r="E31" s="138"/>
+      <c r="F31" s="139"/>
+      <c r="G31" s="139"/>
+      <c r="H31" s="139"/>
+      <c r="I31" s="140" t="s">
         <v>16</v>
       </c>
-      <c r="J31" s="77"/>
-      <c r="K31" s="78"/>
+      <c r="J31" s="141"/>
+      <c r="K31" s="142"/>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" s="37"/>
@@ -2413,12 +2413,12 @@
       <c r="C32" s="4"/>
       <c r="D32" s="38"/>
       <c r="E32" s="3"/>
-      <c r="F32" s="79"/>
-      <c r="G32" s="80"/>
-      <c r="H32" s="81"/>
-      <c r="I32" s="79"/>
-      <c r="J32" s="80"/>
-      <c r="K32" s="82"/>
+      <c r="F32" s="143"/>
+      <c r="G32" s="94"/>
+      <c r="H32" s="110"/>
+      <c r="I32" s="143"/>
+      <c r="J32" s="94"/>
+      <c r="K32" s="144"/>
     </row>
     <row r="33" spans="1:11">
       <c r="A33" s="39"/>
@@ -2497,32 +2497,11 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J30:K30"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="E1:G2"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="A5:C6"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="E6:G6"/>
-    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="E31:H31"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="I32:K32"/>
     <mergeCell ref="A26:E30"/>
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="J9:K9"/>
@@ -2539,11 +2518,32 @@
     <mergeCell ref="J13:K13"/>
     <mergeCell ref="J14:K14"/>
     <mergeCell ref="J15:K15"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="E31:H31"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="A5:C6"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="E1:G2"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J30:K30"/>
   </mergeCells>
   <conditionalFormatting sqref="F12:G15 I12 F17:F22 G17:G19 G21:G22">
     <cfRule type="expression" dxfId="7" priority="1">
@@ -2595,39 +2595,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.6" customHeight="1">
-      <c r="A1" s="128" t="s">
+      <c r="A1" s="73" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="129"/>
-      <c r="C1" s="150"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="145"/>
       <c r="D1" s="58"/>
-      <c r="E1" s="152" t="s">
+      <c r="E1" s="147" t="s">
         <v>18</v>
       </c>
-      <c r="F1" s="153"/>
-      <c r="G1" s="154"/>
+      <c r="F1" s="148"/>
+      <c r="G1" s="149"/>
       <c r="H1" s="29"/>
-      <c r="I1" s="139" t="s">
+      <c r="I1" s="84" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="140"/>
-      <c r="K1" s="141"/>
+      <c r="J1" s="85"/>
+      <c r="K1" s="86"/>
     </row>
     <row r="2" spans="1:11" ht="15.75">
-      <c r="A2" s="130"/>
-      <c r="B2" s="131"/>
-      <c r="C2" s="151"/>
+      <c r="A2" s="75"/>
+      <c r="B2" s="76"/>
+      <c r="C2" s="146"/>
       <c r="D2" s="52"/>
-      <c r="E2" s="155"/>
-      <c r="F2" s="156"/>
-      <c r="G2" s="157"/>
+      <c r="E2" s="150"/>
+      <c r="F2" s="151"/>
+      <c r="G2" s="152"/>
       <c r="H2" s="15"/>
-      <c r="I2" s="142">
+      <c r="I2" s="87">
         <f ca="1">TODAY()</f>
-        <v>45864</v>
-      </c>
-      <c r="J2" s="137"/>
-      <c r="K2" s="138"/>
+        <v>45865</v>
+      </c>
+      <c r="J2" s="82"/>
+      <c r="K2" s="83"/>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="32"/>
@@ -2643,11 +2643,11 @@
       <c r="K3" s="33"/>
     </row>
     <row r="4" spans="1:11" ht="17.25">
-      <c r="A4" s="158" t="s">
+      <c r="A4" s="153" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="159"/>
-      <c r="C4" s="131"/>
+      <c r="B4" s="154"/>
+      <c r="C4" s="76"/>
       <c r="D4" s="52"/>
       <c r="E4" s="26" t="s">
         <v>19</v>
@@ -2658,46 +2658,46 @@
       <c r="I4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="144"/>
-      <c r="K4" s="115"/>
+      <c r="J4" s="91"/>
+      <c r="K4" s="92"/>
     </row>
     <row r="5" spans="1:11" ht="18.75">
-      <c r="A5" s="145" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="146"/>
-      <c r="C5" s="132"/>
+      <c r="A5" s="155" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="156"/>
+      <c r="C5" s="77"/>
       <c r="D5" s="14"/>
-      <c r="E5" s="122" t="s">
+      <c r="E5" s="98" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="123"/>
-      <c r="G5" s="124"/>
+      <c r="F5" s="99"/>
+      <c r="G5" s="100"/>
       <c r="H5" s="22"/>
       <c r="I5" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="J5" s="125"/>
-      <c r="K5" s="115"/>
+      <c r="J5" s="101"/>
+      <c r="K5" s="92"/>
     </row>
     <row r="6" spans="1:11" ht="15.75">
-      <c r="A6" s="130"/>
-      <c r="B6" s="131"/>
-      <c r="C6" s="147"/>
+      <c r="A6" s="75"/>
+      <c r="B6" s="76"/>
+      <c r="C6" s="157"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="148" t="s">
+      <c r="E6" s="158" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="131"/>
-      <c r="G6" s="149"/>
+      <c r="F6" s="76"/>
+      <c r="G6" s="159"/>
       <c r="H6" s="46"/>
       <c r="I6" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="127">
+      <c r="J6" s="104">
         <v>1230</v>
       </c>
-      <c r="K6" s="115"/>
+      <c r="K6" s="92"/>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="32"/>
@@ -2713,44 +2713,44 @@
       <c r="K7" s="33"/>
     </row>
     <row r="8" spans="1:11" ht="15.75">
-      <c r="A8" s="107" t="s">
+      <c r="A8" s="127" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="109"/>
-      <c r="D8" s="110"/>
-      <c r="E8" s="111"/>
+      <c r="C8" s="129"/>
+      <c r="D8" s="130"/>
+      <c r="E8" s="131"/>
       <c r="F8" s="14"/>
-      <c r="G8" s="112" t="s">
+      <c r="G8" s="132" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="113"/>
+      <c r="H8" s="89"/>
       <c r="I8" s="14"/>
-      <c r="J8" s="114" t="s">
+      <c r="J8" s="133" t="s">
         <v>11</v>
       </c>
-      <c r="K8" s="115"/>
+      <c r="K8" s="92"/>
     </row>
     <row r="9" spans="1:11" ht="17.25">
-      <c r="A9" s="108"/>
+      <c r="A9" s="128"/>
       <c r="B9" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="116" t="s">
+      <c r="C9" s="134" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="72"/>
-      <c r="E9" s="81"/>
+      <c r="D9" s="90"/>
+      <c r="E9" s="110"/>
       <c r="F9" s="22"/>
-      <c r="G9" s="87">
+      <c r="G9" s="109">
         <v>1</v>
       </c>
-      <c r="H9" s="81"/>
+      <c r="H9" s="110"/>
       <c r="I9" s="22"/>
-      <c r="J9" s="88"/>
-      <c r="K9" s="89"/>
+      <c r="J9" s="111"/>
+      <c r="K9" s="103"/>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="32"/>
@@ -2766,128 +2766,128 @@
       <c r="K10" s="34"/>
     </row>
     <row r="11" spans="1:11" ht="18.75">
-      <c r="A11" s="90" t="s">
+      <c r="A11" s="112" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="91"/>
-      <c r="C11" s="91"/>
-      <c r="D11" s="91"/>
-      <c r="E11" s="92"/>
-      <c r="F11" s="93"/>
-      <c r="G11" s="91"/>
-      <c r="H11" s="91"/>
-      <c r="I11" s="91"/>
-      <c r="J11" s="91"/>
-      <c r="K11" s="94"/>
+      <c r="B11" s="113"/>
+      <c r="C11" s="113"/>
+      <c r="D11" s="113"/>
+      <c r="E11" s="114"/>
+      <c r="F11" s="115"/>
+      <c r="G11" s="113"/>
+      <c r="H11" s="113"/>
+      <c r="I11" s="113"/>
+      <c r="J11" s="113"/>
+      <c r="K11" s="116"/>
     </row>
     <row r="12" spans="1:11" ht="12.6" customHeight="1">
-      <c r="A12" s="95" t="s">
-        <v>21</v>
-      </c>
-      <c r="B12" s="96"/>
-      <c r="C12" s="96"/>
-      <c r="D12" s="96"/>
-      <c r="E12" s="81"/>
+      <c r="A12" s="117" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="95"/>
+      <c r="C12" s="95"/>
+      <c r="D12" s="95"/>
+      <c r="E12" s="110"/>
       <c r="F12" s="59"/>
       <c r="G12" s="31"/>
       <c r="H12" s="60"/>
       <c r="I12" s="31"/>
-      <c r="J12" s="117"/>
-      <c r="K12" s="118"/>
+      <c r="J12" s="135"/>
+      <c r="K12" s="136"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="97"/>
-      <c r="B13" s="72"/>
-      <c r="C13" s="72"/>
-      <c r="D13" s="72"/>
-      <c r="E13" s="73"/>
+      <c r="A13" s="96"/>
+      <c r="B13" s="90"/>
+      <c r="C13" s="90"/>
+      <c r="D13" s="90"/>
+      <c r="E13" s="97"/>
       <c r="F13" s="27"/>
       <c r="G13" s="61"/>
       <c r="H13" s="62"/>
       <c r="I13" s="2"/>
-      <c r="J13" s="117"/>
-      <c r="K13" s="118"/>
+      <c r="J13" s="135"/>
+      <c r="K13" s="136"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="98" t="str">
+      <c r="A14" s="118" t="str">
         <f>"*"&amp;A12&amp;"*"</f>
-        <v>*GOFEMM20052025002*</v>
-      </c>
-      <c r="B14" s="99"/>
-      <c r="C14" s="99"/>
-      <c r="D14" s="99"/>
-      <c r="E14" s="100"/>
+        <v>*GMKEMM20052025002*</v>
+      </c>
+      <c r="B14" s="119"/>
+      <c r="C14" s="119"/>
+      <c r="D14" s="119"/>
+      <c r="E14" s="120"/>
       <c r="F14" s="27"/>
       <c r="G14" s="62"/>
       <c r="H14" s="62"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="117"/>
-      <c r="K14" s="118"/>
+      <c r="J14" s="135"/>
+      <c r="K14" s="136"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="101"/>
-      <c r="B15" s="102"/>
-      <c r="C15" s="102"/>
-      <c r="D15" s="102"/>
-      <c r="E15" s="103"/>
+      <c r="A15" s="121"/>
+      <c r="B15" s="122"/>
+      <c r="C15" s="122"/>
+      <c r="D15" s="122"/>
+      <c r="E15" s="123"/>
       <c r="F15" s="27"/>
       <c r="G15" s="62"/>
       <c r="H15" s="62"/>
       <c r="I15" s="2"/>
-      <c r="J15" s="117"/>
-      <c r="K15" s="118"/>
+      <c r="J15" s="135"/>
+      <c r="K15" s="136"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="101"/>
-      <c r="B16" s="102"/>
-      <c r="C16" s="102"/>
-      <c r="D16" s="102"/>
-      <c r="E16" s="103"/>
+      <c r="A16" s="121"/>
+      <c r="B16" s="122"/>
+      <c r="C16" s="122"/>
+      <c r="D16" s="122"/>
+      <c r="E16" s="123"/>
       <c r="F16" s="8"/>
       <c r="G16" s="62"/>
       <c r="H16" s="62"/>
       <c r="I16" s="2"/>
-      <c r="J16" s="117"/>
-      <c r="K16" s="118"/>
+      <c r="J16" s="135"/>
+      <c r="K16" s="136"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="101"/>
-      <c r="B17" s="102"/>
-      <c r="C17" s="102"/>
-      <c r="D17" s="102"/>
-      <c r="E17" s="103"/>
+      <c r="A17" s="121"/>
+      <c r="B17" s="122"/>
+      <c r="C17" s="122"/>
+      <c r="D17" s="122"/>
+      <c r="E17" s="123"/>
       <c r="F17" s="27"/>
       <c r="G17" s="62"/>
       <c r="H17" s="62"/>
       <c r="I17" s="2"/>
-      <c r="J17" s="117"/>
-      <c r="K17" s="118"/>
+      <c r="J17" s="135"/>
+      <c r="K17" s="136"/>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="101"/>
-      <c r="B18" s="102"/>
-      <c r="C18" s="102"/>
-      <c r="D18" s="102"/>
-      <c r="E18" s="103"/>
+      <c r="A18" s="121"/>
+      <c r="B18" s="122"/>
+      <c r="C18" s="122"/>
+      <c r="D18" s="122"/>
+      <c r="E18" s="123"/>
       <c r="F18" s="27"/>
       <c r="G18" s="62"/>
       <c r="H18" s="62"/>
       <c r="I18" s="8"/>
-      <c r="J18" s="117"/>
-      <c r="K18" s="118"/>
+      <c r="J18" s="135"/>
+      <c r="K18" s="136"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="104"/>
-      <c r="B19" s="105"/>
-      <c r="C19" s="105"/>
-      <c r="D19" s="105"/>
-      <c r="E19" s="106"/>
+      <c r="A19" s="124"/>
+      <c r="B19" s="125"/>
+      <c r="C19" s="125"/>
+      <c r="D19" s="125"/>
+      <c r="E19" s="126"/>
       <c r="F19" s="63"/>
       <c r="G19" s="62"/>
       <c r="H19" s="62"/>
       <c r="I19" s="27"/>
-      <c r="J19" s="117"/>
-      <c r="K19" s="118"/>
+      <c r="J19" s="135"/>
+      <c r="K19" s="136"/>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="32"/>
@@ -2899,8 +2899,8 @@
       <c r="G20" s="64"/>
       <c r="H20" s="62"/>
       <c r="I20" s="27"/>
-      <c r="J20" s="117"/>
-      <c r="K20" s="118"/>
+      <c r="J20" s="135"/>
+      <c r="K20" s="136"/>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="32"/>
@@ -2912,8 +2912,8 @@
       <c r="G21" s="62"/>
       <c r="H21" s="62"/>
       <c r="I21" s="27"/>
-      <c r="J21" s="117"/>
-      <c r="K21" s="118"/>
+      <c r="J21" s="135"/>
+      <c r="K21" s="136"/>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="32"/>
@@ -2925,8 +2925,8 @@
       <c r="G22" s="62"/>
       <c r="H22" s="62"/>
       <c r="I22" s="27"/>
-      <c r="J22" s="117"/>
-      <c r="K22" s="118"/>
+      <c r="J22" s="135"/>
+      <c r="K22" s="136"/>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="32"/>
@@ -2938,8 +2938,8 @@
       <c r="G23" s="27"/>
       <c r="H23" s="27"/>
       <c r="I23" s="27"/>
-      <c r="J23" s="117"/>
-      <c r="K23" s="118"/>
+      <c r="J23" s="135"/>
+      <c r="K23" s="136"/>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" s="32"/>
@@ -2951,8 +2951,8 @@
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
-      <c r="J24" s="117"/>
-      <c r="K24" s="118"/>
+      <c r="J24" s="135"/>
+      <c r="K24" s="136"/>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="32"/>
@@ -2964,90 +2964,90 @@
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
       <c r="I25" s="9"/>
-      <c r="J25" s="117"/>
-      <c r="K25" s="118"/>
+      <c r="J25" s="135"/>
+      <c r="K25" s="136"/>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="83"/>
-      <c r="B26" s="80"/>
-      <c r="C26" s="80"/>
-      <c r="D26" s="80"/>
-      <c r="E26" s="84"/>
+      <c r="A26" s="105"/>
+      <c r="B26" s="94"/>
+      <c r="C26" s="94"/>
+      <c r="D26" s="94"/>
+      <c r="E26" s="106"/>
       <c r="F26" s="66"/>
       <c r="G26" s="67"/>
       <c r="H26" s="8"/>
       <c r="I26" s="9"/>
-      <c r="J26" s="117"/>
-      <c r="K26" s="118"/>
+      <c r="J26" s="135"/>
+      <c r="K26" s="136"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="80"/>
-      <c r="B27" s="80"/>
-      <c r="C27" s="80"/>
-      <c r="D27" s="80"/>
-      <c r="E27" s="84"/>
+      <c r="A27" s="94"/>
+      <c r="B27" s="94"/>
+      <c r="C27" s="94"/>
+      <c r="D27" s="94"/>
+      <c r="E27" s="106"/>
       <c r="F27" s="68"/>
       <c r="G27" s="67"/>
       <c r="H27" s="8"/>
       <c r="I27" s="9"/>
-      <c r="J27" s="117"/>
-      <c r="K27" s="118"/>
+      <c r="J27" s="135"/>
+      <c r="K27" s="136"/>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="80"/>
-      <c r="B28" s="80"/>
-      <c r="C28" s="80"/>
-      <c r="D28" s="80"/>
-      <c r="E28" s="84"/>
+      <c r="A28" s="94"/>
+      <c r="B28" s="94"/>
+      <c r="C28" s="94"/>
+      <c r="D28" s="94"/>
+      <c r="E28" s="106"/>
       <c r="F28" s="68"/>
       <c r="G28" s="67"/>
       <c r="H28" s="8"/>
       <c r="I28" s="9"/>
-      <c r="J28" s="117"/>
-      <c r="K28" s="118"/>
+      <c r="J28" s="135"/>
+      <c r="K28" s="136"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="80"/>
-      <c r="B29" s="80"/>
-      <c r="C29" s="80"/>
-      <c r="D29" s="80"/>
-      <c r="E29" s="84"/>
+      <c r="A29" s="94"/>
+      <c r="B29" s="94"/>
+      <c r="C29" s="94"/>
+      <c r="D29" s="94"/>
+      <c r="E29" s="106"/>
       <c r="F29" s="69"/>
       <c r="G29" s="70"/>
       <c r="H29" s="65"/>
       <c r="I29" s="23"/>
-      <c r="J29" s="117"/>
-      <c r="K29" s="118"/>
+      <c r="J29" s="135"/>
+      <c r="K29" s="136"/>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="85"/>
-      <c r="B30" s="85"/>
-      <c r="C30" s="85"/>
-      <c r="D30" s="85"/>
-      <c r="E30" s="86"/>
+      <c r="A30" s="107"/>
+      <c r="B30" s="107"/>
+      <c r="C30" s="107"/>
+      <c r="D30" s="107"/>
+      <c r="E30" s="108"/>
       <c r="F30" s="49"/>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
-      <c r="J30" s="117"/>
-      <c r="K30" s="118"/>
+      <c r="J30" s="135"/>
+      <c r="K30" s="136"/>
     </row>
     <row r="31" spans="1:11" ht="15.75">
-      <c r="A31" s="71" t="s">
+      <c r="A31" s="137" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="72"/>
-      <c r="C31" s="73"/>
+      <c r="B31" s="90"/>
+      <c r="C31" s="97"/>
       <c r="D31" s="50"/>
-      <c r="E31" s="74"/>
-      <c r="F31" s="75"/>
-      <c r="G31" s="75"/>
-      <c r="H31" s="75"/>
-      <c r="I31" s="76" t="s">
+      <c r="E31" s="138"/>
+      <c r="F31" s="139"/>
+      <c r="G31" s="139"/>
+      <c r="H31" s="139"/>
+      <c r="I31" s="140" t="s">
         <v>16</v>
       </c>
-      <c r="J31" s="77"/>
-      <c r="K31" s="78"/>
+      <c r="J31" s="141"/>
+      <c r="K31" s="142"/>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" s="37"/>
@@ -3055,12 +3055,12 @@
       <c r="C32" s="4"/>
       <c r="D32" s="38"/>
       <c r="E32" s="3"/>
-      <c r="F32" s="79"/>
-      <c r="G32" s="80"/>
-      <c r="H32" s="81"/>
-      <c r="I32" s="79"/>
-      <c r="J32" s="80"/>
-      <c r="K32" s="82"/>
+      <c r="F32" s="143"/>
+      <c r="G32" s="94"/>
+      <c r="H32" s="110"/>
+      <c r="I32" s="143"/>
+      <c r="J32" s="94"/>
+      <c r="K32" s="144"/>
     </row>
     <row r="33" spans="1:11">
       <c r="A33" s="39"/>
@@ -3139,27 +3139,16 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="E1:G2"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="A26:E30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="E31:H31"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J30:K30"/>
     <mergeCell ref="A14:E19"/>
     <mergeCell ref="A5:C6"/>
     <mergeCell ref="E5:G5"/>
@@ -3176,16 +3165,27 @@
     <mergeCell ref="A11:E11"/>
     <mergeCell ref="F11:K11"/>
     <mergeCell ref="A12:E13"/>
-    <mergeCell ref="A26:E30"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="E31:H31"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="E1:G2"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J26:K26"/>
   </mergeCells>
   <conditionalFormatting sqref="F12:G15 I12 F17:F22 G17:G19 G21:G22">
     <cfRule type="expression" dxfId="3" priority="1">

</xml_diff>

<commit_message>
add all changes for rabat and fix some bugs
</commit_message>
<xml_diff>
--- a/dummy-content/ECHEC-RETOUR_CLIENT-CASABLANCA.xlsx
+++ b/dummy-content/ECHEC-RETOUR_CLIENT-CASABLANCA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UNK\Desktop\GoFleet-Enhancer\dummy-content\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1B4C9ED-1BAA-4ECD-9F77-33AFFD184B73}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14B10EDF-8959-4DC4-A661-4FA6F5E8F07C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ECHEC CASA" sheetId="5" r:id="rId1"/>
@@ -84,13 +84,13 @@
     <t xml:space="preserve">                                                       Destination</t>
   </si>
   <si>
-    <t>GOFEMM20052025001</t>
+    <t>GO FLEET RABAT</t>
   </si>
   <si>
-    <t>GOFEMM20052025002</t>
+    <t>GRBEMM20052025001</t>
   </si>
   <si>
-    <t>GO FLEET RABAT</t>
+    <t>GRBEMM20052025002</t>
   </si>
 </sst>
 </file>
@@ -1400,24 +1400,66 @@
     <xf numFmtId="0" fontId="15" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="5" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
@@ -1425,10 +1467,10 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="11" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1441,8 +1483,6 @@
     <xf numFmtId="0" fontId="21" fillId="12" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="24" fillId="3" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1466,11 +1506,9 @@
     <xf numFmtId="0" fontId="8" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1480,67 +1518,20 @@
     <xf numFmtId="0" fontId="15" fillId="15" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="5" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="20" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="19" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="17" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1555,6 +1546,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="19" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1955,37 +1955,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.6" customHeight="1">
-      <c r="A1" s="128"/>
-      <c r="B1" s="129"/>
-      <c r="C1" s="129"/>
+      <c r="A1" s="73"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
       <c r="D1" s="53"/>
-      <c r="E1" s="133" t="s">
+      <c r="E1" s="78" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="134"/>
-      <c r="G1" s="135"/>
+      <c r="F1" s="79"/>
+      <c r="G1" s="80"/>
       <c r="H1" s="29"/>
-      <c r="I1" s="139" t="s">
+      <c r="I1" s="84" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="140"/>
-      <c r="K1" s="141"/>
+      <c r="J1" s="85"/>
+      <c r="K1" s="86"/>
     </row>
     <row r="2" spans="1:11" ht="15.75">
-      <c r="A2" s="130"/>
-      <c r="B2" s="131"/>
-      <c r="C2" s="132"/>
+      <c r="A2" s="75"/>
+      <c r="B2" s="76"/>
+      <c r="C2" s="77"/>
       <c r="D2" s="53"/>
-      <c r="E2" s="136"/>
-      <c r="F2" s="137"/>
-      <c r="G2" s="138"/>
+      <c r="E2" s="81"/>
+      <c r="F2" s="82"/>
+      <c r="G2" s="83"/>
       <c r="H2" s="15"/>
-      <c r="I2" s="142">
+      <c r="I2" s="87">
         <f ca="1">TODAY()</f>
-        <v>45864</v>
-      </c>
-      <c r="J2" s="137"/>
-      <c r="K2" s="138"/>
+        <v>45865</v>
+      </c>
+      <c r="J2" s="82"/>
+      <c r="K2" s="83"/>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="32"/>
@@ -2001,11 +2001,11 @@
       <c r="K3" s="33"/>
     </row>
     <row r="4" spans="1:11" ht="17.25">
-      <c r="A4" s="143" t="s">
+      <c r="A4" s="88" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="113"/>
-      <c r="C4" s="72"/>
+      <c r="B4" s="89"/>
+      <c r="C4" s="90"/>
       <c r="D4" s="52"/>
       <c r="E4" s="16" t="s">
         <v>19</v>
@@ -2016,46 +2016,46 @@
       <c r="I4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="144"/>
-      <c r="K4" s="115"/>
+      <c r="J4" s="91"/>
+      <c r="K4" s="92"/>
     </row>
     <row r="5" spans="1:11" ht="18.75">
-      <c r="A5" s="121" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="80"/>
-      <c r="C5" s="96"/>
+      <c r="A5" s="93" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="94"/>
+      <c r="C5" s="95"/>
       <c r="D5" s="14"/>
-      <c r="E5" s="122" t="s">
+      <c r="E5" s="98" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="123"/>
-      <c r="G5" s="124"/>
+      <c r="F5" s="99"/>
+      <c r="G5" s="100"/>
       <c r="H5" s="22"/>
       <c r="I5" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="J5" s="125"/>
-      <c r="K5" s="115"/>
+      <c r="J5" s="101"/>
+      <c r="K5" s="92"/>
     </row>
     <row r="6" spans="1:11" ht="15.75">
-      <c r="A6" s="97"/>
-      <c r="B6" s="72"/>
-      <c r="C6" s="73"/>
+      <c r="A6" s="96"/>
+      <c r="B6" s="90"/>
+      <c r="C6" s="97"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="126" t="s">
+      <c r="E6" s="102" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="72"/>
-      <c r="G6" s="89"/>
+      <c r="F6" s="90"/>
+      <c r="G6" s="103"/>
       <c r="H6" s="46"/>
       <c r="I6" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="127">
+      <c r="J6" s="104">
         <v>1230</v>
       </c>
-      <c r="K6" s="115"/>
+      <c r="K6" s="92"/>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="32"/>
@@ -2071,44 +2071,44 @@
       <c r="K7" s="33"/>
     </row>
     <row r="8" spans="1:11" ht="15.75">
-      <c r="A8" s="107" t="s">
+      <c r="A8" s="127" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="109"/>
-      <c r="D8" s="110"/>
-      <c r="E8" s="111"/>
+      <c r="C8" s="129"/>
+      <c r="D8" s="130"/>
+      <c r="E8" s="131"/>
       <c r="F8" s="14"/>
-      <c r="G8" s="112" t="s">
+      <c r="G8" s="132" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="113"/>
+      <c r="H8" s="89"/>
       <c r="I8" s="14"/>
-      <c r="J8" s="114" t="s">
+      <c r="J8" s="133" t="s">
         <v>11</v>
       </c>
-      <c r="K8" s="115"/>
+      <c r="K8" s="92"/>
     </row>
     <row r="9" spans="1:11" ht="17.25">
-      <c r="A9" s="108"/>
+      <c r="A9" s="128"/>
       <c r="B9" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="116" t="s">
+      <c r="C9" s="134" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="72"/>
-      <c r="E9" s="81"/>
+      <c r="D9" s="90"/>
+      <c r="E9" s="110"/>
       <c r="F9" s="22"/>
-      <c r="G9" s="87">
+      <c r="G9" s="109">
         <v>1</v>
       </c>
-      <c r="H9" s="81"/>
+      <c r="H9" s="110"/>
       <c r="I9" s="22"/>
-      <c r="J9" s="88"/>
-      <c r="K9" s="89"/>
+      <c r="J9" s="111"/>
+      <c r="K9" s="103"/>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="32"/>
@@ -2124,128 +2124,128 @@
       <c r="K10" s="34"/>
     </row>
     <row r="11" spans="1:11" ht="18.75">
-      <c r="A11" s="90" t="s">
+      <c r="A11" s="112" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="91"/>
-      <c r="C11" s="91"/>
-      <c r="D11" s="91"/>
-      <c r="E11" s="92"/>
-      <c r="F11" s="93"/>
-      <c r="G11" s="91"/>
-      <c r="H11" s="91"/>
-      <c r="I11" s="91"/>
-      <c r="J11" s="91"/>
-      <c r="K11" s="94"/>
+      <c r="B11" s="113"/>
+      <c r="C11" s="113"/>
+      <c r="D11" s="113"/>
+      <c r="E11" s="114"/>
+      <c r="F11" s="115"/>
+      <c r="G11" s="113"/>
+      <c r="H11" s="113"/>
+      <c r="I11" s="113"/>
+      <c r="J11" s="113"/>
+      <c r="K11" s="116"/>
     </row>
     <row r="12" spans="1:11">
-      <c r="A12" s="95" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" s="96"/>
-      <c r="C12" s="96"/>
-      <c r="D12" s="96"/>
-      <c r="E12" s="81"/>
+      <c r="A12" s="117" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="95"/>
+      <c r="C12" s="95"/>
+      <c r="D12" s="95"/>
+      <c r="E12" s="110"/>
       <c r="F12" s="59"/>
       <c r="G12" s="31"/>
       <c r="H12" s="60"/>
       <c r="I12" s="31"/>
-      <c r="J12" s="117"/>
-      <c r="K12" s="118"/>
+      <c r="J12" s="135"/>
+      <c r="K12" s="136"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="97"/>
-      <c r="B13" s="72"/>
-      <c r="C13" s="72"/>
-      <c r="D13" s="72"/>
-      <c r="E13" s="73"/>
+      <c r="A13" s="96"/>
+      <c r="B13" s="90"/>
+      <c r="C13" s="90"/>
+      <c r="D13" s="90"/>
+      <c r="E13" s="97"/>
       <c r="F13" s="27"/>
       <c r="G13" s="61"/>
       <c r="H13" s="62"/>
       <c r="I13" s="2"/>
-      <c r="J13" s="119"/>
-      <c r="K13" s="120"/>
+      <c r="J13" s="71"/>
+      <c r="K13" s="72"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="98" t="str">
+      <c r="A14" s="118" t="str">
         <f>"*"&amp;A12&amp;"*"</f>
-        <v>*GOFEMM20052025001*</v>
-      </c>
-      <c r="B14" s="99"/>
-      <c r="C14" s="99"/>
-      <c r="D14" s="99"/>
-      <c r="E14" s="100"/>
+        <v>*GRBEMM20052025001*</v>
+      </c>
+      <c r="B14" s="119"/>
+      <c r="C14" s="119"/>
+      <c r="D14" s="119"/>
+      <c r="E14" s="120"/>
       <c r="F14" s="27"/>
       <c r="G14" s="62"/>
       <c r="H14" s="62"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="119"/>
-      <c r="K14" s="120"/>
+      <c r="J14" s="71"/>
+      <c r="K14" s="72"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="101"/>
-      <c r="B15" s="102"/>
-      <c r="C15" s="102"/>
-      <c r="D15" s="102"/>
-      <c r="E15" s="103"/>
+      <c r="A15" s="121"/>
+      <c r="B15" s="122"/>
+      <c r="C15" s="122"/>
+      <c r="D15" s="122"/>
+      <c r="E15" s="123"/>
       <c r="F15" s="27"/>
       <c r="G15" s="62"/>
       <c r="H15" s="62"/>
       <c r="I15" s="2"/>
-      <c r="J15" s="119"/>
-      <c r="K15" s="120"/>
+      <c r="J15" s="71"/>
+      <c r="K15" s="72"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="101"/>
-      <c r="B16" s="102"/>
-      <c r="C16" s="102"/>
-      <c r="D16" s="102"/>
-      <c r="E16" s="103"/>
+      <c r="A16" s="121"/>
+      <c r="B16" s="122"/>
+      <c r="C16" s="122"/>
+      <c r="D16" s="122"/>
+      <c r="E16" s="123"/>
       <c r="F16" s="8"/>
       <c r="G16" s="62"/>
       <c r="H16" s="62"/>
       <c r="I16" s="2"/>
-      <c r="J16" s="119"/>
-      <c r="K16" s="120"/>
+      <c r="J16" s="71"/>
+      <c r="K16" s="72"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="101"/>
-      <c r="B17" s="102"/>
-      <c r="C17" s="102"/>
-      <c r="D17" s="102"/>
-      <c r="E17" s="103"/>
+      <c r="A17" s="121"/>
+      <c r="B17" s="122"/>
+      <c r="C17" s="122"/>
+      <c r="D17" s="122"/>
+      <c r="E17" s="123"/>
       <c r="F17" s="27"/>
       <c r="G17" s="62"/>
       <c r="H17" s="62"/>
       <c r="I17" s="2"/>
-      <c r="J17" s="119"/>
-      <c r="K17" s="120"/>
+      <c r="J17" s="71"/>
+      <c r="K17" s="72"/>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="101"/>
-      <c r="B18" s="102"/>
-      <c r="C18" s="102"/>
-      <c r="D18" s="102"/>
-      <c r="E18" s="103"/>
+      <c r="A18" s="121"/>
+      <c r="B18" s="122"/>
+      <c r="C18" s="122"/>
+      <c r="D18" s="122"/>
+      <c r="E18" s="123"/>
       <c r="F18" s="27"/>
       <c r="G18" s="62"/>
       <c r="H18" s="62"/>
       <c r="I18" s="8"/>
-      <c r="J18" s="119"/>
-      <c r="K18" s="120"/>
+      <c r="J18" s="71"/>
+      <c r="K18" s="72"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="104"/>
-      <c r="B19" s="105"/>
-      <c r="C19" s="105"/>
-      <c r="D19" s="105"/>
-      <c r="E19" s="106"/>
+      <c r="A19" s="124"/>
+      <c r="B19" s="125"/>
+      <c r="C19" s="125"/>
+      <c r="D19" s="125"/>
+      <c r="E19" s="126"/>
       <c r="F19" s="63"/>
       <c r="G19" s="62"/>
       <c r="H19" s="62"/>
       <c r="I19" s="27"/>
-      <c r="J19" s="119"/>
-      <c r="K19" s="120"/>
+      <c r="J19" s="71"/>
+      <c r="K19" s="72"/>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="32"/>
@@ -2257,8 +2257,8 @@
       <c r="G20" s="64"/>
       <c r="H20" s="62"/>
       <c r="I20" s="27"/>
-      <c r="J20" s="119"/>
-      <c r="K20" s="120"/>
+      <c r="J20" s="71"/>
+      <c r="K20" s="72"/>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="32"/>
@@ -2270,8 +2270,8 @@
       <c r="G21" s="62"/>
       <c r="H21" s="62"/>
       <c r="I21" s="27"/>
-      <c r="J21" s="119"/>
-      <c r="K21" s="120"/>
+      <c r="J21" s="71"/>
+      <c r="K21" s="72"/>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="32"/>
@@ -2283,8 +2283,8 @@
       <c r="G22" s="62"/>
       <c r="H22" s="62"/>
       <c r="I22" s="27"/>
-      <c r="J22" s="119"/>
-      <c r="K22" s="120"/>
+      <c r="J22" s="71"/>
+      <c r="K22" s="72"/>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="32"/>
@@ -2296,8 +2296,8 @@
       <c r="G23" s="27"/>
       <c r="H23" s="27"/>
       <c r="I23" s="27"/>
-      <c r="J23" s="119"/>
-      <c r="K23" s="120"/>
+      <c r="J23" s="71"/>
+      <c r="K23" s="72"/>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" s="32"/>
@@ -2309,8 +2309,8 @@
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
-      <c r="J24" s="119"/>
-      <c r="K24" s="120"/>
+      <c r="J24" s="71"/>
+      <c r="K24" s="72"/>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="32"/>
@@ -2322,90 +2322,90 @@
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
       <c r="I25" s="9"/>
-      <c r="J25" s="119"/>
-      <c r="K25" s="120"/>
+      <c r="J25" s="71"/>
+      <c r="K25" s="72"/>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="83"/>
-      <c r="B26" s="80"/>
-      <c r="C26" s="80"/>
-      <c r="D26" s="80"/>
-      <c r="E26" s="84"/>
+      <c r="A26" s="105"/>
+      <c r="B26" s="94"/>
+      <c r="C26" s="94"/>
+      <c r="D26" s="94"/>
+      <c r="E26" s="106"/>
       <c r="F26" s="66"/>
       <c r="G26" s="67"/>
       <c r="H26" s="8"/>
       <c r="I26" s="9"/>
-      <c r="J26" s="119"/>
-      <c r="K26" s="120"/>
+      <c r="J26" s="71"/>
+      <c r="K26" s="72"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="80"/>
-      <c r="B27" s="80"/>
-      <c r="C27" s="80"/>
-      <c r="D27" s="80"/>
-      <c r="E27" s="84"/>
+      <c r="A27" s="94"/>
+      <c r="B27" s="94"/>
+      <c r="C27" s="94"/>
+      <c r="D27" s="94"/>
+      <c r="E27" s="106"/>
       <c r="F27" s="68"/>
       <c r="G27" s="67"/>
       <c r="H27" s="8"/>
       <c r="I27" s="9"/>
-      <c r="J27" s="119"/>
-      <c r="K27" s="120"/>
+      <c r="J27" s="71"/>
+      <c r="K27" s="72"/>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="80"/>
-      <c r="B28" s="80"/>
-      <c r="C28" s="80"/>
-      <c r="D28" s="80"/>
-      <c r="E28" s="84"/>
+      <c r="A28" s="94"/>
+      <c r="B28" s="94"/>
+      <c r="C28" s="94"/>
+      <c r="D28" s="94"/>
+      <c r="E28" s="106"/>
       <c r="F28" s="68"/>
       <c r="G28" s="67"/>
       <c r="H28" s="8"/>
       <c r="I28" s="9"/>
-      <c r="J28" s="119"/>
-      <c r="K28" s="120"/>
+      <c r="J28" s="71"/>
+      <c r="K28" s="72"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="80"/>
-      <c r="B29" s="80"/>
-      <c r="C29" s="80"/>
-      <c r="D29" s="80"/>
-      <c r="E29" s="84"/>
+      <c r="A29" s="94"/>
+      <c r="B29" s="94"/>
+      <c r="C29" s="94"/>
+      <c r="D29" s="94"/>
+      <c r="E29" s="106"/>
       <c r="F29" s="69"/>
       <c r="G29" s="70"/>
       <c r="H29" s="65"/>
       <c r="I29" s="23"/>
-      <c r="J29" s="119"/>
-      <c r="K29" s="120"/>
+      <c r="J29" s="71"/>
+      <c r="K29" s="72"/>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="85"/>
-      <c r="B30" s="85"/>
-      <c r="C30" s="85"/>
-      <c r="D30" s="85"/>
-      <c r="E30" s="86"/>
+      <c r="A30" s="107"/>
+      <c r="B30" s="107"/>
+      <c r="C30" s="107"/>
+      <c r="D30" s="107"/>
+      <c r="E30" s="108"/>
       <c r="F30" s="49"/>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
-      <c r="J30" s="119"/>
-      <c r="K30" s="120"/>
+      <c r="J30" s="71"/>
+      <c r="K30" s="72"/>
     </row>
     <row r="31" spans="1:11" ht="15.75">
-      <c r="A31" s="71" t="s">
+      <c r="A31" s="137" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="72"/>
-      <c r="C31" s="73"/>
+      <c r="B31" s="90"/>
+      <c r="C31" s="97"/>
       <c r="D31" s="50"/>
-      <c r="E31" s="74"/>
-      <c r="F31" s="75"/>
-      <c r="G31" s="75"/>
-      <c r="H31" s="75"/>
-      <c r="I31" s="76" t="s">
+      <c r="E31" s="138"/>
+      <c r="F31" s="139"/>
+      <c r="G31" s="139"/>
+      <c r="H31" s="139"/>
+      <c r="I31" s="140" t="s">
         <v>16</v>
       </c>
-      <c r="J31" s="77"/>
-      <c r="K31" s="78"/>
+      <c r="J31" s="141"/>
+      <c r="K31" s="142"/>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" s="37"/>
@@ -2413,12 +2413,12 @@
       <c r="C32" s="4"/>
       <c r="D32" s="38"/>
       <c r="E32" s="3"/>
-      <c r="F32" s="79"/>
-      <c r="G32" s="80"/>
-      <c r="H32" s="81"/>
-      <c r="I32" s="79"/>
-      <c r="J32" s="80"/>
-      <c r="K32" s="82"/>
+      <c r="F32" s="143"/>
+      <c r="G32" s="94"/>
+      <c r="H32" s="110"/>
+      <c r="I32" s="143"/>
+      <c r="J32" s="94"/>
+      <c r="K32" s="144"/>
     </row>
     <row r="33" spans="1:11">
       <c r="A33" s="39"/>
@@ -2497,32 +2497,11 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J30:K30"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="E1:G2"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="A5:C6"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="E6:G6"/>
-    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="E31:H31"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="I32:K32"/>
     <mergeCell ref="A26:E30"/>
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="J9:K9"/>
@@ -2539,11 +2518,32 @@
     <mergeCell ref="J13:K13"/>
     <mergeCell ref="J14:K14"/>
     <mergeCell ref="J15:K15"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="E31:H31"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="A5:C6"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="E1:G2"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J30:K30"/>
   </mergeCells>
   <conditionalFormatting sqref="F12:G15 I12 F17:F22 G17:G19 G21:G22">
     <cfRule type="expression" dxfId="7" priority="1">
@@ -2595,39 +2595,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.6" customHeight="1">
-      <c r="A1" s="128" t="s">
+      <c r="A1" s="73" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="129"/>
-      <c r="C1" s="150"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="145"/>
       <c r="D1" s="58"/>
-      <c r="E1" s="152" t="s">
+      <c r="E1" s="147" t="s">
         <v>18</v>
       </c>
-      <c r="F1" s="153"/>
-      <c r="G1" s="154"/>
+      <c r="F1" s="148"/>
+      <c r="G1" s="149"/>
       <c r="H1" s="29"/>
-      <c r="I1" s="139" t="s">
+      <c r="I1" s="84" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="140"/>
-      <c r="K1" s="141"/>
+      <c r="J1" s="85"/>
+      <c r="K1" s="86"/>
     </row>
     <row r="2" spans="1:11" ht="15.75">
-      <c r="A2" s="130"/>
-      <c r="B2" s="131"/>
-      <c r="C2" s="151"/>
+      <c r="A2" s="75"/>
+      <c r="B2" s="76"/>
+      <c r="C2" s="146"/>
       <c r="D2" s="52"/>
-      <c r="E2" s="155"/>
-      <c r="F2" s="156"/>
-      <c r="G2" s="157"/>
+      <c r="E2" s="150"/>
+      <c r="F2" s="151"/>
+      <c r="G2" s="152"/>
       <c r="H2" s="15"/>
-      <c r="I2" s="142">
+      <c r="I2" s="87">
         <f ca="1">TODAY()</f>
-        <v>45864</v>
-      </c>
-      <c r="J2" s="137"/>
-      <c r="K2" s="138"/>
+        <v>45865</v>
+      </c>
+      <c r="J2" s="82"/>
+      <c r="K2" s="83"/>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="32"/>
@@ -2643,11 +2643,11 @@
       <c r="K3" s="33"/>
     </row>
     <row r="4" spans="1:11" ht="17.25">
-      <c r="A4" s="158" t="s">
+      <c r="A4" s="153" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="159"/>
-      <c r="C4" s="131"/>
+      <c r="B4" s="154"/>
+      <c r="C4" s="76"/>
       <c r="D4" s="52"/>
       <c r="E4" s="26" t="s">
         <v>19</v>
@@ -2658,46 +2658,46 @@
       <c r="I4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="144"/>
-      <c r="K4" s="115"/>
+      <c r="J4" s="91"/>
+      <c r="K4" s="92"/>
     </row>
     <row r="5" spans="1:11" ht="18.75">
-      <c r="A5" s="145" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="146"/>
-      <c r="C5" s="132"/>
+      <c r="A5" s="155" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="156"/>
+      <c r="C5" s="77"/>
       <c r="D5" s="14"/>
-      <c r="E5" s="122" t="s">
+      <c r="E5" s="98" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="123"/>
-      <c r="G5" s="124"/>
+      <c r="F5" s="99"/>
+      <c r="G5" s="100"/>
       <c r="H5" s="22"/>
       <c r="I5" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="J5" s="125"/>
-      <c r="K5" s="115"/>
+      <c r="J5" s="101"/>
+      <c r="K5" s="92"/>
     </row>
     <row r="6" spans="1:11" ht="15.75">
-      <c r="A6" s="130"/>
-      <c r="B6" s="131"/>
-      <c r="C6" s="147"/>
+      <c r="A6" s="75"/>
+      <c r="B6" s="76"/>
+      <c r="C6" s="157"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="148" t="s">
+      <c r="E6" s="158" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="131"/>
-      <c r="G6" s="149"/>
+      <c r="F6" s="76"/>
+      <c r="G6" s="159"/>
       <c r="H6" s="46"/>
       <c r="I6" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="127">
+      <c r="J6" s="104">
         <v>1230</v>
       </c>
-      <c r="K6" s="115"/>
+      <c r="K6" s="92"/>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="32"/>
@@ -2713,44 +2713,44 @@
       <c r="K7" s="33"/>
     </row>
     <row r="8" spans="1:11" ht="15.75">
-      <c r="A8" s="107" t="s">
+      <c r="A8" s="127" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="109"/>
-      <c r="D8" s="110"/>
-      <c r="E8" s="111"/>
+      <c r="C8" s="129"/>
+      <c r="D8" s="130"/>
+      <c r="E8" s="131"/>
       <c r="F8" s="14"/>
-      <c r="G8" s="112" t="s">
+      <c r="G8" s="132" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="113"/>
+      <c r="H8" s="89"/>
       <c r="I8" s="14"/>
-      <c r="J8" s="114" t="s">
+      <c r="J8" s="133" t="s">
         <v>11</v>
       </c>
-      <c r="K8" s="115"/>
+      <c r="K8" s="92"/>
     </row>
     <row r="9" spans="1:11" ht="17.25">
-      <c r="A9" s="108"/>
+      <c r="A9" s="128"/>
       <c r="B9" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="116" t="s">
+      <c r="C9" s="134" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="72"/>
-      <c r="E9" s="81"/>
+      <c r="D9" s="90"/>
+      <c r="E9" s="110"/>
       <c r="F9" s="22"/>
-      <c r="G9" s="87">
+      <c r="G9" s="109">
         <v>1</v>
       </c>
-      <c r="H9" s="81"/>
+      <c r="H9" s="110"/>
       <c r="I9" s="22"/>
-      <c r="J9" s="88"/>
-      <c r="K9" s="89"/>
+      <c r="J9" s="111"/>
+      <c r="K9" s="103"/>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="32"/>
@@ -2766,128 +2766,128 @@
       <c r="K10" s="34"/>
     </row>
     <row r="11" spans="1:11" ht="18.75">
-      <c r="A11" s="90" t="s">
+      <c r="A11" s="112" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="91"/>
-      <c r="C11" s="91"/>
-      <c r="D11" s="91"/>
-      <c r="E11" s="92"/>
-      <c r="F11" s="93"/>
-      <c r="G11" s="91"/>
-      <c r="H11" s="91"/>
-      <c r="I11" s="91"/>
-      <c r="J11" s="91"/>
-      <c r="K11" s="94"/>
+      <c r="B11" s="113"/>
+      <c r="C11" s="113"/>
+      <c r="D11" s="113"/>
+      <c r="E11" s="114"/>
+      <c r="F11" s="115"/>
+      <c r="G11" s="113"/>
+      <c r="H11" s="113"/>
+      <c r="I11" s="113"/>
+      <c r="J11" s="113"/>
+      <c r="K11" s="116"/>
     </row>
     <row r="12" spans="1:11" ht="12.6" customHeight="1">
-      <c r="A12" s="95" t="s">
-        <v>21</v>
-      </c>
-      <c r="B12" s="96"/>
-      <c r="C12" s="96"/>
-      <c r="D12" s="96"/>
-      <c r="E12" s="81"/>
+      <c r="A12" s="117" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="95"/>
+      <c r="C12" s="95"/>
+      <c r="D12" s="95"/>
+      <c r="E12" s="110"/>
       <c r="F12" s="59"/>
       <c r="G12" s="31"/>
       <c r="H12" s="60"/>
       <c r="I12" s="31"/>
-      <c r="J12" s="117"/>
-      <c r="K12" s="118"/>
+      <c r="J12" s="135"/>
+      <c r="K12" s="136"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="97"/>
-      <c r="B13" s="72"/>
-      <c r="C13" s="72"/>
-      <c r="D13" s="72"/>
-      <c r="E13" s="73"/>
+      <c r="A13" s="96"/>
+      <c r="B13" s="90"/>
+      <c r="C13" s="90"/>
+      <c r="D13" s="90"/>
+      <c r="E13" s="97"/>
       <c r="F13" s="27"/>
       <c r="G13" s="61"/>
       <c r="H13" s="62"/>
       <c r="I13" s="2"/>
-      <c r="J13" s="117"/>
-      <c r="K13" s="118"/>
+      <c r="J13" s="135"/>
+      <c r="K13" s="136"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="98" t="str">
+      <c r="A14" s="118" t="str">
         <f>"*"&amp;A12&amp;"*"</f>
-        <v>*GOFEMM20052025002*</v>
-      </c>
-      <c r="B14" s="99"/>
-      <c r="C14" s="99"/>
-      <c r="D14" s="99"/>
-      <c r="E14" s="100"/>
+        <v>*GRBEMM20052025002*</v>
+      </c>
+      <c r="B14" s="119"/>
+      <c r="C14" s="119"/>
+      <c r="D14" s="119"/>
+      <c r="E14" s="120"/>
       <c r="F14" s="27"/>
       <c r="G14" s="62"/>
       <c r="H14" s="62"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="117"/>
-      <c r="K14" s="118"/>
+      <c r="J14" s="135"/>
+      <c r="K14" s="136"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="101"/>
-      <c r="B15" s="102"/>
-      <c r="C15" s="102"/>
-      <c r="D15" s="102"/>
-      <c r="E15" s="103"/>
+      <c r="A15" s="121"/>
+      <c r="B15" s="122"/>
+      <c r="C15" s="122"/>
+      <c r="D15" s="122"/>
+      <c r="E15" s="123"/>
       <c r="F15" s="27"/>
       <c r="G15" s="62"/>
       <c r="H15" s="62"/>
       <c r="I15" s="2"/>
-      <c r="J15" s="117"/>
-      <c r="K15" s="118"/>
+      <c r="J15" s="135"/>
+      <c r="K15" s="136"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="101"/>
-      <c r="B16" s="102"/>
-      <c r="C16" s="102"/>
-      <c r="D16" s="102"/>
-      <c r="E16" s="103"/>
+      <c r="A16" s="121"/>
+      <c r="B16" s="122"/>
+      <c r="C16" s="122"/>
+      <c r="D16" s="122"/>
+      <c r="E16" s="123"/>
       <c r="F16" s="8"/>
       <c r="G16" s="62"/>
       <c r="H16" s="62"/>
       <c r="I16" s="2"/>
-      <c r="J16" s="117"/>
-      <c r="K16" s="118"/>
+      <c r="J16" s="135"/>
+      <c r="K16" s="136"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="101"/>
-      <c r="B17" s="102"/>
-      <c r="C17" s="102"/>
-      <c r="D17" s="102"/>
-      <c r="E17" s="103"/>
+      <c r="A17" s="121"/>
+      <c r="B17" s="122"/>
+      <c r="C17" s="122"/>
+      <c r="D17" s="122"/>
+      <c r="E17" s="123"/>
       <c r="F17" s="27"/>
       <c r="G17" s="62"/>
       <c r="H17" s="62"/>
       <c r="I17" s="2"/>
-      <c r="J17" s="117"/>
-      <c r="K17" s="118"/>
+      <c r="J17" s="135"/>
+      <c r="K17" s="136"/>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="101"/>
-      <c r="B18" s="102"/>
-      <c r="C18" s="102"/>
-      <c r="D18" s="102"/>
-      <c r="E18" s="103"/>
+      <c r="A18" s="121"/>
+      <c r="B18" s="122"/>
+      <c r="C18" s="122"/>
+      <c r="D18" s="122"/>
+      <c r="E18" s="123"/>
       <c r="F18" s="27"/>
       <c r="G18" s="62"/>
       <c r="H18" s="62"/>
       <c r="I18" s="8"/>
-      <c r="J18" s="117"/>
-      <c r="K18" s="118"/>
+      <c r="J18" s="135"/>
+      <c r="K18" s="136"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="104"/>
-      <c r="B19" s="105"/>
-      <c r="C19" s="105"/>
-      <c r="D19" s="105"/>
-      <c r="E19" s="106"/>
+      <c r="A19" s="124"/>
+      <c r="B19" s="125"/>
+      <c r="C19" s="125"/>
+      <c r="D19" s="125"/>
+      <c r="E19" s="126"/>
       <c r="F19" s="63"/>
       <c r="G19" s="62"/>
       <c r="H19" s="62"/>
       <c r="I19" s="27"/>
-      <c r="J19" s="117"/>
-      <c r="K19" s="118"/>
+      <c r="J19" s="135"/>
+      <c r="K19" s="136"/>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="32"/>
@@ -2899,8 +2899,8 @@
       <c r="G20" s="64"/>
       <c r="H20" s="62"/>
       <c r="I20" s="27"/>
-      <c r="J20" s="117"/>
-      <c r="K20" s="118"/>
+      <c r="J20" s="135"/>
+      <c r="K20" s="136"/>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="32"/>
@@ -2912,8 +2912,8 @@
       <c r="G21" s="62"/>
       <c r="H21" s="62"/>
       <c r="I21" s="27"/>
-      <c r="J21" s="117"/>
-      <c r="K21" s="118"/>
+      <c r="J21" s="135"/>
+      <c r="K21" s="136"/>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="32"/>
@@ -2925,8 +2925,8 @@
       <c r="G22" s="62"/>
       <c r="H22" s="62"/>
       <c r="I22" s="27"/>
-      <c r="J22" s="117"/>
-      <c r="K22" s="118"/>
+      <c r="J22" s="135"/>
+      <c r="K22" s="136"/>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="32"/>
@@ -2938,8 +2938,8 @@
       <c r="G23" s="27"/>
       <c r="H23" s="27"/>
       <c r="I23" s="27"/>
-      <c r="J23" s="117"/>
-      <c r="K23" s="118"/>
+      <c r="J23" s="135"/>
+      <c r="K23" s="136"/>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" s="32"/>
@@ -2951,8 +2951,8 @@
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
-      <c r="J24" s="117"/>
-      <c r="K24" s="118"/>
+      <c r="J24" s="135"/>
+      <c r="K24" s="136"/>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="32"/>
@@ -2964,90 +2964,90 @@
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
       <c r="I25" s="9"/>
-      <c r="J25" s="117"/>
-      <c r="K25" s="118"/>
+      <c r="J25" s="135"/>
+      <c r="K25" s="136"/>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="83"/>
-      <c r="B26" s="80"/>
-      <c r="C26" s="80"/>
-      <c r="D26" s="80"/>
-      <c r="E26" s="84"/>
+      <c r="A26" s="105"/>
+      <c r="B26" s="94"/>
+      <c r="C26" s="94"/>
+      <c r="D26" s="94"/>
+      <c r="E26" s="106"/>
       <c r="F26" s="66"/>
       <c r="G26" s="67"/>
       <c r="H26" s="8"/>
       <c r="I26" s="9"/>
-      <c r="J26" s="117"/>
-      <c r="K26" s="118"/>
+      <c r="J26" s="135"/>
+      <c r="K26" s="136"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="80"/>
-      <c r="B27" s="80"/>
-      <c r="C27" s="80"/>
-      <c r="D27" s="80"/>
-      <c r="E27" s="84"/>
+      <c r="A27" s="94"/>
+      <c r="B27" s="94"/>
+      <c r="C27" s="94"/>
+      <c r="D27" s="94"/>
+      <c r="E27" s="106"/>
       <c r="F27" s="68"/>
       <c r="G27" s="67"/>
       <c r="H27" s="8"/>
       <c r="I27" s="9"/>
-      <c r="J27" s="117"/>
-      <c r="K27" s="118"/>
+      <c r="J27" s="135"/>
+      <c r="K27" s="136"/>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="80"/>
-      <c r="B28" s="80"/>
-      <c r="C28" s="80"/>
-      <c r="D28" s="80"/>
-      <c r="E28" s="84"/>
+      <c r="A28" s="94"/>
+      <c r="B28" s="94"/>
+      <c r="C28" s="94"/>
+      <c r="D28" s="94"/>
+      <c r="E28" s="106"/>
       <c r="F28" s="68"/>
       <c r="G28" s="67"/>
       <c r="H28" s="8"/>
       <c r="I28" s="9"/>
-      <c r="J28" s="117"/>
-      <c r="K28" s="118"/>
+      <c r="J28" s="135"/>
+      <c r="K28" s="136"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="80"/>
-      <c r="B29" s="80"/>
-      <c r="C29" s="80"/>
-      <c r="D29" s="80"/>
-      <c r="E29" s="84"/>
+      <c r="A29" s="94"/>
+      <c r="B29" s="94"/>
+      <c r="C29" s="94"/>
+      <c r="D29" s="94"/>
+      <c r="E29" s="106"/>
       <c r="F29" s="69"/>
       <c r="G29" s="70"/>
       <c r="H29" s="65"/>
       <c r="I29" s="23"/>
-      <c r="J29" s="117"/>
-      <c r="K29" s="118"/>
+      <c r="J29" s="135"/>
+      <c r="K29" s="136"/>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="85"/>
-      <c r="B30" s="85"/>
-      <c r="C30" s="85"/>
-      <c r="D30" s="85"/>
-      <c r="E30" s="86"/>
+      <c r="A30" s="107"/>
+      <c r="B30" s="107"/>
+      <c r="C30" s="107"/>
+      <c r="D30" s="107"/>
+      <c r="E30" s="108"/>
       <c r="F30" s="49"/>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
-      <c r="J30" s="117"/>
-      <c r="K30" s="118"/>
+      <c r="J30" s="135"/>
+      <c r="K30" s="136"/>
     </row>
     <row r="31" spans="1:11" ht="15.75">
-      <c r="A31" s="71" t="s">
+      <c r="A31" s="137" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="72"/>
-      <c r="C31" s="73"/>
+      <c r="B31" s="90"/>
+      <c r="C31" s="97"/>
       <c r="D31" s="50"/>
-      <c r="E31" s="74"/>
-      <c r="F31" s="75"/>
-      <c r="G31" s="75"/>
-      <c r="H31" s="75"/>
-      <c r="I31" s="76" t="s">
+      <c r="E31" s="138"/>
+      <c r="F31" s="139"/>
+      <c r="G31" s="139"/>
+      <c r="H31" s="139"/>
+      <c r="I31" s="140" t="s">
         <v>16</v>
       </c>
-      <c r="J31" s="77"/>
-      <c r="K31" s="78"/>
+      <c r="J31" s="141"/>
+      <c r="K31" s="142"/>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" s="37"/>
@@ -3055,12 +3055,12 @@
       <c r="C32" s="4"/>
       <c r="D32" s="38"/>
       <c r="E32" s="3"/>
-      <c r="F32" s="79"/>
-      <c r="G32" s="80"/>
-      <c r="H32" s="81"/>
-      <c r="I32" s="79"/>
-      <c r="J32" s="80"/>
-      <c r="K32" s="82"/>
+      <c r="F32" s="143"/>
+      <c r="G32" s="94"/>
+      <c r="H32" s="110"/>
+      <c r="I32" s="143"/>
+      <c r="J32" s="94"/>
+      <c r="K32" s="144"/>
     </row>
     <row r="33" spans="1:11">
       <c r="A33" s="39"/>
@@ -3139,27 +3139,16 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="E1:G2"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="A26:E30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="E31:H31"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J30:K30"/>
     <mergeCell ref="A14:E19"/>
     <mergeCell ref="A5:C6"/>
     <mergeCell ref="E5:G5"/>
@@ -3176,16 +3165,27 @@
     <mergeCell ref="A11:E11"/>
     <mergeCell ref="F11:K11"/>
     <mergeCell ref="A12:E13"/>
-    <mergeCell ref="A26:E30"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="E31:H31"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="E1:G2"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J26:K26"/>
   </mergeCells>
   <conditionalFormatting sqref="F12:G15 I12 F17:F22 G17:G19 G21:G22">
     <cfRule type="expression" dxfId="3" priority="1">

</xml_diff>

<commit_message>
feat: add inline timeline badges and live parcel counter, also update excel for mohammedia one if they will use it
</commit_message>
<xml_diff>
--- a/dummy-content/ECHEC-RETOUR_CLIENT-CASABLANCA.xlsx
+++ b/dummy-content/ECHEC-RETOUR_CLIENT-CASABLANCA.xlsx
@@ -1,22 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User1\Desktop\GoFleet-Enhancer\dummy-content\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\simok\Bureau\GoFleet-Enhancer\dummy-content\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEC0E857-1BC1-4997-AA17-053272EDFA2F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD93109A-227B-48BD-805E-7B20E976355F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12110" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="ECHEC CASA" sheetId="5" r:id="rId1"/>
-    <sheet name="RTC CASA" sheetId="6" r:id="rId2"/>
+    <sheet name="ECHEC MOHAMMEDIA" sheetId="5" r:id="rId1"/>
+    <sheet name="RTC MOHAMMEDIA" sheetId="6" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -33,9 +46,6 @@
   </si>
   <si>
     <t>N° Expedition</t>
-  </si>
-  <si>
-    <t>GO FLEET CASABLANCA</t>
   </si>
   <si>
     <t>ENTREPOT MARJANE MALL</t>
@@ -94,6 +104,9 @@
   </si>
   <si>
     <t>GOFEMM20052025002</t>
+  </si>
+  <si>
+    <t>GO FLEET MOHAMMEDIA</t>
   </si>
 </sst>
 </file>
@@ -1273,14 +1286,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="160">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+  <cellXfs count="158">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="13" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1296,83 +1309,81 @@
     <xf numFmtId="0" fontId="17" fillId="15" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="23" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="17" fillId="15" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="21" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="11" fontId="16" fillId="21" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="20" fillId="19" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="19" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="15" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="69" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="69" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="71" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="71" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="21" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="16" fillId="13" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1382,7 +1393,7 @@
     <xf numFmtId="11" fontId="15" fillId="21" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="15" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1403,10 +1414,107 @@
     <xf numFmtId="0" fontId="15" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="65" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="15" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1415,7 +1523,7 @@
     <xf numFmtId="0" fontId="2" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1435,106 +1543,18 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="19" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="65" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="17" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1549,15 +1569,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="20" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="19" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1879,123 +1890,123 @@
     <tabColor rgb="FF003399"/>
   </sheetPr>
   <dimension ref="A1:K67"/>
-  <sheetFormatPr defaultRowHeight="12.5"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
-    <col min="1" max="1" width="23.54296875" style="28" customWidth="1"/>
-    <col min="2" max="2" width="13.26953125" style="28" customWidth="1"/>
-    <col min="3" max="3" width="4.90625" style="28" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="8.7265625" style="28"/>
-    <col min="5" max="5" width="29.81640625" style="28" customWidth="1"/>
-    <col min="6" max="9" width="14.54296875" style="28" customWidth="1"/>
-    <col min="10" max="10" width="8.7265625" style="28"/>
-    <col min="11" max="11" width="17.453125" style="28" customWidth="1"/>
+    <col min="1" max="1" width="23.5703125" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" customWidth="1"/>
+    <col min="3" max="3" width="4.85546875" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="8.7109375"/>
+    <col min="5" max="5" width="29.85546875" customWidth="1"/>
+    <col min="6" max="9" width="14.5703125" customWidth="1"/>
+    <col min="10" max="10" width="8.7109375"/>
+    <col min="11" max="11" width="17.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.5" customHeight="1">
-      <c r="A1" s="73"/>
-      <c r="B1" s="74"/>
-      <c r="C1" s="74"/>
-      <c r="D1" s="53"/>
-      <c r="E1" s="78" t="s">
+    <row r="1" spans="1:11" ht="15.6" customHeight="1">
+      <c r="A1" s="126"/>
+      <c r="B1" s="127"/>
+      <c r="C1" s="127"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="131" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="79"/>
-      <c r="G1" s="80"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="84" t="s">
+      <c r="F1" s="132"/>
+      <c r="G1" s="133"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="137" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="85"/>
-      <c r="K1" s="86"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.5">
-      <c r="A2" s="75"/>
-      <c r="B2" s="76"/>
-      <c r="C2" s="77"/>
-      <c r="D2" s="53"/>
-      <c r="E2" s="81"/>
-      <c r="F2" s="82"/>
-      <c r="G2" s="83"/>
+      <c r="J1" s="138"/>
+      <c r="K1" s="139"/>
+    </row>
+    <row r="2" spans="1:11" ht="15.75">
+      <c r="A2" s="128"/>
+      <c r="B2" s="129"/>
+      <c r="C2" s="130"/>
+      <c r="D2" s="51"/>
+      <c r="E2" s="134"/>
+      <c r="F2" s="135"/>
+      <c r="G2" s="136"/>
       <c r="H2" s="15"/>
-      <c r="I2" s="87">
+      <c r="I2" s="140">
         <f ca="1">TODAY()</f>
-        <v>45833</v>
-      </c>
-      <c r="J2" s="82"/>
-      <c r="K2" s="83"/>
+        <v>46250</v>
+      </c>
+      <c r="J2" s="135"/>
+      <c r="K2" s="136"/>
     </row>
     <row r="3" spans="1:11">
-      <c r="A3" s="32"/>
+      <c r="A3" s="30"/>
       <c r="B3" s="22"/>
       <c r="C3" s="13"/>
-      <c r="D3" s="36"/>
+      <c r="D3" s="34"/>
       <c r="E3" s="11"/>
       <c r="F3" s="22"/>
-      <c r="G3" s="33"/>
+      <c r="G3" s="31"/>
       <c r="H3" s="25"/>
       <c r="I3" s="22"/>
       <c r="J3" s="22"/>
-      <c r="K3" s="33"/>
-    </row>
-    <row r="4" spans="1:11" ht="17">
-      <c r="A4" s="88" t="s">
+      <c r="K3" s="31"/>
+    </row>
+    <row r="4" spans="1:11" ht="17.25">
+      <c r="A4" s="141" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="89"/>
-      <c r="C4" s="90"/>
-      <c r="D4" s="52"/>
+      <c r="B4" s="111"/>
+      <c r="C4" s="70"/>
+      <c r="D4" s="50"/>
       <c r="E4" s="16" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F4" s="1"/>
-      <c r="G4" s="55"/>
+      <c r="G4" s="53"/>
       <c r="H4" s="15"/>
       <c r="I4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="91"/>
-      <c r="K4" s="92"/>
-    </row>
-    <row r="5" spans="1:11" ht="18.5">
-      <c r="A5" s="93" t="s">
+      <c r="J4" s="142"/>
+      <c r="K4" s="113"/>
+    </row>
+    <row r="5" spans="1:11" ht="18.75">
+      <c r="A5" s="119" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="78"/>
+      <c r="C5" s="94"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="120" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="94"/>
-      <c r="C5" s="95"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="98" t="s">
-        <v>5</v>
-      </c>
-      <c r="F5" s="99"/>
-      <c r="G5" s="100"/>
+      <c r="F5" s="121"/>
+      <c r="G5" s="122"/>
       <c r="H5" s="22"/>
       <c r="I5" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="J5" s="123"/>
+      <c r="K5" s="113"/>
+    </row>
+    <row r="6" spans="1:11" ht="15.75">
+      <c r="A6" s="95"/>
+      <c r="B6" s="70"/>
+      <c r="C6" s="71"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="124" t="s">
         <v>6</v>
       </c>
-      <c r="J5" s="101"/>
-      <c r="K5" s="92"/>
-    </row>
-    <row r="6" spans="1:11" ht="15.5">
-      <c r="A6" s="96"/>
-      <c r="B6" s="90"/>
-      <c r="C6" s="97"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="102" t="s">
+      <c r="F6" s="70"/>
+      <c r="G6" s="87"/>
+      <c r="H6" s="44"/>
+      <c r="I6" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="90"/>
-      <c r="G6" s="103"/>
-      <c r="H6" s="46"/>
-      <c r="I6" s="21" t="s">
-        <v>8</v>
-      </c>
-      <c r="J6" s="104">
+      <c r="J6" s="125">
         <v>1230</v>
       </c>
-      <c r="K6" s="92"/>
+      <c r="K6" s="113"/>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="32"/>
+      <c r="A7" s="30"/>
       <c r="B7" s="22"/>
       <c r="C7" s="22"/>
       <c r="D7" s="22"/>
@@ -2005,52 +2016,52 @@
       <c r="H7" s="22"/>
       <c r="I7" s="22"/>
       <c r="J7" s="22"/>
-      <c r="K7" s="33"/>
-    </row>
-    <row r="8" spans="1:11" ht="15.5">
-      <c r="A8" s="127" t="s">
+      <c r="K7" s="31"/>
+    </row>
+    <row r="8" spans="1:11" ht="15.75">
+      <c r="A8" s="105" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="54" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="56" t="s">
+      <c r="C8" s="107" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="129" t="s">
+      <c r="D8" s="108"/>
+      <c r="E8" s="109"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="110" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="130"/>
-      <c r="E8" s="131"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="132" t="s">
+      <c r="H8" s="111"/>
+      <c r="I8" s="14"/>
+      <c r="J8" s="112" t="s">
         <v>12</v>
       </c>
-      <c r="H8" s="89"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="133" t="s">
+      <c r="K8" s="113"/>
+    </row>
+    <row r="9" spans="1:11" ht="17.25">
+      <c r="A9" s="106"/>
+      <c r="B9" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="K8" s="92"/>
-    </row>
-    <row r="9" spans="1:11" ht="17">
-      <c r="A9" s="128"/>
-      <c r="B9" s="57" t="s">
+      <c r="C9" s="114" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="134" t="s">
-        <v>15</v>
-      </c>
-      <c r="D9" s="90"/>
-      <c r="E9" s="110"/>
+      <c r="D9" s="70"/>
+      <c r="E9" s="79"/>
       <c r="F9" s="22"/>
-      <c r="G9" s="109">
+      <c r="G9" s="85">
         <v>1</v>
       </c>
-      <c r="H9" s="110"/>
+      <c r="H9" s="79"/>
       <c r="I9" s="22"/>
-      <c r="J9" s="111"/>
-      <c r="K9" s="103"/>
+      <c r="J9" s="86"/>
+      <c r="K9" s="87"/>
     </row>
     <row r="10" spans="1:11">
-      <c r="A10" s="32"/>
+      <c r="A10" s="30"/>
       <c r="B10" s="22"/>
       <c r="C10" s="22"/>
       <c r="D10" s="22"/>
@@ -2060,173 +2071,173 @@
       <c r="H10" s="19"/>
       <c r="I10" s="19"/>
       <c r="J10" s="22"/>
-      <c r="K10" s="34"/>
-    </row>
-    <row r="11" spans="1:11" ht="18.5">
-      <c r="A11" s="112" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="113"/>
-      <c r="C11" s="113"/>
-      <c r="D11" s="113"/>
-      <c r="E11" s="114"/>
-      <c r="F11" s="115"/>
-      <c r="G11" s="113"/>
-      <c r="H11" s="113"/>
-      <c r="I11" s="113"/>
-      <c r="J11" s="113"/>
-      <c r="K11" s="116"/>
+      <c r="K10" s="32"/>
+    </row>
+    <row r="11" spans="1:11" ht="18.75">
+      <c r="A11" s="88" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="89"/>
+      <c r="C11" s="89"/>
+      <c r="D11" s="89"/>
+      <c r="E11" s="90"/>
+      <c r="F11" s="91"/>
+      <c r="G11" s="89"/>
+      <c r="H11" s="89"/>
+      <c r="I11" s="89"/>
+      <c r="J11" s="89"/>
+      <c r="K11" s="92"/>
     </row>
     <row r="12" spans="1:11">
-      <c r="A12" s="117" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" s="95"/>
-      <c r="C12" s="95"/>
-      <c r="D12" s="95"/>
-      <c r="E12" s="110"/>
-      <c r="F12" s="59"/>
-      <c r="G12" s="31"/>
-      <c r="H12" s="60"/>
-      <c r="I12" s="31"/>
-      <c r="J12" s="135"/>
-      <c r="K12" s="136"/>
+      <c r="A12" s="93" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="94"/>
+      <c r="C12" s="94"/>
+      <c r="D12" s="94"/>
+      <c r="E12" s="79"/>
+      <c r="F12" s="57"/>
+      <c r="G12" s="29"/>
+      <c r="H12" s="58"/>
+      <c r="I12" s="29"/>
+      <c r="J12" s="115"/>
+      <c r="K12" s="116"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="96"/>
-      <c r="B13" s="90"/>
-      <c r="C13" s="90"/>
-      <c r="D13" s="90"/>
-      <c r="E13" s="97"/>
+      <c r="A13" s="95"/>
+      <c r="B13" s="70"/>
+      <c r="C13" s="70"/>
+      <c r="D13" s="70"/>
+      <c r="E13" s="71"/>
       <c r="F13" s="27"/>
-      <c r="G13" s="61"/>
-      <c r="H13" s="62"/>
+      <c r="G13" s="59"/>
+      <c r="H13" s="60"/>
       <c r="I13" s="2"/>
-      <c r="J13" s="71"/>
-      <c r="K13" s="72"/>
+      <c r="J13" s="117"/>
+      <c r="K13" s="118"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="118" t="str">
+      <c r="A14" s="96" t="str">
         <f>"*"&amp;A12&amp;"*"</f>
         <v>*GOFEMM20052025001*</v>
       </c>
-      <c r="B14" s="119"/>
-      <c r="C14" s="119"/>
-      <c r="D14" s="119"/>
-      <c r="E14" s="120"/>
+      <c r="B14" s="97"/>
+      <c r="C14" s="97"/>
+      <c r="D14" s="97"/>
+      <c r="E14" s="98"/>
       <c r="F14" s="27"/>
-      <c r="G14" s="62"/>
-      <c r="H14" s="62"/>
+      <c r="G14" s="60"/>
+      <c r="H14" s="60"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="71"/>
-      <c r="K14" s="72"/>
+      <c r="J14" s="117"/>
+      <c r="K14" s="118"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="121"/>
-      <c r="B15" s="122"/>
-      <c r="C15" s="122"/>
-      <c r="D15" s="122"/>
-      <c r="E15" s="123"/>
+      <c r="A15" s="99"/>
+      <c r="B15" s="100"/>
+      <c r="C15" s="100"/>
+      <c r="D15" s="100"/>
+      <c r="E15" s="101"/>
       <c r="F15" s="27"/>
-      <c r="G15" s="62"/>
-      <c r="H15" s="62"/>
+      <c r="G15" s="60"/>
+      <c r="H15" s="60"/>
       <c r="I15" s="2"/>
-      <c r="J15" s="71"/>
-      <c r="K15" s="72"/>
+      <c r="J15" s="117"/>
+      <c r="K15" s="118"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="121"/>
-      <c r="B16" s="122"/>
-      <c r="C16" s="122"/>
-      <c r="D16" s="122"/>
-      <c r="E16" s="123"/>
+      <c r="A16" s="99"/>
+      <c r="B16" s="100"/>
+      <c r="C16" s="100"/>
+      <c r="D16" s="100"/>
+      <c r="E16" s="101"/>
       <c r="F16" s="8"/>
-      <c r="G16" s="62"/>
-      <c r="H16" s="62"/>
+      <c r="G16" s="60"/>
+      <c r="H16" s="60"/>
       <c r="I16" s="2"/>
-      <c r="J16" s="71"/>
-      <c r="K16" s="72"/>
+      <c r="J16" s="117"/>
+      <c r="K16" s="118"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="121"/>
-      <c r="B17" s="122"/>
-      <c r="C17" s="122"/>
-      <c r="D17" s="122"/>
-      <c r="E17" s="123"/>
+      <c r="A17" s="99"/>
+      <c r="B17" s="100"/>
+      <c r="C17" s="100"/>
+      <c r="D17" s="100"/>
+      <c r="E17" s="101"/>
       <c r="F17" s="27"/>
-      <c r="G17" s="62"/>
-      <c r="H17" s="62"/>
+      <c r="G17" s="60"/>
+      <c r="H17" s="60"/>
       <c r="I17" s="2"/>
-      <c r="J17" s="71"/>
-      <c r="K17" s="72"/>
+      <c r="J17" s="117"/>
+      <c r="K17" s="118"/>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="121"/>
-      <c r="B18" s="122"/>
-      <c r="C18" s="122"/>
-      <c r="D18" s="122"/>
-      <c r="E18" s="123"/>
+      <c r="A18" s="99"/>
+      <c r="B18" s="100"/>
+      <c r="C18" s="100"/>
+      <c r="D18" s="100"/>
+      <c r="E18" s="101"/>
       <c r="F18" s="27"/>
-      <c r="G18" s="62"/>
-      <c r="H18" s="62"/>
+      <c r="G18" s="60"/>
+      <c r="H18" s="60"/>
       <c r="I18" s="8"/>
-      <c r="J18" s="71"/>
-      <c r="K18" s="72"/>
+      <c r="J18" s="117"/>
+      <c r="K18" s="118"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="124"/>
-      <c r="B19" s="125"/>
-      <c r="C19" s="125"/>
-      <c r="D19" s="125"/>
-      <c r="E19" s="126"/>
-      <c r="F19" s="63"/>
-      <c r="G19" s="62"/>
-      <c r="H19" s="62"/>
+      <c r="A19" s="102"/>
+      <c r="B19" s="103"/>
+      <c r="C19" s="103"/>
+      <c r="D19" s="103"/>
+      <c r="E19" s="104"/>
+      <c r="F19" s="61"/>
+      <c r="G19" s="60"/>
+      <c r="H19" s="60"/>
       <c r="I19" s="27"/>
-      <c r="J19" s="71"/>
-      <c r="K19" s="72"/>
+      <c r="J19" s="117"/>
+      <c r="K19" s="118"/>
     </row>
     <row r="20" spans="1:11">
-      <c r="A20" s="32"/>
+      <c r="A20" s="30"/>
       <c r="B20" s="22"/>
       <c r="C20" s="22"/>
       <c r="D20" s="22"/>
       <c r="E20" s="22"/>
-      <c r="F20" s="63"/>
-      <c r="G20" s="64"/>
-      <c r="H20" s="62"/>
+      <c r="F20" s="61"/>
+      <c r="G20" s="62"/>
+      <c r="H20" s="60"/>
       <c r="I20" s="27"/>
-      <c r="J20" s="71"/>
-      <c r="K20" s="72"/>
+      <c r="J20" s="117"/>
+      <c r="K20" s="118"/>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="32"/>
+      <c r="A21" s="30"/>
       <c r="B21" s="22"/>
       <c r="C21" s="22"/>
       <c r="D21" s="22"/>
-      <c r="E21" s="35"/>
-      <c r="F21" s="63"/>
-      <c r="G21" s="62"/>
-      <c r="H21" s="62"/>
+      <c r="E21" s="33"/>
+      <c r="F21" s="61"/>
+      <c r="G21" s="60"/>
+      <c r="H21" s="60"/>
       <c r="I21" s="27"/>
-      <c r="J21" s="71"/>
-      <c r="K21" s="72"/>
+      <c r="J21" s="117"/>
+      <c r="K21" s="118"/>
     </row>
     <row r="22" spans="1:11">
-      <c r="A22" s="32"/>
+      <c r="A22" s="30"/>
       <c r="B22" s="22"/>
       <c r="C22" s="22"/>
       <c r="D22" s="22"/>
-      <c r="E22" s="35"/>
-      <c r="F22" s="63"/>
-      <c r="G22" s="62"/>
-      <c r="H22" s="62"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="61"/>
+      <c r="G22" s="60"/>
+      <c r="H22" s="60"/>
       <c r="I22" s="27"/>
-      <c r="J22" s="71"/>
-      <c r="K22" s="72"/>
+      <c r="J22" s="117"/>
+      <c r="K22" s="118"/>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="32"/>
+      <c r="A23" s="30"/>
       <c r="B23" s="22"/>
       <c r="C23" s="22"/>
       <c r="D23" s="22"/>
@@ -2235,11 +2246,11 @@
       <c r="G23" s="27"/>
       <c r="H23" s="27"/>
       <c r="I23" s="27"/>
-      <c r="J23" s="71"/>
-      <c r="K23" s="72"/>
+      <c r="J23" s="117"/>
+      <c r="K23" s="118"/>
     </row>
     <row r="24" spans="1:11">
-      <c r="A24" s="32"/>
+      <c r="A24" s="30"/>
       <c r="B24" s="22"/>
       <c r="C24" s="22"/>
       <c r="D24" s="22"/>
@@ -2248,187 +2259,164 @@
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
-      <c r="J24" s="71"/>
-      <c r="K24" s="72"/>
+      <c r="J24" s="117"/>
+      <c r="K24" s="118"/>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="32"/>
+      <c r="A25" s="30"/>
       <c r="B25" s="22"/>
       <c r="C25" s="22"/>
       <c r="D25" s="22"/>
       <c r="E25" s="22"/>
-      <c r="F25" s="65"/>
+      <c r="F25" s="63"/>
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
       <c r="I25" s="9"/>
-      <c r="J25" s="71"/>
-      <c r="K25" s="72"/>
+      <c r="J25" s="117"/>
+      <c r="K25" s="118"/>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="105"/>
-      <c r="B26" s="94"/>
-      <c r="C26" s="94"/>
-      <c r="D26" s="94"/>
-      <c r="E26" s="106"/>
-      <c r="F26" s="66"/>
-      <c r="G26" s="67"/>
+      <c r="A26" s="81"/>
+      <c r="B26" s="78"/>
+      <c r="C26" s="78"/>
+      <c r="D26" s="78"/>
+      <c r="E26" s="82"/>
+      <c r="F26" s="64"/>
+      <c r="G26" s="65"/>
       <c r="H26" s="8"/>
       <c r="I26" s="9"/>
-      <c r="J26" s="71"/>
-      <c r="K26" s="72"/>
+      <c r="J26" s="117"/>
+      <c r="K26" s="118"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="94"/>
-      <c r="B27" s="94"/>
-      <c r="C27" s="94"/>
-      <c r="D27" s="94"/>
-      <c r="E27" s="106"/>
-      <c r="F27" s="68"/>
-      <c r="G27" s="67"/>
+      <c r="A27" s="78"/>
+      <c r="B27" s="78"/>
+      <c r="C27" s="78"/>
+      <c r="D27" s="78"/>
+      <c r="E27" s="82"/>
+      <c r="F27" s="66"/>
+      <c r="G27" s="65"/>
       <c r="H27" s="8"/>
       <c r="I27" s="9"/>
-      <c r="J27" s="71"/>
-      <c r="K27" s="72"/>
+      <c r="J27" s="117"/>
+      <c r="K27" s="118"/>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="94"/>
-      <c r="B28" s="94"/>
-      <c r="C28" s="94"/>
-      <c r="D28" s="94"/>
-      <c r="E28" s="106"/>
-      <c r="F28" s="68"/>
-      <c r="G28" s="67"/>
+      <c r="A28" s="78"/>
+      <c r="B28" s="78"/>
+      <c r="C28" s="78"/>
+      <c r="D28" s="78"/>
+      <c r="E28" s="82"/>
+      <c r="F28" s="66"/>
+      <c r="G28" s="65"/>
       <c r="H28" s="8"/>
       <c r="I28" s="9"/>
-      <c r="J28" s="71"/>
-      <c r="K28" s="72"/>
+      <c r="J28" s="117"/>
+      <c r="K28" s="118"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="94"/>
-      <c r="B29" s="94"/>
-      <c r="C29" s="94"/>
-      <c r="D29" s="94"/>
-      <c r="E29" s="106"/>
-      <c r="F29" s="69"/>
-      <c r="G29" s="70"/>
-      <c r="H29" s="65"/>
+      <c r="A29" s="78"/>
+      <c r="B29" s="78"/>
+      <c r="C29" s="78"/>
+      <c r="D29" s="78"/>
+      <c r="E29" s="82"/>
+      <c r="F29" s="67"/>
+      <c r="G29" s="68"/>
+      <c r="H29" s="63"/>
       <c r="I29" s="23"/>
-      <c r="J29" s="71"/>
-      <c r="K29" s="72"/>
+      <c r="J29" s="117"/>
+      <c r="K29" s="118"/>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="107"/>
-      <c r="B30" s="107"/>
-      <c r="C30" s="107"/>
-      <c r="D30" s="107"/>
-      <c r="E30" s="108"/>
-      <c r="F30" s="49"/>
+      <c r="A30" s="83"/>
+      <c r="B30" s="83"/>
+      <c r="C30" s="83"/>
+      <c r="D30" s="83"/>
+      <c r="E30" s="84"/>
+      <c r="F30" s="47"/>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
-      <c r="J30" s="71"/>
-      <c r="K30" s="72"/>
-    </row>
-    <row r="31" spans="1:11" ht="15.5">
-      <c r="A31" s="137" t="s">
+      <c r="J30" s="117"/>
+      <c r="K30" s="118"/>
+    </row>
+    <row r="31" spans="1:11" ht="15.75">
+      <c r="A31" s="69" t="s">
+        <v>16</v>
+      </c>
+      <c r="B31" s="70"/>
+      <c r="C31" s="71"/>
+      <c r="D31" s="48"/>
+      <c r="E31" s="72"/>
+      <c r="F31" s="73"/>
+      <c r="G31" s="73"/>
+      <c r="H31" s="73"/>
+      <c r="I31" s="74" t="s">
         <v>17</v>
       </c>
-      <c r="B31" s="90"/>
-      <c r="C31" s="97"/>
-      <c r="D31" s="50"/>
-      <c r="E31" s="138"/>
-      <c r="F31" s="139"/>
-      <c r="G31" s="139"/>
-      <c r="H31" s="139"/>
-      <c r="I31" s="140" t="s">
-        <v>18</v>
-      </c>
-      <c r="J31" s="141"/>
-      <c r="K31" s="142"/>
+      <c r="J31" s="75"/>
+      <c r="K31" s="76"/>
     </row>
     <row r="32" spans="1:11">
-      <c r="A32" s="37"/>
-      <c r="B32" s="54"/>
+      <c r="A32" s="35"/>
+      <c r="B32" s="52"/>
       <c r="C32" s="4"/>
-      <c r="D32" s="38"/>
+      <c r="D32" s="36"/>
       <c r="E32" s="3"/>
-      <c r="F32" s="143"/>
-      <c r="G32" s="94"/>
-      <c r="H32" s="110"/>
-      <c r="I32" s="143"/>
-      <c r="J32" s="94"/>
-      <c r="K32" s="144"/>
+      <c r="F32" s="77"/>
+      <c r="G32" s="78"/>
+      <c r="H32" s="79"/>
+      <c r="I32" s="77"/>
+      <c r="J32" s="78"/>
+      <c r="K32" s="80"/>
     </row>
     <row r="33" spans="1:11">
-      <c r="A33" s="39"/>
-      <c r="B33" s="45"/>
-      <c r="C33" s="41"/>
-      <c r="D33" s="42"/>
-      <c r="E33" s="43"/>
-      <c r="F33" s="40"/>
-      <c r="G33" s="40"/>
-      <c r="H33" s="44"/>
-      <c r="I33" s="40"/>
-      <c r="J33" s="40"/>
-      <c r="K33" s="45"/>
-    </row>
-    <row r="34" spans="1:11">
-      <c r="A34" s="30"/>
-      <c r="B34" s="30"/>
-      <c r="C34" s="30"/>
-      <c r="D34" s="30"/>
-      <c r="E34" s="30"/>
-    </row>
-    <row r="35" spans="1:11">
-      <c r="A35" s="30"/>
-      <c r="B35" s="30"/>
-      <c r="C35" s="30"/>
-      <c r="D35" s="30"/>
-      <c r="E35" s="30"/>
-    </row>
-    <row r="36" spans="1:11">
-      <c r="A36" s="30"/>
-    </row>
-    <row r="37" spans="1:11">
-      <c r="A37" s="30"/>
-    </row>
-    <row r="38" spans="1:11">
-      <c r="A38" s="30"/>
-    </row>
-    <row r="45" spans="1:11" ht="15.5">
+      <c r="A33" s="37"/>
+      <c r="B33" s="43"/>
+      <c r="C33" s="39"/>
+      <c r="D33" s="40"/>
+      <c r="E33" s="41"/>
+      <c r="F33" s="38"/>
+      <c r="G33" s="38"/>
+      <c r="H33" s="42"/>
+      <c r="I33" s="38"/>
+      <c r="J33" s="38"/>
+      <c r="K33" s="43"/>
+    </row>
+    <row r="45" spans="1:11" ht="15.75">
       <c r="J45" s="5"/>
     </row>
-    <row r="46" spans="1:11" ht="13">
+    <row r="46" spans="1:11">
       <c r="J46" s="6"/>
     </row>
-    <row r="47" spans="1:11" ht="15.5">
+    <row r="47" spans="1:11" ht="15.75">
       <c r="J47" s="5"/>
     </row>
-    <row r="48" spans="1:11" ht="13">
+    <row r="48" spans="1:11">
       <c r="J48" s="6"/>
     </row>
-    <row r="49" spans="10:10" ht="15.5">
+    <row r="49" spans="10:10" ht="15.75">
       <c r="J49" s="5"/>
     </row>
-    <row r="50" spans="10:10" ht="13">
+    <row r="50" spans="10:10">
       <c r="J50" s="6"/>
     </row>
-    <row r="51" spans="10:10" ht="15.5">
+    <row r="51" spans="10:10" ht="15.75">
       <c r="J51" s="5"/>
     </row>
-    <row r="52" spans="10:10" ht="13">
+    <row r="52" spans="10:10">
       <c r="J52" s="6"/>
     </row>
-    <row r="53" spans="10:10" ht="15.5">
+    <row r="53" spans="10:10" ht="15.75">
       <c r="J53" s="5"/>
     </row>
-    <row r="54" spans="10:10" ht="13">
+    <row r="54" spans="10:10">
       <c r="J54" s="6"/>
     </row>
-    <row r="55" spans="10:10" ht="15.5">
+    <row r="55" spans="10:10" ht="15.75">
       <c r="J55" s="5"/>
     </row>
-    <row r="56" spans="10:10" ht="13">
+    <row r="56" spans="10:10">
       <c r="J56" s="6"/>
     </row>
     <row r="67" spans="11:11">
@@ -2436,11 +2424,32 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="E31:H31"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="E1:G2"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="A5:C6"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="J6:K6"/>
     <mergeCell ref="A26:E30"/>
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="J9:K9"/>
@@ -2457,51 +2466,30 @@
     <mergeCell ref="J13:K13"/>
     <mergeCell ref="J14:K14"/>
     <mergeCell ref="J15:K15"/>
-    <mergeCell ref="A5:C6"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="E6:G6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="E1:G2"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="E31:H31"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="I32:K32"/>
   </mergeCells>
-  <conditionalFormatting sqref="F12:G15 I12 F17:F22 G17:G19 G21:G22">
-    <cfRule type="expression" dxfId="7" priority="1">
-      <formula>COUNTIF($F12:$G35,F12)&gt;1</formula>
+  <conditionalFormatting sqref="G12:G19 F12:F24 I12:I24 H13:H24 G21:G25">
+    <cfRule type="expression" dxfId="7" priority="4">
+      <formula>COUNTIF($F12:$K27,F12)&gt;1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G19 H19:I21 G21">
+    <cfRule type="expression" dxfId="6" priority="3">
+      <formula>COUNTIF($F12:$K27,G19)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G22:I23">
-    <cfRule type="expression" dxfId="6" priority="2">
+    <cfRule type="expression" dxfId="5" priority="2">
       <formula>COUNTIF($F16:$K31,G22)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G19 H19:I21 G21">
-    <cfRule type="expression" dxfId="5" priority="3">
-      <formula>COUNTIF($F12:$K27,G19)&gt;1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F12:F24 G12:G19 I12:I24 H13:H24 G21:G25">
-    <cfRule type="expression" dxfId="4" priority="4">
-      <formula>COUNTIF($F12:$K27,F12)&gt;1</formula>
+  <conditionalFormatting sqref="I12 F12:G15 G17:G19 F17:F22 G21:G22">
+    <cfRule type="expression" dxfId="4" priority="1">
+      <formula>COUNTIF($F12:$G35,F12)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -2519,127 +2507,127 @@
     <tabColor theme="9" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:K67"/>
-  <sheetFormatPr defaultRowHeight="12.5"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
-    <col min="1" max="1" width="23.54296875" style="28" customWidth="1"/>
-    <col min="2" max="2" width="13.26953125" style="28" customWidth="1"/>
-    <col min="3" max="3" width="4.90625" style="28" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="8.7265625" style="28"/>
-    <col min="5" max="5" width="30.26953125" style="28" customWidth="1"/>
-    <col min="6" max="6" width="16.54296875" style="28" customWidth="1"/>
-    <col min="7" max="8" width="15.54296875" style="28" customWidth="1"/>
-    <col min="9" max="9" width="13.7265625" style="28" customWidth="1"/>
-    <col min="10" max="10" width="9.81640625" style="28" customWidth="1"/>
-    <col min="11" max="11" width="16.1796875" style="28" customWidth="1"/>
+    <col min="1" max="1" width="23.5703125" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" customWidth="1"/>
+    <col min="3" max="3" width="4.85546875" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="8.7109375"/>
+    <col min="5" max="5" width="30.28515625" customWidth="1"/>
+    <col min="6" max="6" width="16.5703125" customWidth="1"/>
+    <col min="7" max="8" width="15.5703125" customWidth="1"/>
+    <col min="9" max="9" width="13.7109375" customWidth="1"/>
+    <col min="10" max="10" width="9.85546875" customWidth="1"/>
+    <col min="11" max="11" width="16.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.5" customHeight="1">
-      <c r="A1" s="73" t="s">
+    <row r="1" spans="1:11" ht="15.6" customHeight="1">
+      <c r="A1" s="126" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="127"/>
+      <c r="C1" s="148"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="150" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="74"/>
-      <c r="C1" s="145"/>
-      <c r="D1" s="58"/>
-      <c r="E1" s="147" t="s">
-        <v>20</v>
-      </c>
-      <c r="F1" s="148"/>
-      <c r="G1" s="149"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="84" t="s">
+      <c r="F1" s="151"/>
+      <c r="G1" s="152"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="137" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="85"/>
-      <c r="K1" s="86"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.5">
-      <c r="A2" s="75"/>
-      <c r="B2" s="76"/>
-      <c r="C2" s="146"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="150"/>
-      <c r="F2" s="151"/>
-      <c r="G2" s="152"/>
+      <c r="J1" s="138"/>
+      <c r="K1" s="139"/>
+    </row>
+    <row r="2" spans="1:11" ht="15.75">
+      <c r="A2" s="128"/>
+      <c r="B2" s="129"/>
+      <c r="C2" s="149"/>
+      <c r="D2" s="50"/>
+      <c r="E2" s="153"/>
+      <c r="F2" s="154"/>
+      <c r="G2" s="155"/>
       <c r="H2" s="15"/>
-      <c r="I2" s="87">
+      <c r="I2" s="140">
         <f ca="1">TODAY()</f>
-        <v>45833</v>
-      </c>
-      <c r="J2" s="82"/>
-      <c r="K2" s="83"/>
+        <v>46250</v>
+      </c>
+      <c r="J2" s="135"/>
+      <c r="K2" s="136"/>
     </row>
     <row r="3" spans="1:11">
-      <c r="A3" s="32"/>
+      <c r="A3" s="30"/>
       <c r="B3" s="22"/>
       <c r="C3" s="13"/>
-      <c r="D3" s="36"/>
+      <c r="D3" s="34"/>
       <c r="E3" s="11"/>
       <c r="F3" s="22"/>
-      <c r="G3" s="51"/>
+      <c r="G3" s="49"/>
       <c r="H3" s="25"/>
       <c r="I3" s="22"/>
       <c r="J3" s="22"/>
-      <c r="K3" s="33"/>
-    </row>
-    <row r="4" spans="1:11" ht="17">
-      <c r="A4" s="153" t="s">
+      <c r="K3" s="31"/>
+    </row>
+    <row r="4" spans="1:11" ht="17.25">
+      <c r="A4" s="156" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="154"/>
-      <c r="C4" s="76"/>
-      <c r="D4" s="52"/>
+      <c r="B4" s="157"/>
+      <c r="C4" s="129"/>
+      <c r="D4" s="50"/>
       <c r="E4" s="26" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" s="47"/>
-      <c r="G4" s="48"/>
+        <v>20</v>
+      </c>
+      <c r="F4" s="45"/>
+      <c r="G4" s="46"/>
       <c r="H4" s="15"/>
       <c r="I4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="91"/>
-      <c r="K4" s="92"/>
-    </row>
-    <row r="5" spans="1:11" ht="18.5">
-      <c r="A5" s="155" t="s">
+      <c r="J4" s="142"/>
+      <c r="K4" s="113"/>
+    </row>
+    <row r="5" spans="1:11" ht="18.75">
+      <c r="A5" s="143" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="144"/>
+      <c r="C5" s="130"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="120" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="156"/>
-      <c r="C5" s="77"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="98" t="s">
-        <v>5</v>
-      </c>
-      <c r="F5" s="99"/>
-      <c r="G5" s="100"/>
+      <c r="F5" s="121"/>
+      <c r="G5" s="122"/>
       <c r="H5" s="22"/>
       <c r="I5" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="J5" s="123"/>
+      <c r="K5" s="113"/>
+    </row>
+    <row r="6" spans="1:11" ht="15.75">
+      <c r="A6" s="128"/>
+      <c r="B6" s="129"/>
+      <c r="C6" s="145"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="146" t="s">
         <v>6</v>
       </c>
-      <c r="J5" s="101"/>
-      <c r="K5" s="92"/>
-    </row>
-    <row r="6" spans="1:11" ht="15.5">
-      <c r="A6" s="75"/>
-      <c r="B6" s="76"/>
-      <c r="C6" s="157"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="158" t="s">
+      <c r="F6" s="129"/>
+      <c r="G6" s="147"/>
+      <c r="H6" s="44"/>
+      <c r="I6" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="76"/>
-      <c r="G6" s="159"/>
-      <c r="H6" s="46"/>
-      <c r="I6" s="21" t="s">
-        <v>8</v>
-      </c>
-      <c r="J6" s="104">
+      <c r="J6" s="125">
         <v>1230</v>
       </c>
-      <c r="K6" s="92"/>
+      <c r="K6" s="113"/>
     </row>
     <row r="7" spans="1:11">
-      <c r="A7" s="32"/>
+      <c r="A7" s="30"/>
       <c r="B7" s="22"/>
       <c r="C7" s="22"/>
       <c r="D7" s="22"/>
@@ -2649,52 +2637,52 @@
       <c r="H7" s="22"/>
       <c r="I7" s="22"/>
       <c r="J7" s="22"/>
-      <c r="K7" s="33"/>
-    </row>
-    <row r="8" spans="1:11" ht="15.5">
-      <c r="A8" s="127" t="s">
+      <c r="K7" s="31"/>
+    </row>
+    <row r="8" spans="1:11" ht="15.75">
+      <c r="A8" s="105" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="54" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="56" t="s">
+      <c r="C8" s="107" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="129" t="s">
+      <c r="D8" s="108"/>
+      <c r="E8" s="109"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="110" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="130"/>
-      <c r="E8" s="131"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="132" t="s">
+      <c r="H8" s="111"/>
+      <c r="I8" s="14"/>
+      <c r="J8" s="112" t="s">
         <v>12</v>
       </c>
-      <c r="H8" s="89"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="133" t="s">
+      <c r="K8" s="113"/>
+    </row>
+    <row r="9" spans="1:11" ht="17.25">
+      <c r="A9" s="106"/>
+      <c r="B9" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="K8" s="92"/>
-    </row>
-    <row r="9" spans="1:11" ht="17">
-      <c r="A9" s="128"/>
-      <c r="B9" s="57" t="s">
+      <c r="C9" s="114" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="134" t="s">
-        <v>15</v>
-      </c>
-      <c r="D9" s="90"/>
-      <c r="E9" s="110"/>
+      <c r="D9" s="70"/>
+      <c r="E9" s="79"/>
       <c r="F9" s="22"/>
-      <c r="G9" s="109">
+      <c r="G9" s="85">
         <v>1</v>
       </c>
-      <c r="H9" s="110"/>
+      <c r="H9" s="79"/>
       <c r="I9" s="22"/>
-      <c r="J9" s="111"/>
-      <c r="K9" s="103"/>
+      <c r="J9" s="86"/>
+      <c r="K9" s="87"/>
     </row>
     <row r="10" spans="1:11">
-      <c r="A10" s="32"/>
+      <c r="A10" s="30"/>
       <c r="B10" s="22"/>
       <c r="C10" s="22"/>
       <c r="D10" s="22"/>
@@ -2704,173 +2692,173 @@
       <c r="H10" s="19"/>
       <c r="I10" s="19"/>
       <c r="J10" s="22"/>
-      <c r="K10" s="34"/>
-    </row>
-    <row r="11" spans="1:11" ht="18.5">
-      <c r="A11" s="112" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="113"/>
-      <c r="C11" s="113"/>
-      <c r="D11" s="113"/>
-      <c r="E11" s="114"/>
-      <c r="F11" s="115"/>
-      <c r="G11" s="113"/>
-      <c r="H11" s="113"/>
-      <c r="I11" s="113"/>
-      <c r="J11" s="113"/>
-      <c r="K11" s="116"/>
-    </row>
-    <row r="12" spans="1:11" ht="12.5" customHeight="1">
-      <c r="A12" s="117" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" s="95"/>
-      <c r="C12" s="95"/>
-      <c r="D12" s="95"/>
-      <c r="E12" s="110"/>
-      <c r="F12" s="59"/>
-      <c r="G12" s="31"/>
-      <c r="H12" s="60"/>
-      <c r="I12" s="31"/>
-      <c r="J12" s="135"/>
-      <c r="K12" s="136"/>
+      <c r="K10" s="32"/>
+    </row>
+    <row r="11" spans="1:11" ht="18.75">
+      <c r="A11" s="88" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="89"/>
+      <c r="C11" s="89"/>
+      <c r="D11" s="89"/>
+      <c r="E11" s="90"/>
+      <c r="F11" s="91"/>
+      <c r="G11" s="89"/>
+      <c r="H11" s="89"/>
+      <c r="I11" s="89"/>
+      <c r="J11" s="89"/>
+      <c r="K11" s="92"/>
+    </row>
+    <row r="12" spans="1:11" ht="12.6" customHeight="1">
+      <c r="A12" s="93" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="94"/>
+      <c r="C12" s="94"/>
+      <c r="D12" s="94"/>
+      <c r="E12" s="79"/>
+      <c r="F12" s="57"/>
+      <c r="G12" s="29"/>
+      <c r="H12" s="58"/>
+      <c r="I12" s="29"/>
+      <c r="J12" s="115"/>
+      <c r="K12" s="116"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="96"/>
-      <c r="B13" s="90"/>
-      <c r="C13" s="90"/>
-      <c r="D13" s="90"/>
-      <c r="E13" s="97"/>
+      <c r="A13" s="95"/>
+      <c r="B13" s="70"/>
+      <c r="C13" s="70"/>
+      <c r="D13" s="70"/>
+      <c r="E13" s="71"/>
       <c r="F13" s="27"/>
-      <c r="G13" s="61"/>
-      <c r="H13" s="62"/>
+      <c r="G13" s="59"/>
+      <c r="H13" s="60"/>
       <c r="I13" s="2"/>
-      <c r="J13" s="135"/>
-      <c r="K13" s="136"/>
+      <c r="J13" s="115"/>
+      <c r="K13" s="116"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="118" t="str">
+      <c r="A14" s="96" t="str">
         <f>"*"&amp;A12&amp;"*"</f>
         <v>*GOFEMM20052025002*</v>
       </c>
-      <c r="B14" s="119"/>
-      <c r="C14" s="119"/>
-      <c r="D14" s="119"/>
-      <c r="E14" s="120"/>
+      <c r="B14" s="97"/>
+      <c r="C14" s="97"/>
+      <c r="D14" s="97"/>
+      <c r="E14" s="98"/>
       <c r="F14" s="27"/>
-      <c r="G14" s="62"/>
-      <c r="H14" s="62"/>
+      <c r="G14" s="60"/>
+      <c r="H14" s="60"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="135"/>
-      <c r="K14" s="136"/>
+      <c r="J14" s="115"/>
+      <c r="K14" s="116"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="121"/>
-      <c r="B15" s="122"/>
-      <c r="C15" s="122"/>
-      <c r="D15" s="122"/>
-      <c r="E15" s="123"/>
+      <c r="A15" s="99"/>
+      <c r="B15" s="100"/>
+      <c r="C15" s="100"/>
+      <c r="D15" s="100"/>
+      <c r="E15" s="101"/>
       <c r="F15" s="27"/>
-      <c r="G15" s="62"/>
-      <c r="H15" s="62"/>
+      <c r="G15" s="60"/>
+      <c r="H15" s="60"/>
       <c r="I15" s="2"/>
-      <c r="J15" s="135"/>
-      <c r="K15" s="136"/>
+      <c r="J15" s="115"/>
+      <c r="K15" s="116"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="121"/>
-      <c r="B16" s="122"/>
-      <c r="C16" s="122"/>
-      <c r="D16" s="122"/>
-      <c r="E16" s="123"/>
+      <c r="A16" s="99"/>
+      <c r="B16" s="100"/>
+      <c r="C16" s="100"/>
+      <c r="D16" s="100"/>
+      <c r="E16" s="101"/>
       <c r="F16" s="8"/>
-      <c r="G16" s="62"/>
-      <c r="H16" s="62"/>
+      <c r="G16" s="60"/>
+      <c r="H16" s="60"/>
       <c r="I16" s="2"/>
-      <c r="J16" s="135"/>
-      <c r="K16" s="136"/>
+      <c r="J16" s="115"/>
+      <c r="K16" s="116"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="121"/>
-      <c r="B17" s="122"/>
-      <c r="C17" s="122"/>
-      <c r="D17" s="122"/>
-      <c r="E17" s="123"/>
+      <c r="A17" s="99"/>
+      <c r="B17" s="100"/>
+      <c r="C17" s="100"/>
+      <c r="D17" s="100"/>
+      <c r="E17" s="101"/>
       <c r="F17" s="27"/>
-      <c r="G17" s="62"/>
-      <c r="H17" s="62"/>
+      <c r="G17" s="60"/>
+      <c r="H17" s="60"/>
       <c r="I17" s="2"/>
-      <c r="J17" s="135"/>
-      <c r="K17" s="136"/>
+      <c r="J17" s="115"/>
+      <c r="K17" s="116"/>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="121"/>
-      <c r="B18" s="122"/>
-      <c r="C18" s="122"/>
-      <c r="D18" s="122"/>
-      <c r="E18" s="123"/>
+      <c r="A18" s="99"/>
+      <c r="B18" s="100"/>
+      <c r="C18" s="100"/>
+      <c r="D18" s="100"/>
+      <c r="E18" s="101"/>
       <c r="F18" s="27"/>
-      <c r="G18" s="62"/>
-      <c r="H18" s="62"/>
+      <c r="G18" s="60"/>
+      <c r="H18" s="60"/>
       <c r="I18" s="8"/>
-      <c r="J18" s="135"/>
-      <c r="K18" s="136"/>
+      <c r="J18" s="115"/>
+      <c r="K18" s="116"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="124"/>
-      <c r="B19" s="125"/>
-      <c r="C19" s="125"/>
-      <c r="D19" s="125"/>
-      <c r="E19" s="126"/>
-      <c r="F19" s="63"/>
-      <c r="G19" s="62"/>
-      <c r="H19" s="62"/>
+      <c r="A19" s="102"/>
+      <c r="B19" s="103"/>
+      <c r="C19" s="103"/>
+      <c r="D19" s="103"/>
+      <c r="E19" s="104"/>
+      <c r="F19" s="61"/>
+      <c r="G19" s="60"/>
+      <c r="H19" s="60"/>
       <c r="I19" s="27"/>
-      <c r="J19" s="135"/>
-      <c r="K19" s="136"/>
+      <c r="J19" s="115"/>
+      <c r="K19" s="116"/>
     </row>
     <row r="20" spans="1:11">
-      <c r="A20" s="32"/>
+      <c r="A20" s="30"/>
       <c r="B20" s="22"/>
       <c r="C20" s="22"/>
       <c r="D20" s="22"/>
       <c r="E20" s="22"/>
-      <c r="F20" s="63"/>
-      <c r="G20" s="64"/>
-      <c r="H20" s="62"/>
+      <c r="F20" s="61"/>
+      <c r="G20" s="62"/>
+      <c r="H20" s="60"/>
       <c r="I20" s="27"/>
-      <c r="J20" s="135"/>
-      <c r="K20" s="136"/>
+      <c r="J20" s="115"/>
+      <c r="K20" s="116"/>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="32"/>
+      <c r="A21" s="30"/>
       <c r="B21" s="22"/>
       <c r="C21" s="22"/>
       <c r="D21" s="22"/>
-      <c r="E21" s="35"/>
-      <c r="F21" s="63"/>
-      <c r="G21" s="62"/>
-      <c r="H21" s="62"/>
+      <c r="E21" s="33"/>
+      <c r="F21" s="61"/>
+      <c r="G21" s="60"/>
+      <c r="H21" s="60"/>
       <c r="I21" s="27"/>
-      <c r="J21" s="135"/>
-      <c r="K21" s="136"/>
+      <c r="J21" s="115"/>
+      <c r="K21" s="116"/>
     </row>
     <row r="22" spans="1:11">
-      <c r="A22" s="32"/>
+      <c r="A22" s="30"/>
       <c r="B22" s="22"/>
       <c r="C22" s="22"/>
       <c r="D22" s="22"/>
-      <c r="E22" s="35"/>
-      <c r="F22" s="63"/>
-      <c r="G22" s="62"/>
-      <c r="H22" s="62"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="61"/>
+      <c r="G22" s="60"/>
+      <c r="H22" s="60"/>
       <c r="I22" s="27"/>
-      <c r="J22" s="135"/>
-      <c r="K22" s="136"/>
+      <c r="J22" s="115"/>
+      <c r="K22" s="116"/>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="32"/>
+      <c r="A23" s="30"/>
       <c r="B23" s="22"/>
       <c r="C23" s="22"/>
       <c r="D23" s="22"/>
@@ -2879,11 +2867,11 @@
       <c r="G23" s="27"/>
       <c r="H23" s="27"/>
       <c r="I23" s="27"/>
-      <c r="J23" s="135"/>
-      <c r="K23" s="136"/>
+      <c r="J23" s="115"/>
+      <c r="K23" s="116"/>
     </row>
     <row r="24" spans="1:11">
-      <c r="A24" s="32"/>
+      <c r="A24" s="30"/>
       <c r="B24" s="22"/>
       <c r="C24" s="22"/>
       <c r="D24" s="22"/>
@@ -2892,187 +2880,164 @@
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
-      <c r="J24" s="135"/>
-      <c r="K24" s="136"/>
+      <c r="J24" s="115"/>
+      <c r="K24" s="116"/>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="32"/>
+      <c r="A25" s="30"/>
       <c r="B25" s="22"/>
       <c r="C25" s="22"/>
       <c r="D25" s="22"/>
       <c r="E25" s="22"/>
-      <c r="F25" s="65"/>
+      <c r="F25" s="63"/>
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
       <c r="I25" s="9"/>
-      <c r="J25" s="135"/>
-      <c r="K25" s="136"/>
+      <c r="J25" s="115"/>
+      <c r="K25" s="116"/>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="105"/>
-      <c r="B26" s="94"/>
-      <c r="C26" s="94"/>
-      <c r="D26" s="94"/>
-      <c r="E26" s="106"/>
-      <c r="F26" s="66"/>
-      <c r="G26" s="67"/>
+      <c r="A26" s="81"/>
+      <c r="B26" s="78"/>
+      <c r="C26" s="78"/>
+      <c r="D26" s="78"/>
+      <c r="E26" s="82"/>
+      <c r="F26" s="64"/>
+      <c r="G26" s="65"/>
       <c r="H26" s="8"/>
       <c r="I26" s="9"/>
-      <c r="J26" s="135"/>
-      <c r="K26" s="136"/>
+      <c r="J26" s="115"/>
+      <c r="K26" s="116"/>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="94"/>
-      <c r="B27" s="94"/>
-      <c r="C27" s="94"/>
-      <c r="D27" s="94"/>
-      <c r="E27" s="106"/>
-      <c r="F27" s="68"/>
-      <c r="G27" s="67"/>
+      <c r="A27" s="78"/>
+      <c r="B27" s="78"/>
+      <c r="C27" s="78"/>
+      <c r="D27" s="78"/>
+      <c r="E27" s="82"/>
+      <c r="F27" s="66"/>
+      <c r="G27" s="65"/>
       <c r="H27" s="8"/>
       <c r="I27" s="9"/>
-      <c r="J27" s="135"/>
-      <c r="K27" s="136"/>
+      <c r="J27" s="115"/>
+      <c r="K27" s="116"/>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="94"/>
-      <c r="B28" s="94"/>
-      <c r="C28" s="94"/>
-      <c r="D28" s="94"/>
-      <c r="E28" s="106"/>
-      <c r="F28" s="68"/>
-      <c r="G28" s="67"/>
+      <c r="A28" s="78"/>
+      <c r="B28" s="78"/>
+      <c r="C28" s="78"/>
+      <c r="D28" s="78"/>
+      <c r="E28" s="82"/>
+      <c r="F28" s="66"/>
+      <c r="G28" s="65"/>
       <c r="H28" s="8"/>
       <c r="I28" s="9"/>
-      <c r="J28" s="135"/>
-      <c r="K28" s="136"/>
+      <c r="J28" s="115"/>
+      <c r="K28" s="116"/>
     </row>
     <row r="29" spans="1:11">
-      <c r="A29" s="94"/>
-      <c r="B29" s="94"/>
-      <c r="C29" s="94"/>
-      <c r="D29" s="94"/>
-      <c r="E29" s="106"/>
-      <c r="F29" s="69"/>
-      <c r="G29" s="70"/>
-      <c r="H29" s="65"/>
+      <c r="A29" s="78"/>
+      <c r="B29" s="78"/>
+      <c r="C29" s="78"/>
+      <c r="D29" s="78"/>
+      <c r="E29" s="82"/>
+      <c r="F29" s="67"/>
+      <c r="G29" s="68"/>
+      <c r="H29" s="63"/>
       <c r="I29" s="23"/>
-      <c r="J29" s="135"/>
-      <c r="K29" s="136"/>
+      <c r="J29" s="115"/>
+      <c r="K29" s="116"/>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="107"/>
-      <c r="B30" s="107"/>
-      <c r="C30" s="107"/>
-      <c r="D30" s="107"/>
-      <c r="E30" s="108"/>
-      <c r="F30" s="49"/>
+      <c r="A30" s="83"/>
+      <c r="B30" s="83"/>
+      <c r="C30" s="83"/>
+      <c r="D30" s="83"/>
+      <c r="E30" s="84"/>
+      <c r="F30" s="47"/>
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
-      <c r="J30" s="135"/>
-      <c r="K30" s="136"/>
-    </row>
-    <row r="31" spans="1:11" ht="15.5">
-      <c r="A31" s="137" t="s">
+      <c r="J30" s="115"/>
+      <c r="K30" s="116"/>
+    </row>
+    <row r="31" spans="1:11" ht="15.75">
+      <c r="A31" s="69" t="s">
+        <v>16</v>
+      </c>
+      <c r="B31" s="70"/>
+      <c r="C31" s="71"/>
+      <c r="D31" s="48"/>
+      <c r="E31" s="72"/>
+      <c r="F31" s="73"/>
+      <c r="G31" s="73"/>
+      <c r="H31" s="73"/>
+      <c r="I31" s="74" t="s">
         <v>17</v>
       </c>
-      <c r="B31" s="90"/>
-      <c r="C31" s="97"/>
-      <c r="D31" s="50"/>
-      <c r="E31" s="138"/>
-      <c r="F31" s="139"/>
-      <c r="G31" s="139"/>
-      <c r="H31" s="139"/>
-      <c r="I31" s="140" t="s">
-        <v>18</v>
-      </c>
-      <c r="J31" s="141"/>
-      <c r="K31" s="142"/>
+      <c r="J31" s="75"/>
+      <c r="K31" s="76"/>
     </row>
     <row r="32" spans="1:11">
-      <c r="A32" s="37"/>
-      <c r="B32" s="54"/>
+      <c r="A32" s="35"/>
+      <c r="B32" s="52"/>
       <c r="C32" s="4"/>
-      <c r="D32" s="38"/>
+      <c r="D32" s="36"/>
       <c r="E32" s="3"/>
-      <c r="F32" s="143"/>
-      <c r="G32" s="94"/>
-      <c r="H32" s="110"/>
-      <c r="I32" s="143"/>
-      <c r="J32" s="94"/>
-      <c r="K32" s="144"/>
+      <c r="F32" s="77"/>
+      <c r="G32" s="78"/>
+      <c r="H32" s="79"/>
+      <c r="I32" s="77"/>
+      <c r="J32" s="78"/>
+      <c r="K32" s="80"/>
     </row>
     <row r="33" spans="1:11">
-      <c r="A33" s="39"/>
-      <c r="B33" s="45"/>
-      <c r="C33" s="41"/>
-      <c r="D33" s="42"/>
-      <c r="E33" s="43"/>
-      <c r="F33" s="40"/>
-      <c r="G33" s="40"/>
-      <c r="H33" s="44"/>
-      <c r="I33" s="40"/>
-      <c r="J33" s="40"/>
-      <c r="K33" s="45"/>
-    </row>
-    <row r="34" spans="1:11">
-      <c r="A34" s="30"/>
-      <c r="B34" s="30"/>
-      <c r="C34" s="30"/>
-      <c r="D34" s="30"/>
-      <c r="E34" s="30"/>
-    </row>
-    <row r="35" spans="1:11">
-      <c r="A35" s="30"/>
-      <c r="B35" s="30"/>
-      <c r="C35" s="30"/>
-      <c r="D35" s="30"/>
-      <c r="E35" s="30"/>
-    </row>
-    <row r="36" spans="1:11">
-      <c r="A36" s="30"/>
-    </row>
-    <row r="37" spans="1:11">
-      <c r="A37" s="30"/>
-    </row>
-    <row r="38" spans="1:11">
-      <c r="A38" s="30"/>
-    </row>
-    <row r="45" spans="1:11" ht="15.5">
+      <c r="A33" s="37"/>
+      <c r="B33" s="43"/>
+      <c r="C33" s="39"/>
+      <c r="D33" s="40"/>
+      <c r="E33" s="41"/>
+      <c r="F33" s="38"/>
+      <c r="G33" s="38"/>
+      <c r="H33" s="42"/>
+      <c r="I33" s="38"/>
+      <c r="J33" s="38"/>
+      <c r="K33" s="43"/>
+    </row>
+    <row r="45" spans="1:11" ht="15.75">
       <c r="J45" s="5"/>
     </row>
-    <row r="46" spans="1:11" ht="13">
+    <row r="46" spans="1:11">
       <c r="J46" s="6"/>
     </row>
-    <row r="47" spans="1:11" ht="15.5">
+    <row r="47" spans="1:11" ht="15.75">
       <c r="J47" s="5"/>
     </row>
-    <row r="48" spans="1:11" ht="13">
+    <row r="48" spans="1:11">
       <c r="J48" s="6"/>
     </row>
-    <row r="49" spans="10:10" ht="15.5">
+    <row r="49" spans="10:10" ht="15.75">
       <c r="J49" s="5"/>
     </row>
-    <row r="50" spans="10:10" ht="13">
+    <row r="50" spans="10:10">
       <c r="J50" s="6"/>
     </row>
-    <row r="51" spans="10:10" ht="15.5">
+    <row r="51" spans="10:10" ht="15.75">
       <c r="J51" s="5"/>
     </row>
-    <row r="52" spans="10:10" ht="13">
+    <row r="52" spans="10:10">
       <c r="J52" s="6"/>
     </row>
-    <row r="53" spans="10:10" ht="15.5">
+    <row r="53" spans="10:10" ht="15.75">
       <c r="J53" s="5"/>
     </row>
-    <row r="54" spans="10:10" ht="13">
+    <row r="54" spans="10:10">
       <c r="J54" s="6"/>
     </row>
-    <row r="55" spans="10:10" ht="15.5">
+    <row r="55" spans="10:10" ht="15.75">
       <c r="J55" s="5"/>
     </row>
-    <row r="56" spans="10:10" ht="13">
+    <row r="56" spans="10:10">
       <c r="J56" s="6"/>
     </row>
     <row r="67" spans="11:11">
@@ -3080,16 +3045,27 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="A26:E30"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="E31:H31"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="E1:G2"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="J4:K4"/>
     <mergeCell ref="A14:E19"/>
     <mergeCell ref="A5:C6"/>
     <mergeCell ref="E5:G5"/>
@@ -3106,46 +3082,35 @@
     <mergeCell ref="A11:E11"/>
     <mergeCell ref="F11:K11"/>
     <mergeCell ref="A12:E13"/>
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="E1:G2"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="A26:E30"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="E31:H31"/>
+    <mergeCell ref="I31:K31"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J30:K30"/>
   </mergeCells>
-  <conditionalFormatting sqref="F12:G15 I12 F17:F22 G17:G19 G21:G22">
-    <cfRule type="expression" dxfId="3" priority="1">
-      <formula>COUNTIF($F12:$G35,F12)&gt;1</formula>
+  <conditionalFormatting sqref="G12:G19 F12:F24 I12:I24 H13:H24 G21:G25">
+    <cfRule type="expression" dxfId="3" priority="4">
+      <formula>COUNTIF($F12:$K27,F12)&gt;1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G19 H19:I21 G21">
+    <cfRule type="expression" dxfId="2" priority="3">
+      <formula>COUNTIF($F12:$K27,G19)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G22:I23">
-    <cfRule type="expression" dxfId="2" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>COUNTIF($F16:$K31,G22)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G19 H19:I21 G21">
-    <cfRule type="expression" dxfId="1" priority="3">
-      <formula>COUNTIF($F12:$K27,G19)&gt;1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F12:F24 G12:G19 I12:I24 H13:H24 G21:G25">
-    <cfRule type="expression" dxfId="0" priority="4">
-      <formula>COUNTIF($F12:$K27,F12)&gt;1</formula>
+  <conditionalFormatting sqref="I12 F12:G15 G17:G19 F17:F22 G21:G22">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>COUNTIF($F12:$G35,F12)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>